<commit_message>
Tenant form upgraded with dropdowns and default Tenant ID
</commit_message>
<xml_diff>
--- a/Tenant_Manager.xlsx
+++ b/Tenant_Manager.xlsx
@@ -1930,7 +1930,11 @@
           <t>Tenant ID</t>
         </is>
       </c>
-      <c r="D6" s="56" t="n"/>
+      <c r="D6" s="56" t="inlineStr">
+        <is>
+          <t>T-001</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="B7" s="55" t="inlineStr">

</xml_diff>

<commit_message>
Added emergency contacts to form and tenant register
</commit_message>
<xml_diff>
--- a/Tenant_Manager.xlsx
+++ b/Tenant_Manager.xlsx
@@ -278,7 +278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -475,6 +475,9 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -2189,7 +2192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R53"/>
+  <dimension ref="A1:V53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2210,6 +2213,10 @@
     <col width="14" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2317,6 +2324,26 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="S3" s="62" t="inlineStr">
+        <is>
+          <t>Emergency Contact</t>
+        </is>
+      </c>
+      <c r="T3" s="62" t="inlineStr">
+        <is>
+          <t>Relationship</t>
+        </is>
+      </c>
+      <c r="U3" s="62" t="inlineStr">
+        <is>
+          <t>Emergency Phone</t>
+        </is>
+      </c>
+      <c r="V3" s="62" t="inlineStr">
+        <is>
+          <t>Residential Address</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="63" t="inlineStr">
@@ -2402,27 +2429,31 @@
         <f>IFERROR(IF(B4="","Vacant",IF(Q4&lt;0,"Expired",IF(Q4&lt;=30,"Expiring Soon",IF(Q4&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S4" s="69" t="n"/>
+      <c r="T4" s="69" t="n"/>
+      <c r="U4" s="69" t="n"/>
+      <c r="V4" s="69" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="69" t="n"/>
-      <c r="B5" s="69" t="n"/>
-      <c r="C5" s="69" t="n"/>
-      <c r="D5" s="69" t="n"/>
-      <c r="E5" s="69" t="n"/>
-      <c r="F5" s="69" t="n"/>
-      <c r="G5" s="69" t="n"/>
-      <c r="H5" s="69" t="n"/>
-      <c r="I5" s="70" t="n"/>
-      <c r="J5" s="70" t="n"/>
+      <c r="A5" s="70" t="n"/>
+      <c r="B5" s="70" t="n"/>
+      <c r="C5" s="70" t="n"/>
+      <c r="D5" s="70" t="n"/>
+      <c r="E5" s="70" t="n"/>
+      <c r="F5" s="70" t="n"/>
+      <c r="G5" s="70" t="n"/>
+      <c r="H5" s="70" t="n"/>
+      <c r="I5" s="71" t="n"/>
+      <c r="J5" s="71" t="n"/>
       <c r="K5" s="65">
         <f>IFERROR(DATEDIF(I5,J5,"M"),"")</f>
         <v/>
       </c>
-      <c r="L5" s="71" t="n"/>
-      <c r="M5" s="69" t="n"/>
-      <c r="N5" s="69" t="n"/>
-      <c r="O5" s="71" t="n"/>
-      <c r="P5" s="69" t="n"/>
+      <c r="L5" s="72" t="n"/>
+      <c r="M5" s="70" t="n"/>
+      <c r="N5" s="70" t="n"/>
+      <c r="O5" s="72" t="n"/>
+      <c r="P5" s="70" t="n"/>
       <c r="Q5" s="67">
         <f>IFERROR(IF(J5="","",J5-TODAY()),"")</f>
         <v/>
@@ -2431,27 +2462,31 @@
         <f>IFERROR(IF(B5="","Vacant",IF(Q5&lt;0,"Expired",IF(Q5&lt;=30,"Expiring Soon",IF(Q5&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S5" s="69" t="n"/>
+      <c r="T5" s="69" t="n"/>
+      <c r="U5" s="69" t="n"/>
+      <c r="V5" s="69" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="72" t="n"/>
-      <c r="B6" s="72" t="n"/>
-      <c r="C6" s="72" t="n"/>
-      <c r="D6" s="72" t="n"/>
-      <c r="E6" s="72" t="n"/>
-      <c r="F6" s="72" t="n"/>
-      <c r="G6" s="72" t="n"/>
-      <c r="H6" s="72" t="n"/>
-      <c r="I6" s="73" t="n"/>
-      <c r="J6" s="73" t="n"/>
+      <c r="A6" s="73" t="n"/>
+      <c r="B6" s="73" t="n"/>
+      <c r="C6" s="73" t="n"/>
+      <c r="D6" s="73" t="n"/>
+      <c r="E6" s="73" t="n"/>
+      <c r="F6" s="73" t="n"/>
+      <c r="G6" s="73" t="n"/>
+      <c r="H6" s="73" t="n"/>
+      <c r="I6" s="74" t="n"/>
+      <c r="J6" s="74" t="n"/>
       <c r="K6" s="65">
         <f>IFERROR(DATEDIF(I6,J6,"M"),"")</f>
         <v/>
       </c>
-      <c r="L6" s="74" t="n"/>
-      <c r="M6" s="72" t="n"/>
-      <c r="N6" s="72" t="n"/>
-      <c r="O6" s="74" t="n"/>
-      <c r="P6" s="72" t="n"/>
+      <c r="L6" s="75" t="n"/>
+      <c r="M6" s="73" t="n"/>
+      <c r="N6" s="73" t="n"/>
+      <c r="O6" s="75" t="n"/>
+      <c r="P6" s="73" t="n"/>
       <c r="Q6" s="67">
         <f>IFERROR(IF(J6="","",J6-TODAY()),"")</f>
         <v/>
@@ -2460,27 +2495,31 @@
         <f>IFERROR(IF(B6="","Vacant",IF(Q6&lt;0,"Expired",IF(Q6&lt;=30,"Expiring Soon",IF(Q6&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S6" s="69" t="n"/>
+      <c r="T6" s="69" t="n"/>
+      <c r="U6" s="69" t="n"/>
+      <c r="V6" s="69" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="69" t="n"/>
-      <c r="B7" s="69" t="n"/>
-      <c r="C7" s="69" t="n"/>
-      <c r="D7" s="69" t="n"/>
-      <c r="E7" s="69" t="n"/>
-      <c r="F7" s="69" t="n"/>
-      <c r="G7" s="69" t="n"/>
-      <c r="H7" s="69" t="n"/>
-      <c r="I7" s="70" t="n"/>
-      <c r="J7" s="70" t="n"/>
+      <c r="A7" s="70" t="n"/>
+      <c r="B7" s="70" t="n"/>
+      <c r="C7" s="70" t="n"/>
+      <c r="D7" s="70" t="n"/>
+      <c r="E7" s="70" t="n"/>
+      <c r="F7" s="70" t="n"/>
+      <c r="G7" s="70" t="n"/>
+      <c r="H7" s="70" t="n"/>
+      <c r="I7" s="71" t="n"/>
+      <c r="J7" s="71" t="n"/>
       <c r="K7" s="65">
         <f>IFERROR(DATEDIF(I7,J7,"M"),"")</f>
         <v/>
       </c>
-      <c r="L7" s="71" t="n"/>
-      <c r="M7" s="69" t="n"/>
-      <c r="N7" s="69" t="n"/>
-      <c r="O7" s="71" t="n"/>
-      <c r="P7" s="69" t="n"/>
+      <c r="L7" s="72" t="n"/>
+      <c r="M7" s="70" t="n"/>
+      <c r="N7" s="70" t="n"/>
+      <c r="O7" s="72" t="n"/>
+      <c r="P7" s="70" t="n"/>
       <c r="Q7" s="67">
         <f>IFERROR(IF(J7="","",J7-TODAY()),"")</f>
         <v/>
@@ -2489,27 +2528,31 @@
         <f>IFERROR(IF(B7="","Vacant",IF(Q7&lt;0,"Expired",IF(Q7&lt;=30,"Expiring Soon",IF(Q7&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S7" s="69" t="n"/>
+      <c r="T7" s="69" t="n"/>
+      <c r="U7" s="69" t="n"/>
+      <c r="V7" s="69" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="72" t="n"/>
-      <c r="B8" s="72" t="n"/>
-      <c r="C8" s="72" t="n"/>
-      <c r="D8" s="72" t="n"/>
-      <c r="E8" s="72" t="n"/>
-      <c r="F8" s="72" t="n"/>
-      <c r="G8" s="72" t="n"/>
-      <c r="H8" s="72" t="n"/>
-      <c r="I8" s="73" t="n"/>
-      <c r="J8" s="73" t="n"/>
+      <c r="A8" s="73" t="n"/>
+      <c r="B8" s="73" t="n"/>
+      <c r="C8" s="73" t="n"/>
+      <c r="D8" s="73" t="n"/>
+      <c r="E8" s="73" t="n"/>
+      <c r="F8" s="73" t="n"/>
+      <c r="G8" s="73" t="n"/>
+      <c r="H8" s="73" t="n"/>
+      <c r="I8" s="74" t="n"/>
+      <c r="J8" s="74" t="n"/>
       <c r="K8" s="65">
         <f>IFERROR(DATEDIF(I8,J8,"M"),"")</f>
         <v/>
       </c>
-      <c r="L8" s="74" t="n"/>
-      <c r="M8" s="72" t="n"/>
-      <c r="N8" s="72" t="n"/>
-      <c r="O8" s="74" t="n"/>
-      <c r="P8" s="72" t="n"/>
+      <c r="L8" s="75" t="n"/>
+      <c r="M8" s="73" t="n"/>
+      <c r="N8" s="73" t="n"/>
+      <c r="O8" s="75" t="n"/>
+      <c r="P8" s="73" t="n"/>
       <c r="Q8" s="67">
         <f>IFERROR(IF(J8="","",J8-TODAY()),"")</f>
         <v/>
@@ -2518,27 +2561,31 @@
         <f>IFERROR(IF(B8="","Vacant",IF(Q8&lt;0,"Expired",IF(Q8&lt;=30,"Expiring Soon",IF(Q8&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S8" s="69" t="n"/>
+      <c r="T8" s="69" t="n"/>
+      <c r="U8" s="69" t="n"/>
+      <c r="V8" s="69" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="69" t="n"/>
-      <c r="B9" s="69" t="n"/>
-      <c r="C9" s="69" t="n"/>
-      <c r="D9" s="69" t="n"/>
-      <c r="E9" s="69" t="n"/>
-      <c r="F9" s="69" t="n"/>
-      <c r="G9" s="69" t="n"/>
-      <c r="H9" s="69" t="n"/>
-      <c r="I9" s="70" t="n"/>
-      <c r="J9" s="70" t="n"/>
+      <c r="A9" s="70" t="n"/>
+      <c r="B9" s="70" t="n"/>
+      <c r="C9" s="70" t="n"/>
+      <c r="D9" s="70" t="n"/>
+      <c r="E9" s="70" t="n"/>
+      <c r="F9" s="70" t="n"/>
+      <c r="G9" s="70" t="n"/>
+      <c r="H9" s="70" t="n"/>
+      <c r="I9" s="71" t="n"/>
+      <c r="J9" s="71" t="n"/>
       <c r="K9" s="65">
         <f>IFERROR(DATEDIF(I9,J9,"M"),"")</f>
         <v/>
       </c>
-      <c r="L9" s="71" t="n"/>
-      <c r="M9" s="69" t="n"/>
-      <c r="N9" s="69" t="n"/>
-      <c r="O9" s="71" t="n"/>
-      <c r="P9" s="69" t="n"/>
+      <c r="L9" s="72" t="n"/>
+      <c r="M9" s="70" t="n"/>
+      <c r="N9" s="70" t="n"/>
+      <c r="O9" s="72" t="n"/>
+      <c r="P9" s="70" t="n"/>
       <c r="Q9" s="67">
         <f>IFERROR(IF(J9="","",J9-TODAY()),"")</f>
         <v/>
@@ -2547,27 +2594,31 @@
         <f>IFERROR(IF(B9="","Vacant",IF(Q9&lt;0,"Expired",IF(Q9&lt;=30,"Expiring Soon",IF(Q9&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S9" s="69" t="n"/>
+      <c r="T9" s="69" t="n"/>
+      <c r="U9" s="69" t="n"/>
+      <c r="V9" s="69" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="72" t="n"/>
-      <c r="B10" s="72" t="n"/>
-      <c r="C10" s="72" t="n"/>
-      <c r="D10" s="72" t="n"/>
-      <c r="E10" s="72" t="n"/>
-      <c r="F10" s="72" t="n"/>
-      <c r="G10" s="72" t="n"/>
-      <c r="H10" s="72" t="n"/>
-      <c r="I10" s="73" t="n"/>
-      <c r="J10" s="73" t="n"/>
+      <c r="A10" s="73" t="n"/>
+      <c r="B10" s="73" t="n"/>
+      <c r="C10" s="73" t="n"/>
+      <c r="D10" s="73" t="n"/>
+      <c r="E10" s="73" t="n"/>
+      <c r="F10" s="73" t="n"/>
+      <c r="G10" s="73" t="n"/>
+      <c r="H10" s="73" t="n"/>
+      <c r="I10" s="74" t="n"/>
+      <c r="J10" s="74" t="n"/>
       <c r="K10" s="65">
         <f>IFERROR(DATEDIF(I10,J10,"M"),"")</f>
         <v/>
       </c>
-      <c r="L10" s="74" t="n"/>
-      <c r="M10" s="72" t="n"/>
-      <c r="N10" s="72" t="n"/>
-      <c r="O10" s="74" t="n"/>
-      <c r="P10" s="72" t="n"/>
+      <c r="L10" s="75" t="n"/>
+      <c r="M10" s="73" t="n"/>
+      <c r="N10" s="73" t="n"/>
+      <c r="O10" s="75" t="n"/>
+      <c r="P10" s="73" t="n"/>
       <c r="Q10" s="67">
         <f>IFERROR(IF(J10="","",J10-TODAY()),"")</f>
         <v/>
@@ -2576,27 +2627,31 @@
         <f>IFERROR(IF(B10="","Vacant",IF(Q10&lt;0,"Expired",IF(Q10&lt;=30,"Expiring Soon",IF(Q10&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S10" s="69" t="n"/>
+      <c r="T10" s="69" t="n"/>
+      <c r="U10" s="69" t="n"/>
+      <c r="V10" s="69" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="69" t="n"/>
-      <c r="B11" s="69" t="n"/>
-      <c r="C11" s="69" t="n"/>
-      <c r="D11" s="69" t="n"/>
-      <c r="E11" s="69" t="n"/>
-      <c r="F11" s="69" t="n"/>
-      <c r="G11" s="69" t="n"/>
-      <c r="H11" s="69" t="n"/>
-      <c r="I11" s="70" t="n"/>
-      <c r="J11" s="70" t="n"/>
+      <c r="A11" s="70" t="n"/>
+      <c r="B11" s="70" t="n"/>
+      <c r="C11" s="70" t="n"/>
+      <c r="D11" s="70" t="n"/>
+      <c r="E11" s="70" t="n"/>
+      <c r="F11" s="70" t="n"/>
+      <c r="G11" s="70" t="n"/>
+      <c r="H11" s="70" t="n"/>
+      <c r="I11" s="71" t="n"/>
+      <c r="J11" s="71" t="n"/>
       <c r="K11" s="65">
         <f>IFERROR(DATEDIF(I11,J11,"M"),"")</f>
         <v/>
       </c>
-      <c r="L11" s="71" t="n"/>
-      <c r="M11" s="69" t="n"/>
-      <c r="N11" s="69" t="n"/>
-      <c r="O11" s="71" t="n"/>
-      <c r="P11" s="69" t="n"/>
+      <c r="L11" s="72" t="n"/>
+      <c r="M11" s="70" t="n"/>
+      <c r="N11" s="70" t="n"/>
+      <c r="O11" s="72" t="n"/>
+      <c r="P11" s="70" t="n"/>
       <c r="Q11" s="67">
         <f>IFERROR(IF(J11="","",J11-TODAY()),"")</f>
         <v/>
@@ -2605,27 +2660,31 @@
         <f>IFERROR(IF(B11="","Vacant",IF(Q11&lt;0,"Expired",IF(Q11&lt;=30,"Expiring Soon",IF(Q11&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S11" s="69" t="n"/>
+      <c r="T11" s="69" t="n"/>
+      <c r="U11" s="69" t="n"/>
+      <c r="V11" s="69" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="72" t="n"/>
-      <c r="B12" s="72" t="n"/>
-      <c r="C12" s="72" t="n"/>
-      <c r="D12" s="72" t="n"/>
-      <c r="E12" s="72" t="n"/>
-      <c r="F12" s="72" t="n"/>
-      <c r="G12" s="72" t="n"/>
-      <c r="H12" s="72" t="n"/>
-      <c r="I12" s="73" t="n"/>
-      <c r="J12" s="73" t="n"/>
+      <c r="A12" s="73" t="n"/>
+      <c r="B12" s="73" t="n"/>
+      <c r="C12" s="73" t="n"/>
+      <c r="D12" s="73" t="n"/>
+      <c r="E12" s="73" t="n"/>
+      <c r="F12" s="73" t="n"/>
+      <c r="G12" s="73" t="n"/>
+      <c r="H12" s="73" t="n"/>
+      <c r="I12" s="74" t="n"/>
+      <c r="J12" s="74" t="n"/>
       <c r="K12" s="65">
         <f>IFERROR(DATEDIF(I12,J12,"M"),"")</f>
         <v/>
       </c>
-      <c r="L12" s="74" t="n"/>
-      <c r="M12" s="72" t="n"/>
-      <c r="N12" s="72" t="n"/>
-      <c r="O12" s="74" t="n"/>
-      <c r="P12" s="72" t="n"/>
+      <c r="L12" s="75" t="n"/>
+      <c r="M12" s="73" t="n"/>
+      <c r="N12" s="73" t="n"/>
+      <c r="O12" s="75" t="n"/>
+      <c r="P12" s="73" t="n"/>
       <c r="Q12" s="67">
         <f>IFERROR(IF(J12="","",J12-TODAY()),"")</f>
         <v/>
@@ -2634,27 +2693,31 @@
         <f>IFERROR(IF(B12="","Vacant",IF(Q12&lt;0,"Expired",IF(Q12&lt;=30,"Expiring Soon",IF(Q12&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S12" s="69" t="n"/>
+      <c r="T12" s="69" t="n"/>
+      <c r="U12" s="69" t="n"/>
+      <c r="V12" s="69" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="69" t="n"/>
-      <c r="B13" s="69" t="n"/>
-      <c r="C13" s="69" t="n"/>
-      <c r="D13" s="69" t="n"/>
-      <c r="E13" s="69" t="n"/>
-      <c r="F13" s="69" t="n"/>
-      <c r="G13" s="69" t="n"/>
-      <c r="H13" s="69" t="n"/>
-      <c r="I13" s="70" t="n"/>
-      <c r="J13" s="70" t="n"/>
+      <c r="A13" s="70" t="n"/>
+      <c r="B13" s="70" t="n"/>
+      <c r="C13" s="70" t="n"/>
+      <c r="D13" s="70" t="n"/>
+      <c r="E13" s="70" t="n"/>
+      <c r="F13" s="70" t="n"/>
+      <c r="G13" s="70" t="n"/>
+      <c r="H13" s="70" t="n"/>
+      <c r="I13" s="71" t="n"/>
+      <c r="J13" s="71" t="n"/>
       <c r="K13" s="65">
         <f>IFERROR(DATEDIF(I13,J13,"M"),"")</f>
         <v/>
       </c>
-      <c r="L13" s="71" t="n"/>
-      <c r="M13" s="69" t="n"/>
-      <c r="N13" s="69" t="n"/>
-      <c r="O13" s="71" t="n"/>
-      <c r="P13" s="69" t="n"/>
+      <c r="L13" s="72" t="n"/>
+      <c r="M13" s="70" t="n"/>
+      <c r="N13" s="70" t="n"/>
+      <c r="O13" s="72" t="n"/>
+      <c r="P13" s="70" t="n"/>
       <c r="Q13" s="67">
         <f>IFERROR(IF(J13="","",J13-TODAY()),"")</f>
         <v/>
@@ -2663,27 +2726,31 @@
         <f>IFERROR(IF(B13="","Vacant",IF(Q13&lt;0,"Expired",IF(Q13&lt;=30,"Expiring Soon",IF(Q13&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S13" s="69" t="n"/>
+      <c r="T13" s="69" t="n"/>
+      <c r="U13" s="69" t="n"/>
+      <c r="V13" s="69" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="72" t="n"/>
-      <c r="B14" s="72" t="n"/>
-      <c r="C14" s="72" t="n"/>
-      <c r="D14" s="72" t="n"/>
-      <c r="E14" s="72" t="n"/>
-      <c r="F14" s="72" t="n"/>
-      <c r="G14" s="72" t="n"/>
-      <c r="H14" s="72" t="n"/>
-      <c r="I14" s="73" t="n"/>
-      <c r="J14" s="73" t="n"/>
+      <c r="A14" s="73" t="n"/>
+      <c r="B14" s="73" t="n"/>
+      <c r="C14" s="73" t="n"/>
+      <c r="D14" s="73" t="n"/>
+      <c r="E14" s="73" t="n"/>
+      <c r="F14" s="73" t="n"/>
+      <c r="G14" s="73" t="n"/>
+      <c r="H14" s="73" t="n"/>
+      <c r="I14" s="74" t="n"/>
+      <c r="J14" s="74" t="n"/>
       <c r="K14" s="65">
         <f>IFERROR(DATEDIF(I14,J14,"M"),"")</f>
         <v/>
       </c>
-      <c r="L14" s="74" t="n"/>
-      <c r="M14" s="72" t="n"/>
-      <c r="N14" s="72" t="n"/>
-      <c r="O14" s="74" t="n"/>
-      <c r="P14" s="72" t="n"/>
+      <c r="L14" s="75" t="n"/>
+      <c r="M14" s="73" t="n"/>
+      <c r="N14" s="73" t="n"/>
+      <c r="O14" s="75" t="n"/>
+      <c r="P14" s="73" t="n"/>
       <c r="Q14" s="67">
         <f>IFERROR(IF(J14="","",J14-TODAY()),"")</f>
         <v/>
@@ -2692,27 +2759,31 @@
         <f>IFERROR(IF(B14="","Vacant",IF(Q14&lt;0,"Expired",IF(Q14&lt;=30,"Expiring Soon",IF(Q14&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S14" s="69" t="n"/>
+      <c r="T14" s="69" t="n"/>
+      <c r="U14" s="69" t="n"/>
+      <c r="V14" s="69" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="69" t="n"/>
-      <c r="B15" s="69" t="n"/>
-      <c r="C15" s="69" t="n"/>
-      <c r="D15" s="69" t="n"/>
-      <c r="E15" s="69" t="n"/>
-      <c r="F15" s="69" t="n"/>
-      <c r="G15" s="69" t="n"/>
-      <c r="H15" s="69" t="n"/>
-      <c r="I15" s="70" t="n"/>
-      <c r="J15" s="70" t="n"/>
+      <c r="A15" s="70" t="n"/>
+      <c r="B15" s="70" t="n"/>
+      <c r="C15" s="70" t="n"/>
+      <c r="D15" s="70" t="n"/>
+      <c r="E15" s="70" t="n"/>
+      <c r="F15" s="70" t="n"/>
+      <c r="G15" s="70" t="n"/>
+      <c r="H15" s="70" t="n"/>
+      <c r="I15" s="71" t="n"/>
+      <c r="J15" s="71" t="n"/>
       <c r="K15" s="65">
         <f>IFERROR(DATEDIF(I15,J15,"M"),"")</f>
         <v/>
       </c>
-      <c r="L15" s="71" t="n"/>
-      <c r="M15" s="69" t="n"/>
-      <c r="N15" s="69" t="n"/>
-      <c r="O15" s="71" t="n"/>
-      <c r="P15" s="69" t="n"/>
+      <c r="L15" s="72" t="n"/>
+      <c r="M15" s="70" t="n"/>
+      <c r="N15" s="70" t="n"/>
+      <c r="O15" s="72" t="n"/>
+      <c r="P15" s="70" t="n"/>
       <c r="Q15" s="67">
         <f>IFERROR(IF(J15="","",J15-TODAY()),"")</f>
         <v/>
@@ -2721,27 +2792,31 @@
         <f>IFERROR(IF(B15="","Vacant",IF(Q15&lt;0,"Expired",IF(Q15&lt;=30,"Expiring Soon",IF(Q15&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S15" s="69" t="n"/>
+      <c r="T15" s="69" t="n"/>
+      <c r="U15" s="69" t="n"/>
+      <c r="V15" s="69" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="72" t="n"/>
-      <c r="B16" s="72" t="n"/>
-      <c r="C16" s="72" t="n"/>
-      <c r="D16" s="72" t="n"/>
-      <c r="E16" s="72" t="n"/>
-      <c r="F16" s="72" t="n"/>
-      <c r="G16" s="72" t="n"/>
-      <c r="H16" s="72" t="n"/>
-      <c r="I16" s="73" t="n"/>
-      <c r="J16" s="73" t="n"/>
+      <c r="A16" s="73" t="n"/>
+      <c r="B16" s="73" t="n"/>
+      <c r="C16" s="73" t="n"/>
+      <c r="D16" s="73" t="n"/>
+      <c r="E16" s="73" t="n"/>
+      <c r="F16" s="73" t="n"/>
+      <c r="G16" s="73" t="n"/>
+      <c r="H16" s="73" t="n"/>
+      <c r="I16" s="74" t="n"/>
+      <c r="J16" s="74" t="n"/>
       <c r="K16" s="65">
         <f>IFERROR(DATEDIF(I16,J16,"M"),"")</f>
         <v/>
       </c>
-      <c r="L16" s="74" t="n"/>
-      <c r="M16" s="72" t="n"/>
-      <c r="N16" s="72" t="n"/>
-      <c r="O16" s="74" t="n"/>
-      <c r="P16" s="72" t="n"/>
+      <c r="L16" s="75" t="n"/>
+      <c r="M16" s="73" t="n"/>
+      <c r="N16" s="73" t="n"/>
+      <c r="O16" s="75" t="n"/>
+      <c r="P16" s="73" t="n"/>
       <c r="Q16" s="67">
         <f>IFERROR(IF(J16="","",J16-TODAY()),"")</f>
         <v/>
@@ -2750,27 +2825,31 @@
         <f>IFERROR(IF(B16="","Vacant",IF(Q16&lt;0,"Expired",IF(Q16&lt;=30,"Expiring Soon",IF(Q16&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S16" s="69" t="n"/>
+      <c r="T16" s="69" t="n"/>
+      <c r="U16" s="69" t="n"/>
+      <c r="V16" s="69" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="69" t="n"/>
-      <c r="B17" s="69" t="n"/>
-      <c r="C17" s="69" t="n"/>
-      <c r="D17" s="69" t="n"/>
-      <c r="E17" s="69" t="n"/>
-      <c r="F17" s="69" t="n"/>
-      <c r="G17" s="69" t="n"/>
-      <c r="H17" s="69" t="n"/>
-      <c r="I17" s="70" t="n"/>
-      <c r="J17" s="70" t="n"/>
+      <c r="A17" s="70" t="n"/>
+      <c r="B17" s="70" t="n"/>
+      <c r="C17" s="70" t="n"/>
+      <c r="D17" s="70" t="n"/>
+      <c r="E17" s="70" t="n"/>
+      <c r="F17" s="70" t="n"/>
+      <c r="G17" s="70" t="n"/>
+      <c r="H17" s="70" t="n"/>
+      <c r="I17" s="71" t="n"/>
+      <c r="J17" s="71" t="n"/>
       <c r="K17" s="65">
         <f>IFERROR(DATEDIF(I17,J17,"M"),"")</f>
         <v/>
       </c>
-      <c r="L17" s="71" t="n"/>
-      <c r="M17" s="69" t="n"/>
-      <c r="N17" s="69" t="n"/>
-      <c r="O17" s="71" t="n"/>
-      <c r="P17" s="69" t="n"/>
+      <c r="L17" s="72" t="n"/>
+      <c r="M17" s="70" t="n"/>
+      <c r="N17" s="70" t="n"/>
+      <c r="O17" s="72" t="n"/>
+      <c r="P17" s="70" t="n"/>
       <c r="Q17" s="67">
         <f>IFERROR(IF(J17="","",J17-TODAY()),"")</f>
         <v/>
@@ -2779,27 +2858,31 @@
         <f>IFERROR(IF(B17="","Vacant",IF(Q17&lt;0,"Expired",IF(Q17&lt;=30,"Expiring Soon",IF(Q17&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S17" s="69" t="n"/>
+      <c r="T17" s="69" t="n"/>
+      <c r="U17" s="69" t="n"/>
+      <c r="V17" s="69" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="72" t="n"/>
-      <c r="B18" s="72" t="n"/>
-      <c r="C18" s="72" t="n"/>
-      <c r="D18" s="72" t="n"/>
-      <c r="E18" s="72" t="n"/>
-      <c r="F18" s="72" t="n"/>
-      <c r="G18" s="72" t="n"/>
-      <c r="H18" s="72" t="n"/>
-      <c r="I18" s="73" t="n"/>
-      <c r="J18" s="73" t="n"/>
+      <c r="A18" s="73" t="n"/>
+      <c r="B18" s="73" t="n"/>
+      <c r="C18" s="73" t="n"/>
+      <c r="D18" s="73" t="n"/>
+      <c r="E18" s="73" t="n"/>
+      <c r="F18" s="73" t="n"/>
+      <c r="G18" s="73" t="n"/>
+      <c r="H18" s="73" t="n"/>
+      <c r="I18" s="74" t="n"/>
+      <c r="J18" s="74" t="n"/>
       <c r="K18" s="65">
         <f>IFERROR(DATEDIF(I18,J18,"M"),"")</f>
         <v/>
       </c>
-      <c r="L18" s="74" t="n"/>
-      <c r="M18" s="72" t="n"/>
-      <c r="N18" s="72" t="n"/>
-      <c r="O18" s="74" t="n"/>
-      <c r="P18" s="72" t="n"/>
+      <c r="L18" s="75" t="n"/>
+      <c r="M18" s="73" t="n"/>
+      <c r="N18" s="73" t="n"/>
+      <c r="O18" s="75" t="n"/>
+      <c r="P18" s="73" t="n"/>
       <c r="Q18" s="67">
         <f>IFERROR(IF(J18="","",J18-TODAY()),"")</f>
         <v/>
@@ -2808,27 +2891,31 @@
         <f>IFERROR(IF(B18="","Vacant",IF(Q18&lt;0,"Expired",IF(Q18&lt;=30,"Expiring Soon",IF(Q18&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S18" s="69" t="n"/>
+      <c r="T18" s="69" t="n"/>
+      <c r="U18" s="69" t="n"/>
+      <c r="V18" s="69" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="69" t="n"/>
-      <c r="B19" s="69" t="n"/>
-      <c r="C19" s="69" t="n"/>
-      <c r="D19" s="69" t="n"/>
-      <c r="E19" s="69" t="n"/>
-      <c r="F19" s="69" t="n"/>
-      <c r="G19" s="69" t="n"/>
-      <c r="H19" s="69" t="n"/>
-      <c r="I19" s="70" t="n"/>
-      <c r="J19" s="70" t="n"/>
+      <c r="A19" s="70" t="n"/>
+      <c r="B19" s="70" t="n"/>
+      <c r="C19" s="70" t="n"/>
+      <c r="D19" s="70" t="n"/>
+      <c r="E19" s="70" t="n"/>
+      <c r="F19" s="70" t="n"/>
+      <c r="G19" s="70" t="n"/>
+      <c r="H19" s="70" t="n"/>
+      <c r="I19" s="71" t="n"/>
+      <c r="J19" s="71" t="n"/>
       <c r="K19" s="65">
         <f>IFERROR(DATEDIF(I19,J19,"M"),"")</f>
         <v/>
       </c>
-      <c r="L19" s="71" t="n"/>
-      <c r="M19" s="69" t="n"/>
-      <c r="N19" s="69" t="n"/>
-      <c r="O19" s="71" t="n"/>
-      <c r="P19" s="69" t="n"/>
+      <c r="L19" s="72" t="n"/>
+      <c r="M19" s="70" t="n"/>
+      <c r="N19" s="70" t="n"/>
+      <c r="O19" s="72" t="n"/>
+      <c r="P19" s="70" t="n"/>
       <c r="Q19" s="67">
         <f>IFERROR(IF(J19="","",J19-TODAY()),"")</f>
         <v/>
@@ -2837,27 +2924,31 @@
         <f>IFERROR(IF(B19="","Vacant",IF(Q19&lt;0,"Expired",IF(Q19&lt;=30,"Expiring Soon",IF(Q19&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S19" s="69" t="n"/>
+      <c r="T19" s="69" t="n"/>
+      <c r="U19" s="69" t="n"/>
+      <c r="V19" s="69" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="72" t="n"/>
-      <c r="B20" s="72" t="n"/>
-      <c r="C20" s="72" t="n"/>
-      <c r="D20" s="72" t="n"/>
-      <c r="E20" s="72" t="n"/>
-      <c r="F20" s="72" t="n"/>
-      <c r="G20" s="72" t="n"/>
-      <c r="H20" s="72" t="n"/>
-      <c r="I20" s="73" t="n"/>
-      <c r="J20" s="73" t="n"/>
+      <c r="A20" s="73" t="n"/>
+      <c r="B20" s="73" t="n"/>
+      <c r="C20" s="73" t="n"/>
+      <c r="D20" s="73" t="n"/>
+      <c r="E20" s="73" t="n"/>
+      <c r="F20" s="73" t="n"/>
+      <c r="G20" s="73" t="n"/>
+      <c r="H20" s="73" t="n"/>
+      <c r="I20" s="74" t="n"/>
+      <c r="J20" s="74" t="n"/>
       <c r="K20" s="65">
         <f>IFERROR(DATEDIF(I20,J20,"M"),"")</f>
         <v/>
       </c>
-      <c r="L20" s="74" t="n"/>
-      <c r="M20" s="72" t="n"/>
-      <c r="N20" s="72" t="n"/>
-      <c r="O20" s="74" t="n"/>
-      <c r="P20" s="72" t="n"/>
+      <c r="L20" s="75" t="n"/>
+      <c r="M20" s="73" t="n"/>
+      <c r="N20" s="73" t="n"/>
+      <c r="O20" s="75" t="n"/>
+      <c r="P20" s="73" t="n"/>
       <c r="Q20" s="67">
         <f>IFERROR(IF(J20="","",J20-TODAY()),"")</f>
         <v/>
@@ -2866,27 +2957,31 @@
         <f>IFERROR(IF(B20="","Vacant",IF(Q20&lt;0,"Expired",IF(Q20&lt;=30,"Expiring Soon",IF(Q20&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S20" s="69" t="n"/>
+      <c r="T20" s="69" t="n"/>
+      <c r="U20" s="69" t="n"/>
+      <c r="V20" s="69" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="69" t="n"/>
-      <c r="B21" s="69" t="n"/>
-      <c r="C21" s="69" t="n"/>
-      <c r="D21" s="69" t="n"/>
-      <c r="E21" s="69" t="n"/>
-      <c r="F21" s="69" t="n"/>
-      <c r="G21" s="69" t="n"/>
-      <c r="H21" s="69" t="n"/>
-      <c r="I21" s="70" t="n"/>
-      <c r="J21" s="70" t="n"/>
+      <c r="A21" s="70" t="n"/>
+      <c r="B21" s="70" t="n"/>
+      <c r="C21" s="70" t="n"/>
+      <c r="D21" s="70" t="n"/>
+      <c r="E21" s="70" t="n"/>
+      <c r="F21" s="70" t="n"/>
+      <c r="G21" s="70" t="n"/>
+      <c r="H21" s="70" t="n"/>
+      <c r="I21" s="71" t="n"/>
+      <c r="J21" s="71" t="n"/>
       <c r="K21" s="65">
         <f>IFERROR(DATEDIF(I21,J21,"M"),"")</f>
         <v/>
       </c>
-      <c r="L21" s="71" t="n"/>
-      <c r="M21" s="69" t="n"/>
-      <c r="N21" s="69" t="n"/>
-      <c r="O21" s="71" t="n"/>
-      <c r="P21" s="69" t="n"/>
+      <c r="L21" s="72" t="n"/>
+      <c r="M21" s="70" t="n"/>
+      <c r="N21" s="70" t="n"/>
+      <c r="O21" s="72" t="n"/>
+      <c r="P21" s="70" t="n"/>
       <c r="Q21" s="67">
         <f>IFERROR(IF(J21="","",J21-TODAY()),"")</f>
         <v/>
@@ -2895,27 +2990,31 @@
         <f>IFERROR(IF(B21="","Vacant",IF(Q21&lt;0,"Expired",IF(Q21&lt;=30,"Expiring Soon",IF(Q21&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S21" s="69" t="n"/>
+      <c r="T21" s="69" t="n"/>
+      <c r="U21" s="69" t="n"/>
+      <c r="V21" s="69" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="72" t="n"/>
-      <c r="B22" s="72" t="n"/>
-      <c r="C22" s="72" t="n"/>
-      <c r="D22" s="72" t="n"/>
-      <c r="E22" s="72" t="n"/>
-      <c r="F22" s="72" t="n"/>
-      <c r="G22" s="72" t="n"/>
-      <c r="H22" s="72" t="n"/>
-      <c r="I22" s="73" t="n"/>
-      <c r="J22" s="73" t="n"/>
+      <c r="A22" s="73" t="n"/>
+      <c r="B22" s="73" t="n"/>
+      <c r="C22" s="73" t="n"/>
+      <c r="D22" s="73" t="n"/>
+      <c r="E22" s="73" t="n"/>
+      <c r="F22" s="73" t="n"/>
+      <c r="G22" s="73" t="n"/>
+      <c r="H22" s="73" t="n"/>
+      <c r="I22" s="74" t="n"/>
+      <c r="J22" s="74" t="n"/>
       <c r="K22" s="65">
         <f>IFERROR(DATEDIF(I22,J22,"M"),"")</f>
         <v/>
       </c>
-      <c r="L22" s="74" t="n"/>
-      <c r="M22" s="72" t="n"/>
-      <c r="N22" s="72" t="n"/>
-      <c r="O22" s="74" t="n"/>
-      <c r="P22" s="72" t="n"/>
+      <c r="L22" s="75" t="n"/>
+      <c r="M22" s="73" t="n"/>
+      <c r="N22" s="73" t="n"/>
+      <c r="O22" s="75" t="n"/>
+      <c r="P22" s="73" t="n"/>
       <c r="Q22" s="67">
         <f>IFERROR(IF(J22="","",J22-TODAY()),"")</f>
         <v/>
@@ -2924,27 +3023,31 @@
         <f>IFERROR(IF(B22="","Vacant",IF(Q22&lt;0,"Expired",IF(Q22&lt;=30,"Expiring Soon",IF(Q22&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S22" s="69" t="n"/>
+      <c r="T22" s="69" t="n"/>
+      <c r="U22" s="69" t="n"/>
+      <c r="V22" s="69" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="69" t="n"/>
-      <c r="B23" s="69" t="n"/>
-      <c r="C23" s="69" t="n"/>
-      <c r="D23" s="69" t="n"/>
-      <c r="E23" s="69" t="n"/>
-      <c r="F23" s="69" t="n"/>
-      <c r="G23" s="69" t="n"/>
-      <c r="H23" s="69" t="n"/>
-      <c r="I23" s="70" t="n"/>
-      <c r="J23" s="70" t="n"/>
+      <c r="A23" s="70" t="n"/>
+      <c r="B23" s="70" t="n"/>
+      <c r="C23" s="70" t="n"/>
+      <c r="D23" s="70" t="n"/>
+      <c r="E23" s="70" t="n"/>
+      <c r="F23" s="70" t="n"/>
+      <c r="G23" s="70" t="n"/>
+      <c r="H23" s="70" t="n"/>
+      <c r="I23" s="71" t="n"/>
+      <c r="J23" s="71" t="n"/>
       <c r="K23" s="65">
         <f>IFERROR(DATEDIF(I23,J23,"M"),"")</f>
         <v/>
       </c>
-      <c r="L23" s="71" t="n"/>
-      <c r="M23" s="69" t="n"/>
-      <c r="N23" s="69" t="n"/>
-      <c r="O23" s="71" t="n"/>
-      <c r="P23" s="69" t="n"/>
+      <c r="L23" s="72" t="n"/>
+      <c r="M23" s="70" t="n"/>
+      <c r="N23" s="70" t="n"/>
+      <c r="O23" s="72" t="n"/>
+      <c r="P23" s="70" t="n"/>
       <c r="Q23" s="67">
         <f>IFERROR(IF(J23="","",J23-TODAY()),"")</f>
         <v/>
@@ -2953,27 +3056,31 @@
         <f>IFERROR(IF(B23="","Vacant",IF(Q23&lt;0,"Expired",IF(Q23&lt;=30,"Expiring Soon",IF(Q23&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S23" s="69" t="n"/>
+      <c r="T23" s="69" t="n"/>
+      <c r="U23" s="69" t="n"/>
+      <c r="V23" s="69" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="72" t="n"/>
-      <c r="B24" s="72" t="n"/>
-      <c r="C24" s="72" t="n"/>
-      <c r="D24" s="72" t="n"/>
-      <c r="E24" s="72" t="n"/>
-      <c r="F24" s="72" t="n"/>
-      <c r="G24" s="72" t="n"/>
-      <c r="H24" s="72" t="n"/>
-      <c r="I24" s="73" t="n"/>
-      <c r="J24" s="73" t="n"/>
+      <c r="A24" s="73" t="n"/>
+      <c r="B24" s="73" t="n"/>
+      <c r="C24" s="73" t="n"/>
+      <c r="D24" s="73" t="n"/>
+      <c r="E24" s="73" t="n"/>
+      <c r="F24" s="73" t="n"/>
+      <c r="G24" s="73" t="n"/>
+      <c r="H24" s="73" t="n"/>
+      <c r="I24" s="74" t="n"/>
+      <c r="J24" s="74" t="n"/>
       <c r="K24" s="65">
         <f>IFERROR(DATEDIF(I24,J24,"M"),"")</f>
         <v/>
       </c>
-      <c r="L24" s="74" t="n"/>
-      <c r="M24" s="72" t="n"/>
-      <c r="N24" s="72" t="n"/>
-      <c r="O24" s="74" t="n"/>
-      <c r="P24" s="72" t="n"/>
+      <c r="L24" s="75" t="n"/>
+      <c r="M24" s="73" t="n"/>
+      <c r="N24" s="73" t="n"/>
+      <c r="O24" s="75" t="n"/>
+      <c r="P24" s="73" t="n"/>
       <c r="Q24" s="67">
         <f>IFERROR(IF(J24="","",J24-TODAY()),"")</f>
         <v/>
@@ -2982,27 +3089,31 @@
         <f>IFERROR(IF(B24="","Vacant",IF(Q24&lt;0,"Expired",IF(Q24&lt;=30,"Expiring Soon",IF(Q24&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S24" s="69" t="n"/>
+      <c r="T24" s="69" t="n"/>
+      <c r="U24" s="69" t="n"/>
+      <c r="V24" s="69" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="69" t="n"/>
-      <c r="B25" s="69" t="n"/>
-      <c r="C25" s="69" t="n"/>
-      <c r="D25" s="69" t="n"/>
-      <c r="E25" s="69" t="n"/>
-      <c r="F25" s="69" t="n"/>
-      <c r="G25" s="69" t="n"/>
-      <c r="H25" s="69" t="n"/>
-      <c r="I25" s="70" t="n"/>
-      <c r="J25" s="70" t="n"/>
+      <c r="A25" s="70" t="n"/>
+      <c r="B25" s="70" t="n"/>
+      <c r="C25" s="70" t="n"/>
+      <c r="D25" s="70" t="n"/>
+      <c r="E25" s="70" t="n"/>
+      <c r="F25" s="70" t="n"/>
+      <c r="G25" s="70" t="n"/>
+      <c r="H25" s="70" t="n"/>
+      <c r="I25" s="71" t="n"/>
+      <c r="J25" s="71" t="n"/>
       <c r="K25" s="65">
         <f>IFERROR(DATEDIF(I25,J25,"M"),"")</f>
         <v/>
       </c>
-      <c r="L25" s="71" t="n"/>
-      <c r="M25" s="69" t="n"/>
-      <c r="N25" s="69" t="n"/>
-      <c r="O25" s="71" t="n"/>
-      <c r="P25" s="69" t="n"/>
+      <c r="L25" s="72" t="n"/>
+      <c r="M25" s="70" t="n"/>
+      <c r="N25" s="70" t="n"/>
+      <c r="O25" s="72" t="n"/>
+      <c r="P25" s="70" t="n"/>
       <c r="Q25" s="67">
         <f>IFERROR(IF(J25="","",J25-TODAY()),"")</f>
         <v/>
@@ -3011,27 +3122,31 @@
         <f>IFERROR(IF(B25="","Vacant",IF(Q25&lt;0,"Expired",IF(Q25&lt;=30,"Expiring Soon",IF(Q25&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S25" s="69" t="n"/>
+      <c r="T25" s="69" t="n"/>
+      <c r="U25" s="69" t="n"/>
+      <c r="V25" s="69" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="72" t="n"/>
-      <c r="B26" s="72" t="n"/>
-      <c r="C26" s="72" t="n"/>
-      <c r="D26" s="72" t="n"/>
-      <c r="E26" s="72" t="n"/>
-      <c r="F26" s="72" t="n"/>
-      <c r="G26" s="72" t="n"/>
-      <c r="H26" s="72" t="n"/>
-      <c r="I26" s="73" t="n"/>
-      <c r="J26" s="73" t="n"/>
+      <c r="A26" s="73" t="n"/>
+      <c r="B26" s="73" t="n"/>
+      <c r="C26" s="73" t="n"/>
+      <c r="D26" s="73" t="n"/>
+      <c r="E26" s="73" t="n"/>
+      <c r="F26" s="73" t="n"/>
+      <c r="G26" s="73" t="n"/>
+      <c r="H26" s="73" t="n"/>
+      <c r="I26" s="74" t="n"/>
+      <c r="J26" s="74" t="n"/>
       <c r="K26" s="65">
         <f>IFERROR(DATEDIF(I26,J26,"M"),"")</f>
         <v/>
       </c>
-      <c r="L26" s="74" t="n"/>
-      <c r="M26" s="72" t="n"/>
-      <c r="N26" s="72" t="n"/>
-      <c r="O26" s="74" t="n"/>
-      <c r="P26" s="72" t="n"/>
+      <c r="L26" s="75" t="n"/>
+      <c r="M26" s="73" t="n"/>
+      <c r="N26" s="73" t="n"/>
+      <c r="O26" s="75" t="n"/>
+      <c r="P26" s="73" t="n"/>
       <c r="Q26" s="67">
         <f>IFERROR(IF(J26="","",J26-TODAY()),"")</f>
         <v/>
@@ -3040,27 +3155,31 @@
         <f>IFERROR(IF(B26="","Vacant",IF(Q26&lt;0,"Expired",IF(Q26&lt;=30,"Expiring Soon",IF(Q26&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S26" s="69" t="n"/>
+      <c r="T26" s="69" t="n"/>
+      <c r="U26" s="69" t="n"/>
+      <c r="V26" s="69" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="69" t="n"/>
-      <c r="B27" s="69" t="n"/>
-      <c r="C27" s="69" t="n"/>
-      <c r="D27" s="69" t="n"/>
-      <c r="E27" s="69" t="n"/>
-      <c r="F27" s="69" t="n"/>
-      <c r="G27" s="69" t="n"/>
-      <c r="H27" s="69" t="n"/>
-      <c r="I27" s="70" t="n"/>
-      <c r="J27" s="70" t="n"/>
+      <c r="A27" s="70" t="n"/>
+      <c r="B27" s="70" t="n"/>
+      <c r="C27" s="70" t="n"/>
+      <c r="D27" s="70" t="n"/>
+      <c r="E27" s="70" t="n"/>
+      <c r="F27" s="70" t="n"/>
+      <c r="G27" s="70" t="n"/>
+      <c r="H27" s="70" t="n"/>
+      <c r="I27" s="71" t="n"/>
+      <c r="J27" s="71" t="n"/>
       <c r="K27" s="65">
         <f>IFERROR(DATEDIF(I27,J27,"M"),"")</f>
         <v/>
       </c>
-      <c r="L27" s="71" t="n"/>
-      <c r="M27" s="69" t="n"/>
-      <c r="N27" s="69" t="n"/>
-      <c r="O27" s="71" t="n"/>
-      <c r="P27" s="69" t="n"/>
+      <c r="L27" s="72" t="n"/>
+      <c r="M27" s="70" t="n"/>
+      <c r="N27" s="70" t="n"/>
+      <c r="O27" s="72" t="n"/>
+      <c r="P27" s="70" t="n"/>
       <c r="Q27" s="67">
         <f>IFERROR(IF(J27="","",J27-TODAY()),"")</f>
         <v/>
@@ -3069,27 +3188,31 @@
         <f>IFERROR(IF(B27="","Vacant",IF(Q27&lt;0,"Expired",IF(Q27&lt;=30,"Expiring Soon",IF(Q27&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S27" s="69" t="n"/>
+      <c r="T27" s="69" t="n"/>
+      <c r="U27" s="69" t="n"/>
+      <c r="V27" s="69" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="72" t="n"/>
-      <c r="B28" s="72" t="n"/>
-      <c r="C28" s="72" t="n"/>
-      <c r="D28" s="72" t="n"/>
-      <c r="E28" s="72" t="n"/>
-      <c r="F28" s="72" t="n"/>
-      <c r="G28" s="72" t="n"/>
-      <c r="H28" s="72" t="n"/>
-      <c r="I28" s="73" t="n"/>
-      <c r="J28" s="73" t="n"/>
+      <c r="A28" s="73" t="n"/>
+      <c r="B28" s="73" t="n"/>
+      <c r="C28" s="73" t="n"/>
+      <c r="D28" s="73" t="n"/>
+      <c r="E28" s="73" t="n"/>
+      <c r="F28" s="73" t="n"/>
+      <c r="G28" s="73" t="n"/>
+      <c r="H28" s="73" t="n"/>
+      <c r="I28" s="74" t="n"/>
+      <c r="J28" s="74" t="n"/>
       <c r="K28" s="65">
         <f>IFERROR(DATEDIF(I28,J28,"M"),"")</f>
         <v/>
       </c>
-      <c r="L28" s="74" t="n"/>
-      <c r="M28" s="72" t="n"/>
-      <c r="N28" s="72" t="n"/>
-      <c r="O28" s="74" t="n"/>
-      <c r="P28" s="72" t="n"/>
+      <c r="L28" s="75" t="n"/>
+      <c r="M28" s="73" t="n"/>
+      <c r="N28" s="73" t="n"/>
+      <c r="O28" s="75" t="n"/>
+      <c r="P28" s="73" t="n"/>
       <c r="Q28" s="67">
         <f>IFERROR(IF(J28="","",J28-TODAY()),"")</f>
         <v/>
@@ -3098,27 +3221,31 @@
         <f>IFERROR(IF(B28="","Vacant",IF(Q28&lt;0,"Expired",IF(Q28&lt;=30,"Expiring Soon",IF(Q28&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S28" s="69" t="n"/>
+      <c r="T28" s="69" t="n"/>
+      <c r="U28" s="69" t="n"/>
+      <c r="V28" s="69" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="69" t="n"/>
-      <c r="B29" s="69" t="n"/>
-      <c r="C29" s="69" t="n"/>
-      <c r="D29" s="69" t="n"/>
-      <c r="E29" s="69" t="n"/>
-      <c r="F29" s="69" t="n"/>
-      <c r="G29" s="69" t="n"/>
-      <c r="H29" s="69" t="n"/>
-      <c r="I29" s="70" t="n"/>
-      <c r="J29" s="70" t="n"/>
+      <c r="A29" s="70" t="n"/>
+      <c r="B29" s="70" t="n"/>
+      <c r="C29" s="70" t="n"/>
+      <c r="D29" s="70" t="n"/>
+      <c r="E29" s="70" t="n"/>
+      <c r="F29" s="70" t="n"/>
+      <c r="G29" s="70" t="n"/>
+      <c r="H29" s="70" t="n"/>
+      <c r="I29" s="71" t="n"/>
+      <c r="J29" s="71" t="n"/>
       <c r="K29" s="65">
         <f>IFERROR(DATEDIF(I29,J29,"M"),"")</f>
         <v/>
       </c>
-      <c r="L29" s="71" t="n"/>
-      <c r="M29" s="69" t="n"/>
-      <c r="N29" s="69" t="n"/>
-      <c r="O29" s="71" t="n"/>
-      <c r="P29" s="69" t="n"/>
+      <c r="L29" s="72" t="n"/>
+      <c r="M29" s="70" t="n"/>
+      <c r="N29" s="70" t="n"/>
+      <c r="O29" s="72" t="n"/>
+      <c r="P29" s="70" t="n"/>
       <c r="Q29" s="67">
         <f>IFERROR(IF(J29="","",J29-TODAY()),"")</f>
         <v/>
@@ -3127,27 +3254,31 @@
         <f>IFERROR(IF(B29="","Vacant",IF(Q29&lt;0,"Expired",IF(Q29&lt;=30,"Expiring Soon",IF(Q29&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S29" s="69" t="n"/>
+      <c r="T29" s="69" t="n"/>
+      <c r="U29" s="69" t="n"/>
+      <c r="V29" s="69" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="72" t="n"/>
-      <c r="B30" s="72" t="n"/>
-      <c r="C30" s="72" t="n"/>
-      <c r="D30" s="72" t="n"/>
-      <c r="E30" s="72" t="n"/>
-      <c r="F30" s="72" t="n"/>
-      <c r="G30" s="72" t="n"/>
-      <c r="H30" s="72" t="n"/>
-      <c r="I30" s="73" t="n"/>
-      <c r="J30" s="73" t="n"/>
+      <c r="A30" s="73" t="n"/>
+      <c r="B30" s="73" t="n"/>
+      <c r="C30" s="73" t="n"/>
+      <c r="D30" s="73" t="n"/>
+      <c r="E30" s="73" t="n"/>
+      <c r="F30" s="73" t="n"/>
+      <c r="G30" s="73" t="n"/>
+      <c r="H30" s="73" t="n"/>
+      <c r="I30" s="74" t="n"/>
+      <c r="J30" s="74" t="n"/>
       <c r="K30" s="65">
         <f>IFERROR(DATEDIF(I30,J30,"M"),"")</f>
         <v/>
       </c>
-      <c r="L30" s="74" t="n"/>
-      <c r="M30" s="72" t="n"/>
-      <c r="N30" s="72" t="n"/>
-      <c r="O30" s="74" t="n"/>
-      <c r="P30" s="72" t="n"/>
+      <c r="L30" s="75" t="n"/>
+      <c r="M30" s="73" t="n"/>
+      <c r="N30" s="73" t="n"/>
+      <c r="O30" s="75" t="n"/>
+      <c r="P30" s="73" t="n"/>
       <c r="Q30" s="67">
         <f>IFERROR(IF(J30="","",J30-TODAY()),"")</f>
         <v/>
@@ -3156,27 +3287,31 @@
         <f>IFERROR(IF(B30="","Vacant",IF(Q30&lt;0,"Expired",IF(Q30&lt;=30,"Expiring Soon",IF(Q30&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S30" s="69" t="n"/>
+      <c r="T30" s="69" t="n"/>
+      <c r="U30" s="69" t="n"/>
+      <c r="V30" s="69" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="69" t="n"/>
-      <c r="B31" s="69" t="n"/>
-      <c r="C31" s="69" t="n"/>
-      <c r="D31" s="69" t="n"/>
-      <c r="E31" s="69" t="n"/>
-      <c r="F31" s="69" t="n"/>
-      <c r="G31" s="69" t="n"/>
-      <c r="H31" s="69" t="n"/>
-      <c r="I31" s="70" t="n"/>
-      <c r="J31" s="70" t="n"/>
+      <c r="A31" s="70" t="n"/>
+      <c r="B31" s="70" t="n"/>
+      <c r="C31" s="70" t="n"/>
+      <c r="D31" s="70" t="n"/>
+      <c r="E31" s="70" t="n"/>
+      <c r="F31" s="70" t="n"/>
+      <c r="G31" s="70" t="n"/>
+      <c r="H31" s="70" t="n"/>
+      <c r="I31" s="71" t="n"/>
+      <c r="J31" s="71" t="n"/>
       <c r="K31" s="65">
         <f>IFERROR(DATEDIF(I31,J31,"M"),"")</f>
         <v/>
       </c>
-      <c r="L31" s="71" t="n"/>
-      <c r="M31" s="69" t="n"/>
-      <c r="N31" s="69" t="n"/>
-      <c r="O31" s="71" t="n"/>
-      <c r="P31" s="69" t="n"/>
+      <c r="L31" s="72" t="n"/>
+      <c r="M31" s="70" t="n"/>
+      <c r="N31" s="70" t="n"/>
+      <c r="O31" s="72" t="n"/>
+      <c r="P31" s="70" t="n"/>
       <c r="Q31" s="67">
         <f>IFERROR(IF(J31="","",J31-TODAY()),"")</f>
         <v/>
@@ -3185,27 +3320,31 @@
         <f>IFERROR(IF(B31="","Vacant",IF(Q31&lt;0,"Expired",IF(Q31&lt;=30,"Expiring Soon",IF(Q31&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S31" s="69" t="n"/>
+      <c r="T31" s="69" t="n"/>
+      <c r="U31" s="69" t="n"/>
+      <c r="V31" s="69" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="72" t="n"/>
-      <c r="B32" s="72" t="n"/>
-      <c r="C32" s="72" t="n"/>
-      <c r="D32" s="72" t="n"/>
-      <c r="E32" s="72" t="n"/>
-      <c r="F32" s="72" t="n"/>
-      <c r="G32" s="72" t="n"/>
-      <c r="H32" s="72" t="n"/>
-      <c r="I32" s="73" t="n"/>
-      <c r="J32" s="73" t="n"/>
+      <c r="A32" s="73" t="n"/>
+      <c r="B32" s="73" t="n"/>
+      <c r="C32" s="73" t="n"/>
+      <c r="D32" s="73" t="n"/>
+      <c r="E32" s="73" t="n"/>
+      <c r="F32" s="73" t="n"/>
+      <c r="G32" s="73" t="n"/>
+      <c r="H32" s="73" t="n"/>
+      <c r="I32" s="74" t="n"/>
+      <c r="J32" s="74" t="n"/>
       <c r="K32" s="65">
         <f>IFERROR(DATEDIF(I32,J32,"M"),"")</f>
         <v/>
       </c>
-      <c r="L32" s="74" t="n"/>
-      <c r="M32" s="72" t="n"/>
-      <c r="N32" s="72" t="n"/>
-      <c r="O32" s="74" t="n"/>
-      <c r="P32" s="72" t="n"/>
+      <c r="L32" s="75" t="n"/>
+      <c r="M32" s="73" t="n"/>
+      <c r="N32" s="73" t="n"/>
+      <c r="O32" s="75" t="n"/>
+      <c r="P32" s="73" t="n"/>
       <c r="Q32" s="67">
         <f>IFERROR(IF(J32="","",J32-TODAY()),"")</f>
         <v/>
@@ -3214,27 +3353,31 @@
         <f>IFERROR(IF(B32="","Vacant",IF(Q32&lt;0,"Expired",IF(Q32&lt;=30,"Expiring Soon",IF(Q32&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S32" s="69" t="n"/>
+      <c r="T32" s="69" t="n"/>
+      <c r="U32" s="69" t="n"/>
+      <c r="V32" s="69" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="69" t="n"/>
-      <c r="B33" s="69" t="n"/>
-      <c r="C33" s="69" t="n"/>
-      <c r="D33" s="69" t="n"/>
-      <c r="E33" s="69" t="n"/>
-      <c r="F33" s="69" t="n"/>
-      <c r="G33" s="69" t="n"/>
-      <c r="H33" s="69" t="n"/>
-      <c r="I33" s="70" t="n"/>
-      <c r="J33" s="70" t="n"/>
+      <c r="A33" s="70" t="n"/>
+      <c r="B33" s="70" t="n"/>
+      <c r="C33" s="70" t="n"/>
+      <c r="D33" s="70" t="n"/>
+      <c r="E33" s="70" t="n"/>
+      <c r="F33" s="70" t="n"/>
+      <c r="G33" s="70" t="n"/>
+      <c r="H33" s="70" t="n"/>
+      <c r="I33" s="71" t="n"/>
+      <c r="J33" s="71" t="n"/>
       <c r="K33" s="65">
         <f>IFERROR(DATEDIF(I33,J33,"M"),"")</f>
         <v/>
       </c>
-      <c r="L33" s="71" t="n"/>
-      <c r="M33" s="69" t="n"/>
-      <c r="N33" s="69" t="n"/>
-      <c r="O33" s="71" t="n"/>
-      <c r="P33" s="69" t="n"/>
+      <c r="L33" s="72" t="n"/>
+      <c r="M33" s="70" t="n"/>
+      <c r="N33" s="70" t="n"/>
+      <c r="O33" s="72" t="n"/>
+      <c r="P33" s="70" t="n"/>
       <c r="Q33" s="67">
         <f>IFERROR(IF(J33="","",J33-TODAY()),"")</f>
         <v/>
@@ -3243,27 +3386,31 @@
         <f>IFERROR(IF(B33="","Vacant",IF(Q33&lt;0,"Expired",IF(Q33&lt;=30,"Expiring Soon",IF(Q33&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S33" s="69" t="n"/>
+      <c r="T33" s="69" t="n"/>
+      <c r="U33" s="69" t="n"/>
+      <c r="V33" s="69" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="72" t="n"/>
-      <c r="B34" s="72" t="n"/>
-      <c r="C34" s="72" t="n"/>
-      <c r="D34" s="72" t="n"/>
-      <c r="E34" s="72" t="n"/>
-      <c r="F34" s="72" t="n"/>
-      <c r="G34" s="72" t="n"/>
-      <c r="H34" s="72" t="n"/>
-      <c r="I34" s="73" t="n"/>
-      <c r="J34" s="73" t="n"/>
+      <c r="A34" s="73" t="n"/>
+      <c r="B34" s="73" t="n"/>
+      <c r="C34" s="73" t="n"/>
+      <c r="D34" s="73" t="n"/>
+      <c r="E34" s="73" t="n"/>
+      <c r="F34" s="73" t="n"/>
+      <c r="G34" s="73" t="n"/>
+      <c r="H34" s="73" t="n"/>
+      <c r="I34" s="74" t="n"/>
+      <c r="J34" s="74" t="n"/>
       <c r="K34" s="65">
         <f>IFERROR(DATEDIF(I34,J34,"M"),"")</f>
         <v/>
       </c>
-      <c r="L34" s="74" t="n"/>
-      <c r="M34" s="72" t="n"/>
-      <c r="N34" s="72" t="n"/>
-      <c r="O34" s="74" t="n"/>
-      <c r="P34" s="72" t="n"/>
+      <c r="L34" s="75" t="n"/>
+      <c r="M34" s="73" t="n"/>
+      <c r="N34" s="73" t="n"/>
+      <c r="O34" s="75" t="n"/>
+      <c r="P34" s="73" t="n"/>
       <c r="Q34" s="67">
         <f>IFERROR(IF(J34="","",J34-TODAY()),"")</f>
         <v/>
@@ -3272,27 +3419,31 @@
         <f>IFERROR(IF(B34="","Vacant",IF(Q34&lt;0,"Expired",IF(Q34&lt;=30,"Expiring Soon",IF(Q34&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S34" s="69" t="n"/>
+      <c r="T34" s="69" t="n"/>
+      <c r="U34" s="69" t="n"/>
+      <c r="V34" s="69" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="69" t="n"/>
-      <c r="B35" s="69" t="n"/>
-      <c r="C35" s="69" t="n"/>
-      <c r="D35" s="69" t="n"/>
-      <c r="E35" s="69" t="n"/>
-      <c r="F35" s="69" t="n"/>
-      <c r="G35" s="69" t="n"/>
-      <c r="H35" s="69" t="n"/>
-      <c r="I35" s="70" t="n"/>
-      <c r="J35" s="70" t="n"/>
+      <c r="A35" s="70" t="n"/>
+      <c r="B35" s="70" t="n"/>
+      <c r="C35" s="70" t="n"/>
+      <c r="D35" s="70" t="n"/>
+      <c r="E35" s="70" t="n"/>
+      <c r="F35" s="70" t="n"/>
+      <c r="G35" s="70" t="n"/>
+      <c r="H35" s="70" t="n"/>
+      <c r="I35" s="71" t="n"/>
+      <c r="J35" s="71" t="n"/>
       <c r="K35" s="65">
         <f>IFERROR(DATEDIF(I35,J35,"M"),"")</f>
         <v/>
       </c>
-      <c r="L35" s="71" t="n"/>
-      <c r="M35" s="69" t="n"/>
-      <c r="N35" s="69" t="n"/>
-      <c r="O35" s="71" t="n"/>
-      <c r="P35" s="69" t="n"/>
+      <c r="L35" s="72" t="n"/>
+      <c r="M35" s="70" t="n"/>
+      <c r="N35" s="70" t="n"/>
+      <c r="O35" s="72" t="n"/>
+      <c r="P35" s="70" t="n"/>
       <c r="Q35" s="67">
         <f>IFERROR(IF(J35="","",J35-TODAY()),"")</f>
         <v/>
@@ -3301,27 +3452,31 @@
         <f>IFERROR(IF(B35="","Vacant",IF(Q35&lt;0,"Expired",IF(Q35&lt;=30,"Expiring Soon",IF(Q35&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S35" s="69" t="n"/>
+      <c r="T35" s="69" t="n"/>
+      <c r="U35" s="69" t="n"/>
+      <c r="V35" s="69" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="72" t="n"/>
-      <c r="B36" s="72" t="n"/>
-      <c r="C36" s="72" t="n"/>
-      <c r="D36" s="72" t="n"/>
-      <c r="E36" s="72" t="n"/>
-      <c r="F36" s="72" t="n"/>
-      <c r="G36" s="72" t="n"/>
-      <c r="H36" s="72" t="n"/>
-      <c r="I36" s="73" t="n"/>
-      <c r="J36" s="73" t="n"/>
+      <c r="A36" s="73" t="n"/>
+      <c r="B36" s="73" t="n"/>
+      <c r="C36" s="73" t="n"/>
+      <c r="D36" s="73" t="n"/>
+      <c r="E36" s="73" t="n"/>
+      <c r="F36" s="73" t="n"/>
+      <c r="G36" s="73" t="n"/>
+      <c r="H36" s="73" t="n"/>
+      <c r="I36" s="74" t="n"/>
+      <c r="J36" s="74" t="n"/>
       <c r="K36" s="65">
         <f>IFERROR(DATEDIF(I36,J36,"M"),"")</f>
         <v/>
       </c>
-      <c r="L36" s="74" t="n"/>
-      <c r="M36" s="72" t="n"/>
-      <c r="N36" s="72" t="n"/>
-      <c r="O36" s="74" t="n"/>
-      <c r="P36" s="72" t="n"/>
+      <c r="L36" s="75" t="n"/>
+      <c r="M36" s="73" t="n"/>
+      <c r="N36" s="73" t="n"/>
+      <c r="O36" s="75" t="n"/>
+      <c r="P36" s="73" t="n"/>
       <c r="Q36" s="67">
         <f>IFERROR(IF(J36="","",J36-TODAY()),"")</f>
         <v/>
@@ -3330,27 +3485,31 @@
         <f>IFERROR(IF(B36="","Vacant",IF(Q36&lt;0,"Expired",IF(Q36&lt;=30,"Expiring Soon",IF(Q36&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S36" s="69" t="n"/>
+      <c r="T36" s="69" t="n"/>
+      <c r="U36" s="69" t="n"/>
+      <c r="V36" s="69" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="69" t="n"/>
-      <c r="B37" s="69" t="n"/>
-      <c r="C37" s="69" t="n"/>
-      <c r="D37" s="69" t="n"/>
-      <c r="E37" s="69" t="n"/>
-      <c r="F37" s="69" t="n"/>
-      <c r="G37" s="69" t="n"/>
-      <c r="H37" s="69" t="n"/>
-      <c r="I37" s="70" t="n"/>
-      <c r="J37" s="70" t="n"/>
+      <c r="A37" s="70" t="n"/>
+      <c r="B37" s="70" t="n"/>
+      <c r="C37" s="70" t="n"/>
+      <c r="D37" s="70" t="n"/>
+      <c r="E37" s="70" t="n"/>
+      <c r="F37" s="70" t="n"/>
+      <c r="G37" s="70" t="n"/>
+      <c r="H37" s="70" t="n"/>
+      <c r="I37" s="71" t="n"/>
+      <c r="J37" s="71" t="n"/>
       <c r="K37" s="65">
         <f>IFERROR(DATEDIF(I37,J37,"M"),"")</f>
         <v/>
       </c>
-      <c r="L37" s="71" t="n"/>
-      <c r="M37" s="69" t="n"/>
-      <c r="N37" s="69" t="n"/>
-      <c r="O37" s="71" t="n"/>
-      <c r="P37" s="69" t="n"/>
+      <c r="L37" s="72" t="n"/>
+      <c r="M37" s="70" t="n"/>
+      <c r="N37" s="70" t="n"/>
+      <c r="O37" s="72" t="n"/>
+      <c r="P37" s="70" t="n"/>
       <c r="Q37" s="67">
         <f>IFERROR(IF(J37="","",J37-TODAY()),"")</f>
         <v/>
@@ -3359,27 +3518,31 @@
         <f>IFERROR(IF(B37="","Vacant",IF(Q37&lt;0,"Expired",IF(Q37&lt;=30,"Expiring Soon",IF(Q37&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S37" s="69" t="n"/>
+      <c r="T37" s="69" t="n"/>
+      <c r="U37" s="69" t="n"/>
+      <c r="V37" s="69" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="72" t="n"/>
-      <c r="B38" s="72" t="n"/>
-      <c r="C38" s="72" t="n"/>
-      <c r="D38" s="72" t="n"/>
-      <c r="E38" s="72" t="n"/>
-      <c r="F38" s="72" t="n"/>
-      <c r="G38" s="72" t="n"/>
-      <c r="H38" s="72" t="n"/>
-      <c r="I38" s="73" t="n"/>
-      <c r="J38" s="73" t="n"/>
+      <c r="A38" s="73" t="n"/>
+      <c r="B38" s="73" t="n"/>
+      <c r="C38" s="73" t="n"/>
+      <c r="D38" s="73" t="n"/>
+      <c r="E38" s="73" t="n"/>
+      <c r="F38" s="73" t="n"/>
+      <c r="G38" s="73" t="n"/>
+      <c r="H38" s="73" t="n"/>
+      <c r="I38" s="74" t="n"/>
+      <c r="J38" s="74" t="n"/>
       <c r="K38" s="65">
         <f>IFERROR(DATEDIF(I38,J38,"M"),"")</f>
         <v/>
       </c>
-      <c r="L38" s="74" t="n"/>
-      <c r="M38" s="72" t="n"/>
-      <c r="N38" s="72" t="n"/>
-      <c r="O38" s="74" t="n"/>
-      <c r="P38" s="72" t="n"/>
+      <c r="L38" s="75" t="n"/>
+      <c r="M38" s="73" t="n"/>
+      <c r="N38" s="73" t="n"/>
+      <c r="O38" s="75" t="n"/>
+      <c r="P38" s="73" t="n"/>
       <c r="Q38" s="67">
         <f>IFERROR(IF(J38="","",J38-TODAY()),"")</f>
         <v/>
@@ -3388,27 +3551,31 @@
         <f>IFERROR(IF(B38="","Vacant",IF(Q38&lt;0,"Expired",IF(Q38&lt;=30,"Expiring Soon",IF(Q38&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S38" s="69" t="n"/>
+      <c r="T38" s="69" t="n"/>
+      <c r="U38" s="69" t="n"/>
+      <c r="V38" s="69" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="69" t="n"/>
-      <c r="B39" s="69" t="n"/>
-      <c r="C39" s="69" t="n"/>
-      <c r="D39" s="69" t="n"/>
-      <c r="E39" s="69" t="n"/>
-      <c r="F39" s="69" t="n"/>
-      <c r="G39" s="69" t="n"/>
-      <c r="H39" s="69" t="n"/>
-      <c r="I39" s="70" t="n"/>
-      <c r="J39" s="70" t="n"/>
+      <c r="A39" s="70" t="n"/>
+      <c r="B39" s="70" t="n"/>
+      <c r="C39" s="70" t="n"/>
+      <c r="D39" s="70" t="n"/>
+      <c r="E39" s="70" t="n"/>
+      <c r="F39" s="70" t="n"/>
+      <c r="G39" s="70" t="n"/>
+      <c r="H39" s="70" t="n"/>
+      <c r="I39" s="71" t="n"/>
+      <c r="J39" s="71" t="n"/>
       <c r="K39" s="65">
         <f>IFERROR(DATEDIF(I39,J39,"M"),"")</f>
         <v/>
       </c>
-      <c r="L39" s="71" t="n"/>
-      <c r="M39" s="69" t="n"/>
-      <c r="N39" s="69" t="n"/>
-      <c r="O39" s="71" t="n"/>
-      <c r="P39" s="69" t="n"/>
+      <c r="L39" s="72" t="n"/>
+      <c r="M39" s="70" t="n"/>
+      <c r="N39" s="70" t="n"/>
+      <c r="O39" s="72" t="n"/>
+      <c r="P39" s="70" t="n"/>
       <c r="Q39" s="67">
         <f>IFERROR(IF(J39="","",J39-TODAY()),"")</f>
         <v/>
@@ -3417,27 +3584,31 @@
         <f>IFERROR(IF(B39="","Vacant",IF(Q39&lt;0,"Expired",IF(Q39&lt;=30,"Expiring Soon",IF(Q39&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S39" s="69" t="n"/>
+      <c r="T39" s="69" t="n"/>
+      <c r="U39" s="69" t="n"/>
+      <c r="V39" s="69" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="72" t="n"/>
-      <c r="B40" s="72" t="n"/>
-      <c r="C40" s="72" t="n"/>
-      <c r="D40" s="72" t="n"/>
-      <c r="E40" s="72" t="n"/>
-      <c r="F40" s="72" t="n"/>
-      <c r="G40" s="72" t="n"/>
-      <c r="H40" s="72" t="n"/>
-      <c r="I40" s="73" t="n"/>
-      <c r="J40" s="73" t="n"/>
+      <c r="A40" s="73" t="n"/>
+      <c r="B40" s="73" t="n"/>
+      <c r="C40" s="73" t="n"/>
+      <c r="D40" s="73" t="n"/>
+      <c r="E40" s="73" t="n"/>
+      <c r="F40" s="73" t="n"/>
+      <c r="G40" s="73" t="n"/>
+      <c r="H40" s="73" t="n"/>
+      <c r="I40" s="74" t="n"/>
+      <c r="J40" s="74" t="n"/>
       <c r="K40" s="65">
         <f>IFERROR(DATEDIF(I40,J40,"M"),"")</f>
         <v/>
       </c>
-      <c r="L40" s="74" t="n"/>
-      <c r="M40" s="72" t="n"/>
-      <c r="N40" s="72" t="n"/>
-      <c r="O40" s="74" t="n"/>
-      <c r="P40" s="72" t="n"/>
+      <c r="L40" s="75" t="n"/>
+      <c r="M40" s="73" t="n"/>
+      <c r="N40" s="73" t="n"/>
+      <c r="O40" s="75" t="n"/>
+      <c r="P40" s="73" t="n"/>
       <c r="Q40" s="67">
         <f>IFERROR(IF(J40="","",J40-TODAY()),"")</f>
         <v/>
@@ -3446,27 +3617,31 @@
         <f>IFERROR(IF(B40="","Vacant",IF(Q40&lt;0,"Expired",IF(Q40&lt;=30,"Expiring Soon",IF(Q40&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S40" s="69" t="n"/>
+      <c r="T40" s="69" t="n"/>
+      <c r="U40" s="69" t="n"/>
+      <c r="V40" s="69" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="69" t="n"/>
-      <c r="B41" s="69" t="n"/>
-      <c r="C41" s="69" t="n"/>
-      <c r="D41" s="69" t="n"/>
-      <c r="E41" s="69" t="n"/>
-      <c r="F41" s="69" t="n"/>
-      <c r="G41" s="69" t="n"/>
-      <c r="H41" s="69" t="n"/>
-      <c r="I41" s="70" t="n"/>
-      <c r="J41" s="70" t="n"/>
+      <c r="A41" s="70" t="n"/>
+      <c r="B41" s="70" t="n"/>
+      <c r="C41" s="70" t="n"/>
+      <c r="D41" s="70" t="n"/>
+      <c r="E41" s="70" t="n"/>
+      <c r="F41" s="70" t="n"/>
+      <c r="G41" s="70" t="n"/>
+      <c r="H41" s="70" t="n"/>
+      <c r="I41" s="71" t="n"/>
+      <c r="J41" s="71" t="n"/>
       <c r="K41" s="65">
         <f>IFERROR(DATEDIF(I41,J41,"M"),"")</f>
         <v/>
       </c>
-      <c r="L41" s="71" t="n"/>
-      <c r="M41" s="69" t="n"/>
-      <c r="N41" s="69" t="n"/>
-      <c r="O41" s="71" t="n"/>
-      <c r="P41" s="69" t="n"/>
+      <c r="L41" s="72" t="n"/>
+      <c r="M41" s="70" t="n"/>
+      <c r="N41" s="70" t="n"/>
+      <c r="O41" s="72" t="n"/>
+      <c r="P41" s="70" t="n"/>
       <c r="Q41" s="67">
         <f>IFERROR(IF(J41="","",J41-TODAY()),"")</f>
         <v/>
@@ -3475,27 +3650,31 @@
         <f>IFERROR(IF(B41="","Vacant",IF(Q41&lt;0,"Expired",IF(Q41&lt;=30,"Expiring Soon",IF(Q41&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S41" s="69" t="n"/>
+      <c r="T41" s="69" t="n"/>
+      <c r="U41" s="69" t="n"/>
+      <c r="V41" s="69" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="72" t="n"/>
-      <c r="B42" s="72" t="n"/>
-      <c r="C42" s="72" t="n"/>
-      <c r="D42" s="72" t="n"/>
-      <c r="E42" s="72" t="n"/>
-      <c r="F42" s="72" t="n"/>
-      <c r="G42" s="72" t="n"/>
-      <c r="H42" s="72" t="n"/>
-      <c r="I42" s="73" t="n"/>
-      <c r="J42" s="73" t="n"/>
+      <c r="A42" s="73" t="n"/>
+      <c r="B42" s="73" t="n"/>
+      <c r="C42" s="73" t="n"/>
+      <c r="D42" s="73" t="n"/>
+      <c r="E42" s="73" t="n"/>
+      <c r="F42" s="73" t="n"/>
+      <c r="G42" s="73" t="n"/>
+      <c r="H42" s="73" t="n"/>
+      <c r="I42" s="74" t="n"/>
+      <c r="J42" s="74" t="n"/>
       <c r="K42" s="65">
         <f>IFERROR(DATEDIF(I42,J42,"M"),"")</f>
         <v/>
       </c>
-      <c r="L42" s="74" t="n"/>
-      <c r="M42" s="72" t="n"/>
-      <c r="N42" s="72" t="n"/>
-      <c r="O42" s="74" t="n"/>
-      <c r="P42" s="72" t="n"/>
+      <c r="L42" s="75" t="n"/>
+      <c r="M42" s="73" t="n"/>
+      <c r="N42" s="73" t="n"/>
+      <c r="O42" s="75" t="n"/>
+      <c r="P42" s="73" t="n"/>
       <c r="Q42" s="67">
         <f>IFERROR(IF(J42="","",J42-TODAY()),"")</f>
         <v/>
@@ -3504,27 +3683,31 @@
         <f>IFERROR(IF(B42="","Vacant",IF(Q42&lt;0,"Expired",IF(Q42&lt;=30,"Expiring Soon",IF(Q42&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S42" s="69" t="n"/>
+      <c r="T42" s="69" t="n"/>
+      <c r="U42" s="69" t="n"/>
+      <c r="V42" s="69" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="69" t="n"/>
-      <c r="B43" s="69" t="n"/>
-      <c r="C43" s="69" t="n"/>
-      <c r="D43" s="69" t="n"/>
-      <c r="E43" s="69" t="n"/>
-      <c r="F43" s="69" t="n"/>
-      <c r="G43" s="69" t="n"/>
-      <c r="H43" s="69" t="n"/>
-      <c r="I43" s="70" t="n"/>
-      <c r="J43" s="70" t="n"/>
+      <c r="A43" s="70" t="n"/>
+      <c r="B43" s="70" t="n"/>
+      <c r="C43" s="70" t="n"/>
+      <c r="D43" s="70" t="n"/>
+      <c r="E43" s="70" t="n"/>
+      <c r="F43" s="70" t="n"/>
+      <c r="G43" s="70" t="n"/>
+      <c r="H43" s="70" t="n"/>
+      <c r="I43" s="71" t="n"/>
+      <c r="J43" s="71" t="n"/>
       <c r="K43" s="65">
         <f>IFERROR(DATEDIF(I43,J43,"M"),"")</f>
         <v/>
       </c>
-      <c r="L43" s="71" t="n"/>
-      <c r="M43" s="69" t="n"/>
-      <c r="N43" s="69" t="n"/>
-      <c r="O43" s="71" t="n"/>
-      <c r="P43" s="69" t="n"/>
+      <c r="L43" s="72" t="n"/>
+      <c r="M43" s="70" t="n"/>
+      <c r="N43" s="70" t="n"/>
+      <c r="O43" s="72" t="n"/>
+      <c r="P43" s="70" t="n"/>
       <c r="Q43" s="67">
         <f>IFERROR(IF(J43="","",J43-TODAY()),"")</f>
         <v/>
@@ -3533,27 +3716,31 @@
         <f>IFERROR(IF(B43="","Vacant",IF(Q43&lt;0,"Expired",IF(Q43&lt;=30,"Expiring Soon",IF(Q43&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S43" s="69" t="n"/>
+      <c r="T43" s="69" t="n"/>
+      <c r="U43" s="69" t="n"/>
+      <c r="V43" s="69" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="72" t="n"/>
-      <c r="B44" s="72" t="n"/>
-      <c r="C44" s="72" t="n"/>
-      <c r="D44" s="72" t="n"/>
-      <c r="E44" s="72" t="n"/>
-      <c r="F44" s="72" t="n"/>
-      <c r="G44" s="72" t="n"/>
-      <c r="H44" s="72" t="n"/>
-      <c r="I44" s="73" t="n"/>
-      <c r="J44" s="73" t="n"/>
+      <c r="A44" s="73" t="n"/>
+      <c r="B44" s="73" t="n"/>
+      <c r="C44" s="73" t="n"/>
+      <c r="D44" s="73" t="n"/>
+      <c r="E44" s="73" t="n"/>
+      <c r="F44" s="73" t="n"/>
+      <c r="G44" s="73" t="n"/>
+      <c r="H44" s="73" t="n"/>
+      <c r="I44" s="74" t="n"/>
+      <c r="J44" s="74" t="n"/>
       <c r="K44" s="65">
         <f>IFERROR(DATEDIF(I44,J44,"M"),"")</f>
         <v/>
       </c>
-      <c r="L44" s="74" t="n"/>
-      <c r="M44" s="72" t="n"/>
-      <c r="N44" s="72" t="n"/>
-      <c r="O44" s="74" t="n"/>
-      <c r="P44" s="72" t="n"/>
+      <c r="L44" s="75" t="n"/>
+      <c r="M44" s="73" t="n"/>
+      <c r="N44" s="73" t="n"/>
+      <c r="O44" s="75" t="n"/>
+      <c r="P44" s="73" t="n"/>
       <c r="Q44" s="67">
         <f>IFERROR(IF(J44="","",J44-TODAY()),"")</f>
         <v/>
@@ -3562,27 +3749,31 @@
         <f>IFERROR(IF(B44="","Vacant",IF(Q44&lt;0,"Expired",IF(Q44&lt;=30,"Expiring Soon",IF(Q44&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S44" s="69" t="n"/>
+      <c r="T44" s="69" t="n"/>
+      <c r="U44" s="69" t="n"/>
+      <c r="V44" s="69" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="69" t="n"/>
-      <c r="B45" s="69" t="n"/>
-      <c r="C45" s="69" t="n"/>
-      <c r="D45" s="69" t="n"/>
-      <c r="E45" s="69" t="n"/>
-      <c r="F45" s="69" t="n"/>
-      <c r="G45" s="69" t="n"/>
-      <c r="H45" s="69" t="n"/>
-      <c r="I45" s="70" t="n"/>
-      <c r="J45" s="70" t="n"/>
+      <c r="A45" s="70" t="n"/>
+      <c r="B45" s="70" t="n"/>
+      <c r="C45" s="70" t="n"/>
+      <c r="D45" s="70" t="n"/>
+      <c r="E45" s="70" t="n"/>
+      <c r="F45" s="70" t="n"/>
+      <c r="G45" s="70" t="n"/>
+      <c r="H45" s="70" t="n"/>
+      <c r="I45" s="71" t="n"/>
+      <c r="J45" s="71" t="n"/>
       <c r="K45" s="65">
         <f>IFERROR(DATEDIF(I45,J45,"M"),"")</f>
         <v/>
       </c>
-      <c r="L45" s="71" t="n"/>
-      <c r="M45" s="69" t="n"/>
-      <c r="N45" s="69" t="n"/>
-      <c r="O45" s="71" t="n"/>
-      <c r="P45" s="69" t="n"/>
+      <c r="L45" s="72" t="n"/>
+      <c r="M45" s="70" t="n"/>
+      <c r="N45" s="70" t="n"/>
+      <c r="O45" s="72" t="n"/>
+      <c r="P45" s="70" t="n"/>
       <c r="Q45" s="67">
         <f>IFERROR(IF(J45="","",J45-TODAY()),"")</f>
         <v/>
@@ -3591,27 +3782,31 @@
         <f>IFERROR(IF(B45="","Vacant",IF(Q45&lt;0,"Expired",IF(Q45&lt;=30,"Expiring Soon",IF(Q45&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S45" s="69" t="n"/>
+      <c r="T45" s="69" t="n"/>
+      <c r="U45" s="69" t="n"/>
+      <c r="V45" s="69" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="72" t="n"/>
-      <c r="B46" s="72" t="n"/>
-      <c r="C46" s="72" t="n"/>
-      <c r="D46" s="72" t="n"/>
-      <c r="E46" s="72" t="n"/>
-      <c r="F46" s="72" t="n"/>
-      <c r="G46" s="72" t="n"/>
-      <c r="H46" s="72" t="n"/>
-      <c r="I46" s="73" t="n"/>
-      <c r="J46" s="73" t="n"/>
+      <c r="A46" s="73" t="n"/>
+      <c r="B46" s="73" t="n"/>
+      <c r="C46" s="73" t="n"/>
+      <c r="D46" s="73" t="n"/>
+      <c r="E46" s="73" t="n"/>
+      <c r="F46" s="73" t="n"/>
+      <c r="G46" s="73" t="n"/>
+      <c r="H46" s="73" t="n"/>
+      <c r="I46" s="74" t="n"/>
+      <c r="J46" s="74" t="n"/>
       <c r="K46" s="65">
         <f>IFERROR(DATEDIF(I46,J46,"M"),"")</f>
         <v/>
       </c>
-      <c r="L46" s="74" t="n"/>
-      <c r="M46" s="72" t="n"/>
-      <c r="N46" s="72" t="n"/>
-      <c r="O46" s="74" t="n"/>
-      <c r="P46" s="72" t="n"/>
+      <c r="L46" s="75" t="n"/>
+      <c r="M46" s="73" t="n"/>
+      <c r="N46" s="73" t="n"/>
+      <c r="O46" s="75" t="n"/>
+      <c r="P46" s="73" t="n"/>
       <c r="Q46" s="67">
         <f>IFERROR(IF(J46="","",J46-TODAY()),"")</f>
         <v/>
@@ -3620,27 +3815,31 @@
         <f>IFERROR(IF(B46="","Vacant",IF(Q46&lt;0,"Expired",IF(Q46&lt;=30,"Expiring Soon",IF(Q46&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S46" s="69" t="n"/>
+      <c r="T46" s="69" t="n"/>
+      <c r="U46" s="69" t="n"/>
+      <c r="V46" s="69" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="69" t="n"/>
-      <c r="B47" s="69" t="n"/>
-      <c r="C47" s="69" t="n"/>
-      <c r="D47" s="69" t="n"/>
-      <c r="E47" s="69" t="n"/>
-      <c r="F47" s="69" t="n"/>
-      <c r="G47" s="69" t="n"/>
-      <c r="H47" s="69" t="n"/>
-      <c r="I47" s="70" t="n"/>
-      <c r="J47" s="70" t="n"/>
+      <c r="A47" s="70" t="n"/>
+      <c r="B47" s="70" t="n"/>
+      <c r="C47" s="70" t="n"/>
+      <c r="D47" s="70" t="n"/>
+      <c r="E47" s="70" t="n"/>
+      <c r="F47" s="70" t="n"/>
+      <c r="G47" s="70" t="n"/>
+      <c r="H47" s="70" t="n"/>
+      <c r="I47" s="71" t="n"/>
+      <c r="J47" s="71" t="n"/>
       <c r="K47" s="65">
         <f>IFERROR(DATEDIF(I47,J47,"M"),"")</f>
         <v/>
       </c>
-      <c r="L47" s="71" t="n"/>
-      <c r="M47" s="69" t="n"/>
-      <c r="N47" s="69" t="n"/>
-      <c r="O47" s="71" t="n"/>
-      <c r="P47" s="69" t="n"/>
+      <c r="L47" s="72" t="n"/>
+      <c r="M47" s="70" t="n"/>
+      <c r="N47" s="70" t="n"/>
+      <c r="O47" s="72" t="n"/>
+      <c r="P47" s="70" t="n"/>
       <c r="Q47" s="67">
         <f>IFERROR(IF(J47="","",J47-TODAY()),"")</f>
         <v/>
@@ -3649,27 +3848,31 @@
         <f>IFERROR(IF(B47="","Vacant",IF(Q47&lt;0,"Expired",IF(Q47&lt;=30,"Expiring Soon",IF(Q47&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S47" s="69" t="n"/>
+      <c r="T47" s="69" t="n"/>
+      <c r="U47" s="69" t="n"/>
+      <c r="V47" s="69" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="72" t="n"/>
-      <c r="B48" s="72" t="n"/>
-      <c r="C48" s="72" t="n"/>
-      <c r="D48" s="72" t="n"/>
-      <c r="E48" s="72" t="n"/>
-      <c r="F48" s="72" t="n"/>
-      <c r="G48" s="72" t="n"/>
-      <c r="H48" s="72" t="n"/>
-      <c r="I48" s="73" t="n"/>
-      <c r="J48" s="73" t="n"/>
+      <c r="A48" s="73" t="n"/>
+      <c r="B48" s="73" t="n"/>
+      <c r="C48" s="73" t="n"/>
+      <c r="D48" s="73" t="n"/>
+      <c r="E48" s="73" t="n"/>
+      <c r="F48" s="73" t="n"/>
+      <c r="G48" s="73" t="n"/>
+      <c r="H48" s="73" t="n"/>
+      <c r="I48" s="74" t="n"/>
+      <c r="J48" s="74" t="n"/>
       <c r="K48" s="65">
         <f>IFERROR(DATEDIF(I48,J48,"M"),"")</f>
         <v/>
       </c>
-      <c r="L48" s="74" t="n"/>
-      <c r="M48" s="72" t="n"/>
-      <c r="N48" s="72" t="n"/>
-      <c r="O48" s="74" t="n"/>
-      <c r="P48" s="72" t="n"/>
+      <c r="L48" s="75" t="n"/>
+      <c r="M48" s="73" t="n"/>
+      <c r="N48" s="73" t="n"/>
+      <c r="O48" s="75" t="n"/>
+      <c r="P48" s="73" t="n"/>
       <c r="Q48" s="67">
         <f>IFERROR(IF(J48="","",J48-TODAY()),"")</f>
         <v/>
@@ -3678,27 +3881,31 @@
         <f>IFERROR(IF(B48="","Vacant",IF(Q48&lt;0,"Expired",IF(Q48&lt;=30,"Expiring Soon",IF(Q48&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S48" s="69" t="n"/>
+      <c r="T48" s="69" t="n"/>
+      <c r="U48" s="69" t="n"/>
+      <c r="V48" s="69" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="69" t="n"/>
-      <c r="B49" s="69" t="n"/>
-      <c r="C49" s="69" t="n"/>
-      <c r="D49" s="69" t="n"/>
-      <c r="E49" s="69" t="n"/>
-      <c r="F49" s="69" t="n"/>
-      <c r="G49" s="69" t="n"/>
-      <c r="H49" s="69" t="n"/>
-      <c r="I49" s="70" t="n"/>
-      <c r="J49" s="70" t="n"/>
+      <c r="A49" s="70" t="n"/>
+      <c r="B49" s="70" t="n"/>
+      <c r="C49" s="70" t="n"/>
+      <c r="D49" s="70" t="n"/>
+      <c r="E49" s="70" t="n"/>
+      <c r="F49" s="70" t="n"/>
+      <c r="G49" s="70" t="n"/>
+      <c r="H49" s="70" t="n"/>
+      <c r="I49" s="71" t="n"/>
+      <c r="J49" s="71" t="n"/>
       <c r="K49" s="65">
         <f>IFERROR(DATEDIF(I49,J49,"M"),"")</f>
         <v/>
       </c>
-      <c r="L49" s="71" t="n"/>
-      <c r="M49" s="69" t="n"/>
-      <c r="N49" s="69" t="n"/>
-      <c r="O49" s="71" t="n"/>
-      <c r="P49" s="69" t="n"/>
+      <c r="L49" s="72" t="n"/>
+      <c r="M49" s="70" t="n"/>
+      <c r="N49" s="70" t="n"/>
+      <c r="O49" s="72" t="n"/>
+      <c r="P49" s="70" t="n"/>
       <c r="Q49" s="67">
         <f>IFERROR(IF(J49="","",J49-TODAY()),"")</f>
         <v/>
@@ -3707,27 +3914,31 @@
         <f>IFERROR(IF(B49="","Vacant",IF(Q49&lt;0,"Expired",IF(Q49&lt;=30,"Expiring Soon",IF(Q49&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S49" s="69" t="n"/>
+      <c r="T49" s="69" t="n"/>
+      <c r="U49" s="69" t="n"/>
+      <c r="V49" s="69" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="72" t="n"/>
-      <c r="B50" s="72" t="n"/>
-      <c r="C50" s="72" t="n"/>
-      <c r="D50" s="72" t="n"/>
-      <c r="E50" s="72" t="n"/>
-      <c r="F50" s="72" t="n"/>
-      <c r="G50" s="72" t="n"/>
-      <c r="H50" s="72" t="n"/>
-      <c r="I50" s="73" t="n"/>
-      <c r="J50" s="73" t="n"/>
+      <c r="A50" s="73" t="n"/>
+      <c r="B50" s="73" t="n"/>
+      <c r="C50" s="73" t="n"/>
+      <c r="D50" s="73" t="n"/>
+      <c r="E50" s="73" t="n"/>
+      <c r="F50" s="73" t="n"/>
+      <c r="G50" s="73" t="n"/>
+      <c r="H50" s="73" t="n"/>
+      <c r="I50" s="74" t="n"/>
+      <c r="J50" s="74" t="n"/>
       <c r="K50" s="65">
         <f>IFERROR(DATEDIF(I50,J50,"M"),"")</f>
         <v/>
       </c>
-      <c r="L50" s="74" t="n"/>
-      <c r="M50" s="72" t="n"/>
-      <c r="N50" s="72" t="n"/>
-      <c r="O50" s="74" t="n"/>
-      <c r="P50" s="72" t="n"/>
+      <c r="L50" s="75" t="n"/>
+      <c r="M50" s="73" t="n"/>
+      <c r="N50" s="73" t="n"/>
+      <c r="O50" s="75" t="n"/>
+      <c r="P50" s="73" t="n"/>
       <c r="Q50" s="67">
         <f>IFERROR(IF(J50="","",J50-TODAY()),"")</f>
         <v/>
@@ -3736,27 +3947,31 @@
         <f>IFERROR(IF(B50="","Vacant",IF(Q50&lt;0,"Expired",IF(Q50&lt;=30,"Expiring Soon",IF(Q50&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S50" s="69" t="n"/>
+      <c r="T50" s="69" t="n"/>
+      <c r="U50" s="69" t="n"/>
+      <c r="V50" s="69" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="69" t="n"/>
-      <c r="B51" s="69" t="n"/>
-      <c r="C51" s="69" t="n"/>
-      <c r="D51" s="69" t="n"/>
-      <c r="E51" s="69" t="n"/>
-      <c r="F51" s="69" t="n"/>
-      <c r="G51" s="69" t="n"/>
-      <c r="H51" s="69" t="n"/>
-      <c r="I51" s="70" t="n"/>
-      <c r="J51" s="70" t="n"/>
+      <c r="A51" s="70" t="n"/>
+      <c r="B51" s="70" t="n"/>
+      <c r="C51" s="70" t="n"/>
+      <c r="D51" s="70" t="n"/>
+      <c r="E51" s="70" t="n"/>
+      <c r="F51" s="70" t="n"/>
+      <c r="G51" s="70" t="n"/>
+      <c r="H51" s="70" t="n"/>
+      <c r="I51" s="71" t="n"/>
+      <c r="J51" s="71" t="n"/>
       <c r="K51" s="65">
         <f>IFERROR(DATEDIF(I51,J51,"M"),"")</f>
         <v/>
       </c>
-      <c r="L51" s="71" t="n"/>
-      <c r="M51" s="69" t="n"/>
-      <c r="N51" s="69" t="n"/>
-      <c r="O51" s="71" t="n"/>
-      <c r="P51" s="69" t="n"/>
+      <c r="L51" s="72" t="n"/>
+      <c r="M51" s="70" t="n"/>
+      <c r="N51" s="70" t="n"/>
+      <c r="O51" s="72" t="n"/>
+      <c r="P51" s="70" t="n"/>
       <c r="Q51" s="67">
         <f>IFERROR(IF(J51="","",J51-TODAY()),"")</f>
         <v/>
@@ -3765,27 +3980,31 @@
         <f>IFERROR(IF(B51="","Vacant",IF(Q51&lt;0,"Expired",IF(Q51&lt;=30,"Expiring Soon",IF(Q51&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S51" s="69" t="n"/>
+      <c r="T51" s="69" t="n"/>
+      <c r="U51" s="69" t="n"/>
+      <c r="V51" s="69" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="72" t="n"/>
-      <c r="B52" s="72" t="n"/>
-      <c r="C52" s="72" t="n"/>
-      <c r="D52" s="72" t="n"/>
-      <c r="E52" s="72" t="n"/>
-      <c r="F52" s="72" t="n"/>
-      <c r="G52" s="72" t="n"/>
-      <c r="H52" s="72" t="n"/>
-      <c r="I52" s="73" t="n"/>
-      <c r="J52" s="73" t="n"/>
+      <c r="A52" s="73" t="n"/>
+      <c r="B52" s="73" t="n"/>
+      <c r="C52" s="73" t="n"/>
+      <c r="D52" s="73" t="n"/>
+      <c r="E52" s="73" t="n"/>
+      <c r="F52" s="73" t="n"/>
+      <c r="G52" s="73" t="n"/>
+      <c r="H52" s="73" t="n"/>
+      <c r="I52" s="74" t="n"/>
+      <c r="J52" s="74" t="n"/>
       <c r="K52" s="65">
         <f>IFERROR(DATEDIF(I52,J52,"M"),"")</f>
         <v/>
       </c>
-      <c r="L52" s="74" t="n"/>
-      <c r="M52" s="72" t="n"/>
-      <c r="N52" s="72" t="n"/>
-      <c r="O52" s="74" t="n"/>
-      <c r="P52" s="72" t="n"/>
+      <c r="L52" s="75" t="n"/>
+      <c r="M52" s="73" t="n"/>
+      <c r="N52" s="73" t="n"/>
+      <c r="O52" s="75" t="n"/>
+      <c r="P52" s="73" t="n"/>
       <c r="Q52" s="67">
         <f>IFERROR(IF(J52="","",J52-TODAY()),"")</f>
         <v/>
@@ -3794,27 +4013,31 @@
         <f>IFERROR(IF(B52="","Vacant",IF(Q52&lt;0,"Expired",IF(Q52&lt;=30,"Expiring Soon",IF(Q52&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S52" s="69" t="n"/>
+      <c r="T52" s="69" t="n"/>
+      <c r="U52" s="69" t="n"/>
+      <c r="V52" s="69" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="69" t="n"/>
-      <c r="B53" s="69" t="n"/>
-      <c r="C53" s="69" t="n"/>
-      <c r="D53" s="69" t="n"/>
-      <c r="E53" s="69" t="n"/>
-      <c r="F53" s="69" t="n"/>
-      <c r="G53" s="69" t="n"/>
-      <c r="H53" s="69" t="n"/>
-      <c r="I53" s="70" t="n"/>
-      <c r="J53" s="70" t="n"/>
+      <c r="A53" s="70" t="n"/>
+      <c r="B53" s="70" t="n"/>
+      <c r="C53" s="70" t="n"/>
+      <c r="D53" s="70" t="n"/>
+      <c r="E53" s="70" t="n"/>
+      <c r="F53" s="70" t="n"/>
+      <c r="G53" s="70" t="n"/>
+      <c r="H53" s="70" t="n"/>
+      <c r="I53" s="71" t="n"/>
+      <c r="J53" s="71" t="n"/>
       <c r="K53" s="65">
         <f>IFERROR(DATEDIF(I53,J53,"M"),"")</f>
         <v/>
       </c>
-      <c r="L53" s="71" t="n"/>
-      <c r="M53" s="69" t="n"/>
-      <c r="N53" s="69" t="n"/>
-      <c r="O53" s="71" t="n"/>
-      <c r="P53" s="69" t="n"/>
+      <c r="L53" s="72" t="n"/>
+      <c r="M53" s="70" t="n"/>
+      <c r="N53" s="70" t="n"/>
+      <c r="O53" s="72" t="n"/>
+      <c r="P53" s="70" t="n"/>
       <c r="Q53" s="67">
         <f>IFERROR(IF(J53="","",J53-TODAY()),"")</f>
         <v/>
@@ -3823,11 +4046,15 @@
         <f>IFERROR(IF(B53="","Vacant",IF(Q53&lt;0,"Expired",IF(Q53&lt;=30,"Expiring Soon",IF(Q53&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
+      <c r="S53" s="69" t="n"/>
+      <c r="T53" s="69" t="n"/>
+      <c r="U53" s="69" t="n"/>
+      <c r="V53" s="69" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:R2"/>
-    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A2:V2"/>
+    <mergeCell ref="A1:V1"/>
   </mergeCells>
   <conditionalFormatting sqref="R4:R53">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -4031,7 +4258,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="75" t="inlineStr">
+      <c r="A1" s="76" t="inlineStr">
         <is>
           <t>📋  LEASE AGREEMENTS &amp; RENEWALS</t>
         </is>
@@ -4045,82 +4272,82 @@
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="76" t="inlineStr">
+      <c r="A3" s="77" t="inlineStr">
         <is>
           <t>Agr. ID</t>
         </is>
       </c>
-      <c r="B3" s="76" t="inlineStr">
+      <c r="B3" s="77" t="inlineStr">
         <is>
           <t>Tenant ID</t>
         </is>
       </c>
-      <c r="C3" s="76" t="inlineStr">
+      <c r="C3" s="77" t="inlineStr">
         <is>
           <t>Tenant Name</t>
         </is>
       </c>
-      <c r="D3" s="76" t="inlineStr">
+      <c r="D3" s="77" t="inlineStr">
         <is>
           <t>Unit No.</t>
         </is>
       </c>
-      <c r="E3" s="76" t="inlineStr">
+      <c r="E3" s="77" t="inlineStr">
         <is>
           <t>Original Start</t>
         </is>
       </c>
-      <c r="F3" s="76" t="inlineStr">
+      <c r="F3" s="77" t="inlineStr">
         <is>
           <t>Lease Start</t>
         </is>
       </c>
-      <c r="G3" s="76" t="inlineStr">
+      <c r="G3" s="77" t="inlineStr">
         <is>
           <t>Lease End</t>
         </is>
       </c>
-      <c r="H3" s="76" t="inlineStr">
+      <c r="H3" s="77" t="inlineStr">
         <is>
           <t>Renewal?</t>
         </is>
       </c>
-      <c r="I3" s="76" t="inlineStr">
+      <c r="I3" s="77" t="inlineStr">
         <is>
           <t>Renewal No.</t>
         </is>
       </c>
-      <c r="J3" s="76" t="inlineStr">
+      <c r="J3" s="77" t="inlineStr">
         <is>
           <t>Term (months)</t>
         </is>
       </c>
-      <c r="K3" s="76" t="inlineStr">
+      <c r="K3" s="77" t="inlineStr">
         <is>
           <t>Annual Rent</t>
         </is>
       </c>
-      <c r="L3" s="76" t="inlineStr">
+      <c r="L3" s="77" t="inlineStr">
         <is>
           <t>Monthly Rent</t>
         </is>
       </c>
-      <c r="M3" s="76" t="inlineStr">
+      <c r="M3" s="77" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="N3" s="76" t="inlineStr">
+      <c r="N3" s="77" t="inlineStr">
         <is>
           <t>Rent Increment%</t>
         </is>
       </c>
-      <c r="O3" s="76" t="inlineStr">
+      <c r="O3" s="77" t="inlineStr">
         <is>
           <t>Next Review Date</t>
         </is>
       </c>
-      <c r="P3" s="76" t="inlineStr">
+      <c r="P3" s="77" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -4171,7 +4398,7 @@
       <c r="K4" s="66" t="n">
         <v>42000</v>
       </c>
-      <c r="L4" s="77">
+      <c r="L4" s="78">
         <f>IFERROR(IF(K4="","",K4/12),"")</f>
         <v/>
       </c>
@@ -4180,1337 +4407,1337 @@
           <t>GHS</t>
         </is>
       </c>
-      <c r="N4" s="78" t="n">
+      <c r="N4" s="79" t="n">
         <v>0.05</v>
       </c>
-      <c r="O4" s="79">
+      <c r="O4" s="80">
         <f>IFERROR(IF(G4="","",G4-365),"")</f>
         <v/>
       </c>
       <c r="P4" s="63" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="69" t="n"/>
-      <c r="B5" s="69" t="n"/>
-      <c r="C5" s="69" t="n"/>
-      <c r="D5" s="69" t="n"/>
-      <c r="E5" s="70" t="n"/>
-      <c r="F5" s="70" t="n"/>
-      <c r="G5" s="70" t="n"/>
-      <c r="H5" s="69" t="n"/>
-      <c r="I5" s="69" t="n"/>
+      <c r="A5" s="70" t="n"/>
+      <c r="B5" s="70" t="n"/>
+      <c r="C5" s="70" t="n"/>
+      <c r="D5" s="70" t="n"/>
+      <c r="E5" s="71" t="n"/>
+      <c r="F5" s="71" t="n"/>
+      <c r="G5" s="71" t="n"/>
+      <c r="H5" s="70" t="n"/>
+      <c r="I5" s="70" t="n"/>
       <c r="J5" s="65">
         <f>IFERROR(DATEDIF(F5,G5,"M"),"")</f>
         <v/>
       </c>
-      <c r="K5" s="71" t="n"/>
-      <c r="L5" s="77">
+      <c r="K5" s="72" t="n"/>
+      <c r="L5" s="78">
         <f>IFERROR(IF(K5="","",K5/12),"")</f>
         <v/>
       </c>
-      <c r="M5" s="69" t="n"/>
-      <c r="N5" s="80" t="n"/>
-      <c r="O5" s="79">
+      <c r="M5" s="70" t="n"/>
+      <c r="N5" s="81" t="n"/>
+      <c r="O5" s="80">
         <f>IFERROR(IF(G5="","",G5-365),"")</f>
         <v/>
       </c>
-      <c r="P5" s="69" t="n"/>
+      <c r="P5" s="70" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="72" t="n"/>
-      <c r="B6" s="72" t="n"/>
-      <c r="C6" s="72" t="n"/>
-      <c r="D6" s="72" t="n"/>
-      <c r="E6" s="73" t="n"/>
-      <c r="F6" s="73" t="n"/>
-      <c r="G6" s="73" t="n"/>
-      <c r="H6" s="72" t="n"/>
-      <c r="I6" s="72" t="n"/>
+      <c r="A6" s="73" t="n"/>
+      <c r="B6" s="73" t="n"/>
+      <c r="C6" s="73" t="n"/>
+      <c r="D6" s="73" t="n"/>
+      <c r="E6" s="74" t="n"/>
+      <c r="F6" s="74" t="n"/>
+      <c r="G6" s="74" t="n"/>
+      <c r="H6" s="73" t="n"/>
+      <c r="I6" s="73" t="n"/>
       <c r="J6" s="65">
         <f>IFERROR(DATEDIF(F6,G6,"M"),"")</f>
         <v/>
       </c>
-      <c r="K6" s="74" t="n"/>
-      <c r="L6" s="77">
+      <c r="K6" s="75" t="n"/>
+      <c r="L6" s="78">
         <f>IFERROR(IF(K6="","",K6/12),"")</f>
         <v/>
       </c>
-      <c r="M6" s="72" t="n"/>
-      <c r="N6" s="81" t="n"/>
-      <c r="O6" s="79">
+      <c r="M6" s="73" t="n"/>
+      <c r="N6" s="82" t="n"/>
+      <c r="O6" s="80">
         <f>IFERROR(IF(G6="","",G6-365),"")</f>
         <v/>
       </c>
-      <c r="P6" s="72" t="n"/>
+      <c r="P6" s="73" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="69" t="n"/>
-      <c r="B7" s="69" t="n"/>
-      <c r="C7" s="69" t="n"/>
-      <c r="D7" s="69" t="n"/>
-      <c r="E7" s="70" t="n"/>
-      <c r="F7" s="70" t="n"/>
-      <c r="G7" s="70" t="n"/>
-      <c r="H7" s="69" t="n"/>
-      <c r="I7" s="69" t="n"/>
+      <c r="A7" s="70" t="n"/>
+      <c r="B7" s="70" t="n"/>
+      <c r="C7" s="70" t="n"/>
+      <c r="D7" s="70" t="n"/>
+      <c r="E7" s="71" t="n"/>
+      <c r="F7" s="71" t="n"/>
+      <c r="G7" s="71" t="n"/>
+      <c r="H7" s="70" t="n"/>
+      <c r="I7" s="70" t="n"/>
       <c r="J7" s="65">
         <f>IFERROR(DATEDIF(F7,G7,"M"),"")</f>
         <v/>
       </c>
-      <c r="K7" s="71" t="n"/>
-      <c r="L7" s="77">
+      <c r="K7" s="72" t="n"/>
+      <c r="L7" s="78">
         <f>IFERROR(IF(K7="","",K7/12),"")</f>
         <v/>
       </c>
-      <c r="M7" s="69" t="n"/>
-      <c r="N7" s="80" t="n"/>
-      <c r="O7" s="79">
+      <c r="M7" s="70" t="n"/>
+      <c r="N7" s="81" t="n"/>
+      <c r="O7" s="80">
         <f>IFERROR(IF(G7="","",G7-365),"")</f>
         <v/>
       </c>
-      <c r="P7" s="69" t="n"/>
+      <c r="P7" s="70" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="72" t="n"/>
-      <c r="B8" s="72" t="n"/>
-      <c r="C8" s="72" t="n"/>
-      <c r="D8" s="72" t="n"/>
-      <c r="E8" s="73" t="n"/>
-      <c r="F8" s="73" t="n"/>
-      <c r="G8" s="73" t="n"/>
-      <c r="H8" s="72" t="n"/>
-      <c r="I8" s="72" t="n"/>
+      <c r="A8" s="73" t="n"/>
+      <c r="B8" s="73" t="n"/>
+      <c r="C8" s="73" t="n"/>
+      <c r="D8" s="73" t="n"/>
+      <c r="E8" s="74" t="n"/>
+      <c r="F8" s="74" t="n"/>
+      <c r="G8" s="74" t="n"/>
+      <c r="H8" s="73" t="n"/>
+      <c r="I8" s="73" t="n"/>
       <c r="J8" s="65">
         <f>IFERROR(DATEDIF(F8,G8,"M"),"")</f>
         <v/>
       </c>
-      <c r="K8" s="74" t="n"/>
-      <c r="L8" s="77">
+      <c r="K8" s="75" t="n"/>
+      <c r="L8" s="78">
         <f>IFERROR(IF(K8="","",K8/12),"")</f>
         <v/>
       </c>
-      <c r="M8" s="72" t="n"/>
-      <c r="N8" s="81" t="n"/>
-      <c r="O8" s="79">
+      <c r="M8" s="73" t="n"/>
+      <c r="N8" s="82" t="n"/>
+      <c r="O8" s="80">
         <f>IFERROR(IF(G8="","",G8-365),"")</f>
         <v/>
       </c>
-      <c r="P8" s="72" t="n"/>
+      <c r="P8" s="73" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="69" t="n"/>
-      <c r="B9" s="69" t="n"/>
-      <c r="C9" s="69" t="n"/>
-      <c r="D9" s="69" t="n"/>
-      <c r="E9" s="70" t="n"/>
-      <c r="F9" s="70" t="n"/>
-      <c r="G9" s="70" t="n"/>
-      <c r="H9" s="69" t="n"/>
-      <c r="I9" s="69" t="n"/>
+      <c r="A9" s="70" t="n"/>
+      <c r="B9" s="70" t="n"/>
+      <c r="C9" s="70" t="n"/>
+      <c r="D9" s="70" t="n"/>
+      <c r="E9" s="71" t="n"/>
+      <c r="F9" s="71" t="n"/>
+      <c r="G9" s="71" t="n"/>
+      <c r="H9" s="70" t="n"/>
+      <c r="I9" s="70" t="n"/>
       <c r="J9" s="65">
         <f>IFERROR(DATEDIF(F9,G9,"M"),"")</f>
         <v/>
       </c>
-      <c r="K9" s="71" t="n"/>
-      <c r="L9" s="77">
+      <c r="K9" s="72" t="n"/>
+      <c r="L9" s="78">
         <f>IFERROR(IF(K9="","",K9/12),"")</f>
         <v/>
       </c>
-      <c r="M9" s="69" t="n"/>
-      <c r="N9" s="80" t="n"/>
-      <c r="O9" s="79">
+      <c r="M9" s="70" t="n"/>
+      <c r="N9" s="81" t="n"/>
+      <c r="O9" s="80">
         <f>IFERROR(IF(G9="","",G9-365),"")</f>
         <v/>
       </c>
-      <c r="P9" s="69" t="n"/>
+      <c r="P9" s="70" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="72" t="n"/>
-      <c r="B10" s="72" t="n"/>
-      <c r="C10" s="72" t="n"/>
-      <c r="D10" s="72" t="n"/>
-      <c r="E10" s="73" t="n"/>
-      <c r="F10" s="73" t="n"/>
-      <c r="G10" s="73" t="n"/>
-      <c r="H10" s="72" t="n"/>
-      <c r="I10" s="72" t="n"/>
+      <c r="A10" s="73" t="n"/>
+      <c r="B10" s="73" t="n"/>
+      <c r="C10" s="73" t="n"/>
+      <c r="D10" s="73" t="n"/>
+      <c r="E10" s="74" t="n"/>
+      <c r="F10" s="74" t="n"/>
+      <c r="G10" s="74" t="n"/>
+      <c r="H10" s="73" t="n"/>
+      <c r="I10" s="73" t="n"/>
       <c r="J10" s="65">
         <f>IFERROR(DATEDIF(F10,G10,"M"),"")</f>
         <v/>
       </c>
-      <c r="K10" s="74" t="n"/>
-      <c r="L10" s="77">
+      <c r="K10" s="75" t="n"/>
+      <c r="L10" s="78">
         <f>IFERROR(IF(K10="","",K10/12),"")</f>
         <v/>
       </c>
-      <c r="M10" s="72" t="n"/>
-      <c r="N10" s="81" t="n"/>
-      <c r="O10" s="79">
+      <c r="M10" s="73" t="n"/>
+      <c r="N10" s="82" t="n"/>
+      <c r="O10" s="80">
         <f>IFERROR(IF(G10="","",G10-365),"")</f>
         <v/>
       </c>
-      <c r="P10" s="72" t="n"/>
+      <c r="P10" s="73" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="69" t="n"/>
-      <c r="B11" s="69" t="n"/>
-      <c r="C11" s="69" t="n"/>
-      <c r="D11" s="69" t="n"/>
-      <c r="E11" s="70" t="n"/>
-      <c r="F11" s="70" t="n"/>
-      <c r="G11" s="70" t="n"/>
-      <c r="H11" s="69" t="n"/>
-      <c r="I11" s="69" t="n"/>
+      <c r="A11" s="70" t="n"/>
+      <c r="B11" s="70" t="n"/>
+      <c r="C11" s="70" t="n"/>
+      <c r="D11" s="70" t="n"/>
+      <c r="E11" s="71" t="n"/>
+      <c r="F11" s="71" t="n"/>
+      <c r="G11" s="71" t="n"/>
+      <c r="H11" s="70" t="n"/>
+      <c r="I11" s="70" t="n"/>
       <c r="J11" s="65">
         <f>IFERROR(DATEDIF(F11,G11,"M"),"")</f>
         <v/>
       </c>
-      <c r="K11" s="71" t="n"/>
-      <c r="L11" s="77">
+      <c r="K11" s="72" t="n"/>
+      <c r="L11" s="78">
         <f>IFERROR(IF(K11="","",K11/12),"")</f>
         <v/>
       </c>
-      <c r="M11" s="69" t="n"/>
-      <c r="N11" s="80" t="n"/>
-      <c r="O11" s="79">
+      <c r="M11" s="70" t="n"/>
+      <c r="N11" s="81" t="n"/>
+      <c r="O11" s="80">
         <f>IFERROR(IF(G11="","",G11-365),"")</f>
         <v/>
       </c>
-      <c r="P11" s="69" t="n"/>
+      <c r="P11" s="70" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="72" t="n"/>
-      <c r="B12" s="72" t="n"/>
-      <c r="C12" s="72" t="n"/>
-      <c r="D12" s="72" t="n"/>
-      <c r="E12" s="73" t="n"/>
-      <c r="F12" s="73" t="n"/>
-      <c r="G12" s="73" t="n"/>
-      <c r="H12" s="72" t="n"/>
-      <c r="I12" s="72" t="n"/>
+      <c r="A12" s="73" t="n"/>
+      <c r="B12" s="73" t="n"/>
+      <c r="C12" s="73" t="n"/>
+      <c r="D12" s="73" t="n"/>
+      <c r="E12" s="74" t="n"/>
+      <c r="F12" s="74" t="n"/>
+      <c r="G12" s="74" t="n"/>
+      <c r="H12" s="73" t="n"/>
+      <c r="I12" s="73" t="n"/>
       <c r="J12" s="65">
         <f>IFERROR(DATEDIF(F12,G12,"M"),"")</f>
         <v/>
       </c>
-      <c r="K12" s="74" t="n"/>
-      <c r="L12" s="77">
+      <c r="K12" s="75" t="n"/>
+      <c r="L12" s="78">
         <f>IFERROR(IF(K12="","",K12/12),"")</f>
         <v/>
       </c>
-      <c r="M12" s="72" t="n"/>
-      <c r="N12" s="81" t="n"/>
-      <c r="O12" s="79">
+      <c r="M12" s="73" t="n"/>
+      <c r="N12" s="82" t="n"/>
+      <c r="O12" s="80">
         <f>IFERROR(IF(G12="","",G12-365),"")</f>
         <v/>
       </c>
-      <c r="P12" s="72" t="n"/>
+      <c r="P12" s="73" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="69" t="n"/>
-      <c r="B13" s="69" t="n"/>
-      <c r="C13" s="69" t="n"/>
-      <c r="D13" s="69" t="n"/>
-      <c r="E13" s="70" t="n"/>
-      <c r="F13" s="70" t="n"/>
-      <c r="G13" s="70" t="n"/>
-      <c r="H13" s="69" t="n"/>
-      <c r="I13" s="69" t="n"/>
+      <c r="A13" s="70" t="n"/>
+      <c r="B13" s="70" t="n"/>
+      <c r="C13" s="70" t="n"/>
+      <c r="D13" s="70" t="n"/>
+      <c r="E13" s="71" t="n"/>
+      <c r="F13" s="71" t="n"/>
+      <c r="G13" s="71" t="n"/>
+      <c r="H13" s="70" t="n"/>
+      <c r="I13" s="70" t="n"/>
       <c r="J13" s="65">
         <f>IFERROR(DATEDIF(F13,G13,"M"),"")</f>
         <v/>
       </c>
-      <c r="K13" s="71" t="n"/>
-      <c r="L13" s="77">
+      <c r="K13" s="72" t="n"/>
+      <c r="L13" s="78">
         <f>IFERROR(IF(K13="","",K13/12),"")</f>
         <v/>
       </c>
-      <c r="M13" s="69" t="n"/>
-      <c r="N13" s="80" t="n"/>
-      <c r="O13" s="79">
+      <c r="M13" s="70" t="n"/>
+      <c r="N13" s="81" t="n"/>
+      <c r="O13" s="80">
         <f>IFERROR(IF(G13="","",G13-365),"")</f>
         <v/>
       </c>
-      <c r="P13" s="69" t="n"/>
+      <c r="P13" s="70" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="72" t="n"/>
-      <c r="B14" s="72" t="n"/>
-      <c r="C14" s="72" t="n"/>
-      <c r="D14" s="72" t="n"/>
-      <c r="E14" s="73" t="n"/>
-      <c r="F14" s="73" t="n"/>
-      <c r="G14" s="73" t="n"/>
-      <c r="H14" s="72" t="n"/>
-      <c r="I14" s="72" t="n"/>
+      <c r="A14" s="73" t="n"/>
+      <c r="B14" s="73" t="n"/>
+      <c r="C14" s="73" t="n"/>
+      <c r="D14" s="73" t="n"/>
+      <c r="E14" s="74" t="n"/>
+      <c r="F14" s="74" t="n"/>
+      <c r="G14" s="74" t="n"/>
+      <c r="H14" s="73" t="n"/>
+      <c r="I14" s="73" t="n"/>
       <c r="J14" s="65">
         <f>IFERROR(DATEDIF(F14,G14,"M"),"")</f>
         <v/>
       </c>
-      <c r="K14" s="74" t="n"/>
-      <c r="L14" s="77">
+      <c r="K14" s="75" t="n"/>
+      <c r="L14" s="78">
         <f>IFERROR(IF(K14="","",K14/12),"")</f>
         <v/>
       </c>
-      <c r="M14" s="72" t="n"/>
-      <c r="N14" s="81" t="n"/>
-      <c r="O14" s="79">
+      <c r="M14" s="73" t="n"/>
+      <c r="N14" s="82" t="n"/>
+      <c r="O14" s="80">
         <f>IFERROR(IF(G14="","",G14-365),"")</f>
         <v/>
       </c>
-      <c r="P14" s="72" t="n"/>
+      <c r="P14" s="73" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="69" t="n"/>
-      <c r="B15" s="69" t="n"/>
-      <c r="C15" s="69" t="n"/>
-      <c r="D15" s="69" t="n"/>
-      <c r="E15" s="70" t="n"/>
-      <c r="F15" s="70" t="n"/>
-      <c r="G15" s="70" t="n"/>
-      <c r="H15" s="69" t="n"/>
-      <c r="I15" s="69" t="n"/>
+      <c r="A15" s="70" t="n"/>
+      <c r="B15" s="70" t="n"/>
+      <c r="C15" s="70" t="n"/>
+      <c r="D15" s="70" t="n"/>
+      <c r="E15" s="71" t="n"/>
+      <c r="F15" s="71" t="n"/>
+      <c r="G15" s="71" t="n"/>
+      <c r="H15" s="70" t="n"/>
+      <c r="I15" s="70" t="n"/>
       <c r="J15" s="65">
         <f>IFERROR(DATEDIF(F15,G15,"M"),"")</f>
         <v/>
       </c>
-      <c r="K15" s="71" t="n"/>
-      <c r="L15" s="77">
+      <c r="K15" s="72" t="n"/>
+      <c r="L15" s="78">
         <f>IFERROR(IF(K15="","",K15/12),"")</f>
         <v/>
       </c>
-      <c r="M15" s="69" t="n"/>
-      <c r="N15" s="80" t="n"/>
-      <c r="O15" s="79">
+      <c r="M15" s="70" t="n"/>
+      <c r="N15" s="81" t="n"/>
+      <c r="O15" s="80">
         <f>IFERROR(IF(G15="","",G15-365),"")</f>
         <v/>
       </c>
-      <c r="P15" s="69" t="n"/>
+      <c r="P15" s="70" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="72" t="n"/>
-      <c r="B16" s="72" t="n"/>
-      <c r="C16" s="72" t="n"/>
-      <c r="D16" s="72" t="n"/>
-      <c r="E16" s="73" t="n"/>
-      <c r="F16" s="73" t="n"/>
-      <c r="G16" s="73" t="n"/>
-      <c r="H16" s="72" t="n"/>
-      <c r="I16" s="72" t="n"/>
+      <c r="A16" s="73" t="n"/>
+      <c r="B16" s="73" t="n"/>
+      <c r="C16" s="73" t="n"/>
+      <c r="D16" s="73" t="n"/>
+      <c r="E16" s="74" t="n"/>
+      <c r="F16" s="74" t="n"/>
+      <c r="G16" s="74" t="n"/>
+      <c r="H16" s="73" t="n"/>
+      <c r="I16" s="73" t="n"/>
       <c r="J16" s="65">
         <f>IFERROR(DATEDIF(F16,G16,"M"),"")</f>
         <v/>
       </c>
-      <c r="K16" s="74" t="n"/>
-      <c r="L16" s="77">
+      <c r="K16" s="75" t="n"/>
+      <c r="L16" s="78">
         <f>IFERROR(IF(K16="","",K16/12),"")</f>
         <v/>
       </c>
-      <c r="M16" s="72" t="n"/>
-      <c r="N16" s="81" t="n"/>
-      <c r="O16" s="79">
+      <c r="M16" s="73" t="n"/>
+      <c r="N16" s="82" t="n"/>
+      <c r="O16" s="80">
         <f>IFERROR(IF(G16="","",G16-365),"")</f>
         <v/>
       </c>
-      <c r="P16" s="72" t="n"/>
+      <c r="P16" s="73" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="69" t="n"/>
-      <c r="B17" s="69" t="n"/>
-      <c r="C17" s="69" t="n"/>
-      <c r="D17" s="69" t="n"/>
-      <c r="E17" s="70" t="n"/>
-      <c r="F17" s="70" t="n"/>
-      <c r="G17" s="70" t="n"/>
-      <c r="H17" s="69" t="n"/>
-      <c r="I17" s="69" t="n"/>
+      <c r="A17" s="70" t="n"/>
+      <c r="B17" s="70" t="n"/>
+      <c r="C17" s="70" t="n"/>
+      <c r="D17" s="70" t="n"/>
+      <c r="E17" s="71" t="n"/>
+      <c r="F17" s="71" t="n"/>
+      <c r="G17" s="71" t="n"/>
+      <c r="H17" s="70" t="n"/>
+      <c r="I17" s="70" t="n"/>
       <c r="J17" s="65">
         <f>IFERROR(DATEDIF(F17,G17,"M"),"")</f>
         <v/>
       </c>
-      <c r="K17" s="71" t="n"/>
-      <c r="L17" s="77">
+      <c r="K17" s="72" t="n"/>
+      <c r="L17" s="78">
         <f>IFERROR(IF(K17="","",K17/12),"")</f>
         <v/>
       </c>
-      <c r="M17" s="69" t="n"/>
-      <c r="N17" s="80" t="n"/>
-      <c r="O17" s="79">
+      <c r="M17" s="70" t="n"/>
+      <c r="N17" s="81" t="n"/>
+      <c r="O17" s="80">
         <f>IFERROR(IF(G17="","",G17-365),"")</f>
         <v/>
       </c>
-      <c r="P17" s="69" t="n"/>
+      <c r="P17" s="70" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="72" t="n"/>
-      <c r="B18" s="72" t="n"/>
-      <c r="C18" s="72" t="n"/>
-      <c r="D18" s="72" t="n"/>
-      <c r="E18" s="73" t="n"/>
-      <c r="F18" s="73" t="n"/>
-      <c r="G18" s="73" t="n"/>
-      <c r="H18" s="72" t="n"/>
-      <c r="I18" s="72" t="n"/>
+      <c r="A18" s="73" t="n"/>
+      <c r="B18" s="73" t="n"/>
+      <c r="C18" s="73" t="n"/>
+      <c r="D18" s="73" t="n"/>
+      <c r="E18" s="74" t="n"/>
+      <c r="F18" s="74" t="n"/>
+      <c r="G18" s="74" t="n"/>
+      <c r="H18" s="73" t="n"/>
+      <c r="I18" s="73" t="n"/>
       <c r="J18" s="65">
         <f>IFERROR(DATEDIF(F18,G18,"M"),"")</f>
         <v/>
       </c>
-      <c r="K18" s="74" t="n"/>
-      <c r="L18" s="77">
+      <c r="K18" s="75" t="n"/>
+      <c r="L18" s="78">
         <f>IFERROR(IF(K18="","",K18/12),"")</f>
         <v/>
       </c>
-      <c r="M18" s="72" t="n"/>
-      <c r="N18" s="81" t="n"/>
-      <c r="O18" s="79">
+      <c r="M18" s="73" t="n"/>
+      <c r="N18" s="82" t="n"/>
+      <c r="O18" s="80">
         <f>IFERROR(IF(G18="","",G18-365),"")</f>
         <v/>
       </c>
-      <c r="P18" s="72" t="n"/>
+      <c r="P18" s="73" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="69" t="n"/>
-      <c r="B19" s="69" t="n"/>
-      <c r="C19" s="69" t="n"/>
-      <c r="D19" s="69" t="n"/>
-      <c r="E19" s="70" t="n"/>
-      <c r="F19" s="70" t="n"/>
-      <c r="G19" s="70" t="n"/>
-      <c r="H19" s="69" t="n"/>
-      <c r="I19" s="69" t="n"/>
+      <c r="A19" s="70" t="n"/>
+      <c r="B19" s="70" t="n"/>
+      <c r="C19" s="70" t="n"/>
+      <c r="D19" s="70" t="n"/>
+      <c r="E19" s="71" t="n"/>
+      <c r="F19" s="71" t="n"/>
+      <c r="G19" s="71" t="n"/>
+      <c r="H19" s="70" t="n"/>
+      <c r="I19" s="70" t="n"/>
       <c r="J19" s="65">
         <f>IFERROR(DATEDIF(F19,G19,"M"),"")</f>
         <v/>
       </c>
-      <c r="K19" s="71" t="n"/>
-      <c r="L19" s="77">
+      <c r="K19" s="72" t="n"/>
+      <c r="L19" s="78">
         <f>IFERROR(IF(K19="","",K19/12),"")</f>
         <v/>
       </c>
-      <c r="M19" s="69" t="n"/>
-      <c r="N19" s="80" t="n"/>
-      <c r="O19" s="79">
+      <c r="M19" s="70" t="n"/>
+      <c r="N19" s="81" t="n"/>
+      <c r="O19" s="80">
         <f>IFERROR(IF(G19="","",G19-365),"")</f>
         <v/>
       </c>
-      <c r="P19" s="69" t="n"/>
+      <c r="P19" s="70" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="72" t="n"/>
-      <c r="B20" s="72" t="n"/>
-      <c r="C20" s="72" t="n"/>
-      <c r="D20" s="72" t="n"/>
-      <c r="E20" s="73" t="n"/>
-      <c r="F20" s="73" t="n"/>
-      <c r="G20" s="73" t="n"/>
-      <c r="H20" s="72" t="n"/>
-      <c r="I20" s="72" t="n"/>
+      <c r="A20" s="73" t="n"/>
+      <c r="B20" s="73" t="n"/>
+      <c r="C20" s="73" t="n"/>
+      <c r="D20" s="73" t="n"/>
+      <c r="E20" s="74" t="n"/>
+      <c r="F20" s="74" t="n"/>
+      <c r="G20" s="74" t="n"/>
+      <c r="H20" s="73" t="n"/>
+      <c r="I20" s="73" t="n"/>
       <c r="J20" s="65">
         <f>IFERROR(DATEDIF(F20,G20,"M"),"")</f>
         <v/>
       </c>
-      <c r="K20" s="74" t="n"/>
-      <c r="L20" s="77">
+      <c r="K20" s="75" t="n"/>
+      <c r="L20" s="78">
         <f>IFERROR(IF(K20="","",K20/12),"")</f>
         <v/>
       </c>
-      <c r="M20" s="72" t="n"/>
-      <c r="N20" s="81" t="n"/>
-      <c r="O20" s="79">
+      <c r="M20" s="73" t="n"/>
+      <c r="N20" s="82" t="n"/>
+      <c r="O20" s="80">
         <f>IFERROR(IF(G20="","",G20-365),"")</f>
         <v/>
       </c>
-      <c r="P20" s="72" t="n"/>
+      <c r="P20" s="73" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="69" t="n"/>
-      <c r="B21" s="69" t="n"/>
-      <c r="C21" s="69" t="n"/>
-      <c r="D21" s="69" t="n"/>
-      <c r="E21" s="70" t="n"/>
-      <c r="F21" s="70" t="n"/>
-      <c r="G21" s="70" t="n"/>
-      <c r="H21" s="69" t="n"/>
-      <c r="I21" s="69" t="n"/>
+      <c r="A21" s="70" t="n"/>
+      <c r="B21" s="70" t="n"/>
+      <c r="C21" s="70" t="n"/>
+      <c r="D21" s="70" t="n"/>
+      <c r="E21" s="71" t="n"/>
+      <c r="F21" s="71" t="n"/>
+      <c r="G21" s="71" t="n"/>
+      <c r="H21" s="70" t="n"/>
+      <c r="I21" s="70" t="n"/>
       <c r="J21" s="65">
         <f>IFERROR(DATEDIF(F21,G21,"M"),"")</f>
         <v/>
       </c>
-      <c r="K21" s="71" t="n"/>
-      <c r="L21" s="77">
+      <c r="K21" s="72" t="n"/>
+      <c r="L21" s="78">
         <f>IFERROR(IF(K21="","",K21/12),"")</f>
         <v/>
       </c>
-      <c r="M21" s="69" t="n"/>
-      <c r="N21" s="80" t="n"/>
-      <c r="O21" s="79">
+      <c r="M21" s="70" t="n"/>
+      <c r="N21" s="81" t="n"/>
+      <c r="O21" s="80">
         <f>IFERROR(IF(G21="","",G21-365),"")</f>
         <v/>
       </c>
-      <c r="P21" s="69" t="n"/>
+      <c r="P21" s="70" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="72" t="n"/>
-      <c r="B22" s="72" t="n"/>
-      <c r="C22" s="72" t="n"/>
-      <c r="D22" s="72" t="n"/>
-      <c r="E22" s="73" t="n"/>
-      <c r="F22" s="73" t="n"/>
-      <c r="G22" s="73" t="n"/>
-      <c r="H22" s="72" t="n"/>
-      <c r="I22" s="72" t="n"/>
+      <c r="A22" s="73" t="n"/>
+      <c r="B22" s="73" t="n"/>
+      <c r="C22" s="73" t="n"/>
+      <c r="D22" s="73" t="n"/>
+      <c r="E22" s="74" t="n"/>
+      <c r="F22" s="74" t="n"/>
+      <c r="G22" s="74" t="n"/>
+      <c r="H22" s="73" t="n"/>
+      <c r="I22" s="73" t="n"/>
       <c r="J22" s="65">
         <f>IFERROR(DATEDIF(F22,G22,"M"),"")</f>
         <v/>
       </c>
-      <c r="K22" s="74" t="n"/>
-      <c r="L22" s="77">
+      <c r="K22" s="75" t="n"/>
+      <c r="L22" s="78">
         <f>IFERROR(IF(K22="","",K22/12),"")</f>
         <v/>
       </c>
-      <c r="M22" s="72" t="n"/>
-      <c r="N22" s="81" t="n"/>
-      <c r="O22" s="79">
+      <c r="M22" s="73" t="n"/>
+      <c r="N22" s="82" t="n"/>
+      <c r="O22" s="80">
         <f>IFERROR(IF(G22="","",G22-365),"")</f>
         <v/>
       </c>
-      <c r="P22" s="72" t="n"/>
+      <c r="P22" s="73" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="69" t="n"/>
-      <c r="B23" s="69" t="n"/>
-      <c r="C23" s="69" t="n"/>
-      <c r="D23" s="69" t="n"/>
-      <c r="E23" s="70" t="n"/>
-      <c r="F23" s="70" t="n"/>
-      <c r="G23" s="70" t="n"/>
-      <c r="H23" s="69" t="n"/>
-      <c r="I23" s="69" t="n"/>
+      <c r="A23" s="70" t="n"/>
+      <c r="B23" s="70" t="n"/>
+      <c r="C23" s="70" t="n"/>
+      <c r="D23" s="70" t="n"/>
+      <c r="E23" s="71" t="n"/>
+      <c r="F23" s="71" t="n"/>
+      <c r="G23" s="71" t="n"/>
+      <c r="H23" s="70" t="n"/>
+      <c r="I23" s="70" t="n"/>
       <c r="J23" s="65">
         <f>IFERROR(DATEDIF(F23,G23,"M"),"")</f>
         <v/>
       </c>
-      <c r="K23" s="71" t="n"/>
-      <c r="L23" s="77">
+      <c r="K23" s="72" t="n"/>
+      <c r="L23" s="78">
         <f>IFERROR(IF(K23="","",K23/12),"")</f>
         <v/>
       </c>
-      <c r="M23" s="69" t="n"/>
-      <c r="N23" s="80" t="n"/>
-      <c r="O23" s="79">
+      <c r="M23" s="70" t="n"/>
+      <c r="N23" s="81" t="n"/>
+      <c r="O23" s="80">
         <f>IFERROR(IF(G23="","",G23-365),"")</f>
         <v/>
       </c>
-      <c r="P23" s="69" t="n"/>
+      <c r="P23" s="70" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="72" t="n"/>
-      <c r="B24" s="72" t="n"/>
-      <c r="C24" s="72" t="n"/>
-      <c r="D24" s="72" t="n"/>
-      <c r="E24" s="73" t="n"/>
-      <c r="F24" s="73" t="n"/>
-      <c r="G24" s="73" t="n"/>
-      <c r="H24" s="72" t="n"/>
-      <c r="I24" s="72" t="n"/>
+      <c r="A24" s="73" t="n"/>
+      <c r="B24" s="73" t="n"/>
+      <c r="C24" s="73" t="n"/>
+      <c r="D24" s="73" t="n"/>
+      <c r="E24" s="74" t="n"/>
+      <c r="F24" s="74" t="n"/>
+      <c r="G24" s="74" t="n"/>
+      <c r="H24" s="73" t="n"/>
+      <c r="I24" s="73" t="n"/>
       <c r="J24" s="65">
         <f>IFERROR(DATEDIF(F24,G24,"M"),"")</f>
         <v/>
       </c>
-      <c r="K24" s="74" t="n"/>
-      <c r="L24" s="77">
+      <c r="K24" s="75" t="n"/>
+      <c r="L24" s="78">
         <f>IFERROR(IF(K24="","",K24/12),"")</f>
         <v/>
       </c>
-      <c r="M24" s="72" t="n"/>
-      <c r="N24" s="81" t="n"/>
-      <c r="O24" s="79">
+      <c r="M24" s="73" t="n"/>
+      <c r="N24" s="82" t="n"/>
+      <c r="O24" s="80">
         <f>IFERROR(IF(G24="","",G24-365),"")</f>
         <v/>
       </c>
-      <c r="P24" s="72" t="n"/>
+      <c r="P24" s="73" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="69" t="n"/>
-      <c r="B25" s="69" t="n"/>
-      <c r="C25" s="69" t="n"/>
-      <c r="D25" s="69" t="n"/>
-      <c r="E25" s="70" t="n"/>
-      <c r="F25" s="70" t="n"/>
-      <c r="G25" s="70" t="n"/>
-      <c r="H25" s="69" t="n"/>
-      <c r="I25" s="69" t="n"/>
+      <c r="A25" s="70" t="n"/>
+      <c r="B25" s="70" t="n"/>
+      <c r="C25" s="70" t="n"/>
+      <c r="D25" s="70" t="n"/>
+      <c r="E25" s="71" t="n"/>
+      <c r="F25" s="71" t="n"/>
+      <c r="G25" s="71" t="n"/>
+      <c r="H25" s="70" t="n"/>
+      <c r="I25" s="70" t="n"/>
       <c r="J25" s="65">
         <f>IFERROR(DATEDIF(F25,G25,"M"),"")</f>
         <v/>
       </c>
-      <c r="K25" s="71" t="n"/>
-      <c r="L25" s="77">
+      <c r="K25" s="72" t="n"/>
+      <c r="L25" s="78">
         <f>IFERROR(IF(K25="","",K25/12),"")</f>
         <v/>
       </c>
-      <c r="M25" s="69" t="n"/>
-      <c r="N25" s="80" t="n"/>
-      <c r="O25" s="79">
+      <c r="M25" s="70" t="n"/>
+      <c r="N25" s="81" t="n"/>
+      <c r="O25" s="80">
         <f>IFERROR(IF(G25="","",G25-365),"")</f>
         <v/>
       </c>
-      <c r="P25" s="69" t="n"/>
+      <c r="P25" s="70" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="72" t="n"/>
-      <c r="B26" s="72" t="n"/>
-      <c r="C26" s="72" t="n"/>
-      <c r="D26" s="72" t="n"/>
-      <c r="E26" s="73" t="n"/>
-      <c r="F26" s="73" t="n"/>
-      <c r="G26" s="73" t="n"/>
-      <c r="H26" s="72" t="n"/>
-      <c r="I26" s="72" t="n"/>
+      <c r="A26" s="73" t="n"/>
+      <c r="B26" s="73" t="n"/>
+      <c r="C26" s="73" t="n"/>
+      <c r="D26" s="73" t="n"/>
+      <c r="E26" s="74" t="n"/>
+      <c r="F26" s="74" t="n"/>
+      <c r="G26" s="74" t="n"/>
+      <c r="H26" s="73" t="n"/>
+      <c r="I26" s="73" t="n"/>
       <c r="J26" s="65">
         <f>IFERROR(DATEDIF(F26,G26,"M"),"")</f>
         <v/>
       </c>
-      <c r="K26" s="74" t="n"/>
-      <c r="L26" s="77">
+      <c r="K26" s="75" t="n"/>
+      <c r="L26" s="78">
         <f>IFERROR(IF(K26="","",K26/12),"")</f>
         <v/>
       </c>
-      <c r="M26" s="72" t="n"/>
-      <c r="N26" s="81" t="n"/>
-      <c r="O26" s="79">
+      <c r="M26" s="73" t="n"/>
+      <c r="N26" s="82" t="n"/>
+      <c r="O26" s="80">
         <f>IFERROR(IF(G26="","",G26-365),"")</f>
         <v/>
       </c>
-      <c r="P26" s="72" t="n"/>
+      <c r="P26" s="73" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="69" t="n"/>
-      <c r="B27" s="69" t="n"/>
-      <c r="C27" s="69" t="n"/>
-      <c r="D27" s="69" t="n"/>
-      <c r="E27" s="70" t="n"/>
-      <c r="F27" s="70" t="n"/>
-      <c r="G27" s="70" t="n"/>
-      <c r="H27" s="69" t="n"/>
-      <c r="I27" s="69" t="n"/>
+      <c r="A27" s="70" t="n"/>
+      <c r="B27" s="70" t="n"/>
+      <c r="C27" s="70" t="n"/>
+      <c r="D27" s="70" t="n"/>
+      <c r="E27" s="71" t="n"/>
+      <c r="F27" s="71" t="n"/>
+      <c r="G27" s="71" t="n"/>
+      <c r="H27" s="70" t="n"/>
+      <c r="I27" s="70" t="n"/>
       <c r="J27" s="65">
         <f>IFERROR(DATEDIF(F27,G27,"M"),"")</f>
         <v/>
       </c>
-      <c r="K27" s="71" t="n"/>
-      <c r="L27" s="77">
+      <c r="K27" s="72" t="n"/>
+      <c r="L27" s="78">
         <f>IFERROR(IF(K27="","",K27/12),"")</f>
         <v/>
       </c>
-      <c r="M27" s="69" t="n"/>
-      <c r="N27" s="80" t="n"/>
-      <c r="O27" s="79">
+      <c r="M27" s="70" t="n"/>
+      <c r="N27" s="81" t="n"/>
+      <c r="O27" s="80">
         <f>IFERROR(IF(G27="","",G27-365),"")</f>
         <v/>
       </c>
-      <c r="P27" s="69" t="n"/>
+      <c r="P27" s="70" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="72" t="n"/>
-      <c r="B28" s="72" t="n"/>
-      <c r="C28" s="72" t="n"/>
-      <c r="D28" s="72" t="n"/>
-      <c r="E28" s="73" t="n"/>
-      <c r="F28" s="73" t="n"/>
-      <c r="G28" s="73" t="n"/>
-      <c r="H28" s="72" t="n"/>
-      <c r="I28" s="72" t="n"/>
+      <c r="A28" s="73" t="n"/>
+      <c r="B28" s="73" t="n"/>
+      <c r="C28" s="73" t="n"/>
+      <c r="D28" s="73" t="n"/>
+      <c r="E28" s="74" t="n"/>
+      <c r="F28" s="74" t="n"/>
+      <c r="G28" s="74" t="n"/>
+      <c r="H28" s="73" t="n"/>
+      <c r="I28" s="73" t="n"/>
       <c r="J28" s="65">
         <f>IFERROR(DATEDIF(F28,G28,"M"),"")</f>
         <v/>
       </c>
-      <c r="K28" s="74" t="n"/>
-      <c r="L28" s="77">
+      <c r="K28" s="75" t="n"/>
+      <c r="L28" s="78">
         <f>IFERROR(IF(K28="","",K28/12),"")</f>
         <v/>
       </c>
-      <c r="M28" s="72" t="n"/>
-      <c r="N28" s="81" t="n"/>
-      <c r="O28" s="79">
+      <c r="M28" s="73" t="n"/>
+      <c r="N28" s="82" t="n"/>
+      <c r="O28" s="80">
         <f>IFERROR(IF(G28="","",G28-365),"")</f>
         <v/>
       </c>
-      <c r="P28" s="72" t="n"/>
+      <c r="P28" s="73" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="69" t="n"/>
-      <c r="B29" s="69" t="n"/>
-      <c r="C29" s="69" t="n"/>
-      <c r="D29" s="69" t="n"/>
-      <c r="E29" s="70" t="n"/>
-      <c r="F29" s="70" t="n"/>
-      <c r="G29" s="70" t="n"/>
-      <c r="H29" s="69" t="n"/>
-      <c r="I29" s="69" t="n"/>
+      <c r="A29" s="70" t="n"/>
+      <c r="B29" s="70" t="n"/>
+      <c r="C29" s="70" t="n"/>
+      <c r="D29" s="70" t="n"/>
+      <c r="E29" s="71" t="n"/>
+      <c r="F29" s="71" t="n"/>
+      <c r="G29" s="71" t="n"/>
+      <c r="H29" s="70" t="n"/>
+      <c r="I29" s="70" t="n"/>
       <c r="J29" s="65">
         <f>IFERROR(DATEDIF(F29,G29,"M"),"")</f>
         <v/>
       </c>
-      <c r="K29" s="71" t="n"/>
-      <c r="L29" s="77">
+      <c r="K29" s="72" t="n"/>
+      <c r="L29" s="78">
         <f>IFERROR(IF(K29="","",K29/12),"")</f>
         <v/>
       </c>
-      <c r="M29" s="69" t="n"/>
-      <c r="N29" s="80" t="n"/>
-      <c r="O29" s="79">
+      <c r="M29" s="70" t="n"/>
+      <c r="N29" s="81" t="n"/>
+      <c r="O29" s="80">
         <f>IFERROR(IF(G29="","",G29-365),"")</f>
         <v/>
       </c>
-      <c r="P29" s="69" t="n"/>
+      <c r="P29" s="70" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="72" t="n"/>
-      <c r="B30" s="72" t="n"/>
-      <c r="C30" s="72" t="n"/>
-      <c r="D30" s="72" t="n"/>
-      <c r="E30" s="73" t="n"/>
-      <c r="F30" s="73" t="n"/>
-      <c r="G30" s="73" t="n"/>
-      <c r="H30" s="72" t="n"/>
-      <c r="I30" s="72" t="n"/>
+      <c r="A30" s="73" t="n"/>
+      <c r="B30" s="73" t="n"/>
+      <c r="C30" s="73" t="n"/>
+      <c r="D30" s="73" t="n"/>
+      <c r="E30" s="74" t="n"/>
+      <c r="F30" s="74" t="n"/>
+      <c r="G30" s="74" t="n"/>
+      <c r="H30" s="73" t="n"/>
+      <c r="I30" s="73" t="n"/>
       <c r="J30" s="65">
         <f>IFERROR(DATEDIF(F30,G30,"M"),"")</f>
         <v/>
       </c>
-      <c r="K30" s="74" t="n"/>
-      <c r="L30" s="77">
+      <c r="K30" s="75" t="n"/>
+      <c r="L30" s="78">
         <f>IFERROR(IF(K30="","",K30/12),"")</f>
         <v/>
       </c>
-      <c r="M30" s="72" t="n"/>
-      <c r="N30" s="81" t="n"/>
-      <c r="O30" s="79">
+      <c r="M30" s="73" t="n"/>
+      <c r="N30" s="82" t="n"/>
+      <c r="O30" s="80">
         <f>IFERROR(IF(G30="","",G30-365),"")</f>
         <v/>
       </c>
-      <c r="P30" s="72" t="n"/>
+      <c r="P30" s="73" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="69" t="n"/>
-      <c r="B31" s="69" t="n"/>
-      <c r="C31" s="69" t="n"/>
-      <c r="D31" s="69" t="n"/>
-      <c r="E31" s="70" t="n"/>
-      <c r="F31" s="70" t="n"/>
-      <c r="G31" s="70" t="n"/>
-      <c r="H31" s="69" t="n"/>
-      <c r="I31" s="69" t="n"/>
+      <c r="A31" s="70" t="n"/>
+      <c r="B31" s="70" t="n"/>
+      <c r="C31" s="70" t="n"/>
+      <c r="D31" s="70" t="n"/>
+      <c r="E31" s="71" t="n"/>
+      <c r="F31" s="71" t="n"/>
+      <c r="G31" s="71" t="n"/>
+      <c r="H31" s="70" t="n"/>
+      <c r="I31" s="70" t="n"/>
       <c r="J31" s="65">
         <f>IFERROR(DATEDIF(F31,G31,"M"),"")</f>
         <v/>
       </c>
-      <c r="K31" s="71" t="n"/>
-      <c r="L31" s="77">
+      <c r="K31" s="72" t="n"/>
+      <c r="L31" s="78">
         <f>IFERROR(IF(K31="","",K31/12),"")</f>
         <v/>
       </c>
-      <c r="M31" s="69" t="n"/>
-      <c r="N31" s="80" t="n"/>
-      <c r="O31" s="79">
+      <c r="M31" s="70" t="n"/>
+      <c r="N31" s="81" t="n"/>
+      <c r="O31" s="80">
         <f>IFERROR(IF(G31="","",G31-365),"")</f>
         <v/>
       </c>
-      <c r="P31" s="69" t="n"/>
+      <c r="P31" s="70" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="72" t="n"/>
-      <c r="B32" s="72" t="n"/>
-      <c r="C32" s="72" t="n"/>
-      <c r="D32" s="72" t="n"/>
-      <c r="E32" s="73" t="n"/>
-      <c r="F32" s="73" t="n"/>
-      <c r="G32" s="73" t="n"/>
-      <c r="H32" s="72" t="n"/>
-      <c r="I32" s="72" t="n"/>
+      <c r="A32" s="73" t="n"/>
+      <c r="B32" s="73" t="n"/>
+      <c r="C32" s="73" t="n"/>
+      <c r="D32" s="73" t="n"/>
+      <c r="E32" s="74" t="n"/>
+      <c r="F32" s="74" t="n"/>
+      <c r="G32" s="74" t="n"/>
+      <c r="H32" s="73" t="n"/>
+      <c r="I32" s="73" t="n"/>
       <c r="J32" s="65">
         <f>IFERROR(DATEDIF(F32,G32,"M"),"")</f>
         <v/>
       </c>
-      <c r="K32" s="74" t="n"/>
-      <c r="L32" s="77">
+      <c r="K32" s="75" t="n"/>
+      <c r="L32" s="78">
         <f>IFERROR(IF(K32="","",K32/12),"")</f>
         <v/>
       </c>
-      <c r="M32" s="72" t="n"/>
-      <c r="N32" s="81" t="n"/>
-      <c r="O32" s="79">
+      <c r="M32" s="73" t="n"/>
+      <c r="N32" s="82" t="n"/>
+      <c r="O32" s="80">
         <f>IFERROR(IF(G32="","",G32-365),"")</f>
         <v/>
       </c>
-      <c r="P32" s="72" t="n"/>
+      <c r="P32" s="73" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="69" t="n"/>
-      <c r="B33" s="69" t="n"/>
-      <c r="C33" s="69" t="n"/>
-      <c r="D33" s="69" t="n"/>
-      <c r="E33" s="70" t="n"/>
-      <c r="F33" s="70" t="n"/>
-      <c r="G33" s="70" t="n"/>
-      <c r="H33" s="69" t="n"/>
-      <c r="I33" s="69" t="n"/>
+      <c r="A33" s="70" t="n"/>
+      <c r="B33" s="70" t="n"/>
+      <c r="C33" s="70" t="n"/>
+      <c r="D33" s="70" t="n"/>
+      <c r="E33" s="71" t="n"/>
+      <c r="F33" s="71" t="n"/>
+      <c r="G33" s="71" t="n"/>
+      <c r="H33" s="70" t="n"/>
+      <c r="I33" s="70" t="n"/>
       <c r="J33" s="65">
         <f>IFERROR(DATEDIF(F33,G33,"M"),"")</f>
         <v/>
       </c>
-      <c r="K33" s="71" t="n"/>
-      <c r="L33" s="77">
+      <c r="K33" s="72" t="n"/>
+      <c r="L33" s="78">
         <f>IFERROR(IF(K33="","",K33/12),"")</f>
         <v/>
       </c>
-      <c r="M33" s="69" t="n"/>
-      <c r="N33" s="80" t="n"/>
-      <c r="O33" s="79">
+      <c r="M33" s="70" t="n"/>
+      <c r="N33" s="81" t="n"/>
+      <c r="O33" s="80">
         <f>IFERROR(IF(G33="","",G33-365),"")</f>
         <v/>
       </c>
-      <c r="P33" s="69" t="n"/>
+      <c r="P33" s="70" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="72" t="n"/>
-      <c r="B34" s="72" t="n"/>
-      <c r="C34" s="72" t="n"/>
-      <c r="D34" s="72" t="n"/>
-      <c r="E34" s="73" t="n"/>
-      <c r="F34" s="73" t="n"/>
-      <c r="G34" s="73" t="n"/>
-      <c r="H34" s="72" t="n"/>
-      <c r="I34" s="72" t="n"/>
+      <c r="A34" s="73" t="n"/>
+      <c r="B34" s="73" t="n"/>
+      <c r="C34" s="73" t="n"/>
+      <c r="D34" s="73" t="n"/>
+      <c r="E34" s="74" t="n"/>
+      <c r="F34" s="74" t="n"/>
+      <c r="G34" s="74" t="n"/>
+      <c r="H34" s="73" t="n"/>
+      <c r="I34" s="73" t="n"/>
       <c r="J34" s="65">
         <f>IFERROR(DATEDIF(F34,G34,"M"),"")</f>
         <v/>
       </c>
-      <c r="K34" s="74" t="n"/>
-      <c r="L34" s="77">
+      <c r="K34" s="75" t="n"/>
+      <c r="L34" s="78">
         <f>IFERROR(IF(K34="","",K34/12),"")</f>
         <v/>
       </c>
-      <c r="M34" s="72" t="n"/>
-      <c r="N34" s="81" t="n"/>
-      <c r="O34" s="79">
+      <c r="M34" s="73" t="n"/>
+      <c r="N34" s="82" t="n"/>
+      <c r="O34" s="80">
         <f>IFERROR(IF(G34="","",G34-365),"")</f>
         <v/>
       </c>
-      <c r="P34" s="72" t="n"/>
+      <c r="P34" s="73" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="69" t="n"/>
-      <c r="B35" s="69" t="n"/>
-      <c r="C35" s="69" t="n"/>
-      <c r="D35" s="69" t="n"/>
-      <c r="E35" s="70" t="n"/>
-      <c r="F35" s="70" t="n"/>
-      <c r="G35" s="70" t="n"/>
-      <c r="H35" s="69" t="n"/>
-      <c r="I35" s="69" t="n"/>
+      <c r="A35" s="70" t="n"/>
+      <c r="B35" s="70" t="n"/>
+      <c r="C35" s="70" t="n"/>
+      <c r="D35" s="70" t="n"/>
+      <c r="E35" s="71" t="n"/>
+      <c r="F35" s="71" t="n"/>
+      <c r="G35" s="71" t="n"/>
+      <c r="H35" s="70" t="n"/>
+      <c r="I35" s="70" t="n"/>
       <c r="J35" s="65">
         <f>IFERROR(DATEDIF(F35,G35,"M"),"")</f>
         <v/>
       </c>
-      <c r="K35" s="71" t="n"/>
-      <c r="L35" s="77">
+      <c r="K35" s="72" t="n"/>
+      <c r="L35" s="78">
         <f>IFERROR(IF(K35="","",K35/12),"")</f>
         <v/>
       </c>
-      <c r="M35" s="69" t="n"/>
-      <c r="N35" s="80" t="n"/>
-      <c r="O35" s="79">
+      <c r="M35" s="70" t="n"/>
+      <c r="N35" s="81" t="n"/>
+      <c r="O35" s="80">
         <f>IFERROR(IF(G35="","",G35-365),"")</f>
         <v/>
       </c>
-      <c r="P35" s="69" t="n"/>
+      <c r="P35" s="70" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="72" t="n"/>
-      <c r="B36" s="72" t="n"/>
-      <c r="C36" s="72" t="n"/>
-      <c r="D36" s="72" t="n"/>
-      <c r="E36" s="73" t="n"/>
-      <c r="F36" s="73" t="n"/>
-      <c r="G36" s="73" t="n"/>
-      <c r="H36" s="72" t="n"/>
-      <c r="I36" s="72" t="n"/>
+      <c r="A36" s="73" t="n"/>
+      <c r="B36" s="73" t="n"/>
+      <c r="C36" s="73" t="n"/>
+      <c r="D36" s="73" t="n"/>
+      <c r="E36" s="74" t="n"/>
+      <c r="F36" s="74" t="n"/>
+      <c r="G36" s="74" t="n"/>
+      <c r="H36" s="73" t="n"/>
+      <c r="I36" s="73" t="n"/>
       <c r="J36" s="65">
         <f>IFERROR(DATEDIF(F36,G36,"M"),"")</f>
         <v/>
       </c>
-      <c r="K36" s="74" t="n"/>
-      <c r="L36" s="77">
+      <c r="K36" s="75" t="n"/>
+      <c r="L36" s="78">
         <f>IFERROR(IF(K36="","",K36/12),"")</f>
         <v/>
       </c>
-      <c r="M36" s="72" t="n"/>
-      <c r="N36" s="81" t="n"/>
-      <c r="O36" s="79">
+      <c r="M36" s="73" t="n"/>
+      <c r="N36" s="82" t="n"/>
+      <c r="O36" s="80">
         <f>IFERROR(IF(G36="","",G36-365),"")</f>
         <v/>
       </c>
-      <c r="P36" s="72" t="n"/>
+      <c r="P36" s="73" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="69" t="n"/>
-      <c r="B37" s="69" t="n"/>
-      <c r="C37" s="69" t="n"/>
-      <c r="D37" s="69" t="n"/>
-      <c r="E37" s="70" t="n"/>
-      <c r="F37" s="70" t="n"/>
-      <c r="G37" s="70" t="n"/>
-      <c r="H37" s="69" t="n"/>
-      <c r="I37" s="69" t="n"/>
+      <c r="A37" s="70" t="n"/>
+      <c r="B37" s="70" t="n"/>
+      <c r="C37" s="70" t="n"/>
+      <c r="D37" s="70" t="n"/>
+      <c r="E37" s="71" t="n"/>
+      <c r="F37" s="71" t="n"/>
+      <c r="G37" s="71" t="n"/>
+      <c r="H37" s="70" t="n"/>
+      <c r="I37" s="70" t="n"/>
       <c r="J37" s="65">
         <f>IFERROR(DATEDIF(F37,G37,"M"),"")</f>
         <v/>
       </c>
-      <c r="K37" s="71" t="n"/>
-      <c r="L37" s="77">
+      <c r="K37" s="72" t="n"/>
+      <c r="L37" s="78">
         <f>IFERROR(IF(K37="","",K37/12),"")</f>
         <v/>
       </c>
-      <c r="M37" s="69" t="n"/>
-      <c r="N37" s="80" t="n"/>
-      <c r="O37" s="79">
+      <c r="M37" s="70" t="n"/>
+      <c r="N37" s="81" t="n"/>
+      <c r="O37" s="80">
         <f>IFERROR(IF(G37="","",G37-365),"")</f>
         <v/>
       </c>
-      <c r="P37" s="69" t="n"/>
+      <c r="P37" s="70" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="72" t="n"/>
-      <c r="B38" s="72" t="n"/>
-      <c r="C38" s="72" t="n"/>
-      <c r="D38" s="72" t="n"/>
-      <c r="E38" s="73" t="n"/>
-      <c r="F38" s="73" t="n"/>
-      <c r="G38" s="73" t="n"/>
-      <c r="H38" s="72" t="n"/>
-      <c r="I38" s="72" t="n"/>
+      <c r="A38" s="73" t="n"/>
+      <c r="B38" s="73" t="n"/>
+      <c r="C38" s="73" t="n"/>
+      <c r="D38" s="73" t="n"/>
+      <c r="E38" s="74" t="n"/>
+      <c r="F38" s="74" t="n"/>
+      <c r="G38" s="74" t="n"/>
+      <c r="H38" s="73" t="n"/>
+      <c r="I38" s="73" t="n"/>
       <c r="J38" s="65">
         <f>IFERROR(DATEDIF(F38,G38,"M"),"")</f>
         <v/>
       </c>
-      <c r="K38" s="74" t="n"/>
-      <c r="L38" s="77">
+      <c r="K38" s="75" t="n"/>
+      <c r="L38" s="78">
         <f>IFERROR(IF(K38="","",K38/12),"")</f>
         <v/>
       </c>
-      <c r="M38" s="72" t="n"/>
-      <c r="N38" s="81" t="n"/>
-      <c r="O38" s="79">
+      <c r="M38" s="73" t="n"/>
+      <c r="N38" s="82" t="n"/>
+      <c r="O38" s="80">
         <f>IFERROR(IF(G38="","",G38-365),"")</f>
         <v/>
       </c>
-      <c r="P38" s="72" t="n"/>
+      <c r="P38" s="73" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="69" t="n"/>
-      <c r="B39" s="69" t="n"/>
-      <c r="C39" s="69" t="n"/>
-      <c r="D39" s="69" t="n"/>
-      <c r="E39" s="70" t="n"/>
-      <c r="F39" s="70" t="n"/>
-      <c r="G39" s="70" t="n"/>
-      <c r="H39" s="69" t="n"/>
-      <c r="I39" s="69" t="n"/>
+      <c r="A39" s="70" t="n"/>
+      <c r="B39" s="70" t="n"/>
+      <c r="C39" s="70" t="n"/>
+      <c r="D39" s="70" t="n"/>
+      <c r="E39" s="71" t="n"/>
+      <c r="F39" s="71" t="n"/>
+      <c r="G39" s="71" t="n"/>
+      <c r="H39" s="70" t="n"/>
+      <c r="I39" s="70" t="n"/>
       <c r="J39" s="65">
         <f>IFERROR(DATEDIF(F39,G39,"M"),"")</f>
         <v/>
       </c>
-      <c r="K39" s="71" t="n"/>
-      <c r="L39" s="77">
+      <c r="K39" s="72" t="n"/>
+      <c r="L39" s="78">
         <f>IFERROR(IF(K39="","",K39/12),"")</f>
         <v/>
       </c>
-      <c r="M39" s="69" t="n"/>
-      <c r="N39" s="80" t="n"/>
-      <c r="O39" s="79">
+      <c r="M39" s="70" t="n"/>
+      <c r="N39" s="81" t="n"/>
+      <c r="O39" s="80">
         <f>IFERROR(IF(G39="","",G39-365),"")</f>
         <v/>
       </c>
-      <c r="P39" s="69" t="n"/>
+      <c r="P39" s="70" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="72" t="n"/>
-      <c r="B40" s="72" t="n"/>
-      <c r="C40" s="72" t="n"/>
-      <c r="D40" s="72" t="n"/>
-      <c r="E40" s="73" t="n"/>
-      <c r="F40" s="73" t="n"/>
-      <c r="G40" s="73" t="n"/>
-      <c r="H40" s="72" t="n"/>
-      <c r="I40" s="72" t="n"/>
+      <c r="A40" s="73" t="n"/>
+      <c r="B40" s="73" t="n"/>
+      <c r="C40" s="73" t="n"/>
+      <c r="D40" s="73" t="n"/>
+      <c r="E40" s="74" t="n"/>
+      <c r="F40" s="74" t="n"/>
+      <c r="G40" s="74" t="n"/>
+      <c r="H40" s="73" t="n"/>
+      <c r="I40" s="73" t="n"/>
       <c r="J40" s="65">
         <f>IFERROR(DATEDIF(F40,G40,"M"),"")</f>
         <v/>
       </c>
-      <c r="K40" s="74" t="n"/>
-      <c r="L40" s="77">
+      <c r="K40" s="75" t="n"/>
+      <c r="L40" s="78">
         <f>IFERROR(IF(K40="","",K40/12),"")</f>
         <v/>
       </c>
-      <c r="M40" s="72" t="n"/>
-      <c r="N40" s="81" t="n"/>
-      <c r="O40" s="79">
+      <c r="M40" s="73" t="n"/>
+      <c r="N40" s="82" t="n"/>
+      <c r="O40" s="80">
         <f>IFERROR(IF(G40="","",G40-365),"")</f>
         <v/>
       </c>
-      <c r="P40" s="72" t="n"/>
+      <c r="P40" s="73" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="69" t="n"/>
-      <c r="B41" s="69" t="n"/>
-      <c r="C41" s="69" t="n"/>
-      <c r="D41" s="69" t="n"/>
-      <c r="E41" s="70" t="n"/>
-      <c r="F41" s="70" t="n"/>
-      <c r="G41" s="70" t="n"/>
-      <c r="H41" s="69" t="n"/>
-      <c r="I41" s="69" t="n"/>
+      <c r="A41" s="70" t="n"/>
+      <c r="B41" s="70" t="n"/>
+      <c r="C41" s="70" t="n"/>
+      <c r="D41" s="70" t="n"/>
+      <c r="E41" s="71" t="n"/>
+      <c r="F41" s="71" t="n"/>
+      <c r="G41" s="71" t="n"/>
+      <c r="H41" s="70" t="n"/>
+      <c r="I41" s="70" t="n"/>
       <c r="J41" s="65">
         <f>IFERROR(DATEDIF(F41,G41,"M"),"")</f>
         <v/>
       </c>
-      <c r="K41" s="71" t="n"/>
-      <c r="L41" s="77">
+      <c r="K41" s="72" t="n"/>
+      <c r="L41" s="78">
         <f>IFERROR(IF(K41="","",K41/12),"")</f>
         <v/>
       </c>
-      <c r="M41" s="69" t="n"/>
-      <c r="N41" s="80" t="n"/>
-      <c r="O41" s="79">
+      <c r="M41" s="70" t="n"/>
+      <c r="N41" s="81" t="n"/>
+      <c r="O41" s="80">
         <f>IFERROR(IF(G41="","",G41-365),"")</f>
         <v/>
       </c>
-      <c r="P41" s="69" t="n"/>
+      <c r="P41" s="70" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="72" t="n"/>
-      <c r="B42" s="72" t="n"/>
-      <c r="C42" s="72" t="n"/>
-      <c r="D42" s="72" t="n"/>
-      <c r="E42" s="73" t="n"/>
-      <c r="F42" s="73" t="n"/>
-      <c r="G42" s="73" t="n"/>
-      <c r="H42" s="72" t="n"/>
-      <c r="I42" s="72" t="n"/>
+      <c r="A42" s="73" t="n"/>
+      <c r="B42" s="73" t="n"/>
+      <c r="C42" s="73" t="n"/>
+      <c r="D42" s="73" t="n"/>
+      <c r="E42" s="74" t="n"/>
+      <c r="F42" s="74" t="n"/>
+      <c r="G42" s="74" t="n"/>
+      <c r="H42" s="73" t="n"/>
+      <c r="I42" s="73" t="n"/>
       <c r="J42" s="65">
         <f>IFERROR(DATEDIF(F42,G42,"M"),"")</f>
         <v/>
       </c>
-      <c r="K42" s="74" t="n"/>
-      <c r="L42" s="77">
+      <c r="K42" s="75" t="n"/>
+      <c r="L42" s="78">
         <f>IFERROR(IF(K42="","",K42/12),"")</f>
         <v/>
       </c>
-      <c r="M42" s="72" t="n"/>
-      <c r="N42" s="81" t="n"/>
-      <c r="O42" s="79">
+      <c r="M42" s="73" t="n"/>
+      <c r="N42" s="82" t="n"/>
+      <c r="O42" s="80">
         <f>IFERROR(IF(G42="","",G42-365),"")</f>
         <v/>
       </c>
-      <c r="P42" s="72" t="n"/>
+      <c r="P42" s="73" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="69" t="n"/>
-      <c r="B43" s="69" t="n"/>
-      <c r="C43" s="69" t="n"/>
-      <c r="D43" s="69" t="n"/>
-      <c r="E43" s="70" t="n"/>
-      <c r="F43" s="70" t="n"/>
-      <c r="G43" s="70" t="n"/>
-      <c r="H43" s="69" t="n"/>
-      <c r="I43" s="69" t="n"/>
+      <c r="A43" s="70" t="n"/>
+      <c r="B43" s="70" t="n"/>
+      <c r="C43" s="70" t="n"/>
+      <c r="D43" s="70" t="n"/>
+      <c r="E43" s="71" t="n"/>
+      <c r="F43" s="71" t="n"/>
+      <c r="G43" s="71" t="n"/>
+      <c r="H43" s="70" t="n"/>
+      <c r="I43" s="70" t="n"/>
       <c r="J43" s="65">
         <f>IFERROR(DATEDIF(F43,G43,"M"),"")</f>
         <v/>
       </c>
-      <c r="K43" s="71" t="n"/>
-      <c r="L43" s="77">
+      <c r="K43" s="72" t="n"/>
+      <c r="L43" s="78">
         <f>IFERROR(IF(K43="","",K43/12),"")</f>
         <v/>
       </c>
-      <c r="M43" s="69" t="n"/>
-      <c r="N43" s="80" t="n"/>
-      <c r="O43" s="79">
+      <c r="M43" s="70" t="n"/>
+      <c r="N43" s="81" t="n"/>
+      <c r="O43" s="80">
         <f>IFERROR(IF(G43="","",G43-365),"")</f>
         <v/>
       </c>
-      <c r="P43" s="69" t="n"/>
+      <c r="P43" s="70" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="72" t="n"/>
-      <c r="B44" s="72" t="n"/>
-      <c r="C44" s="72" t="n"/>
-      <c r="D44" s="72" t="n"/>
-      <c r="E44" s="73" t="n"/>
-      <c r="F44" s="73" t="n"/>
-      <c r="G44" s="73" t="n"/>
-      <c r="H44" s="72" t="n"/>
-      <c r="I44" s="72" t="n"/>
+      <c r="A44" s="73" t="n"/>
+      <c r="B44" s="73" t="n"/>
+      <c r="C44" s="73" t="n"/>
+      <c r="D44" s="73" t="n"/>
+      <c r="E44" s="74" t="n"/>
+      <c r="F44" s="74" t="n"/>
+      <c r="G44" s="74" t="n"/>
+      <c r="H44" s="73" t="n"/>
+      <c r="I44" s="73" t="n"/>
       <c r="J44" s="65">
         <f>IFERROR(DATEDIF(F44,G44,"M"),"")</f>
         <v/>
       </c>
-      <c r="K44" s="74" t="n"/>
-      <c r="L44" s="77">
+      <c r="K44" s="75" t="n"/>
+      <c r="L44" s="78">
         <f>IFERROR(IF(K44="","",K44/12),"")</f>
         <v/>
       </c>
-      <c r="M44" s="72" t="n"/>
-      <c r="N44" s="81" t="n"/>
-      <c r="O44" s="79">
+      <c r="M44" s="73" t="n"/>
+      <c r="N44" s="82" t="n"/>
+      <c r="O44" s="80">
         <f>IFERROR(IF(G44="","",G44-365),"")</f>
         <v/>
       </c>
-      <c r="P44" s="72" t="n"/>
+      <c r="P44" s="73" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="69" t="n"/>
-      <c r="B45" s="69" t="n"/>
-      <c r="C45" s="69" t="n"/>
-      <c r="D45" s="69" t="n"/>
-      <c r="E45" s="70" t="n"/>
-      <c r="F45" s="70" t="n"/>
-      <c r="G45" s="70" t="n"/>
-      <c r="H45" s="69" t="n"/>
-      <c r="I45" s="69" t="n"/>
+      <c r="A45" s="70" t="n"/>
+      <c r="B45" s="70" t="n"/>
+      <c r="C45" s="70" t="n"/>
+      <c r="D45" s="70" t="n"/>
+      <c r="E45" s="71" t="n"/>
+      <c r="F45" s="71" t="n"/>
+      <c r="G45" s="71" t="n"/>
+      <c r="H45" s="70" t="n"/>
+      <c r="I45" s="70" t="n"/>
       <c r="J45" s="65">
         <f>IFERROR(DATEDIF(F45,G45,"M"),"")</f>
         <v/>
       </c>
-      <c r="K45" s="71" t="n"/>
-      <c r="L45" s="77">
+      <c r="K45" s="72" t="n"/>
+      <c r="L45" s="78">
         <f>IFERROR(IF(K45="","",K45/12),"")</f>
         <v/>
       </c>
-      <c r="M45" s="69" t="n"/>
-      <c r="N45" s="80" t="n"/>
-      <c r="O45" s="79">
+      <c r="M45" s="70" t="n"/>
+      <c r="N45" s="81" t="n"/>
+      <c r="O45" s="80">
         <f>IFERROR(IF(G45="","",G45-365),"")</f>
         <v/>
       </c>
-      <c r="P45" s="69" t="n"/>
+      <c r="P45" s="70" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="72" t="n"/>
-      <c r="B46" s="72" t="n"/>
-      <c r="C46" s="72" t="n"/>
-      <c r="D46" s="72" t="n"/>
-      <c r="E46" s="73" t="n"/>
-      <c r="F46" s="73" t="n"/>
-      <c r="G46" s="73" t="n"/>
-      <c r="H46" s="72" t="n"/>
-      <c r="I46" s="72" t="n"/>
+      <c r="A46" s="73" t="n"/>
+      <c r="B46" s="73" t="n"/>
+      <c r="C46" s="73" t="n"/>
+      <c r="D46" s="73" t="n"/>
+      <c r="E46" s="74" t="n"/>
+      <c r="F46" s="74" t="n"/>
+      <c r="G46" s="74" t="n"/>
+      <c r="H46" s="73" t="n"/>
+      <c r="I46" s="73" t="n"/>
       <c r="J46" s="65">
         <f>IFERROR(DATEDIF(F46,G46,"M"),"")</f>
         <v/>
       </c>
-      <c r="K46" s="74" t="n"/>
-      <c r="L46" s="77">
+      <c r="K46" s="75" t="n"/>
+      <c r="L46" s="78">
         <f>IFERROR(IF(K46="","",K46/12),"")</f>
         <v/>
       </c>
-      <c r="M46" s="72" t="n"/>
-      <c r="N46" s="81" t="n"/>
-      <c r="O46" s="79">
+      <c r="M46" s="73" t="n"/>
+      <c r="N46" s="82" t="n"/>
+      <c r="O46" s="80">
         <f>IFERROR(IF(G46="","",G46-365),"")</f>
         <v/>
       </c>
-      <c r="P46" s="72" t="n"/>
+      <c r="P46" s="73" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="69" t="n"/>
-      <c r="B47" s="69" t="n"/>
-      <c r="C47" s="69" t="n"/>
-      <c r="D47" s="69" t="n"/>
-      <c r="E47" s="70" t="n"/>
-      <c r="F47" s="70" t="n"/>
-      <c r="G47" s="70" t="n"/>
-      <c r="H47" s="69" t="n"/>
-      <c r="I47" s="69" t="n"/>
+      <c r="A47" s="70" t="n"/>
+      <c r="B47" s="70" t="n"/>
+      <c r="C47" s="70" t="n"/>
+      <c r="D47" s="70" t="n"/>
+      <c r="E47" s="71" t="n"/>
+      <c r="F47" s="71" t="n"/>
+      <c r="G47" s="71" t="n"/>
+      <c r="H47" s="70" t="n"/>
+      <c r="I47" s="70" t="n"/>
       <c r="J47" s="65">
         <f>IFERROR(DATEDIF(F47,G47,"M"),"")</f>
         <v/>
       </c>
-      <c r="K47" s="71" t="n"/>
-      <c r="L47" s="77">
+      <c r="K47" s="72" t="n"/>
+      <c r="L47" s="78">
         <f>IFERROR(IF(K47="","",K47/12),"")</f>
         <v/>
       </c>
-      <c r="M47" s="69" t="n"/>
-      <c r="N47" s="80" t="n"/>
-      <c r="O47" s="79">
+      <c r="M47" s="70" t="n"/>
+      <c r="N47" s="81" t="n"/>
+      <c r="O47" s="80">
         <f>IFERROR(IF(G47="","",G47-365),"")</f>
         <v/>
       </c>
-      <c r="P47" s="69" t="n"/>
+      <c r="P47" s="70" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="72" t="n"/>
-      <c r="B48" s="72" t="n"/>
-      <c r="C48" s="72" t="n"/>
-      <c r="D48" s="72" t="n"/>
-      <c r="E48" s="73" t="n"/>
-      <c r="F48" s="73" t="n"/>
-      <c r="G48" s="73" t="n"/>
-      <c r="H48" s="72" t="n"/>
-      <c r="I48" s="72" t="n"/>
+      <c r="A48" s="73" t="n"/>
+      <c r="B48" s="73" t="n"/>
+      <c r="C48" s="73" t="n"/>
+      <c r="D48" s="73" t="n"/>
+      <c r="E48" s="74" t="n"/>
+      <c r="F48" s="74" t="n"/>
+      <c r="G48" s="74" t="n"/>
+      <c r="H48" s="73" t="n"/>
+      <c r="I48" s="73" t="n"/>
       <c r="J48" s="65">
         <f>IFERROR(DATEDIF(F48,G48,"M"),"")</f>
         <v/>
       </c>
-      <c r="K48" s="74" t="n"/>
-      <c r="L48" s="77">
+      <c r="K48" s="75" t="n"/>
+      <c r="L48" s="78">
         <f>IFERROR(IF(K48="","",K48/12),"")</f>
         <v/>
       </c>
-      <c r="M48" s="72" t="n"/>
-      <c r="N48" s="81" t="n"/>
-      <c r="O48" s="79">
+      <c r="M48" s="73" t="n"/>
+      <c r="N48" s="82" t="n"/>
+      <c r="O48" s="80">
         <f>IFERROR(IF(G48="","",G48-365),"")</f>
         <v/>
       </c>
-      <c r="P48" s="72" t="n"/>
+      <c r="P48" s="73" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="69" t="n"/>
-      <c r="B49" s="69" t="n"/>
-      <c r="C49" s="69" t="n"/>
-      <c r="D49" s="69" t="n"/>
-      <c r="E49" s="70" t="n"/>
-      <c r="F49" s="70" t="n"/>
-      <c r="G49" s="70" t="n"/>
-      <c r="H49" s="69" t="n"/>
-      <c r="I49" s="69" t="n"/>
+      <c r="A49" s="70" t="n"/>
+      <c r="B49" s="70" t="n"/>
+      <c r="C49" s="70" t="n"/>
+      <c r="D49" s="70" t="n"/>
+      <c r="E49" s="71" t="n"/>
+      <c r="F49" s="71" t="n"/>
+      <c r="G49" s="71" t="n"/>
+      <c r="H49" s="70" t="n"/>
+      <c r="I49" s="70" t="n"/>
       <c r="J49" s="65">
         <f>IFERROR(DATEDIF(F49,G49,"M"),"")</f>
         <v/>
       </c>
-      <c r="K49" s="71" t="n"/>
-      <c r="L49" s="77">
+      <c r="K49" s="72" t="n"/>
+      <c r="L49" s="78">
         <f>IFERROR(IF(K49="","",K49/12),"")</f>
         <v/>
       </c>
-      <c r="M49" s="69" t="n"/>
-      <c r="N49" s="80" t="n"/>
-      <c r="O49" s="79">
+      <c r="M49" s="70" t="n"/>
+      <c r="N49" s="81" t="n"/>
+      <c r="O49" s="80">
         <f>IFERROR(IF(G49="","",G49-365),"")</f>
         <v/>
       </c>
-      <c r="P49" s="69" t="n"/>
+      <c r="P49" s="70" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="72" t="n"/>
-      <c r="B50" s="72" t="n"/>
-      <c r="C50" s="72" t="n"/>
-      <c r="D50" s="72" t="n"/>
-      <c r="E50" s="73" t="n"/>
-      <c r="F50" s="73" t="n"/>
-      <c r="G50" s="73" t="n"/>
-      <c r="H50" s="72" t="n"/>
-      <c r="I50" s="72" t="n"/>
+      <c r="A50" s="73" t="n"/>
+      <c r="B50" s="73" t="n"/>
+      <c r="C50" s="73" t="n"/>
+      <c r="D50" s="73" t="n"/>
+      <c r="E50" s="74" t="n"/>
+      <c r="F50" s="74" t="n"/>
+      <c r="G50" s="74" t="n"/>
+      <c r="H50" s="73" t="n"/>
+      <c r="I50" s="73" t="n"/>
       <c r="J50" s="65">
         <f>IFERROR(DATEDIF(F50,G50,"M"),"")</f>
         <v/>
       </c>
-      <c r="K50" s="74" t="n"/>
-      <c r="L50" s="77">
+      <c r="K50" s="75" t="n"/>
+      <c r="L50" s="78">
         <f>IFERROR(IF(K50="","",K50/12),"")</f>
         <v/>
       </c>
-      <c r="M50" s="72" t="n"/>
-      <c r="N50" s="81" t="n"/>
-      <c r="O50" s="79">
+      <c r="M50" s="73" t="n"/>
+      <c r="N50" s="82" t="n"/>
+      <c r="O50" s="80">
         <f>IFERROR(IF(G50="","",G50-365),"")</f>
         <v/>
       </c>
-      <c r="P50" s="72" t="n"/>
+      <c r="P50" s="73" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="69" t="n"/>
-      <c r="B51" s="69" t="n"/>
-      <c r="C51" s="69" t="n"/>
-      <c r="D51" s="69" t="n"/>
-      <c r="E51" s="70" t="n"/>
-      <c r="F51" s="70" t="n"/>
-      <c r="G51" s="70" t="n"/>
-      <c r="H51" s="69" t="n"/>
-      <c r="I51" s="69" t="n"/>
+      <c r="A51" s="70" t="n"/>
+      <c r="B51" s="70" t="n"/>
+      <c r="C51" s="70" t="n"/>
+      <c r="D51" s="70" t="n"/>
+      <c r="E51" s="71" t="n"/>
+      <c r="F51" s="71" t="n"/>
+      <c r="G51" s="71" t="n"/>
+      <c r="H51" s="70" t="n"/>
+      <c r="I51" s="70" t="n"/>
       <c r="J51" s="65">
         <f>IFERROR(DATEDIF(F51,G51,"M"),"")</f>
         <v/>
       </c>
-      <c r="K51" s="71" t="n"/>
-      <c r="L51" s="77">
+      <c r="K51" s="72" t="n"/>
+      <c r="L51" s="78">
         <f>IFERROR(IF(K51="","",K51/12),"")</f>
         <v/>
       </c>
-      <c r="M51" s="69" t="n"/>
-      <c r="N51" s="80" t="n"/>
-      <c r="O51" s="79">
+      <c r="M51" s="70" t="n"/>
+      <c r="N51" s="81" t="n"/>
+      <c r="O51" s="80">
         <f>IFERROR(IF(G51="","",G51-365),"")</f>
         <v/>
       </c>
-      <c r="P51" s="69" t="n"/>
+      <c r="P51" s="70" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="72" t="n"/>
-      <c r="B52" s="72" t="n"/>
-      <c r="C52" s="72" t="n"/>
-      <c r="D52" s="72" t="n"/>
-      <c r="E52" s="73" t="n"/>
-      <c r="F52" s="73" t="n"/>
-      <c r="G52" s="73" t="n"/>
-      <c r="H52" s="72" t="n"/>
-      <c r="I52" s="72" t="n"/>
+      <c r="A52" s="73" t="n"/>
+      <c r="B52" s="73" t="n"/>
+      <c r="C52" s="73" t="n"/>
+      <c r="D52" s="73" t="n"/>
+      <c r="E52" s="74" t="n"/>
+      <c r="F52" s="74" t="n"/>
+      <c r="G52" s="74" t="n"/>
+      <c r="H52" s="73" t="n"/>
+      <c r="I52" s="73" t="n"/>
       <c r="J52" s="65">
         <f>IFERROR(DATEDIF(F52,G52,"M"),"")</f>
         <v/>
       </c>
-      <c r="K52" s="74" t="n"/>
-      <c r="L52" s="77">
+      <c r="K52" s="75" t="n"/>
+      <c r="L52" s="78">
         <f>IFERROR(IF(K52="","",K52/12),"")</f>
         <v/>
       </c>
-      <c r="M52" s="72" t="n"/>
-      <c r="N52" s="81" t="n"/>
-      <c r="O52" s="79">
+      <c r="M52" s="73" t="n"/>
+      <c r="N52" s="82" t="n"/>
+      <c r="O52" s="80">
         <f>IFERROR(IF(G52="","",G52-365),"")</f>
         <v/>
       </c>
-      <c r="P52" s="72" t="n"/>
+      <c r="P52" s="73" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="69" t="n"/>
-      <c r="B53" s="69" t="n"/>
-      <c r="C53" s="69" t="n"/>
-      <c r="D53" s="69" t="n"/>
-      <c r="E53" s="70" t="n"/>
-      <c r="F53" s="70" t="n"/>
-      <c r="G53" s="70" t="n"/>
-      <c r="H53" s="69" t="n"/>
-      <c r="I53" s="69" t="n"/>
+      <c r="A53" s="70" t="n"/>
+      <c r="B53" s="70" t="n"/>
+      <c r="C53" s="70" t="n"/>
+      <c r="D53" s="70" t="n"/>
+      <c r="E53" s="71" t="n"/>
+      <c r="F53" s="71" t="n"/>
+      <c r="G53" s="71" t="n"/>
+      <c r="H53" s="70" t="n"/>
+      <c r="I53" s="70" t="n"/>
       <c r="J53" s="65">
         <f>IFERROR(DATEDIF(F53,G53,"M"),"")</f>
         <v/>
       </c>
-      <c r="K53" s="71" t="n"/>
-      <c r="L53" s="77">
+      <c r="K53" s="72" t="n"/>
+      <c r="L53" s="78">
         <f>IFERROR(IF(K53="","",K53/12),"")</f>
         <v/>
       </c>
-      <c r="M53" s="69" t="n"/>
-      <c r="N53" s="80" t="n"/>
-      <c r="O53" s="79">
+      <c r="M53" s="70" t="n"/>
+      <c r="N53" s="81" t="n"/>
+      <c r="O53" s="80">
         <f>IFERROR(IF(G53="","",G53-365),"")</f>
         <v/>
       </c>
-      <c r="P53" s="69" t="n"/>
+      <c r="P53" s="70" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Emergency contacts added and form layout repaired
</commit_message>
<xml_diff>
--- a/Tenant_Manager.xlsx
+++ b/Tenant_Manager.xlsx
@@ -278,7 +278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -475,9 +475,6 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1903,7 +1900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2092,51 +2089,51 @@
       </c>
       <c r="D24" s="56" t="n"/>
     </row>
-    <row r="27">
-      <c r="B27" s="57" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="57" t="inlineStr">
         <is>
           <t>Additional Notes / Special Conditions</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="58" t="n"/>
-    </row>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
+    <row r="31">
+      <c r="B31" s="58" t="n"/>
+    </row>
     <row r="32"/>
-    <row r="35">
-      <c r="B35" t="inlineStr">
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="38">
+      <c r="B38" t="inlineStr">
         <is>
           <t>Tenant Signature</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Property Manager</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="B36" s="58" t="n"/>
-      <c r="E36" s="58" t="n"/>
-    </row>
     <row r="39">
-      <c r="A39" s="59" t="inlineStr">
+      <c r="B39" s="58" t="n"/>
+      <c r="E39" s="58" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="59" t="inlineStr">
         <is>
           <t>Transfer approved tenant records into TENANTS sheet</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="D41" s="60" t="inlineStr">
+    <row r="44">
+      <c r="D44" s="60" t="inlineStr">
         <is>
           <t>▶ SUBMIT TENANT</t>
         </is>
       </c>
     </row>
-    <row r="42"/>
+    <row r="45"/>
   </sheetData>
   <mergeCells count="28">
     <mergeCell ref="D11:F11"/>
@@ -2144,9 +2141,10 @@
     <mergeCell ref="D17:F17"/>
     <mergeCell ref="D7:F7"/>
     <mergeCell ref="D16:F16"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="E38:F38"/>
+    <mergeCell ref="D44:F45"/>
+    <mergeCell ref="B31:F35"/>
     <mergeCell ref="D12:F12"/>
     <mergeCell ref="D18:F18"/>
     <mergeCell ref="D9:F9"/>
@@ -2156,17 +2154,16 @@
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="D23:F23"/>
-    <mergeCell ref="B35:D35"/>
     <mergeCell ref="D20:F20"/>
-    <mergeCell ref="D41:F42"/>
     <mergeCell ref="D10:F10"/>
+    <mergeCell ref="B30:F30"/>
     <mergeCell ref="D19:F19"/>
-    <mergeCell ref="B28:F32"/>
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="D22:F22"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="D21:F21"/>
     <mergeCell ref="D6:F6"/>
+    <mergeCell ref="A42:G42"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation sqref="D12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -2429,31 +2426,31 @@
         <f>IFERROR(IF(B4="","Vacant",IF(Q4&lt;0,"Expired",IF(Q4&lt;=30,"Expiring Soon",IF(Q4&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S4" s="69" t="n"/>
-      <c r="T4" s="69" t="n"/>
-      <c r="U4" s="69" t="n"/>
-      <c r="V4" s="69" t="n"/>
+      <c r="S4" s="63" t="n"/>
+      <c r="T4" s="63" t="n"/>
+      <c r="U4" s="63" t="n"/>
+      <c r="V4" s="63" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="70" t="n"/>
-      <c r="B5" s="70" t="n"/>
-      <c r="C5" s="70" t="n"/>
-      <c r="D5" s="70" t="n"/>
-      <c r="E5" s="70" t="n"/>
-      <c r="F5" s="70" t="n"/>
-      <c r="G5" s="70" t="n"/>
-      <c r="H5" s="70" t="n"/>
-      <c r="I5" s="71" t="n"/>
-      <c r="J5" s="71" t="n"/>
+      <c r="A5" s="69" t="n"/>
+      <c r="B5" s="69" t="n"/>
+      <c r="C5" s="69" t="n"/>
+      <c r="D5" s="69" t="n"/>
+      <c r="E5" s="69" t="n"/>
+      <c r="F5" s="69" t="n"/>
+      <c r="G5" s="69" t="n"/>
+      <c r="H5" s="69" t="n"/>
+      <c r="I5" s="70" t="n"/>
+      <c r="J5" s="70" t="n"/>
       <c r="K5" s="65">
         <f>IFERROR(DATEDIF(I5,J5,"M"),"")</f>
         <v/>
       </c>
-      <c r="L5" s="72" t="n"/>
-      <c r="M5" s="70" t="n"/>
-      <c r="N5" s="70" t="n"/>
-      <c r="O5" s="72" t="n"/>
-      <c r="P5" s="70" t="n"/>
+      <c r="L5" s="71" t="n"/>
+      <c r="M5" s="69" t="n"/>
+      <c r="N5" s="69" t="n"/>
+      <c r="O5" s="71" t="n"/>
+      <c r="P5" s="69" t="n"/>
       <c r="Q5" s="67">
         <f>IFERROR(IF(J5="","",J5-TODAY()),"")</f>
         <v/>
@@ -2468,25 +2465,25 @@
       <c r="V5" s="69" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="73" t="n"/>
-      <c r="B6" s="73" t="n"/>
-      <c r="C6" s="73" t="n"/>
-      <c r="D6" s="73" t="n"/>
-      <c r="E6" s="73" t="n"/>
-      <c r="F6" s="73" t="n"/>
-      <c r="G6" s="73" t="n"/>
-      <c r="H6" s="73" t="n"/>
-      <c r="I6" s="74" t="n"/>
-      <c r="J6" s="74" t="n"/>
+      <c r="A6" s="72" t="n"/>
+      <c r="B6" s="72" t="n"/>
+      <c r="C6" s="72" t="n"/>
+      <c r="D6" s="72" t="n"/>
+      <c r="E6" s="72" t="n"/>
+      <c r="F6" s="72" t="n"/>
+      <c r="G6" s="72" t="n"/>
+      <c r="H6" s="72" t="n"/>
+      <c r="I6" s="73" t="n"/>
+      <c r="J6" s="73" t="n"/>
       <c r="K6" s="65">
         <f>IFERROR(DATEDIF(I6,J6,"M"),"")</f>
         <v/>
       </c>
-      <c r="L6" s="75" t="n"/>
-      <c r="M6" s="73" t="n"/>
-      <c r="N6" s="73" t="n"/>
-      <c r="O6" s="75" t="n"/>
-      <c r="P6" s="73" t="n"/>
+      <c r="L6" s="74" t="n"/>
+      <c r="M6" s="72" t="n"/>
+      <c r="N6" s="72" t="n"/>
+      <c r="O6" s="74" t="n"/>
+      <c r="P6" s="72" t="n"/>
       <c r="Q6" s="67">
         <f>IFERROR(IF(J6="","",J6-TODAY()),"")</f>
         <v/>
@@ -2495,31 +2492,31 @@
         <f>IFERROR(IF(B6="","Vacant",IF(Q6&lt;0,"Expired",IF(Q6&lt;=30,"Expiring Soon",IF(Q6&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S6" s="69" t="n"/>
-      <c r="T6" s="69" t="n"/>
-      <c r="U6" s="69" t="n"/>
-      <c r="V6" s="69" t="n"/>
+      <c r="S6" s="72" t="n"/>
+      <c r="T6" s="72" t="n"/>
+      <c r="U6" s="72" t="n"/>
+      <c r="V6" s="72" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="70" t="n"/>
-      <c r="B7" s="70" t="n"/>
-      <c r="C7" s="70" t="n"/>
-      <c r="D7" s="70" t="n"/>
-      <c r="E7" s="70" t="n"/>
-      <c r="F7" s="70" t="n"/>
-      <c r="G7" s="70" t="n"/>
-      <c r="H7" s="70" t="n"/>
-      <c r="I7" s="71" t="n"/>
-      <c r="J7" s="71" t="n"/>
+      <c r="A7" s="69" t="n"/>
+      <c r="B7" s="69" t="n"/>
+      <c r="C7" s="69" t="n"/>
+      <c r="D7" s="69" t="n"/>
+      <c r="E7" s="69" t="n"/>
+      <c r="F7" s="69" t="n"/>
+      <c r="G7" s="69" t="n"/>
+      <c r="H7" s="69" t="n"/>
+      <c r="I7" s="70" t="n"/>
+      <c r="J7" s="70" t="n"/>
       <c r="K7" s="65">
         <f>IFERROR(DATEDIF(I7,J7,"M"),"")</f>
         <v/>
       </c>
-      <c r="L7" s="72" t="n"/>
-      <c r="M7" s="70" t="n"/>
-      <c r="N7" s="70" t="n"/>
-      <c r="O7" s="72" t="n"/>
-      <c r="P7" s="70" t="n"/>
+      <c r="L7" s="71" t="n"/>
+      <c r="M7" s="69" t="n"/>
+      <c r="N7" s="69" t="n"/>
+      <c r="O7" s="71" t="n"/>
+      <c r="P7" s="69" t="n"/>
       <c r="Q7" s="67">
         <f>IFERROR(IF(J7="","",J7-TODAY()),"")</f>
         <v/>
@@ -2534,25 +2531,25 @@
       <c r="V7" s="69" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="73" t="n"/>
-      <c r="B8" s="73" t="n"/>
-      <c r="C8" s="73" t="n"/>
-      <c r="D8" s="73" t="n"/>
-      <c r="E8" s="73" t="n"/>
-      <c r="F8" s="73" t="n"/>
-      <c r="G8" s="73" t="n"/>
-      <c r="H8" s="73" t="n"/>
-      <c r="I8" s="74" t="n"/>
-      <c r="J8" s="74" t="n"/>
+      <c r="A8" s="72" t="n"/>
+      <c r="B8" s="72" t="n"/>
+      <c r="C8" s="72" t="n"/>
+      <c r="D8" s="72" t="n"/>
+      <c r="E8" s="72" t="n"/>
+      <c r="F8" s="72" t="n"/>
+      <c r="G8" s="72" t="n"/>
+      <c r="H8" s="72" t="n"/>
+      <c r="I8" s="73" t="n"/>
+      <c r="J8" s="73" t="n"/>
       <c r="K8" s="65">
         <f>IFERROR(DATEDIF(I8,J8,"M"),"")</f>
         <v/>
       </c>
-      <c r="L8" s="75" t="n"/>
-      <c r="M8" s="73" t="n"/>
-      <c r="N8" s="73" t="n"/>
-      <c r="O8" s="75" t="n"/>
-      <c r="P8" s="73" t="n"/>
+      <c r="L8" s="74" t="n"/>
+      <c r="M8" s="72" t="n"/>
+      <c r="N8" s="72" t="n"/>
+      <c r="O8" s="74" t="n"/>
+      <c r="P8" s="72" t="n"/>
       <c r="Q8" s="67">
         <f>IFERROR(IF(J8="","",J8-TODAY()),"")</f>
         <v/>
@@ -2561,31 +2558,31 @@
         <f>IFERROR(IF(B8="","Vacant",IF(Q8&lt;0,"Expired",IF(Q8&lt;=30,"Expiring Soon",IF(Q8&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S8" s="69" t="n"/>
-      <c r="T8" s="69" t="n"/>
-      <c r="U8" s="69" t="n"/>
-      <c r="V8" s="69" t="n"/>
+      <c r="S8" s="72" t="n"/>
+      <c r="T8" s="72" t="n"/>
+      <c r="U8" s="72" t="n"/>
+      <c r="V8" s="72" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="70" t="n"/>
-      <c r="B9" s="70" t="n"/>
-      <c r="C9" s="70" t="n"/>
-      <c r="D9" s="70" t="n"/>
-      <c r="E9" s="70" t="n"/>
-      <c r="F9" s="70" t="n"/>
-      <c r="G9" s="70" t="n"/>
-      <c r="H9" s="70" t="n"/>
-      <c r="I9" s="71" t="n"/>
-      <c r="J9" s="71" t="n"/>
+      <c r="A9" s="69" t="n"/>
+      <c r="B9" s="69" t="n"/>
+      <c r="C9" s="69" t="n"/>
+      <c r="D9" s="69" t="n"/>
+      <c r="E9" s="69" t="n"/>
+      <c r="F9" s="69" t="n"/>
+      <c r="G9" s="69" t="n"/>
+      <c r="H9" s="69" t="n"/>
+      <c r="I9" s="70" t="n"/>
+      <c r="J9" s="70" t="n"/>
       <c r="K9" s="65">
         <f>IFERROR(DATEDIF(I9,J9,"M"),"")</f>
         <v/>
       </c>
-      <c r="L9" s="72" t="n"/>
-      <c r="M9" s="70" t="n"/>
-      <c r="N9" s="70" t="n"/>
-      <c r="O9" s="72" t="n"/>
-      <c r="P9" s="70" t="n"/>
+      <c r="L9" s="71" t="n"/>
+      <c r="M9" s="69" t="n"/>
+      <c r="N9" s="69" t="n"/>
+      <c r="O9" s="71" t="n"/>
+      <c r="P9" s="69" t="n"/>
       <c r="Q9" s="67">
         <f>IFERROR(IF(J9="","",J9-TODAY()),"")</f>
         <v/>
@@ -2600,25 +2597,25 @@
       <c r="V9" s="69" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="73" t="n"/>
-      <c r="B10" s="73" t="n"/>
-      <c r="C10" s="73" t="n"/>
-      <c r="D10" s="73" t="n"/>
-      <c r="E10" s="73" t="n"/>
-      <c r="F10" s="73" t="n"/>
-      <c r="G10" s="73" t="n"/>
-      <c r="H10" s="73" t="n"/>
-      <c r="I10" s="74" t="n"/>
-      <c r="J10" s="74" t="n"/>
+      <c r="A10" s="72" t="n"/>
+      <c r="B10" s="72" t="n"/>
+      <c r="C10" s="72" t="n"/>
+      <c r="D10" s="72" t="n"/>
+      <c r="E10" s="72" t="n"/>
+      <c r="F10" s="72" t="n"/>
+      <c r="G10" s="72" t="n"/>
+      <c r="H10" s="72" t="n"/>
+      <c r="I10" s="73" t="n"/>
+      <c r="J10" s="73" t="n"/>
       <c r="K10" s="65">
         <f>IFERROR(DATEDIF(I10,J10,"M"),"")</f>
         <v/>
       </c>
-      <c r="L10" s="75" t="n"/>
-      <c r="M10" s="73" t="n"/>
-      <c r="N10" s="73" t="n"/>
-      <c r="O10" s="75" t="n"/>
-      <c r="P10" s="73" t="n"/>
+      <c r="L10" s="74" t="n"/>
+      <c r="M10" s="72" t="n"/>
+      <c r="N10" s="72" t="n"/>
+      <c r="O10" s="74" t="n"/>
+      <c r="P10" s="72" t="n"/>
       <c r="Q10" s="67">
         <f>IFERROR(IF(J10="","",J10-TODAY()),"")</f>
         <v/>
@@ -2627,31 +2624,31 @@
         <f>IFERROR(IF(B10="","Vacant",IF(Q10&lt;0,"Expired",IF(Q10&lt;=30,"Expiring Soon",IF(Q10&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S10" s="69" t="n"/>
-      <c r="T10" s="69" t="n"/>
-      <c r="U10" s="69" t="n"/>
-      <c r="V10" s="69" t="n"/>
+      <c r="S10" s="72" t="n"/>
+      <c r="T10" s="72" t="n"/>
+      <c r="U10" s="72" t="n"/>
+      <c r="V10" s="72" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="70" t="n"/>
-      <c r="B11" s="70" t="n"/>
-      <c r="C11" s="70" t="n"/>
-      <c r="D11" s="70" t="n"/>
-      <c r="E11" s="70" t="n"/>
-      <c r="F11" s="70" t="n"/>
-      <c r="G11" s="70" t="n"/>
-      <c r="H11" s="70" t="n"/>
-      <c r="I11" s="71" t="n"/>
-      <c r="J11" s="71" t="n"/>
+      <c r="A11" s="69" t="n"/>
+      <c r="B11" s="69" t="n"/>
+      <c r="C11" s="69" t="n"/>
+      <c r="D11" s="69" t="n"/>
+      <c r="E11" s="69" t="n"/>
+      <c r="F11" s="69" t="n"/>
+      <c r="G11" s="69" t="n"/>
+      <c r="H11" s="69" t="n"/>
+      <c r="I11" s="70" t="n"/>
+      <c r="J11" s="70" t="n"/>
       <c r="K11" s="65">
         <f>IFERROR(DATEDIF(I11,J11,"M"),"")</f>
         <v/>
       </c>
-      <c r="L11" s="72" t="n"/>
-      <c r="M11" s="70" t="n"/>
-      <c r="N11" s="70" t="n"/>
-      <c r="O11" s="72" t="n"/>
-      <c r="P11" s="70" t="n"/>
+      <c r="L11" s="71" t="n"/>
+      <c r="M11" s="69" t="n"/>
+      <c r="N11" s="69" t="n"/>
+      <c r="O11" s="71" t="n"/>
+      <c r="P11" s="69" t="n"/>
       <c r="Q11" s="67">
         <f>IFERROR(IF(J11="","",J11-TODAY()),"")</f>
         <v/>
@@ -2666,25 +2663,25 @@
       <c r="V11" s="69" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="73" t="n"/>
-      <c r="B12" s="73" t="n"/>
-      <c r="C12" s="73" t="n"/>
-      <c r="D12" s="73" t="n"/>
-      <c r="E12" s="73" t="n"/>
-      <c r="F12" s="73" t="n"/>
-      <c r="G12" s="73" t="n"/>
-      <c r="H12" s="73" t="n"/>
-      <c r="I12" s="74" t="n"/>
-      <c r="J12" s="74" t="n"/>
+      <c r="A12" s="72" t="n"/>
+      <c r="B12" s="72" t="n"/>
+      <c r="C12" s="72" t="n"/>
+      <c r="D12" s="72" t="n"/>
+      <c r="E12" s="72" t="n"/>
+      <c r="F12" s="72" t="n"/>
+      <c r="G12" s="72" t="n"/>
+      <c r="H12" s="72" t="n"/>
+      <c r="I12" s="73" t="n"/>
+      <c r="J12" s="73" t="n"/>
       <c r="K12" s="65">
         <f>IFERROR(DATEDIF(I12,J12,"M"),"")</f>
         <v/>
       </c>
-      <c r="L12" s="75" t="n"/>
-      <c r="M12" s="73" t="n"/>
-      <c r="N12" s="73" t="n"/>
-      <c r="O12" s="75" t="n"/>
-      <c r="P12" s="73" t="n"/>
+      <c r="L12" s="74" t="n"/>
+      <c r="M12" s="72" t="n"/>
+      <c r="N12" s="72" t="n"/>
+      <c r="O12" s="74" t="n"/>
+      <c r="P12" s="72" t="n"/>
       <c r="Q12" s="67">
         <f>IFERROR(IF(J12="","",J12-TODAY()),"")</f>
         <v/>
@@ -2693,31 +2690,31 @@
         <f>IFERROR(IF(B12="","Vacant",IF(Q12&lt;0,"Expired",IF(Q12&lt;=30,"Expiring Soon",IF(Q12&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S12" s="69" t="n"/>
-      <c r="T12" s="69" t="n"/>
-      <c r="U12" s="69" t="n"/>
-      <c r="V12" s="69" t="n"/>
+      <c r="S12" s="72" t="n"/>
+      <c r="T12" s="72" t="n"/>
+      <c r="U12" s="72" t="n"/>
+      <c r="V12" s="72" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="70" t="n"/>
-      <c r="B13" s="70" t="n"/>
-      <c r="C13" s="70" t="n"/>
-      <c r="D13" s="70" t="n"/>
-      <c r="E13" s="70" t="n"/>
-      <c r="F13" s="70" t="n"/>
-      <c r="G13" s="70" t="n"/>
-      <c r="H13" s="70" t="n"/>
-      <c r="I13" s="71" t="n"/>
-      <c r="J13" s="71" t="n"/>
+      <c r="A13" s="69" t="n"/>
+      <c r="B13" s="69" t="n"/>
+      <c r="C13" s="69" t="n"/>
+      <c r="D13" s="69" t="n"/>
+      <c r="E13" s="69" t="n"/>
+      <c r="F13" s="69" t="n"/>
+      <c r="G13" s="69" t="n"/>
+      <c r="H13" s="69" t="n"/>
+      <c r="I13" s="70" t="n"/>
+      <c r="J13" s="70" t="n"/>
       <c r="K13" s="65">
         <f>IFERROR(DATEDIF(I13,J13,"M"),"")</f>
         <v/>
       </c>
-      <c r="L13" s="72" t="n"/>
-      <c r="M13" s="70" t="n"/>
-      <c r="N13" s="70" t="n"/>
-      <c r="O13" s="72" t="n"/>
-      <c r="P13" s="70" t="n"/>
+      <c r="L13" s="71" t="n"/>
+      <c r="M13" s="69" t="n"/>
+      <c r="N13" s="69" t="n"/>
+      <c r="O13" s="71" t="n"/>
+      <c r="P13" s="69" t="n"/>
       <c r="Q13" s="67">
         <f>IFERROR(IF(J13="","",J13-TODAY()),"")</f>
         <v/>
@@ -2732,25 +2729,25 @@
       <c r="V13" s="69" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="73" t="n"/>
-      <c r="B14" s="73" t="n"/>
-      <c r="C14" s="73" t="n"/>
-      <c r="D14" s="73" t="n"/>
-      <c r="E14" s="73" t="n"/>
-      <c r="F14" s="73" t="n"/>
-      <c r="G14" s="73" t="n"/>
-      <c r="H14" s="73" t="n"/>
-      <c r="I14" s="74" t="n"/>
-      <c r="J14" s="74" t="n"/>
+      <c r="A14" s="72" t="n"/>
+      <c r="B14" s="72" t="n"/>
+      <c r="C14" s="72" t="n"/>
+      <c r="D14" s="72" t="n"/>
+      <c r="E14" s="72" t="n"/>
+      <c r="F14" s="72" t="n"/>
+      <c r="G14" s="72" t="n"/>
+      <c r="H14" s="72" t="n"/>
+      <c r="I14" s="73" t="n"/>
+      <c r="J14" s="73" t="n"/>
       <c r="K14" s="65">
         <f>IFERROR(DATEDIF(I14,J14,"M"),"")</f>
         <v/>
       </c>
-      <c r="L14" s="75" t="n"/>
-      <c r="M14" s="73" t="n"/>
-      <c r="N14" s="73" t="n"/>
-      <c r="O14" s="75" t="n"/>
-      <c r="P14" s="73" t="n"/>
+      <c r="L14" s="74" t="n"/>
+      <c r="M14" s="72" t="n"/>
+      <c r="N14" s="72" t="n"/>
+      <c r="O14" s="74" t="n"/>
+      <c r="P14" s="72" t="n"/>
       <c r="Q14" s="67">
         <f>IFERROR(IF(J14="","",J14-TODAY()),"")</f>
         <v/>
@@ -2759,31 +2756,31 @@
         <f>IFERROR(IF(B14="","Vacant",IF(Q14&lt;0,"Expired",IF(Q14&lt;=30,"Expiring Soon",IF(Q14&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S14" s="69" t="n"/>
-      <c r="T14" s="69" t="n"/>
-      <c r="U14" s="69" t="n"/>
-      <c r="V14" s="69" t="n"/>
+      <c r="S14" s="72" t="n"/>
+      <c r="T14" s="72" t="n"/>
+      <c r="U14" s="72" t="n"/>
+      <c r="V14" s="72" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="70" t="n"/>
-      <c r="B15" s="70" t="n"/>
-      <c r="C15" s="70" t="n"/>
-      <c r="D15" s="70" t="n"/>
-      <c r="E15" s="70" t="n"/>
-      <c r="F15" s="70" t="n"/>
-      <c r="G15" s="70" t="n"/>
-      <c r="H15" s="70" t="n"/>
-      <c r="I15" s="71" t="n"/>
-      <c r="J15" s="71" t="n"/>
+      <c r="A15" s="69" t="n"/>
+      <c r="B15" s="69" t="n"/>
+      <c r="C15" s="69" t="n"/>
+      <c r="D15" s="69" t="n"/>
+      <c r="E15" s="69" t="n"/>
+      <c r="F15" s="69" t="n"/>
+      <c r="G15" s="69" t="n"/>
+      <c r="H15" s="69" t="n"/>
+      <c r="I15" s="70" t="n"/>
+      <c r="J15" s="70" t="n"/>
       <c r="K15" s="65">
         <f>IFERROR(DATEDIF(I15,J15,"M"),"")</f>
         <v/>
       </c>
-      <c r="L15" s="72" t="n"/>
-      <c r="M15" s="70" t="n"/>
-      <c r="N15" s="70" t="n"/>
-      <c r="O15" s="72" t="n"/>
-      <c r="P15" s="70" t="n"/>
+      <c r="L15" s="71" t="n"/>
+      <c r="M15" s="69" t="n"/>
+      <c r="N15" s="69" t="n"/>
+      <c r="O15" s="71" t="n"/>
+      <c r="P15" s="69" t="n"/>
       <c r="Q15" s="67">
         <f>IFERROR(IF(J15="","",J15-TODAY()),"")</f>
         <v/>
@@ -2798,25 +2795,25 @@
       <c r="V15" s="69" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="73" t="n"/>
-      <c r="B16" s="73" t="n"/>
-      <c r="C16" s="73" t="n"/>
-      <c r="D16" s="73" t="n"/>
-      <c r="E16" s="73" t="n"/>
-      <c r="F16" s="73" t="n"/>
-      <c r="G16" s="73" t="n"/>
-      <c r="H16" s="73" t="n"/>
-      <c r="I16" s="74" t="n"/>
-      <c r="J16" s="74" t="n"/>
+      <c r="A16" s="72" t="n"/>
+      <c r="B16" s="72" t="n"/>
+      <c r="C16" s="72" t="n"/>
+      <c r="D16" s="72" t="n"/>
+      <c r="E16" s="72" t="n"/>
+      <c r="F16" s="72" t="n"/>
+      <c r="G16" s="72" t="n"/>
+      <c r="H16" s="72" t="n"/>
+      <c r="I16" s="73" t="n"/>
+      <c r="J16" s="73" t="n"/>
       <c r="K16" s="65">
         <f>IFERROR(DATEDIF(I16,J16,"M"),"")</f>
         <v/>
       </c>
-      <c r="L16" s="75" t="n"/>
-      <c r="M16" s="73" t="n"/>
-      <c r="N16" s="73" t="n"/>
-      <c r="O16" s="75" t="n"/>
-      <c r="P16" s="73" t="n"/>
+      <c r="L16" s="74" t="n"/>
+      <c r="M16" s="72" t="n"/>
+      <c r="N16" s="72" t="n"/>
+      <c r="O16" s="74" t="n"/>
+      <c r="P16" s="72" t="n"/>
       <c r="Q16" s="67">
         <f>IFERROR(IF(J16="","",J16-TODAY()),"")</f>
         <v/>
@@ -2825,31 +2822,31 @@
         <f>IFERROR(IF(B16="","Vacant",IF(Q16&lt;0,"Expired",IF(Q16&lt;=30,"Expiring Soon",IF(Q16&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S16" s="69" t="n"/>
-      <c r="T16" s="69" t="n"/>
-      <c r="U16" s="69" t="n"/>
-      <c r="V16" s="69" t="n"/>
+      <c r="S16" s="72" t="n"/>
+      <c r="T16" s="72" t="n"/>
+      <c r="U16" s="72" t="n"/>
+      <c r="V16" s="72" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="70" t="n"/>
-      <c r="B17" s="70" t="n"/>
-      <c r="C17" s="70" t="n"/>
-      <c r="D17" s="70" t="n"/>
-      <c r="E17" s="70" t="n"/>
-      <c r="F17" s="70" t="n"/>
-      <c r="G17" s="70" t="n"/>
-      <c r="H17" s="70" t="n"/>
-      <c r="I17" s="71" t="n"/>
-      <c r="J17" s="71" t="n"/>
+      <c r="A17" s="69" t="n"/>
+      <c r="B17" s="69" t="n"/>
+      <c r="C17" s="69" t="n"/>
+      <c r="D17" s="69" t="n"/>
+      <c r="E17" s="69" t="n"/>
+      <c r="F17" s="69" t="n"/>
+      <c r="G17" s="69" t="n"/>
+      <c r="H17" s="69" t="n"/>
+      <c r="I17" s="70" t="n"/>
+      <c r="J17" s="70" t="n"/>
       <c r="K17" s="65">
         <f>IFERROR(DATEDIF(I17,J17,"M"),"")</f>
         <v/>
       </c>
-      <c r="L17" s="72" t="n"/>
-      <c r="M17" s="70" t="n"/>
-      <c r="N17" s="70" t="n"/>
-      <c r="O17" s="72" t="n"/>
-      <c r="P17" s="70" t="n"/>
+      <c r="L17" s="71" t="n"/>
+      <c r="M17" s="69" t="n"/>
+      <c r="N17" s="69" t="n"/>
+      <c r="O17" s="71" t="n"/>
+      <c r="P17" s="69" t="n"/>
       <c r="Q17" s="67">
         <f>IFERROR(IF(J17="","",J17-TODAY()),"")</f>
         <v/>
@@ -2864,25 +2861,25 @@
       <c r="V17" s="69" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="73" t="n"/>
-      <c r="B18" s="73" t="n"/>
-      <c r="C18" s="73" t="n"/>
-      <c r="D18" s="73" t="n"/>
-      <c r="E18" s="73" t="n"/>
-      <c r="F18" s="73" t="n"/>
-      <c r="G18" s="73" t="n"/>
-      <c r="H18" s="73" t="n"/>
-      <c r="I18" s="74" t="n"/>
-      <c r="J18" s="74" t="n"/>
+      <c r="A18" s="72" t="n"/>
+      <c r="B18" s="72" t="n"/>
+      <c r="C18" s="72" t="n"/>
+      <c r="D18" s="72" t="n"/>
+      <c r="E18" s="72" t="n"/>
+      <c r="F18" s="72" t="n"/>
+      <c r="G18" s="72" t="n"/>
+      <c r="H18" s="72" t="n"/>
+      <c r="I18" s="73" t="n"/>
+      <c r="J18" s="73" t="n"/>
       <c r="K18" s="65">
         <f>IFERROR(DATEDIF(I18,J18,"M"),"")</f>
         <v/>
       </c>
-      <c r="L18" s="75" t="n"/>
-      <c r="M18" s="73" t="n"/>
-      <c r="N18" s="73" t="n"/>
-      <c r="O18" s="75" t="n"/>
-      <c r="P18" s="73" t="n"/>
+      <c r="L18" s="74" t="n"/>
+      <c r="M18" s="72" t="n"/>
+      <c r="N18" s="72" t="n"/>
+      <c r="O18" s="74" t="n"/>
+      <c r="P18" s="72" t="n"/>
       <c r="Q18" s="67">
         <f>IFERROR(IF(J18="","",J18-TODAY()),"")</f>
         <v/>
@@ -2891,31 +2888,31 @@
         <f>IFERROR(IF(B18="","Vacant",IF(Q18&lt;0,"Expired",IF(Q18&lt;=30,"Expiring Soon",IF(Q18&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S18" s="69" t="n"/>
-      <c r="T18" s="69" t="n"/>
-      <c r="U18" s="69" t="n"/>
-      <c r="V18" s="69" t="n"/>
+      <c r="S18" s="72" t="n"/>
+      <c r="T18" s="72" t="n"/>
+      <c r="U18" s="72" t="n"/>
+      <c r="V18" s="72" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="70" t="n"/>
-      <c r="B19" s="70" t="n"/>
-      <c r="C19" s="70" t="n"/>
-      <c r="D19" s="70" t="n"/>
-      <c r="E19" s="70" t="n"/>
-      <c r="F19" s="70" t="n"/>
-      <c r="G19" s="70" t="n"/>
-      <c r="H19" s="70" t="n"/>
-      <c r="I19" s="71" t="n"/>
-      <c r="J19" s="71" t="n"/>
+      <c r="A19" s="69" t="n"/>
+      <c r="B19" s="69" t="n"/>
+      <c r="C19" s="69" t="n"/>
+      <c r="D19" s="69" t="n"/>
+      <c r="E19" s="69" t="n"/>
+      <c r="F19" s="69" t="n"/>
+      <c r="G19" s="69" t="n"/>
+      <c r="H19" s="69" t="n"/>
+      <c r="I19" s="70" t="n"/>
+      <c r="J19" s="70" t="n"/>
       <c r="K19" s="65">
         <f>IFERROR(DATEDIF(I19,J19,"M"),"")</f>
         <v/>
       </c>
-      <c r="L19" s="72" t="n"/>
-      <c r="M19" s="70" t="n"/>
-      <c r="N19" s="70" t="n"/>
-      <c r="O19" s="72" t="n"/>
-      <c r="P19" s="70" t="n"/>
+      <c r="L19" s="71" t="n"/>
+      <c r="M19" s="69" t="n"/>
+      <c r="N19" s="69" t="n"/>
+      <c r="O19" s="71" t="n"/>
+      <c r="P19" s="69" t="n"/>
       <c r="Q19" s="67">
         <f>IFERROR(IF(J19="","",J19-TODAY()),"")</f>
         <v/>
@@ -2930,25 +2927,25 @@
       <c r="V19" s="69" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="73" t="n"/>
-      <c r="B20" s="73" t="n"/>
-      <c r="C20" s="73" t="n"/>
-      <c r="D20" s="73" t="n"/>
-      <c r="E20" s="73" t="n"/>
-      <c r="F20" s="73" t="n"/>
-      <c r="G20" s="73" t="n"/>
-      <c r="H20" s="73" t="n"/>
-      <c r="I20" s="74" t="n"/>
-      <c r="J20" s="74" t="n"/>
+      <c r="A20" s="72" t="n"/>
+      <c r="B20" s="72" t="n"/>
+      <c r="C20" s="72" t="n"/>
+      <c r="D20" s="72" t="n"/>
+      <c r="E20" s="72" t="n"/>
+      <c r="F20" s="72" t="n"/>
+      <c r="G20" s="72" t="n"/>
+      <c r="H20" s="72" t="n"/>
+      <c r="I20" s="73" t="n"/>
+      <c r="J20" s="73" t="n"/>
       <c r="K20" s="65">
         <f>IFERROR(DATEDIF(I20,J20,"M"),"")</f>
         <v/>
       </c>
-      <c r="L20" s="75" t="n"/>
-      <c r="M20" s="73" t="n"/>
-      <c r="N20" s="73" t="n"/>
-      <c r="O20" s="75" t="n"/>
-      <c r="P20" s="73" t="n"/>
+      <c r="L20" s="74" t="n"/>
+      <c r="M20" s="72" t="n"/>
+      <c r="N20" s="72" t="n"/>
+      <c r="O20" s="74" t="n"/>
+      <c r="P20" s="72" t="n"/>
       <c r="Q20" s="67">
         <f>IFERROR(IF(J20="","",J20-TODAY()),"")</f>
         <v/>
@@ -2957,31 +2954,31 @@
         <f>IFERROR(IF(B20="","Vacant",IF(Q20&lt;0,"Expired",IF(Q20&lt;=30,"Expiring Soon",IF(Q20&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S20" s="69" t="n"/>
-      <c r="T20" s="69" t="n"/>
-      <c r="U20" s="69" t="n"/>
-      <c r="V20" s="69" t="n"/>
+      <c r="S20" s="72" t="n"/>
+      <c r="T20" s="72" t="n"/>
+      <c r="U20" s="72" t="n"/>
+      <c r="V20" s="72" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="70" t="n"/>
-      <c r="B21" s="70" t="n"/>
-      <c r="C21" s="70" t="n"/>
-      <c r="D21" s="70" t="n"/>
-      <c r="E21" s="70" t="n"/>
-      <c r="F21" s="70" t="n"/>
-      <c r="G21" s="70" t="n"/>
-      <c r="H21" s="70" t="n"/>
-      <c r="I21" s="71" t="n"/>
-      <c r="J21" s="71" t="n"/>
+      <c r="A21" s="69" t="n"/>
+      <c r="B21" s="69" t="n"/>
+      <c r="C21" s="69" t="n"/>
+      <c r="D21" s="69" t="n"/>
+      <c r="E21" s="69" t="n"/>
+      <c r="F21" s="69" t="n"/>
+      <c r="G21" s="69" t="n"/>
+      <c r="H21" s="69" t="n"/>
+      <c r="I21" s="70" t="n"/>
+      <c r="J21" s="70" t="n"/>
       <c r="K21" s="65">
         <f>IFERROR(DATEDIF(I21,J21,"M"),"")</f>
         <v/>
       </c>
-      <c r="L21" s="72" t="n"/>
-      <c r="M21" s="70" t="n"/>
-      <c r="N21" s="70" t="n"/>
-      <c r="O21" s="72" t="n"/>
-      <c r="P21" s="70" t="n"/>
+      <c r="L21" s="71" t="n"/>
+      <c r="M21" s="69" t="n"/>
+      <c r="N21" s="69" t="n"/>
+      <c r="O21" s="71" t="n"/>
+      <c r="P21" s="69" t="n"/>
       <c r="Q21" s="67">
         <f>IFERROR(IF(J21="","",J21-TODAY()),"")</f>
         <v/>
@@ -2996,25 +2993,25 @@
       <c r="V21" s="69" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="73" t="n"/>
-      <c r="B22" s="73" t="n"/>
-      <c r="C22" s="73" t="n"/>
-      <c r="D22" s="73" t="n"/>
-      <c r="E22" s="73" t="n"/>
-      <c r="F22" s="73" t="n"/>
-      <c r="G22" s="73" t="n"/>
-      <c r="H22" s="73" t="n"/>
-      <c r="I22" s="74" t="n"/>
-      <c r="J22" s="74" t="n"/>
+      <c r="A22" s="72" t="n"/>
+      <c r="B22" s="72" t="n"/>
+      <c r="C22" s="72" t="n"/>
+      <c r="D22" s="72" t="n"/>
+      <c r="E22" s="72" t="n"/>
+      <c r="F22" s="72" t="n"/>
+      <c r="G22" s="72" t="n"/>
+      <c r="H22" s="72" t="n"/>
+      <c r="I22" s="73" t="n"/>
+      <c r="J22" s="73" t="n"/>
       <c r="K22" s="65">
         <f>IFERROR(DATEDIF(I22,J22,"M"),"")</f>
         <v/>
       </c>
-      <c r="L22" s="75" t="n"/>
-      <c r="M22" s="73" t="n"/>
-      <c r="N22" s="73" t="n"/>
-      <c r="O22" s="75" t="n"/>
-      <c r="P22" s="73" t="n"/>
+      <c r="L22" s="74" t="n"/>
+      <c r="M22" s="72" t="n"/>
+      <c r="N22" s="72" t="n"/>
+      <c r="O22" s="74" t="n"/>
+      <c r="P22" s="72" t="n"/>
       <c r="Q22" s="67">
         <f>IFERROR(IF(J22="","",J22-TODAY()),"")</f>
         <v/>
@@ -3023,31 +3020,31 @@
         <f>IFERROR(IF(B22="","Vacant",IF(Q22&lt;0,"Expired",IF(Q22&lt;=30,"Expiring Soon",IF(Q22&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S22" s="69" t="n"/>
-      <c r="T22" s="69" t="n"/>
-      <c r="U22" s="69" t="n"/>
-      <c r="V22" s="69" t="n"/>
+      <c r="S22" s="72" t="n"/>
+      <c r="T22" s="72" t="n"/>
+      <c r="U22" s="72" t="n"/>
+      <c r="V22" s="72" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="70" t="n"/>
-      <c r="B23" s="70" t="n"/>
-      <c r="C23" s="70" t="n"/>
-      <c r="D23" s="70" t="n"/>
-      <c r="E23" s="70" t="n"/>
-      <c r="F23" s="70" t="n"/>
-      <c r="G23" s="70" t="n"/>
-      <c r="H23" s="70" t="n"/>
-      <c r="I23" s="71" t="n"/>
-      <c r="J23" s="71" t="n"/>
+      <c r="A23" s="69" t="n"/>
+      <c r="B23" s="69" t="n"/>
+      <c r="C23" s="69" t="n"/>
+      <c r="D23" s="69" t="n"/>
+      <c r="E23" s="69" t="n"/>
+      <c r="F23" s="69" t="n"/>
+      <c r="G23" s="69" t="n"/>
+      <c r="H23" s="69" t="n"/>
+      <c r="I23" s="70" t="n"/>
+      <c r="J23" s="70" t="n"/>
       <c r="K23" s="65">
         <f>IFERROR(DATEDIF(I23,J23,"M"),"")</f>
         <v/>
       </c>
-      <c r="L23" s="72" t="n"/>
-      <c r="M23" s="70" t="n"/>
-      <c r="N23" s="70" t="n"/>
-      <c r="O23" s="72" t="n"/>
-      <c r="P23" s="70" t="n"/>
+      <c r="L23" s="71" t="n"/>
+      <c r="M23" s="69" t="n"/>
+      <c r="N23" s="69" t="n"/>
+      <c r="O23" s="71" t="n"/>
+      <c r="P23" s="69" t="n"/>
       <c r="Q23" s="67">
         <f>IFERROR(IF(J23="","",J23-TODAY()),"")</f>
         <v/>
@@ -3062,25 +3059,25 @@
       <c r="V23" s="69" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="73" t="n"/>
-      <c r="B24" s="73" t="n"/>
-      <c r="C24" s="73" t="n"/>
-      <c r="D24" s="73" t="n"/>
-      <c r="E24" s="73" t="n"/>
-      <c r="F24" s="73" t="n"/>
-      <c r="G24" s="73" t="n"/>
-      <c r="H24" s="73" t="n"/>
-      <c r="I24" s="74" t="n"/>
-      <c r="J24" s="74" t="n"/>
+      <c r="A24" s="72" t="n"/>
+      <c r="B24" s="72" t="n"/>
+      <c r="C24" s="72" t="n"/>
+      <c r="D24" s="72" t="n"/>
+      <c r="E24" s="72" t="n"/>
+      <c r="F24" s="72" t="n"/>
+      <c r="G24" s="72" t="n"/>
+      <c r="H24" s="72" t="n"/>
+      <c r="I24" s="73" t="n"/>
+      <c r="J24" s="73" t="n"/>
       <c r="K24" s="65">
         <f>IFERROR(DATEDIF(I24,J24,"M"),"")</f>
         <v/>
       </c>
-      <c r="L24" s="75" t="n"/>
-      <c r="M24" s="73" t="n"/>
-      <c r="N24" s="73" t="n"/>
-      <c r="O24" s="75" t="n"/>
-      <c r="P24" s="73" t="n"/>
+      <c r="L24" s="74" t="n"/>
+      <c r="M24" s="72" t="n"/>
+      <c r="N24" s="72" t="n"/>
+      <c r="O24" s="74" t="n"/>
+      <c r="P24" s="72" t="n"/>
       <c r="Q24" s="67">
         <f>IFERROR(IF(J24="","",J24-TODAY()),"")</f>
         <v/>
@@ -3089,31 +3086,31 @@
         <f>IFERROR(IF(B24="","Vacant",IF(Q24&lt;0,"Expired",IF(Q24&lt;=30,"Expiring Soon",IF(Q24&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S24" s="69" t="n"/>
-      <c r="T24" s="69" t="n"/>
-      <c r="U24" s="69" t="n"/>
-      <c r="V24" s="69" t="n"/>
+      <c r="S24" s="72" t="n"/>
+      <c r="T24" s="72" t="n"/>
+      <c r="U24" s="72" t="n"/>
+      <c r="V24" s="72" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="70" t="n"/>
-      <c r="B25" s="70" t="n"/>
-      <c r="C25" s="70" t="n"/>
-      <c r="D25" s="70" t="n"/>
-      <c r="E25" s="70" t="n"/>
-      <c r="F25" s="70" t="n"/>
-      <c r="G25" s="70" t="n"/>
-      <c r="H25" s="70" t="n"/>
-      <c r="I25" s="71" t="n"/>
-      <c r="J25" s="71" t="n"/>
+      <c r="A25" s="69" t="n"/>
+      <c r="B25" s="69" t="n"/>
+      <c r="C25" s="69" t="n"/>
+      <c r="D25" s="69" t="n"/>
+      <c r="E25" s="69" t="n"/>
+      <c r="F25" s="69" t="n"/>
+      <c r="G25" s="69" t="n"/>
+      <c r="H25" s="69" t="n"/>
+      <c r="I25" s="70" t="n"/>
+      <c r="J25" s="70" t="n"/>
       <c r="K25" s="65">
         <f>IFERROR(DATEDIF(I25,J25,"M"),"")</f>
         <v/>
       </c>
-      <c r="L25" s="72" t="n"/>
-      <c r="M25" s="70" t="n"/>
-      <c r="N25" s="70" t="n"/>
-      <c r="O25" s="72" t="n"/>
-      <c r="P25" s="70" t="n"/>
+      <c r="L25" s="71" t="n"/>
+      <c r="M25" s="69" t="n"/>
+      <c r="N25" s="69" t="n"/>
+      <c r="O25" s="71" t="n"/>
+      <c r="P25" s="69" t="n"/>
       <c r="Q25" s="67">
         <f>IFERROR(IF(J25="","",J25-TODAY()),"")</f>
         <v/>
@@ -3128,25 +3125,25 @@
       <c r="V25" s="69" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="73" t="n"/>
-      <c r="B26" s="73" t="n"/>
-      <c r="C26" s="73" t="n"/>
-      <c r="D26" s="73" t="n"/>
-      <c r="E26" s="73" t="n"/>
-      <c r="F26" s="73" t="n"/>
-      <c r="G26" s="73" t="n"/>
-      <c r="H26" s="73" t="n"/>
-      <c r="I26" s="74" t="n"/>
-      <c r="J26" s="74" t="n"/>
+      <c r="A26" s="72" t="n"/>
+      <c r="B26" s="72" t="n"/>
+      <c r="C26" s="72" t="n"/>
+      <c r="D26" s="72" t="n"/>
+      <c r="E26" s="72" t="n"/>
+      <c r="F26" s="72" t="n"/>
+      <c r="G26" s="72" t="n"/>
+      <c r="H26" s="72" t="n"/>
+      <c r="I26" s="73" t="n"/>
+      <c r="J26" s="73" t="n"/>
       <c r="K26" s="65">
         <f>IFERROR(DATEDIF(I26,J26,"M"),"")</f>
         <v/>
       </c>
-      <c r="L26" s="75" t="n"/>
-      <c r="M26" s="73" t="n"/>
-      <c r="N26" s="73" t="n"/>
-      <c r="O26" s="75" t="n"/>
-      <c r="P26" s="73" t="n"/>
+      <c r="L26" s="74" t="n"/>
+      <c r="M26" s="72" t="n"/>
+      <c r="N26" s="72" t="n"/>
+      <c r="O26" s="74" t="n"/>
+      <c r="P26" s="72" t="n"/>
       <c r="Q26" s="67">
         <f>IFERROR(IF(J26="","",J26-TODAY()),"")</f>
         <v/>
@@ -3155,31 +3152,31 @@
         <f>IFERROR(IF(B26="","Vacant",IF(Q26&lt;0,"Expired",IF(Q26&lt;=30,"Expiring Soon",IF(Q26&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S26" s="69" t="n"/>
-      <c r="T26" s="69" t="n"/>
-      <c r="U26" s="69" t="n"/>
-      <c r="V26" s="69" t="n"/>
+      <c r="S26" s="72" t="n"/>
+      <c r="T26" s="72" t="n"/>
+      <c r="U26" s="72" t="n"/>
+      <c r="V26" s="72" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="70" t="n"/>
-      <c r="B27" s="70" t="n"/>
-      <c r="C27" s="70" t="n"/>
-      <c r="D27" s="70" t="n"/>
-      <c r="E27" s="70" t="n"/>
-      <c r="F27" s="70" t="n"/>
-      <c r="G27" s="70" t="n"/>
-      <c r="H27" s="70" t="n"/>
-      <c r="I27" s="71" t="n"/>
-      <c r="J27" s="71" t="n"/>
+      <c r="A27" s="69" t="n"/>
+      <c r="B27" s="69" t="n"/>
+      <c r="C27" s="69" t="n"/>
+      <c r="D27" s="69" t="n"/>
+      <c r="E27" s="69" t="n"/>
+      <c r="F27" s="69" t="n"/>
+      <c r="G27" s="69" t="n"/>
+      <c r="H27" s="69" t="n"/>
+      <c r="I27" s="70" t="n"/>
+      <c r="J27" s="70" t="n"/>
       <c r="K27" s="65">
         <f>IFERROR(DATEDIF(I27,J27,"M"),"")</f>
         <v/>
       </c>
-      <c r="L27" s="72" t="n"/>
-      <c r="M27" s="70" t="n"/>
-      <c r="N27" s="70" t="n"/>
-      <c r="O27" s="72" t="n"/>
-      <c r="P27" s="70" t="n"/>
+      <c r="L27" s="71" t="n"/>
+      <c r="M27" s="69" t="n"/>
+      <c r="N27" s="69" t="n"/>
+      <c r="O27" s="71" t="n"/>
+      <c r="P27" s="69" t="n"/>
       <c r="Q27" s="67">
         <f>IFERROR(IF(J27="","",J27-TODAY()),"")</f>
         <v/>
@@ -3194,25 +3191,25 @@
       <c r="V27" s="69" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="73" t="n"/>
-      <c r="B28" s="73" t="n"/>
-      <c r="C28" s="73" t="n"/>
-      <c r="D28" s="73" t="n"/>
-      <c r="E28" s="73" t="n"/>
-      <c r="F28" s="73" t="n"/>
-      <c r="G28" s="73" t="n"/>
-      <c r="H28" s="73" t="n"/>
-      <c r="I28" s="74" t="n"/>
-      <c r="J28" s="74" t="n"/>
+      <c r="A28" s="72" t="n"/>
+      <c r="B28" s="72" t="n"/>
+      <c r="C28" s="72" t="n"/>
+      <c r="D28" s="72" t="n"/>
+      <c r="E28" s="72" t="n"/>
+      <c r="F28" s="72" t="n"/>
+      <c r="G28" s="72" t="n"/>
+      <c r="H28" s="72" t="n"/>
+      <c r="I28" s="73" t="n"/>
+      <c r="J28" s="73" t="n"/>
       <c r="K28" s="65">
         <f>IFERROR(DATEDIF(I28,J28,"M"),"")</f>
         <v/>
       </c>
-      <c r="L28" s="75" t="n"/>
-      <c r="M28" s="73" t="n"/>
-      <c r="N28" s="73" t="n"/>
-      <c r="O28" s="75" t="n"/>
-      <c r="P28" s="73" t="n"/>
+      <c r="L28" s="74" t="n"/>
+      <c r="M28" s="72" t="n"/>
+      <c r="N28" s="72" t="n"/>
+      <c r="O28" s="74" t="n"/>
+      <c r="P28" s="72" t="n"/>
       <c r="Q28" s="67">
         <f>IFERROR(IF(J28="","",J28-TODAY()),"")</f>
         <v/>
@@ -3221,31 +3218,31 @@
         <f>IFERROR(IF(B28="","Vacant",IF(Q28&lt;0,"Expired",IF(Q28&lt;=30,"Expiring Soon",IF(Q28&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S28" s="69" t="n"/>
-      <c r="T28" s="69" t="n"/>
-      <c r="U28" s="69" t="n"/>
-      <c r="V28" s="69" t="n"/>
+      <c r="S28" s="72" t="n"/>
+      <c r="T28" s="72" t="n"/>
+      <c r="U28" s="72" t="n"/>
+      <c r="V28" s="72" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="70" t="n"/>
-      <c r="B29" s="70" t="n"/>
-      <c r="C29" s="70" t="n"/>
-      <c r="D29" s="70" t="n"/>
-      <c r="E29" s="70" t="n"/>
-      <c r="F29" s="70" t="n"/>
-      <c r="G29" s="70" t="n"/>
-      <c r="H29" s="70" t="n"/>
-      <c r="I29" s="71" t="n"/>
-      <c r="J29" s="71" t="n"/>
+      <c r="A29" s="69" t="n"/>
+      <c r="B29" s="69" t="n"/>
+      <c r="C29" s="69" t="n"/>
+      <c r="D29" s="69" t="n"/>
+      <c r="E29" s="69" t="n"/>
+      <c r="F29" s="69" t="n"/>
+      <c r="G29" s="69" t="n"/>
+      <c r="H29" s="69" t="n"/>
+      <c r="I29" s="70" t="n"/>
+      <c r="J29" s="70" t="n"/>
       <c r="K29" s="65">
         <f>IFERROR(DATEDIF(I29,J29,"M"),"")</f>
         <v/>
       </c>
-      <c r="L29" s="72" t="n"/>
-      <c r="M29" s="70" t="n"/>
-      <c r="N29" s="70" t="n"/>
-      <c r="O29" s="72" t="n"/>
-      <c r="P29" s="70" t="n"/>
+      <c r="L29" s="71" t="n"/>
+      <c r="M29" s="69" t="n"/>
+      <c r="N29" s="69" t="n"/>
+      <c r="O29" s="71" t="n"/>
+      <c r="P29" s="69" t="n"/>
       <c r="Q29" s="67">
         <f>IFERROR(IF(J29="","",J29-TODAY()),"")</f>
         <v/>
@@ -3260,25 +3257,25 @@
       <c r="V29" s="69" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="73" t="n"/>
-      <c r="B30" s="73" t="n"/>
-      <c r="C30" s="73" t="n"/>
-      <c r="D30" s="73" t="n"/>
-      <c r="E30" s="73" t="n"/>
-      <c r="F30" s="73" t="n"/>
-      <c r="G30" s="73" t="n"/>
-      <c r="H30" s="73" t="n"/>
-      <c r="I30" s="74" t="n"/>
-      <c r="J30" s="74" t="n"/>
+      <c r="A30" s="72" t="n"/>
+      <c r="B30" s="72" t="n"/>
+      <c r="C30" s="72" t="n"/>
+      <c r="D30" s="72" t="n"/>
+      <c r="E30" s="72" t="n"/>
+      <c r="F30" s="72" t="n"/>
+      <c r="G30" s="72" t="n"/>
+      <c r="H30" s="72" t="n"/>
+      <c r="I30" s="73" t="n"/>
+      <c r="J30" s="73" t="n"/>
       <c r="K30" s="65">
         <f>IFERROR(DATEDIF(I30,J30,"M"),"")</f>
         <v/>
       </c>
-      <c r="L30" s="75" t="n"/>
-      <c r="M30" s="73" t="n"/>
-      <c r="N30" s="73" t="n"/>
-      <c r="O30" s="75" t="n"/>
-      <c r="P30" s="73" t="n"/>
+      <c r="L30" s="74" t="n"/>
+      <c r="M30" s="72" t="n"/>
+      <c r="N30" s="72" t="n"/>
+      <c r="O30" s="74" t="n"/>
+      <c r="P30" s="72" t="n"/>
       <c r="Q30" s="67">
         <f>IFERROR(IF(J30="","",J30-TODAY()),"")</f>
         <v/>
@@ -3287,31 +3284,31 @@
         <f>IFERROR(IF(B30="","Vacant",IF(Q30&lt;0,"Expired",IF(Q30&lt;=30,"Expiring Soon",IF(Q30&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S30" s="69" t="n"/>
-      <c r="T30" s="69" t="n"/>
-      <c r="U30" s="69" t="n"/>
-      <c r="V30" s="69" t="n"/>
+      <c r="S30" s="72" t="n"/>
+      <c r="T30" s="72" t="n"/>
+      <c r="U30" s="72" t="n"/>
+      <c r="V30" s="72" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="70" t="n"/>
-      <c r="B31" s="70" t="n"/>
-      <c r="C31" s="70" t="n"/>
-      <c r="D31" s="70" t="n"/>
-      <c r="E31" s="70" t="n"/>
-      <c r="F31" s="70" t="n"/>
-      <c r="G31" s="70" t="n"/>
-      <c r="H31" s="70" t="n"/>
-      <c r="I31" s="71" t="n"/>
-      <c r="J31" s="71" t="n"/>
+      <c r="A31" s="69" t="n"/>
+      <c r="B31" s="69" t="n"/>
+      <c r="C31" s="69" t="n"/>
+      <c r="D31" s="69" t="n"/>
+      <c r="E31" s="69" t="n"/>
+      <c r="F31" s="69" t="n"/>
+      <c r="G31" s="69" t="n"/>
+      <c r="H31" s="69" t="n"/>
+      <c r="I31" s="70" t="n"/>
+      <c r="J31" s="70" t="n"/>
       <c r="K31" s="65">
         <f>IFERROR(DATEDIF(I31,J31,"M"),"")</f>
         <v/>
       </c>
-      <c r="L31" s="72" t="n"/>
-      <c r="M31" s="70" t="n"/>
-      <c r="N31" s="70" t="n"/>
-      <c r="O31" s="72" t="n"/>
-      <c r="P31" s="70" t="n"/>
+      <c r="L31" s="71" t="n"/>
+      <c r="M31" s="69" t="n"/>
+      <c r="N31" s="69" t="n"/>
+      <c r="O31" s="71" t="n"/>
+      <c r="P31" s="69" t="n"/>
       <c r="Q31" s="67">
         <f>IFERROR(IF(J31="","",J31-TODAY()),"")</f>
         <v/>
@@ -3326,25 +3323,25 @@
       <c r="V31" s="69" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="73" t="n"/>
-      <c r="B32" s="73" t="n"/>
-      <c r="C32" s="73" t="n"/>
-      <c r="D32" s="73" t="n"/>
-      <c r="E32" s="73" t="n"/>
-      <c r="F32" s="73" t="n"/>
-      <c r="G32" s="73" t="n"/>
-      <c r="H32" s="73" t="n"/>
-      <c r="I32" s="74" t="n"/>
-      <c r="J32" s="74" t="n"/>
+      <c r="A32" s="72" t="n"/>
+      <c r="B32" s="72" t="n"/>
+      <c r="C32" s="72" t="n"/>
+      <c r="D32" s="72" t="n"/>
+      <c r="E32" s="72" t="n"/>
+      <c r="F32" s="72" t="n"/>
+      <c r="G32" s="72" t="n"/>
+      <c r="H32" s="72" t="n"/>
+      <c r="I32" s="73" t="n"/>
+      <c r="J32" s="73" t="n"/>
       <c r="K32" s="65">
         <f>IFERROR(DATEDIF(I32,J32,"M"),"")</f>
         <v/>
       </c>
-      <c r="L32" s="75" t="n"/>
-      <c r="M32" s="73" t="n"/>
-      <c r="N32" s="73" t="n"/>
-      <c r="O32" s="75" t="n"/>
-      <c r="P32" s="73" t="n"/>
+      <c r="L32" s="74" t="n"/>
+      <c r="M32" s="72" t="n"/>
+      <c r="N32" s="72" t="n"/>
+      <c r="O32" s="74" t="n"/>
+      <c r="P32" s="72" t="n"/>
       <c r="Q32" s="67">
         <f>IFERROR(IF(J32="","",J32-TODAY()),"")</f>
         <v/>
@@ -3353,31 +3350,31 @@
         <f>IFERROR(IF(B32="","Vacant",IF(Q32&lt;0,"Expired",IF(Q32&lt;=30,"Expiring Soon",IF(Q32&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S32" s="69" t="n"/>
-      <c r="T32" s="69" t="n"/>
-      <c r="U32" s="69" t="n"/>
-      <c r="V32" s="69" t="n"/>
+      <c r="S32" s="72" t="n"/>
+      <c r="T32" s="72" t="n"/>
+      <c r="U32" s="72" t="n"/>
+      <c r="V32" s="72" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="70" t="n"/>
-      <c r="B33" s="70" t="n"/>
-      <c r="C33" s="70" t="n"/>
-      <c r="D33" s="70" t="n"/>
-      <c r="E33" s="70" t="n"/>
-      <c r="F33" s="70" t="n"/>
-      <c r="G33" s="70" t="n"/>
-      <c r="H33" s="70" t="n"/>
-      <c r="I33" s="71" t="n"/>
-      <c r="J33" s="71" t="n"/>
+      <c r="A33" s="69" t="n"/>
+      <c r="B33" s="69" t="n"/>
+      <c r="C33" s="69" t="n"/>
+      <c r="D33" s="69" t="n"/>
+      <c r="E33" s="69" t="n"/>
+      <c r="F33" s="69" t="n"/>
+      <c r="G33" s="69" t="n"/>
+      <c r="H33" s="69" t="n"/>
+      <c r="I33" s="70" t="n"/>
+      <c r="J33" s="70" t="n"/>
       <c r="K33" s="65">
         <f>IFERROR(DATEDIF(I33,J33,"M"),"")</f>
         <v/>
       </c>
-      <c r="L33" s="72" t="n"/>
-      <c r="M33" s="70" t="n"/>
-      <c r="N33" s="70" t="n"/>
-      <c r="O33" s="72" t="n"/>
-      <c r="P33" s="70" t="n"/>
+      <c r="L33" s="71" t="n"/>
+      <c r="M33" s="69" t="n"/>
+      <c r="N33" s="69" t="n"/>
+      <c r="O33" s="71" t="n"/>
+      <c r="P33" s="69" t="n"/>
       <c r="Q33" s="67">
         <f>IFERROR(IF(J33="","",J33-TODAY()),"")</f>
         <v/>
@@ -3392,25 +3389,25 @@
       <c r="V33" s="69" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="73" t="n"/>
-      <c r="B34" s="73" t="n"/>
-      <c r="C34" s="73" t="n"/>
-      <c r="D34" s="73" t="n"/>
-      <c r="E34" s="73" t="n"/>
-      <c r="F34" s="73" t="n"/>
-      <c r="G34" s="73" t="n"/>
-      <c r="H34" s="73" t="n"/>
-      <c r="I34" s="74" t="n"/>
-      <c r="J34" s="74" t="n"/>
+      <c r="A34" s="72" t="n"/>
+      <c r="B34" s="72" t="n"/>
+      <c r="C34" s="72" t="n"/>
+      <c r="D34" s="72" t="n"/>
+      <c r="E34" s="72" t="n"/>
+      <c r="F34" s="72" t="n"/>
+      <c r="G34" s="72" t="n"/>
+      <c r="H34" s="72" t="n"/>
+      <c r="I34" s="73" t="n"/>
+      <c r="J34" s="73" t="n"/>
       <c r="K34" s="65">
         <f>IFERROR(DATEDIF(I34,J34,"M"),"")</f>
         <v/>
       </c>
-      <c r="L34" s="75" t="n"/>
-      <c r="M34" s="73" t="n"/>
-      <c r="N34" s="73" t="n"/>
-      <c r="O34" s="75" t="n"/>
-      <c r="P34" s="73" t="n"/>
+      <c r="L34" s="74" t="n"/>
+      <c r="M34" s="72" t="n"/>
+      <c r="N34" s="72" t="n"/>
+      <c r="O34" s="74" t="n"/>
+      <c r="P34" s="72" t="n"/>
       <c r="Q34" s="67">
         <f>IFERROR(IF(J34="","",J34-TODAY()),"")</f>
         <v/>
@@ -3419,31 +3416,31 @@
         <f>IFERROR(IF(B34="","Vacant",IF(Q34&lt;0,"Expired",IF(Q34&lt;=30,"Expiring Soon",IF(Q34&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S34" s="69" t="n"/>
-      <c r="T34" s="69" t="n"/>
-      <c r="U34" s="69" t="n"/>
-      <c r="V34" s="69" t="n"/>
+      <c r="S34" s="72" t="n"/>
+      <c r="T34" s="72" t="n"/>
+      <c r="U34" s="72" t="n"/>
+      <c r="V34" s="72" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="70" t="n"/>
-      <c r="B35" s="70" t="n"/>
-      <c r="C35" s="70" t="n"/>
-      <c r="D35" s="70" t="n"/>
-      <c r="E35" s="70" t="n"/>
-      <c r="F35" s="70" t="n"/>
-      <c r="G35" s="70" t="n"/>
-      <c r="H35" s="70" t="n"/>
-      <c r="I35" s="71" t="n"/>
-      <c r="J35" s="71" t="n"/>
+      <c r="A35" s="69" t="n"/>
+      <c r="B35" s="69" t="n"/>
+      <c r="C35" s="69" t="n"/>
+      <c r="D35" s="69" t="n"/>
+      <c r="E35" s="69" t="n"/>
+      <c r="F35" s="69" t="n"/>
+      <c r="G35" s="69" t="n"/>
+      <c r="H35" s="69" t="n"/>
+      <c r="I35" s="70" t="n"/>
+      <c r="J35" s="70" t="n"/>
       <c r="K35" s="65">
         <f>IFERROR(DATEDIF(I35,J35,"M"),"")</f>
         <v/>
       </c>
-      <c r="L35" s="72" t="n"/>
-      <c r="M35" s="70" t="n"/>
-      <c r="N35" s="70" t="n"/>
-      <c r="O35" s="72" t="n"/>
-      <c r="P35" s="70" t="n"/>
+      <c r="L35" s="71" t="n"/>
+      <c r="M35" s="69" t="n"/>
+      <c r="N35" s="69" t="n"/>
+      <c r="O35" s="71" t="n"/>
+      <c r="P35" s="69" t="n"/>
       <c r="Q35" s="67">
         <f>IFERROR(IF(J35="","",J35-TODAY()),"")</f>
         <v/>
@@ -3458,25 +3455,25 @@
       <c r="V35" s="69" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="73" t="n"/>
-      <c r="B36" s="73" t="n"/>
-      <c r="C36" s="73" t="n"/>
-      <c r="D36" s="73" t="n"/>
-      <c r="E36" s="73" t="n"/>
-      <c r="F36" s="73" t="n"/>
-      <c r="G36" s="73" t="n"/>
-      <c r="H36" s="73" t="n"/>
-      <c r="I36" s="74" t="n"/>
-      <c r="J36" s="74" t="n"/>
+      <c r="A36" s="72" t="n"/>
+      <c r="B36" s="72" t="n"/>
+      <c r="C36" s="72" t="n"/>
+      <c r="D36" s="72" t="n"/>
+      <c r="E36" s="72" t="n"/>
+      <c r="F36" s="72" t="n"/>
+      <c r="G36" s="72" t="n"/>
+      <c r="H36" s="72" t="n"/>
+      <c r="I36" s="73" t="n"/>
+      <c r="J36" s="73" t="n"/>
       <c r="K36" s="65">
         <f>IFERROR(DATEDIF(I36,J36,"M"),"")</f>
         <v/>
       </c>
-      <c r="L36" s="75" t="n"/>
-      <c r="M36" s="73" t="n"/>
-      <c r="N36" s="73" t="n"/>
-      <c r="O36" s="75" t="n"/>
-      <c r="P36" s="73" t="n"/>
+      <c r="L36" s="74" t="n"/>
+      <c r="M36" s="72" t="n"/>
+      <c r="N36" s="72" t="n"/>
+      <c r="O36" s="74" t="n"/>
+      <c r="P36" s="72" t="n"/>
       <c r="Q36" s="67">
         <f>IFERROR(IF(J36="","",J36-TODAY()),"")</f>
         <v/>
@@ -3485,31 +3482,31 @@
         <f>IFERROR(IF(B36="","Vacant",IF(Q36&lt;0,"Expired",IF(Q36&lt;=30,"Expiring Soon",IF(Q36&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S36" s="69" t="n"/>
-      <c r="T36" s="69" t="n"/>
-      <c r="U36" s="69" t="n"/>
-      <c r="V36" s="69" t="n"/>
+      <c r="S36" s="72" t="n"/>
+      <c r="T36" s="72" t="n"/>
+      <c r="U36" s="72" t="n"/>
+      <c r="V36" s="72" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="70" t="n"/>
-      <c r="B37" s="70" t="n"/>
-      <c r="C37" s="70" t="n"/>
-      <c r="D37" s="70" t="n"/>
-      <c r="E37" s="70" t="n"/>
-      <c r="F37" s="70" t="n"/>
-      <c r="G37" s="70" t="n"/>
-      <c r="H37" s="70" t="n"/>
-      <c r="I37" s="71" t="n"/>
-      <c r="J37" s="71" t="n"/>
+      <c r="A37" s="69" t="n"/>
+      <c r="B37" s="69" t="n"/>
+      <c r="C37" s="69" t="n"/>
+      <c r="D37" s="69" t="n"/>
+      <c r="E37" s="69" t="n"/>
+      <c r="F37" s="69" t="n"/>
+      <c r="G37" s="69" t="n"/>
+      <c r="H37" s="69" t="n"/>
+      <c r="I37" s="70" t="n"/>
+      <c r="J37" s="70" t="n"/>
       <c r="K37" s="65">
         <f>IFERROR(DATEDIF(I37,J37,"M"),"")</f>
         <v/>
       </c>
-      <c r="L37" s="72" t="n"/>
-      <c r="M37" s="70" t="n"/>
-      <c r="N37" s="70" t="n"/>
-      <c r="O37" s="72" t="n"/>
-      <c r="P37" s="70" t="n"/>
+      <c r="L37" s="71" t="n"/>
+      <c r="M37" s="69" t="n"/>
+      <c r="N37" s="69" t="n"/>
+      <c r="O37" s="71" t="n"/>
+      <c r="P37" s="69" t="n"/>
       <c r="Q37" s="67">
         <f>IFERROR(IF(J37="","",J37-TODAY()),"")</f>
         <v/>
@@ -3524,25 +3521,25 @@
       <c r="V37" s="69" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="73" t="n"/>
-      <c r="B38" s="73" t="n"/>
-      <c r="C38" s="73" t="n"/>
-      <c r="D38" s="73" t="n"/>
-      <c r="E38" s="73" t="n"/>
-      <c r="F38" s="73" t="n"/>
-      <c r="G38" s="73" t="n"/>
-      <c r="H38" s="73" t="n"/>
-      <c r="I38" s="74" t="n"/>
-      <c r="J38" s="74" t="n"/>
+      <c r="A38" s="72" t="n"/>
+      <c r="B38" s="72" t="n"/>
+      <c r="C38" s="72" t="n"/>
+      <c r="D38" s="72" t="n"/>
+      <c r="E38" s="72" t="n"/>
+      <c r="F38" s="72" t="n"/>
+      <c r="G38" s="72" t="n"/>
+      <c r="H38" s="72" t="n"/>
+      <c r="I38" s="73" t="n"/>
+      <c r="J38" s="73" t="n"/>
       <c r="K38" s="65">
         <f>IFERROR(DATEDIF(I38,J38,"M"),"")</f>
         <v/>
       </c>
-      <c r="L38" s="75" t="n"/>
-      <c r="M38" s="73" t="n"/>
-      <c r="N38" s="73" t="n"/>
-      <c r="O38" s="75" t="n"/>
-      <c r="P38" s="73" t="n"/>
+      <c r="L38" s="74" t="n"/>
+      <c r="M38" s="72" t="n"/>
+      <c r="N38" s="72" t="n"/>
+      <c r="O38" s="74" t="n"/>
+      <c r="P38" s="72" t="n"/>
       <c r="Q38" s="67">
         <f>IFERROR(IF(J38="","",J38-TODAY()),"")</f>
         <v/>
@@ -3551,31 +3548,31 @@
         <f>IFERROR(IF(B38="","Vacant",IF(Q38&lt;0,"Expired",IF(Q38&lt;=30,"Expiring Soon",IF(Q38&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S38" s="69" t="n"/>
-      <c r="T38" s="69" t="n"/>
-      <c r="U38" s="69" t="n"/>
-      <c r="V38" s="69" t="n"/>
+      <c r="S38" s="72" t="n"/>
+      <c r="T38" s="72" t="n"/>
+      <c r="U38" s="72" t="n"/>
+      <c r="V38" s="72" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="70" t="n"/>
-      <c r="B39" s="70" t="n"/>
-      <c r="C39" s="70" t="n"/>
-      <c r="D39" s="70" t="n"/>
-      <c r="E39" s="70" t="n"/>
-      <c r="F39" s="70" t="n"/>
-      <c r="G39" s="70" t="n"/>
-      <c r="H39" s="70" t="n"/>
-      <c r="I39" s="71" t="n"/>
-      <c r="J39" s="71" t="n"/>
+      <c r="A39" s="69" t="n"/>
+      <c r="B39" s="69" t="n"/>
+      <c r="C39" s="69" t="n"/>
+      <c r="D39" s="69" t="n"/>
+      <c r="E39" s="69" t="n"/>
+      <c r="F39" s="69" t="n"/>
+      <c r="G39" s="69" t="n"/>
+      <c r="H39" s="69" t="n"/>
+      <c r="I39" s="70" t="n"/>
+      <c r="J39" s="70" t="n"/>
       <c r="K39" s="65">
         <f>IFERROR(DATEDIF(I39,J39,"M"),"")</f>
         <v/>
       </c>
-      <c r="L39" s="72" t="n"/>
-      <c r="M39" s="70" t="n"/>
-      <c r="N39" s="70" t="n"/>
-      <c r="O39" s="72" t="n"/>
-      <c r="P39" s="70" t="n"/>
+      <c r="L39" s="71" t="n"/>
+      <c r="M39" s="69" t="n"/>
+      <c r="N39" s="69" t="n"/>
+      <c r="O39" s="71" t="n"/>
+      <c r="P39" s="69" t="n"/>
       <c r="Q39" s="67">
         <f>IFERROR(IF(J39="","",J39-TODAY()),"")</f>
         <v/>
@@ -3590,25 +3587,25 @@
       <c r="V39" s="69" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="73" t="n"/>
-      <c r="B40" s="73" t="n"/>
-      <c r="C40" s="73" t="n"/>
-      <c r="D40" s="73" t="n"/>
-      <c r="E40" s="73" t="n"/>
-      <c r="F40" s="73" t="n"/>
-      <c r="G40" s="73" t="n"/>
-      <c r="H40" s="73" t="n"/>
-      <c r="I40" s="74" t="n"/>
-      <c r="J40" s="74" t="n"/>
+      <c r="A40" s="72" t="n"/>
+      <c r="B40" s="72" t="n"/>
+      <c r="C40" s="72" t="n"/>
+      <c r="D40" s="72" t="n"/>
+      <c r="E40" s="72" t="n"/>
+      <c r="F40" s="72" t="n"/>
+      <c r="G40" s="72" t="n"/>
+      <c r="H40" s="72" t="n"/>
+      <c r="I40" s="73" t="n"/>
+      <c r="J40" s="73" t="n"/>
       <c r="K40" s="65">
         <f>IFERROR(DATEDIF(I40,J40,"M"),"")</f>
         <v/>
       </c>
-      <c r="L40" s="75" t="n"/>
-      <c r="M40" s="73" t="n"/>
-      <c r="N40" s="73" t="n"/>
-      <c r="O40" s="75" t="n"/>
-      <c r="P40" s="73" t="n"/>
+      <c r="L40" s="74" t="n"/>
+      <c r="M40" s="72" t="n"/>
+      <c r="N40" s="72" t="n"/>
+      <c r="O40" s="74" t="n"/>
+      <c r="P40" s="72" t="n"/>
       <c r="Q40" s="67">
         <f>IFERROR(IF(J40="","",J40-TODAY()),"")</f>
         <v/>
@@ -3617,31 +3614,31 @@
         <f>IFERROR(IF(B40="","Vacant",IF(Q40&lt;0,"Expired",IF(Q40&lt;=30,"Expiring Soon",IF(Q40&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S40" s="69" t="n"/>
-      <c r="T40" s="69" t="n"/>
-      <c r="U40" s="69" t="n"/>
-      <c r="V40" s="69" t="n"/>
+      <c r="S40" s="72" t="n"/>
+      <c r="T40" s="72" t="n"/>
+      <c r="U40" s="72" t="n"/>
+      <c r="V40" s="72" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="70" t="n"/>
-      <c r="B41" s="70" t="n"/>
-      <c r="C41" s="70" t="n"/>
-      <c r="D41" s="70" t="n"/>
-      <c r="E41" s="70" t="n"/>
-      <c r="F41" s="70" t="n"/>
-      <c r="G41" s="70" t="n"/>
-      <c r="H41" s="70" t="n"/>
-      <c r="I41" s="71" t="n"/>
-      <c r="J41" s="71" t="n"/>
+      <c r="A41" s="69" t="n"/>
+      <c r="B41" s="69" t="n"/>
+      <c r="C41" s="69" t="n"/>
+      <c r="D41" s="69" t="n"/>
+      <c r="E41" s="69" t="n"/>
+      <c r="F41" s="69" t="n"/>
+      <c r="G41" s="69" t="n"/>
+      <c r="H41" s="69" t="n"/>
+      <c r="I41" s="70" t="n"/>
+      <c r="J41" s="70" t="n"/>
       <c r="K41" s="65">
         <f>IFERROR(DATEDIF(I41,J41,"M"),"")</f>
         <v/>
       </c>
-      <c r="L41" s="72" t="n"/>
-      <c r="M41" s="70" t="n"/>
-      <c r="N41" s="70" t="n"/>
-      <c r="O41" s="72" t="n"/>
-      <c r="P41" s="70" t="n"/>
+      <c r="L41" s="71" t="n"/>
+      <c r="M41" s="69" t="n"/>
+      <c r="N41" s="69" t="n"/>
+      <c r="O41" s="71" t="n"/>
+      <c r="P41" s="69" t="n"/>
       <c r="Q41" s="67">
         <f>IFERROR(IF(J41="","",J41-TODAY()),"")</f>
         <v/>
@@ -3656,25 +3653,25 @@
       <c r="V41" s="69" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="73" t="n"/>
-      <c r="B42" s="73" t="n"/>
-      <c r="C42" s="73" t="n"/>
-      <c r="D42" s="73" t="n"/>
-      <c r="E42" s="73" t="n"/>
-      <c r="F42" s="73" t="n"/>
-      <c r="G42" s="73" t="n"/>
-      <c r="H42" s="73" t="n"/>
-      <c r="I42" s="74" t="n"/>
-      <c r="J42" s="74" t="n"/>
+      <c r="A42" s="72" t="n"/>
+      <c r="B42" s="72" t="n"/>
+      <c r="C42" s="72" t="n"/>
+      <c r="D42" s="72" t="n"/>
+      <c r="E42" s="72" t="n"/>
+      <c r="F42" s="72" t="n"/>
+      <c r="G42" s="72" t="n"/>
+      <c r="H42" s="72" t="n"/>
+      <c r="I42" s="73" t="n"/>
+      <c r="J42" s="73" t="n"/>
       <c r="K42" s="65">
         <f>IFERROR(DATEDIF(I42,J42,"M"),"")</f>
         <v/>
       </c>
-      <c r="L42" s="75" t="n"/>
-      <c r="M42" s="73" t="n"/>
-      <c r="N42" s="73" t="n"/>
-      <c r="O42" s="75" t="n"/>
-      <c r="P42" s="73" t="n"/>
+      <c r="L42" s="74" t="n"/>
+      <c r="M42" s="72" t="n"/>
+      <c r="N42" s="72" t="n"/>
+      <c r="O42" s="74" t="n"/>
+      <c r="P42" s="72" t="n"/>
       <c r="Q42" s="67">
         <f>IFERROR(IF(J42="","",J42-TODAY()),"")</f>
         <v/>
@@ -3683,31 +3680,31 @@
         <f>IFERROR(IF(B42="","Vacant",IF(Q42&lt;0,"Expired",IF(Q42&lt;=30,"Expiring Soon",IF(Q42&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S42" s="69" t="n"/>
-      <c r="T42" s="69" t="n"/>
-      <c r="U42" s="69" t="n"/>
-      <c r="V42" s="69" t="n"/>
+      <c r="S42" s="72" t="n"/>
+      <c r="T42" s="72" t="n"/>
+      <c r="U42" s="72" t="n"/>
+      <c r="V42" s="72" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="70" t="n"/>
-      <c r="B43" s="70" t="n"/>
-      <c r="C43" s="70" t="n"/>
-      <c r="D43" s="70" t="n"/>
-      <c r="E43" s="70" t="n"/>
-      <c r="F43" s="70" t="n"/>
-      <c r="G43" s="70" t="n"/>
-      <c r="H43" s="70" t="n"/>
-      <c r="I43" s="71" t="n"/>
-      <c r="J43" s="71" t="n"/>
+      <c r="A43" s="69" t="n"/>
+      <c r="B43" s="69" t="n"/>
+      <c r="C43" s="69" t="n"/>
+      <c r="D43" s="69" t="n"/>
+      <c r="E43" s="69" t="n"/>
+      <c r="F43" s="69" t="n"/>
+      <c r="G43" s="69" t="n"/>
+      <c r="H43" s="69" t="n"/>
+      <c r="I43" s="70" t="n"/>
+      <c r="J43" s="70" t="n"/>
       <c r="K43" s="65">
         <f>IFERROR(DATEDIF(I43,J43,"M"),"")</f>
         <v/>
       </c>
-      <c r="L43" s="72" t="n"/>
-      <c r="M43" s="70" t="n"/>
-      <c r="N43" s="70" t="n"/>
-      <c r="O43" s="72" t="n"/>
-      <c r="P43" s="70" t="n"/>
+      <c r="L43" s="71" t="n"/>
+      <c r="M43" s="69" t="n"/>
+      <c r="N43" s="69" t="n"/>
+      <c r="O43" s="71" t="n"/>
+      <c r="P43" s="69" t="n"/>
       <c r="Q43" s="67">
         <f>IFERROR(IF(J43="","",J43-TODAY()),"")</f>
         <v/>
@@ -3722,25 +3719,25 @@
       <c r="V43" s="69" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="73" t="n"/>
-      <c r="B44" s="73" t="n"/>
-      <c r="C44" s="73" t="n"/>
-      <c r="D44" s="73" t="n"/>
-      <c r="E44" s="73" t="n"/>
-      <c r="F44" s="73" t="n"/>
-      <c r="G44" s="73" t="n"/>
-      <c r="H44" s="73" t="n"/>
-      <c r="I44" s="74" t="n"/>
-      <c r="J44" s="74" t="n"/>
+      <c r="A44" s="72" t="n"/>
+      <c r="B44" s="72" t="n"/>
+      <c r="C44" s="72" t="n"/>
+      <c r="D44" s="72" t="n"/>
+      <c r="E44" s="72" t="n"/>
+      <c r="F44" s="72" t="n"/>
+      <c r="G44" s="72" t="n"/>
+      <c r="H44" s="72" t="n"/>
+      <c r="I44" s="73" t="n"/>
+      <c r="J44" s="73" t="n"/>
       <c r="K44" s="65">
         <f>IFERROR(DATEDIF(I44,J44,"M"),"")</f>
         <v/>
       </c>
-      <c r="L44" s="75" t="n"/>
-      <c r="M44" s="73" t="n"/>
-      <c r="N44" s="73" t="n"/>
-      <c r="O44" s="75" t="n"/>
-      <c r="P44" s="73" t="n"/>
+      <c r="L44" s="74" t="n"/>
+      <c r="M44" s="72" t="n"/>
+      <c r="N44" s="72" t="n"/>
+      <c r="O44" s="74" t="n"/>
+      <c r="P44" s="72" t="n"/>
       <c r="Q44" s="67">
         <f>IFERROR(IF(J44="","",J44-TODAY()),"")</f>
         <v/>
@@ -3749,31 +3746,31 @@
         <f>IFERROR(IF(B44="","Vacant",IF(Q44&lt;0,"Expired",IF(Q44&lt;=30,"Expiring Soon",IF(Q44&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S44" s="69" t="n"/>
-      <c r="T44" s="69" t="n"/>
-      <c r="U44" s="69" t="n"/>
-      <c r="V44" s="69" t="n"/>
+      <c r="S44" s="72" t="n"/>
+      <c r="T44" s="72" t="n"/>
+      <c r="U44" s="72" t="n"/>
+      <c r="V44" s="72" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="70" t="n"/>
-      <c r="B45" s="70" t="n"/>
-      <c r="C45" s="70" t="n"/>
-      <c r="D45" s="70" t="n"/>
-      <c r="E45" s="70" t="n"/>
-      <c r="F45" s="70" t="n"/>
-      <c r="G45" s="70" t="n"/>
-      <c r="H45" s="70" t="n"/>
-      <c r="I45" s="71" t="n"/>
-      <c r="J45" s="71" t="n"/>
+      <c r="A45" s="69" t="n"/>
+      <c r="B45" s="69" t="n"/>
+      <c r="C45" s="69" t="n"/>
+      <c r="D45" s="69" t="n"/>
+      <c r="E45" s="69" t="n"/>
+      <c r="F45" s="69" t="n"/>
+      <c r="G45" s="69" t="n"/>
+      <c r="H45" s="69" t="n"/>
+      <c r="I45" s="70" t="n"/>
+      <c r="J45" s="70" t="n"/>
       <c r="K45" s="65">
         <f>IFERROR(DATEDIF(I45,J45,"M"),"")</f>
         <v/>
       </c>
-      <c r="L45" s="72" t="n"/>
-      <c r="M45" s="70" t="n"/>
-      <c r="N45" s="70" t="n"/>
-      <c r="O45" s="72" t="n"/>
-      <c r="P45" s="70" t="n"/>
+      <c r="L45" s="71" t="n"/>
+      <c r="M45" s="69" t="n"/>
+      <c r="N45" s="69" t="n"/>
+      <c r="O45" s="71" t="n"/>
+      <c r="P45" s="69" t="n"/>
       <c r="Q45" s="67">
         <f>IFERROR(IF(J45="","",J45-TODAY()),"")</f>
         <v/>
@@ -3788,25 +3785,25 @@
       <c r="V45" s="69" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="73" t="n"/>
-      <c r="B46" s="73" t="n"/>
-      <c r="C46" s="73" t="n"/>
-      <c r="D46" s="73" t="n"/>
-      <c r="E46" s="73" t="n"/>
-      <c r="F46" s="73" t="n"/>
-      <c r="G46" s="73" t="n"/>
-      <c r="H46" s="73" t="n"/>
-      <c r="I46" s="74" t="n"/>
-      <c r="J46" s="74" t="n"/>
+      <c r="A46" s="72" t="n"/>
+      <c r="B46" s="72" t="n"/>
+      <c r="C46" s="72" t="n"/>
+      <c r="D46" s="72" t="n"/>
+      <c r="E46" s="72" t="n"/>
+      <c r="F46" s="72" t="n"/>
+      <c r="G46" s="72" t="n"/>
+      <c r="H46" s="72" t="n"/>
+      <c r="I46" s="73" t="n"/>
+      <c r="J46" s="73" t="n"/>
       <c r="K46" s="65">
         <f>IFERROR(DATEDIF(I46,J46,"M"),"")</f>
         <v/>
       </c>
-      <c r="L46" s="75" t="n"/>
-      <c r="M46" s="73" t="n"/>
-      <c r="N46" s="73" t="n"/>
-      <c r="O46" s="75" t="n"/>
-      <c r="P46" s="73" t="n"/>
+      <c r="L46" s="74" t="n"/>
+      <c r="M46" s="72" t="n"/>
+      <c r="N46" s="72" t="n"/>
+      <c r="O46" s="74" t="n"/>
+      <c r="P46" s="72" t="n"/>
       <c r="Q46" s="67">
         <f>IFERROR(IF(J46="","",J46-TODAY()),"")</f>
         <v/>
@@ -3815,31 +3812,31 @@
         <f>IFERROR(IF(B46="","Vacant",IF(Q46&lt;0,"Expired",IF(Q46&lt;=30,"Expiring Soon",IF(Q46&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S46" s="69" t="n"/>
-      <c r="T46" s="69" t="n"/>
-      <c r="U46" s="69" t="n"/>
-      <c r="V46" s="69" t="n"/>
+      <c r="S46" s="72" t="n"/>
+      <c r="T46" s="72" t="n"/>
+      <c r="U46" s="72" t="n"/>
+      <c r="V46" s="72" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="70" t="n"/>
-      <c r="B47" s="70" t="n"/>
-      <c r="C47" s="70" t="n"/>
-      <c r="D47" s="70" t="n"/>
-      <c r="E47" s="70" t="n"/>
-      <c r="F47" s="70" t="n"/>
-      <c r="G47" s="70" t="n"/>
-      <c r="H47" s="70" t="n"/>
-      <c r="I47" s="71" t="n"/>
-      <c r="J47" s="71" t="n"/>
+      <c r="A47" s="69" t="n"/>
+      <c r="B47" s="69" t="n"/>
+      <c r="C47" s="69" t="n"/>
+      <c r="D47" s="69" t="n"/>
+      <c r="E47" s="69" t="n"/>
+      <c r="F47" s="69" t="n"/>
+      <c r="G47" s="69" t="n"/>
+      <c r="H47" s="69" t="n"/>
+      <c r="I47" s="70" t="n"/>
+      <c r="J47" s="70" t="n"/>
       <c r="K47" s="65">
         <f>IFERROR(DATEDIF(I47,J47,"M"),"")</f>
         <v/>
       </c>
-      <c r="L47" s="72" t="n"/>
-      <c r="M47" s="70" t="n"/>
-      <c r="N47" s="70" t="n"/>
-      <c r="O47" s="72" t="n"/>
-      <c r="P47" s="70" t="n"/>
+      <c r="L47" s="71" t="n"/>
+      <c r="M47" s="69" t="n"/>
+      <c r="N47" s="69" t="n"/>
+      <c r="O47" s="71" t="n"/>
+      <c r="P47" s="69" t="n"/>
       <c r="Q47" s="67">
         <f>IFERROR(IF(J47="","",J47-TODAY()),"")</f>
         <v/>
@@ -3854,25 +3851,25 @@
       <c r="V47" s="69" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="73" t="n"/>
-      <c r="B48" s="73" t="n"/>
-      <c r="C48" s="73" t="n"/>
-      <c r="D48" s="73" t="n"/>
-      <c r="E48" s="73" t="n"/>
-      <c r="F48" s="73" t="n"/>
-      <c r="G48" s="73" t="n"/>
-      <c r="H48" s="73" t="n"/>
-      <c r="I48" s="74" t="n"/>
-      <c r="J48" s="74" t="n"/>
+      <c r="A48" s="72" t="n"/>
+      <c r="B48" s="72" t="n"/>
+      <c r="C48" s="72" t="n"/>
+      <c r="D48" s="72" t="n"/>
+      <c r="E48" s="72" t="n"/>
+      <c r="F48" s="72" t="n"/>
+      <c r="G48" s="72" t="n"/>
+      <c r="H48" s="72" t="n"/>
+      <c r="I48" s="73" t="n"/>
+      <c r="J48" s="73" t="n"/>
       <c r="K48" s="65">
         <f>IFERROR(DATEDIF(I48,J48,"M"),"")</f>
         <v/>
       </c>
-      <c r="L48" s="75" t="n"/>
-      <c r="M48" s="73" t="n"/>
-      <c r="N48" s="73" t="n"/>
-      <c r="O48" s="75" t="n"/>
-      <c r="P48" s="73" t="n"/>
+      <c r="L48" s="74" t="n"/>
+      <c r="M48" s="72" t="n"/>
+      <c r="N48" s="72" t="n"/>
+      <c r="O48" s="74" t="n"/>
+      <c r="P48" s="72" t="n"/>
       <c r="Q48" s="67">
         <f>IFERROR(IF(J48="","",J48-TODAY()),"")</f>
         <v/>
@@ -3881,31 +3878,31 @@
         <f>IFERROR(IF(B48="","Vacant",IF(Q48&lt;0,"Expired",IF(Q48&lt;=30,"Expiring Soon",IF(Q48&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S48" s="69" t="n"/>
-      <c r="T48" s="69" t="n"/>
-      <c r="U48" s="69" t="n"/>
-      <c r="V48" s="69" t="n"/>
+      <c r="S48" s="72" t="n"/>
+      <c r="T48" s="72" t="n"/>
+      <c r="U48" s="72" t="n"/>
+      <c r="V48" s="72" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="70" t="n"/>
-      <c r="B49" s="70" t="n"/>
-      <c r="C49" s="70" t="n"/>
-      <c r="D49" s="70" t="n"/>
-      <c r="E49" s="70" t="n"/>
-      <c r="F49" s="70" t="n"/>
-      <c r="G49" s="70" t="n"/>
-      <c r="H49" s="70" t="n"/>
-      <c r="I49" s="71" t="n"/>
-      <c r="J49" s="71" t="n"/>
+      <c r="A49" s="69" t="n"/>
+      <c r="B49" s="69" t="n"/>
+      <c r="C49" s="69" t="n"/>
+      <c r="D49" s="69" t="n"/>
+      <c r="E49" s="69" t="n"/>
+      <c r="F49" s="69" t="n"/>
+      <c r="G49" s="69" t="n"/>
+      <c r="H49" s="69" t="n"/>
+      <c r="I49" s="70" t="n"/>
+      <c r="J49" s="70" t="n"/>
       <c r="K49" s="65">
         <f>IFERROR(DATEDIF(I49,J49,"M"),"")</f>
         <v/>
       </c>
-      <c r="L49" s="72" t="n"/>
-      <c r="M49" s="70" t="n"/>
-      <c r="N49" s="70" t="n"/>
-      <c r="O49" s="72" t="n"/>
-      <c r="P49" s="70" t="n"/>
+      <c r="L49" s="71" t="n"/>
+      <c r="M49" s="69" t="n"/>
+      <c r="N49" s="69" t="n"/>
+      <c r="O49" s="71" t="n"/>
+      <c r="P49" s="69" t="n"/>
       <c r="Q49" s="67">
         <f>IFERROR(IF(J49="","",J49-TODAY()),"")</f>
         <v/>
@@ -3920,25 +3917,25 @@
       <c r="V49" s="69" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="73" t="n"/>
-      <c r="B50" s="73" t="n"/>
-      <c r="C50" s="73" t="n"/>
-      <c r="D50" s="73" t="n"/>
-      <c r="E50" s="73" t="n"/>
-      <c r="F50" s="73" t="n"/>
-      <c r="G50" s="73" t="n"/>
-      <c r="H50" s="73" t="n"/>
-      <c r="I50" s="74" t="n"/>
-      <c r="J50" s="74" t="n"/>
+      <c r="A50" s="72" t="n"/>
+      <c r="B50" s="72" t="n"/>
+      <c r="C50" s="72" t="n"/>
+      <c r="D50" s="72" t="n"/>
+      <c r="E50" s="72" t="n"/>
+      <c r="F50" s="72" t="n"/>
+      <c r="G50" s="72" t="n"/>
+      <c r="H50" s="72" t="n"/>
+      <c r="I50" s="73" t="n"/>
+      <c r="J50" s="73" t="n"/>
       <c r="K50" s="65">
         <f>IFERROR(DATEDIF(I50,J50,"M"),"")</f>
         <v/>
       </c>
-      <c r="L50" s="75" t="n"/>
-      <c r="M50" s="73" t="n"/>
-      <c r="N50" s="73" t="n"/>
-      <c r="O50" s="75" t="n"/>
-      <c r="P50" s="73" t="n"/>
+      <c r="L50" s="74" t="n"/>
+      <c r="M50" s="72" t="n"/>
+      <c r="N50" s="72" t="n"/>
+      <c r="O50" s="74" t="n"/>
+      <c r="P50" s="72" t="n"/>
       <c r="Q50" s="67">
         <f>IFERROR(IF(J50="","",J50-TODAY()),"")</f>
         <v/>
@@ -3947,31 +3944,31 @@
         <f>IFERROR(IF(B50="","Vacant",IF(Q50&lt;0,"Expired",IF(Q50&lt;=30,"Expiring Soon",IF(Q50&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S50" s="69" t="n"/>
-      <c r="T50" s="69" t="n"/>
-      <c r="U50" s="69" t="n"/>
-      <c r="V50" s="69" t="n"/>
+      <c r="S50" s="72" t="n"/>
+      <c r="T50" s="72" t="n"/>
+      <c r="U50" s="72" t="n"/>
+      <c r="V50" s="72" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="70" t="n"/>
-      <c r="B51" s="70" t="n"/>
-      <c r="C51" s="70" t="n"/>
-      <c r="D51" s="70" t="n"/>
-      <c r="E51" s="70" t="n"/>
-      <c r="F51" s="70" t="n"/>
-      <c r="G51" s="70" t="n"/>
-      <c r="H51" s="70" t="n"/>
-      <c r="I51" s="71" t="n"/>
-      <c r="J51" s="71" t="n"/>
+      <c r="A51" s="69" t="n"/>
+      <c r="B51" s="69" t="n"/>
+      <c r="C51" s="69" t="n"/>
+      <c r="D51" s="69" t="n"/>
+      <c r="E51" s="69" t="n"/>
+      <c r="F51" s="69" t="n"/>
+      <c r="G51" s="69" t="n"/>
+      <c r="H51" s="69" t="n"/>
+      <c r="I51" s="70" t="n"/>
+      <c r="J51" s="70" t="n"/>
       <c r="K51" s="65">
         <f>IFERROR(DATEDIF(I51,J51,"M"),"")</f>
         <v/>
       </c>
-      <c r="L51" s="72" t="n"/>
-      <c r="M51" s="70" t="n"/>
-      <c r="N51" s="70" t="n"/>
-      <c r="O51" s="72" t="n"/>
-      <c r="P51" s="70" t="n"/>
+      <c r="L51" s="71" t="n"/>
+      <c r="M51" s="69" t="n"/>
+      <c r="N51" s="69" t="n"/>
+      <c r="O51" s="71" t="n"/>
+      <c r="P51" s="69" t="n"/>
       <c r="Q51" s="67">
         <f>IFERROR(IF(J51="","",J51-TODAY()),"")</f>
         <v/>
@@ -3986,25 +3983,25 @@
       <c r="V51" s="69" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="73" t="n"/>
-      <c r="B52" s="73" t="n"/>
-      <c r="C52" s="73" t="n"/>
-      <c r="D52" s="73" t="n"/>
-      <c r="E52" s="73" t="n"/>
-      <c r="F52" s="73" t="n"/>
-      <c r="G52" s="73" t="n"/>
-      <c r="H52" s="73" t="n"/>
-      <c r="I52" s="74" t="n"/>
-      <c r="J52" s="74" t="n"/>
+      <c r="A52" s="72" t="n"/>
+      <c r="B52" s="72" t="n"/>
+      <c r="C52" s="72" t="n"/>
+      <c r="D52" s="72" t="n"/>
+      <c r="E52" s="72" t="n"/>
+      <c r="F52" s="72" t="n"/>
+      <c r="G52" s="72" t="n"/>
+      <c r="H52" s="72" t="n"/>
+      <c r="I52" s="73" t="n"/>
+      <c r="J52" s="73" t="n"/>
       <c r="K52" s="65">
         <f>IFERROR(DATEDIF(I52,J52,"M"),"")</f>
         <v/>
       </c>
-      <c r="L52" s="75" t="n"/>
-      <c r="M52" s="73" t="n"/>
-      <c r="N52" s="73" t="n"/>
-      <c r="O52" s="75" t="n"/>
-      <c r="P52" s="73" t="n"/>
+      <c r="L52" s="74" t="n"/>
+      <c r="M52" s="72" t="n"/>
+      <c r="N52" s="72" t="n"/>
+      <c r="O52" s="74" t="n"/>
+      <c r="P52" s="72" t="n"/>
       <c r="Q52" s="67">
         <f>IFERROR(IF(J52="","",J52-TODAY()),"")</f>
         <v/>
@@ -4013,31 +4010,31 @@
         <f>IFERROR(IF(B52="","Vacant",IF(Q52&lt;0,"Expired",IF(Q52&lt;=30,"Expiring Soon",IF(Q52&lt;=90,"Active - Review","Active")))),"Vacant")</f>
         <v/>
       </c>
-      <c r="S52" s="69" t="n"/>
-      <c r="T52" s="69" t="n"/>
-      <c r="U52" s="69" t="n"/>
-      <c r="V52" s="69" t="n"/>
+      <c r="S52" s="72" t="n"/>
+      <c r="T52" s="72" t="n"/>
+      <c r="U52" s="72" t="n"/>
+      <c r="V52" s="72" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="70" t="n"/>
-      <c r="B53" s="70" t="n"/>
-      <c r="C53" s="70" t="n"/>
-      <c r="D53" s="70" t="n"/>
-      <c r="E53" s="70" t="n"/>
-      <c r="F53" s="70" t="n"/>
-      <c r="G53" s="70" t="n"/>
-      <c r="H53" s="70" t="n"/>
-      <c r="I53" s="71" t="n"/>
-      <c r="J53" s="71" t="n"/>
+      <c r="A53" s="69" t="n"/>
+      <c r="B53" s="69" t="n"/>
+      <c r="C53" s="69" t="n"/>
+      <c r="D53" s="69" t="n"/>
+      <c r="E53" s="69" t="n"/>
+      <c r="F53" s="69" t="n"/>
+      <c r="G53" s="69" t="n"/>
+      <c r="H53" s="69" t="n"/>
+      <c r="I53" s="70" t="n"/>
+      <c r="J53" s="70" t="n"/>
       <c r="K53" s="65">
         <f>IFERROR(DATEDIF(I53,J53,"M"),"")</f>
         <v/>
       </c>
-      <c r="L53" s="72" t="n"/>
-      <c r="M53" s="70" t="n"/>
-      <c r="N53" s="70" t="n"/>
-      <c r="O53" s="72" t="n"/>
-      <c r="P53" s="70" t="n"/>
+      <c r="L53" s="71" t="n"/>
+      <c r="M53" s="69" t="n"/>
+      <c r="N53" s="69" t="n"/>
+      <c r="O53" s="71" t="n"/>
+      <c r="P53" s="69" t="n"/>
       <c r="Q53" s="67">
         <f>IFERROR(IF(J53="","",J53-TODAY()),"")</f>
         <v/>
@@ -4258,7 +4255,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="76" t="inlineStr">
+      <c r="A1" s="75" t="inlineStr">
         <is>
           <t>📋  LEASE AGREEMENTS &amp; RENEWALS</t>
         </is>
@@ -4272,82 +4269,82 @@
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="77" t="inlineStr">
+      <c r="A3" s="76" t="inlineStr">
         <is>
           <t>Agr. ID</t>
         </is>
       </c>
-      <c r="B3" s="77" t="inlineStr">
+      <c r="B3" s="76" t="inlineStr">
         <is>
           <t>Tenant ID</t>
         </is>
       </c>
-      <c r="C3" s="77" t="inlineStr">
+      <c r="C3" s="76" t="inlineStr">
         <is>
           <t>Tenant Name</t>
         </is>
       </c>
-      <c r="D3" s="77" t="inlineStr">
+      <c r="D3" s="76" t="inlineStr">
         <is>
           <t>Unit No.</t>
         </is>
       </c>
-      <c r="E3" s="77" t="inlineStr">
+      <c r="E3" s="76" t="inlineStr">
         <is>
           <t>Original Start</t>
         </is>
       </c>
-      <c r="F3" s="77" t="inlineStr">
+      <c r="F3" s="76" t="inlineStr">
         <is>
           <t>Lease Start</t>
         </is>
       </c>
-      <c r="G3" s="77" t="inlineStr">
+      <c r="G3" s="76" t="inlineStr">
         <is>
           <t>Lease End</t>
         </is>
       </c>
-      <c r="H3" s="77" t="inlineStr">
+      <c r="H3" s="76" t="inlineStr">
         <is>
           <t>Renewal?</t>
         </is>
       </c>
-      <c r="I3" s="77" t="inlineStr">
+      <c r="I3" s="76" t="inlineStr">
         <is>
           <t>Renewal No.</t>
         </is>
       </c>
-      <c r="J3" s="77" t="inlineStr">
+      <c r="J3" s="76" t="inlineStr">
         <is>
           <t>Term (months)</t>
         </is>
       </c>
-      <c r="K3" s="77" t="inlineStr">
+      <c r="K3" s="76" t="inlineStr">
         <is>
           <t>Annual Rent</t>
         </is>
       </c>
-      <c r="L3" s="77" t="inlineStr">
+      <c r="L3" s="76" t="inlineStr">
         <is>
           <t>Monthly Rent</t>
         </is>
       </c>
-      <c r="M3" s="77" t="inlineStr">
+      <c r="M3" s="76" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="N3" s="77" t="inlineStr">
+      <c r="N3" s="76" t="inlineStr">
         <is>
           <t>Rent Increment%</t>
         </is>
       </c>
-      <c r="O3" s="77" t="inlineStr">
+      <c r="O3" s="76" t="inlineStr">
         <is>
           <t>Next Review Date</t>
         </is>
       </c>
-      <c r="P3" s="77" t="inlineStr">
+      <c r="P3" s="76" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -4398,7 +4395,7 @@
       <c r="K4" s="66" t="n">
         <v>42000</v>
       </c>
-      <c r="L4" s="78">
+      <c r="L4" s="77">
         <f>IFERROR(IF(K4="","",K4/12),"")</f>
         <v/>
       </c>
@@ -4407,1337 +4404,1337 @@
           <t>GHS</t>
         </is>
       </c>
-      <c r="N4" s="79" t="n">
+      <c r="N4" s="78" t="n">
         <v>0.05</v>
       </c>
-      <c r="O4" s="80">
+      <c r="O4" s="79">
         <f>IFERROR(IF(G4="","",G4-365),"")</f>
         <v/>
       </c>
       <c r="P4" s="63" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="70" t="n"/>
-      <c r="B5" s="70" t="n"/>
-      <c r="C5" s="70" t="n"/>
-      <c r="D5" s="70" t="n"/>
-      <c r="E5" s="71" t="n"/>
-      <c r="F5" s="71" t="n"/>
-      <c r="G5" s="71" t="n"/>
-      <c r="H5" s="70" t="n"/>
-      <c r="I5" s="70" t="n"/>
+      <c r="A5" s="69" t="n"/>
+      <c r="B5" s="69" t="n"/>
+      <c r="C5" s="69" t="n"/>
+      <c r="D5" s="69" t="n"/>
+      <c r="E5" s="70" t="n"/>
+      <c r="F5" s="70" t="n"/>
+      <c r="G5" s="70" t="n"/>
+      <c r="H5" s="69" t="n"/>
+      <c r="I5" s="69" t="n"/>
       <c r="J5" s="65">
         <f>IFERROR(DATEDIF(F5,G5,"M"),"")</f>
         <v/>
       </c>
-      <c r="K5" s="72" t="n"/>
-      <c r="L5" s="78">
+      <c r="K5" s="71" t="n"/>
+      <c r="L5" s="77">
         <f>IFERROR(IF(K5="","",K5/12),"")</f>
         <v/>
       </c>
-      <c r="M5" s="70" t="n"/>
-      <c r="N5" s="81" t="n"/>
-      <c r="O5" s="80">
+      <c r="M5" s="69" t="n"/>
+      <c r="N5" s="80" t="n"/>
+      <c r="O5" s="79">
         <f>IFERROR(IF(G5="","",G5-365),"")</f>
         <v/>
       </c>
-      <c r="P5" s="70" t="n"/>
+      <c r="P5" s="69" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="73" t="n"/>
-      <c r="B6" s="73" t="n"/>
-      <c r="C6" s="73" t="n"/>
-      <c r="D6" s="73" t="n"/>
-      <c r="E6" s="74" t="n"/>
-      <c r="F6" s="74" t="n"/>
-      <c r="G6" s="74" t="n"/>
-      <c r="H6" s="73" t="n"/>
-      <c r="I6" s="73" t="n"/>
+      <c r="A6" s="72" t="n"/>
+      <c r="B6" s="72" t="n"/>
+      <c r="C6" s="72" t="n"/>
+      <c r="D6" s="72" t="n"/>
+      <c r="E6" s="73" t="n"/>
+      <c r="F6" s="73" t="n"/>
+      <c r="G6" s="73" t="n"/>
+      <c r="H6" s="72" t="n"/>
+      <c r="I6" s="72" t="n"/>
       <c r="J6" s="65">
         <f>IFERROR(DATEDIF(F6,G6,"M"),"")</f>
         <v/>
       </c>
-      <c r="K6" s="75" t="n"/>
-      <c r="L6" s="78">
+      <c r="K6" s="74" t="n"/>
+      <c r="L6" s="77">
         <f>IFERROR(IF(K6="","",K6/12),"")</f>
         <v/>
       </c>
-      <c r="M6" s="73" t="n"/>
-      <c r="N6" s="82" t="n"/>
-      <c r="O6" s="80">
+      <c r="M6" s="72" t="n"/>
+      <c r="N6" s="81" t="n"/>
+      <c r="O6" s="79">
         <f>IFERROR(IF(G6="","",G6-365),"")</f>
         <v/>
       </c>
-      <c r="P6" s="73" t="n"/>
+      <c r="P6" s="72" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="70" t="n"/>
-      <c r="B7" s="70" t="n"/>
-      <c r="C7" s="70" t="n"/>
-      <c r="D7" s="70" t="n"/>
-      <c r="E7" s="71" t="n"/>
-      <c r="F7" s="71" t="n"/>
-      <c r="G7" s="71" t="n"/>
-      <c r="H7" s="70" t="n"/>
-      <c r="I7" s="70" t="n"/>
+      <c r="A7" s="69" t="n"/>
+      <c r="B7" s="69" t="n"/>
+      <c r="C7" s="69" t="n"/>
+      <c r="D7" s="69" t="n"/>
+      <c r="E7" s="70" t="n"/>
+      <c r="F7" s="70" t="n"/>
+      <c r="G7" s="70" t="n"/>
+      <c r="H7" s="69" t="n"/>
+      <c r="I7" s="69" t="n"/>
       <c r="J7" s="65">
         <f>IFERROR(DATEDIF(F7,G7,"M"),"")</f>
         <v/>
       </c>
-      <c r="K7" s="72" t="n"/>
-      <c r="L7" s="78">
+      <c r="K7" s="71" t="n"/>
+      <c r="L7" s="77">
         <f>IFERROR(IF(K7="","",K7/12),"")</f>
         <v/>
       </c>
-      <c r="M7" s="70" t="n"/>
-      <c r="N7" s="81" t="n"/>
-      <c r="O7" s="80">
+      <c r="M7" s="69" t="n"/>
+      <c r="N7" s="80" t="n"/>
+      <c r="O7" s="79">
         <f>IFERROR(IF(G7="","",G7-365),"")</f>
         <v/>
       </c>
-      <c r="P7" s="70" t="n"/>
+      <c r="P7" s="69" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="73" t="n"/>
-      <c r="B8" s="73" t="n"/>
-      <c r="C8" s="73" t="n"/>
-      <c r="D8" s="73" t="n"/>
-      <c r="E8" s="74" t="n"/>
-      <c r="F8" s="74" t="n"/>
-      <c r="G8" s="74" t="n"/>
-      <c r="H8" s="73" t="n"/>
-      <c r="I8" s="73" t="n"/>
+      <c r="A8" s="72" t="n"/>
+      <c r="B8" s="72" t="n"/>
+      <c r="C8" s="72" t="n"/>
+      <c r="D8" s="72" t="n"/>
+      <c r="E8" s="73" t="n"/>
+      <c r="F8" s="73" t="n"/>
+      <c r="G8" s="73" t="n"/>
+      <c r="H8" s="72" t="n"/>
+      <c r="I8" s="72" t="n"/>
       <c r="J8" s="65">
         <f>IFERROR(DATEDIF(F8,G8,"M"),"")</f>
         <v/>
       </c>
-      <c r="K8" s="75" t="n"/>
-      <c r="L8" s="78">
+      <c r="K8" s="74" t="n"/>
+      <c r="L8" s="77">
         <f>IFERROR(IF(K8="","",K8/12),"")</f>
         <v/>
       </c>
-      <c r="M8" s="73" t="n"/>
-      <c r="N8" s="82" t="n"/>
-      <c r="O8" s="80">
+      <c r="M8" s="72" t="n"/>
+      <c r="N8" s="81" t="n"/>
+      <c r="O8" s="79">
         <f>IFERROR(IF(G8="","",G8-365),"")</f>
         <v/>
       </c>
-      <c r="P8" s="73" t="n"/>
+      <c r="P8" s="72" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="70" t="n"/>
-      <c r="B9" s="70" t="n"/>
-      <c r="C9" s="70" t="n"/>
-      <c r="D9" s="70" t="n"/>
-      <c r="E9" s="71" t="n"/>
-      <c r="F9" s="71" t="n"/>
-      <c r="G9" s="71" t="n"/>
-      <c r="H9" s="70" t="n"/>
-      <c r="I9" s="70" t="n"/>
+      <c r="A9" s="69" t="n"/>
+      <c r="B9" s="69" t="n"/>
+      <c r="C9" s="69" t="n"/>
+      <c r="D9" s="69" t="n"/>
+      <c r="E9" s="70" t="n"/>
+      <c r="F9" s="70" t="n"/>
+      <c r="G9" s="70" t="n"/>
+      <c r="H9" s="69" t="n"/>
+      <c r="I9" s="69" t="n"/>
       <c r="J9" s="65">
         <f>IFERROR(DATEDIF(F9,G9,"M"),"")</f>
         <v/>
       </c>
-      <c r="K9" s="72" t="n"/>
-      <c r="L9" s="78">
+      <c r="K9" s="71" t="n"/>
+      <c r="L9" s="77">
         <f>IFERROR(IF(K9="","",K9/12),"")</f>
         <v/>
       </c>
-      <c r="M9" s="70" t="n"/>
-      <c r="N9" s="81" t="n"/>
-      <c r="O9" s="80">
+      <c r="M9" s="69" t="n"/>
+      <c r="N9" s="80" t="n"/>
+      <c r="O9" s="79">
         <f>IFERROR(IF(G9="","",G9-365),"")</f>
         <v/>
       </c>
-      <c r="P9" s="70" t="n"/>
+      <c r="P9" s="69" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="73" t="n"/>
-      <c r="B10" s="73" t="n"/>
-      <c r="C10" s="73" t="n"/>
-      <c r="D10" s="73" t="n"/>
-      <c r="E10" s="74" t="n"/>
-      <c r="F10" s="74" t="n"/>
-      <c r="G10" s="74" t="n"/>
-      <c r="H10" s="73" t="n"/>
-      <c r="I10" s="73" t="n"/>
+      <c r="A10" s="72" t="n"/>
+      <c r="B10" s="72" t="n"/>
+      <c r="C10" s="72" t="n"/>
+      <c r="D10" s="72" t="n"/>
+      <c r="E10" s="73" t="n"/>
+      <c r="F10" s="73" t="n"/>
+      <c r="G10" s="73" t="n"/>
+      <c r="H10" s="72" t="n"/>
+      <c r="I10" s="72" t="n"/>
       <c r="J10" s="65">
         <f>IFERROR(DATEDIF(F10,G10,"M"),"")</f>
         <v/>
       </c>
-      <c r="K10" s="75" t="n"/>
-      <c r="L10" s="78">
+      <c r="K10" s="74" t="n"/>
+      <c r="L10" s="77">
         <f>IFERROR(IF(K10="","",K10/12),"")</f>
         <v/>
       </c>
-      <c r="M10" s="73" t="n"/>
-      <c r="N10" s="82" t="n"/>
-      <c r="O10" s="80">
+      <c r="M10" s="72" t="n"/>
+      <c r="N10" s="81" t="n"/>
+      <c r="O10" s="79">
         <f>IFERROR(IF(G10="","",G10-365),"")</f>
         <v/>
       </c>
-      <c r="P10" s="73" t="n"/>
+      <c r="P10" s="72" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="70" t="n"/>
-      <c r="B11" s="70" t="n"/>
-      <c r="C11" s="70" t="n"/>
-      <c r="D11" s="70" t="n"/>
-      <c r="E11" s="71" t="n"/>
-      <c r="F11" s="71" t="n"/>
-      <c r="G11" s="71" t="n"/>
-      <c r="H11" s="70" t="n"/>
-      <c r="I11" s="70" t="n"/>
+      <c r="A11" s="69" t="n"/>
+      <c r="B11" s="69" t="n"/>
+      <c r="C11" s="69" t="n"/>
+      <c r="D11" s="69" t="n"/>
+      <c r="E11" s="70" t="n"/>
+      <c r="F11" s="70" t="n"/>
+      <c r="G11" s="70" t="n"/>
+      <c r="H11" s="69" t="n"/>
+      <c r="I11" s="69" t="n"/>
       <c r="J11" s="65">
         <f>IFERROR(DATEDIF(F11,G11,"M"),"")</f>
         <v/>
       </c>
-      <c r="K11" s="72" t="n"/>
-      <c r="L11" s="78">
+      <c r="K11" s="71" t="n"/>
+      <c r="L11" s="77">
         <f>IFERROR(IF(K11="","",K11/12),"")</f>
         <v/>
       </c>
-      <c r="M11" s="70" t="n"/>
-      <c r="N11" s="81" t="n"/>
-      <c r="O11" s="80">
+      <c r="M11" s="69" t="n"/>
+      <c r="N11" s="80" t="n"/>
+      <c r="O11" s="79">
         <f>IFERROR(IF(G11="","",G11-365),"")</f>
         <v/>
       </c>
-      <c r="P11" s="70" t="n"/>
+      <c r="P11" s="69" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="73" t="n"/>
-      <c r="B12" s="73" t="n"/>
-      <c r="C12" s="73" t="n"/>
-      <c r="D12" s="73" t="n"/>
-      <c r="E12" s="74" t="n"/>
-      <c r="F12" s="74" t="n"/>
-      <c r="G12" s="74" t="n"/>
-      <c r="H12" s="73" t="n"/>
-      <c r="I12" s="73" t="n"/>
+      <c r="A12" s="72" t="n"/>
+      <c r="B12" s="72" t="n"/>
+      <c r="C12" s="72" t="n"/>
+      <c r="D12" s="72" t="n"/>
+      <c r="E12" s="73" t="n"/>
+      <c r="F12" s="73" t="n"/>
+      <c r="G12" s="73" t="n"/>
+      <c r="H12" s="72" t="n"/>
+      <c r="I12" s="72" t="n"/>
       <c r="J12" s="65">
         <f>IFERROR(DATEDIF(F12,G12,"M"),"")</f>
         <v/>
       </c>
-      <c r="K12" s="75" t="n"/>
-      <c r="L12" s="78">
+      <c r="K12" s="74" t="n"/>
+      <c r="L12" s="77">
         <f>IFERROR(IF(K12="","",K12/12),"")</f>
         <v/>
       </c>
-      <c r="M12" s="73" t="n"/>
-      <c r="N12" s="82" t="n"/>
-      <c r="O12" s="80">
+      <c r="M12" s="72" t="n"/>
+      <c r="N12" s="81" t="n"/>
+      <c r="O12" s="79">
         <f>IFERROR(IF(G12="","",G12-365),"")</f>
         <v/>
       </c>
-      <c r="P12" s="73" t="n"/>
+      <c r="P12" s="72" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="70" t="n"/>
-      <c r="B13" s="70" t="n"/>
-      <c r="C13" s="70" t="n"/>
-      <c r="D13" s="70" t="n"/>
-      <c r="E13" s="71" t="n"/>
-      <c r="F13" s="71" t="n"/>
-      <c r="G13" s="71" t="n"/>
-      <c r="H13" s="70" t="n"/>
-      <c r="I13" s="70" t="n"/>
+      <c r="A13" s="69" t="n"/>
+      <c r="B13" s="69" t="n"/>
+      <c r="C13" s="69" t="n"/>
+      <c r="D13" s="69" t="n"/>
+      <c r="E13" s="70" t="n"/>
+      <c r="F13" s="70" t="n"/>
+      <c r="G13" s="70" t="n"/>
+      <c r="H13" s="69" t="n"/>
+      <c r="I13" s="69" t="n"/>
       <c r="J13" s="65">
         <f>IFERROR(DATEDIF(F13,G13,"M"),"")</f>
         <v/>
       </c>
-      <c r="K13" s="72" t="n"/>
-      <c r="L13" s="78">
+      <c r="K13" s="71" t="n"/>
+      <c r="L13" s="77">
         <f>IFERROR(IF(K13="","",K13/12),"")</f>
         <v/>
       </c>
-      <c r="M13" s="70" t="n"/>
-      <c r="N13" s="81" t="n"/>
-      <c r="O13" s="80">
+      <c r="M13" s="69" t="n"/>
+      <c r="N13" s="80" t="n"/>
+      <c r="O13" s="79">
         <f>IFERROR(IF(G13="","",G13-365),"")</f>
         <v/>
       </c>
-      <c r="P13" s="70" t="n"/>
+      <c r="P13" s="69" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="73" t="n"/>
-      <c r="B14" s="73" t="n"/>
-      <c r="C14" s="73" t="n"/>
-      <c r="D14" s="73" t="n"/>
-      <c r="E14" s="74" t="n"/>
-      <c r="F14" s="74" t="n"/>
-      <c r="G14" s="74" t="n"/>
-      <c r="H14" s="73" t="n"/>
-      <c r="I14" s="73" t="n"/>
+      <c r="A14" s="72" t="n"/>
+      <c r="B14" s="72" t="n"/>
+      <c r="C14" s="72" t="n"/>
+      <c r="D14" s="72" t="n"/>
+      <c r="E14" s="73" t="n"/>
+      <c r="F14" s="73" t="n"/>
+      <c r="G14" s="73" t="n"/>
+      <c r="H14" s="72" t="n"/>
+      <c r="I14" s="72" t="n"/>
       <c r="J14" s="65">
         <f>IFERROR(DATEDIF(F14,G14,"M"),"")</f>
         <v/>
       </c>
-      <c r="K14" s="75" t="n"/>
-      <c r="L14" s="78">
+      <c r="K14" s="74" t="n"/>
+      <c r="L14" s="77">
         <f>IFERROR(IF(K14="","",K14/12),"")</f>
         <v/>
       </c>
-      <c r="M14" s="73" t="n"/>
-      <c r="N14" s="82" t="n"/>
-      <c r="O14" s="80">
+      <c r="M14" s="72" t="n"/>
+      <c r="N14" s="81" t="n"/>
+      <c r="O14" s="79">
         <f>IFERROR(IF(G14="","",G14-365),"")</f>
         <v/>
       </c>
-      <c r="P14" s="73" t="n"/>
+      <c r="P14" s="72" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="70" t="n"/>
-      <c r="B15" s="70" t="n"/>
-      <c r="C15" s="70" t="n"/>
-      <c r="D15" s="70" t="n"/>
-      <c r="E15" s="71" t="n"/>
-      <c r="F15" s="71" t="n"/>
-      <c r="G15" s="71" t="n"/>
-      <c r="H15" s="70" t="n"/>
-      <c r="I15" s="70" t="n"/>
+      <c r="A15" s="69" t="n"/>
+      <c r="B15" s="69" t="n"/>
+      <c r="C15" s="69" t="n"/>
+      <c r="D15" s="69" t="n"/>
+      <c r="E15" s="70" t="n"/>
+      <c r="F15" s="70" t="n"/>
+      <c r="G15" s="70" t="n"/>
+      <c r="H15" s="69" t="n"/>
+      <c r="I15" s="69" t="n"/>
       <c r="J15" s="65">
         <f>IFERROR(DATEDIF(F15,G15,"M"),"")</f>
         <v/>
       </c>
-      <c r="K15" s="72" t="n"/>
-      <c r="L15" s="78">
+      <c r="K15" s="71" t="n"/>
+      <c r="L15" s="77">
         <f>IFERROR(IF(K15="","",K15/12),"")</f>
         <v/>
       </c>
-      <c r="M15" s="70" t="n"/>
-      <c r="N15" s="81" t="n"/>
-      <c r="O15" s="80">
+      <c r="M15" s="69" t="n"/>
+      <c r="N15" s="80" t="n"/>
+      <c r="O15" s="79">
         <f>IFERROR(IF(G15="","",G15-365),"")</f>
         <v/>
       </c>
-      <c r="P15" s="70" t="n"/>
+      <c r="P15" s="69" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="73" t="n"/>
-      <c r="B16" s="73" t="n"/>
-      <c r="C16" s="73" t="n"/>
-      <c r="D16" s="73" t="n"/>
-      <c r="E16" s="74" t="n"/>
-      <c r="F16" s="74" t="n"/>
-      <c r="G16" s="74" t="n"/>
-      <c r="H16" s="73" t="n"/>
-      <c r="I16" s="73" t="n"/>
+      <c r="A16" s="72" t="n"/>
+      <c r="B16" s="72" t="n"/>
+      <c r="C16" s="72" t="n"/>
+      <c r="D16" s="72" t="n"/>
+      <c r="E16" s="73" t="n"/>
+      <c r="F16" s="73" t="n"/>
+      <c r="G16" s="73" t="n"/>
+      <c r="H16" s="72" t="n"/>
+      <c r="I16" s="72" t="n"/>
       <c r="J16" s="65">
         <f>IFERROR(DATEDIF(F16,G16,"M"),"")</f>
         <v/>
       </c>
-      <c r="K16" s="75" t="n"/>
-      <c r="L16" s="78">
+      <c r="K16" s="74" t="n"/>
+      <c r="L16" s="77">
         <f>IFERROR(IF(K16="","",K16/12),"")</f>
         <v/>
       </c>
-      <c r="M16" s="73" t="n"/>
-      <c r="N16" s="82" t="n"/>
-      <c r="O16" s="80">
+      <c r="M16" s="72" t="n"/>
+      <c r="N16" s="81" t="n"/>
+      <c r="O16" s="79">
         <f>IFERROR(IF(G16="","",G16-365),"")</f>
         <v/>
       </c>
-      <c r="P16" s="73" t="n"/>
+      <c r="P16" s="72" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="70" t="n"/>
-      <c r="B17" s="70" t="n"/>
-      <c r="C17" s="70" t="n"/>
-      <c r="D17" s="70" t="n"/>
-      <c r="E17" s="71" t="n"/>
-      <c r="F17" s="71" t="n"/>
-      <c r="G17" s="71" t="n"/>
-      <c r="H17" s="70" t="n"/>
-      <c r="I17" s="70" t="n"/>
+      <c r="A17" s="69" t="n"/>
+      <c r="B17" s="69" t="n"/>
+      <c r="C17" s="69" t="n"/>
+      <c r="D17" s="69" t="n"/>
+      <c r="E17" s="70" t="n"/>
+      <c r="F17" s="70" t="n"/>
+      <c r="G17" s="70" t="n"/>
+      <c r="H17" s="69" t="n"/>
+      <c r="I17" s="69" t="n"/>
       <c r="J17" s="65">
         <f>IFERROR(DATEDIF(F17,G17,"M"),"")</f>
         <v/>
       </c>
-      <c r="K17" s="72" t="n"/>
-      <c r="L17" s="78">
+      <c r="K17" s="71" t="n"/>
+      <c r="L17" s="77">
         <f>IFERROR(IF(K17="","",K17/12),"")</f>
         <v/>
       </c>
-      <c r="M17" s="70" t="n"/>
-      <c r="N17" s="81" t="n"/>
-      <c r="O17" s="80">
+      <c r="M17" s="69" t="n"/>
+      <c r="N17" s="80" t="n"/>
+      <c r="O17" s="79">
         <f>IFERROR(IF(G17="","",G17-365),"")</f>
         <v/>
       </c>
-      <c r="P17" s="70" t="n"/>
+      <c r="P17" s="69" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="73" t="n"/>
-      <c r="B18" s="73" t="n"/>
-      <c r="C18" s="73" t="n"/>
-      <c r="D18" s="73" t="n"/>
-      <c r="E18" s="74" t="n"/>
-      <c r="F18" s="74" t="n"/>
-      <c r="G18" s="74" t="n"/>
-      <c r="H18" s="73" t="n"/>
-      <c r="I18" s="73" t="n"/>
+      <c r="A18" s="72" t="n"/>
+      <c r="B18" s="72" t="n"/>
+      <c r="C18" s="72" t="n"/>
+      <c r="D18" s="72" t="n"/>
+      <c r="E18" s="73" t="n"/>
+      <c r="F18" s="73" t="n"/>
+      <c r="G18" s="73" t="n"/>
+      <c r="H18" s="72" t="n"/>
+      <c r="I18" s="72" t="n"/>
       <c r="J18" s="65">
         <f>IFERROR(DATEDIF(F18,G18,"M"),"")</f>
         <v/>
       </c>
-      <c r="K18" s="75" t="n"/>
-      <c r="L18" s="78">
+      <c r="K18" s="74" t="n"/>
+      <c r="L18" s="77">
         <f>IFERROR(IF(K18="","",K18/12),"")</f>
         <v/>
       </c>
-      <c r="M18" s="73" t="n"/>
-      <c r="N18" s="82" t="n"/>
-      <c r="O18" s="80">
+      <c r="M18" s="72" t="n"/>
+      <c r="N18" s="81" t="n"/>
+      <c r="O18" s="79">
         <f>IFERROR(IF(G18="","",G18-365),"")</f>
         <v/>
       </c>
-      <c r="P18" s="73" t="n"/>
+      <c r="P18" s="72" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="70" t="n"/>
-      <c r="B19" s="70" t="n"/>
-      <c r="C19" s="70" t="n"/>
-      <c r="D19" s="70" t="n"/>
-      <c r="E19" s="71" t="n"/>
-      <c r="F19" s="71" t="n"/>
-      <c r="G19" s="71" t="n"/>
-      <c r="H19" s="70" t="n"/>
-      <c r="I19" s="70" t="n"/>
+      <c r="A19" s="69" t="n"/>
+      <c r="B19" s="69" t="n"/>
+      <c r="C19" s="69" t="n"/>
+      <c r="D19" s="69" t="n"/>
+      <c r="E19" s="70" t="n"/>
+      <c r="F19" s="70" t="n"/>
+      <c r="G19" s="70" t="n"/>
+      <c r="H19" s="69" t="n"/>
+      <c r="I19" s="69" t="n"/>
       <c r="J19" s="65">
         <f>IFERROR(DATEDIF(F19,G19,"M"),"")</f>
         <v/>
       </c>
-      <c r="K19" s="72" t="n"/>
-      <c r="L19" s="78">
+      <c r="K19" s="71" t="n"/>
+      <c r="L19" s="77">
         <f>IFERROR(IF(K19="","",K19/12),"")</f>
         <v/>
       </c>
-      <c r="M19" s="70" t="n"/>
-      <c r="N19" s="81" t="n"/>
-      <c r="O19" s="80">
+      <c r="M19" s="69" t="n"/>
+      <c r="N19" s="80" t="n"/>
+      <c r="O19" s="79">
         <f>IFERROR(IF(G19="","",G19-365),"")</f>
         <v/>
       </c>
-      <c r="P19" s="70" t="n"/>
+      <c r="P19" s="69" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="73" t="n"/>
-      <c r="B20" s="73" t="n"/>
-      <c r="C20" s="73" t="n"/>
-      <c r="D20" s="73" t="n"/>
-      <c r="E20" s="74" t="n"/>
-      <c r="F20" s="74" t="n"/>
-      <c r="G20" s="74" t="n"/>
-      <c r="H20" s="73" t="n"/>
-      <c r="I20" s="73" t="n"/>
+      <c r="A20" s="72" t="n"/>
+      <c r="B20" s="72" t="n"/>
+      <c r="C20" s="72" t="n"/>
+      <c r="D20" s="72" t="n"/>
+      <c r="E20" s="73" t="n"/>
+      <c r="F20" s="73" t="n"/>
+      <c r="G20" s="73" t="n"/>
+      <c r="H20" s="72" t="n"/>
+      <c r="I20" s="72" t="n"/>
       <c r="J20" s="65">
         <f>IFERROR(DATEDIF(F20,G20,"M"),"")</f>
         <v/>
       </c>
-      <c r="K20" s="75" t="n"/>
-      <c r="L20" s="78">
+      <c r="K20" s="74" t="n"/>
+      <c r="L20" s="77">
         <f>IFERROR(IF(K20="","",K20/12),"")</f>
         <v/>
       </c>
-      <c r="M20" s="73" t="n"/>
-      <c r="N20" s="82" t="n"/>
-      <c r="O20" s="80">
+      <c r="M20" s="72" t="n"/>
+      <c r="N20" s="81" t="n"/>
+      <c r="O20" s="79">
         <f>IFERROR(IF(G20="","",G20-365),"")</f>
         <v/>
       </c>
-      <c r="P20" s="73" t="n"/>
+      <c r="P20" s="72" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="70" t="n"/>
-      <c r="B21" s="70" t="n"/>
-      <c r="C21" s="70" t="n"/>
-      <c r="D21" s="70" t="n"/>
-      <c r="E21" s="71" t="n"/>
-      <c r="F21" s="71" t="n"/>
-      <c r="G21" s="71" t="n"/>
-      <c r="H21" s="70" t="n"/>
-      <c r="I21" s="70" t="n"/>
+      <c r="A21" s="69" t="n"/>
+      <c r="B21" s="69" t="n"/>
+      <c r="C21" s="69" t="n"/>
+      <c r="D21" s="69" t="n"/>
+      <c r="E21" s="70" t="n"/>
+      <c r="F21" s="70" t="n"/>
+      <c r="G21" s="70" t="n"/>
+      <c r="H21" s="69" t="n"/>
+      <c r="I21" s="69" t="n"/>
       <c r="J21" s="65">
         <f>IFERROR(DATEDIF(F21,G21,"M"),"")</f>
         <v/>
       </c>
-      <c r="K21" s="72" t="n"/>
-      <c r="L21" s="78">
+      <c r="K21" s="71" t="n"/>
+      <c r="L21" s="77">
         <f>IFERROR(IF(K21="","",K21/12),"")</f>
         <v/>
       </c>
-      <c r="M21" s="70" t="n"/>
-      <c r="N21" s="81" t="n"/>
-      <c r="O21" s="80">
+      <c r="M21" s="69" t="n"/>
+      <c r="N21" s="80" t="n"/>
+      <c r="O21" s="79">
         <f>IFERROR(IF(G21="","",G21-365),"")</f>
         <v/>
       </c>
-      <c r="P21" s="70" t="n"/>
+      <c r="P21" s="69" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="73" t="n"/>
-      <c r="B22" s="73" t="n"/>
-      <c r="C22" s="73" t="n"/>
-      <c r="D22" s="73" t="n"/>
-      <c r="E22" s="74" t="n"/>
-      <c r="F22" s="74" t="n"/>
-      <c r="G22" s="74" t="n"/>
-      <c r="H22" s="73" t="n"/>
-      <c r="I22" s="73" t="n"/>
+      <c r="A22" s="72" t="n"/>
+      <c r="B22" s="72" t="n"/>
+      <c r="C22" s="72" t="n"/>
+      <c r="D22" s="72" t="n"/>
+      <c r="E22" s="73" t="n"/>
+      <c r="F22" s="73" t="n"/>
+      <c r="G22" s="73" t="n"/>
+      <c r="H22" s="72" t="n"/>
+      <c r="I22" s="72" t="n"/>
       <c r="J22" s="65">
         <f>IFERROR(DATEDIF(F22,G22,"M"),"")</f>
         <v/>
       </c>
-      <c r="K22" s="75" t="n"/>
-      <c r="L22" s="78">
+      <c r="K22" s="74" t="n"/>
+      <c r="L22" s="77">
         <f>IFERROR(IF(K22="","",K22/12),"")</f>
         <v/>
       </c>
-      <c r="M22" s="73" t="n"/>
-      <c r="N22" s="82" t="n"/>
-      <c r="O22" s="80">
+      <c r="M22" s="72" t="n"/>
+      <c r="N22" s="81" t="n"/>
+      <c r="O22" s="79">
         <f>IFERROR(IF(G22="","",G22-365),"")</f>
         <v/>
       </c>
-      <c r="P22" s="73" t="n"/>
+      <c r="P22" s="72" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="70" t="n"/>
-      <c r="B23" s="70" t="n"/>
-      <c r="C23" s="70" t="n"/>
-      <c r="D23" s="70" t="n"/>
-      <c r="E23" s="71" t="n"/>
-      <c r="F23" s="71" t="n"/>
-      <c r="G23" s="71" t="n"/>
-      <c r="H23" s="70" t="n"/>
-      <c r="I23" s="70" t="n"/>
+      <c r="A23" s="69" t="n"/>
+      <c r="B23" s="69" t="n"/>
+      <c r="C23" s="69" t="n"/>
+      <c r="D23" s="69" t="n"/>
+      <c r="E23" s="70" t="n"/>
+      <c r="F23" s="70" t="n"/>
+      <c r="G23" s="70" t="n"/>
+      <c r="H23" s="69" t="n"/>
+      <c r="I23" s="69" t="n"/>
       <c r="J23" s="65">
         <f>IFERROR(DATEDIF(F23,G23,"M"),"")</f>
         <v/>
       </c>
-      <c r="K23" s="72" t="n"/>
-      <c r="L23" s="78">
+      <c r="K23" s="71" t="n"/>
+      <c r="L23" s="77">
         <f>IFERROR(IF(K23="","",K23/12),"")</f>
         <v/>
       </c>
-      <c r="M23" s="70" t="n"/>
-      <c r="N23" s="81" t="n"/>
-      <c r="O23" s="80">
+      <c r="M23" s="69" t="n"/>
+      <c r="N23" s="80" t="n"/>
+      <c r="O23" s="79">
         <f>IFERROR(IF(G23="","",G23-365),"")</f>
         <v/>
       </c>
-      <c r="P23" s="70" t="n"/>
+      <c r="P23" s="69" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="73" t="n"/>
-      <c r="B24" s="73" t="n"/>
-      <c r="C24" s="73" t="n"/>
-      <c r="D24" s="73" t="n"/>
-      <c r="E24" s="74" t="n"/>
-      <c r="F24" s="74" t="n"/>
-      <c r="G24" s="74" t="n"/>
-      <c r="H24" s="73" t="n"/>
-      <c r="I24" s="73" t="n"/>
+      <c r="A24" s="72" t="n"/>
+      <c r="B24" s="72" t="n"/>
+      <c r="C24" s="72" t="n"/>
+      <c r="D24" s="72" t="n"/>
+      <c r="E24" s="73" t="n"/>
+      <c r="F24" s="73" t="n"/>
+      <c r="G24" s="73" t="n"/>
+      <c r="H24" s="72" t="n"/>
+      <c r="I24" s="72" t="n"/>
       <c r="J24" s="65">
         <f>IFERROR(DATEDIF(F24,G24,"M"),"")</f>
         <v/>
       </c>
-      <c r="K24" s="75" t="n"/>
-      <c r="L24" s="78">
+      <c r="K24" s="74" t="n"/>
+      <c r="L24" s="77">
         <f>IFERROR(IF(K24="","",K24/12),"")</f>
         <v/>
       </c>
-      <c r="M24" s="73" t="n"/>
-      <c r="N24" s="82" t="n"/>
-      <c r="O24" s="80">
+      <c r="M24" s="72" t="n"/>
+      <c r="N24" s="81" t="n"/>
+      <c r="O24" s="79">
         <f>IFERROR(IF(G24="","",G24-365),"")</f>
         <v/>
       </c>
-      <c r="P24" s="73" t="n"/>
+      <c r="P24" s="72" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="70" t="n"/>
-      <c r="B25" s="70" t="n"/>
-      <c r="C25" s="70" t="n"/>
-      <c r="D25" s="70" t="n"/>
-      <c r="E25" s="71" t="n"/>
-      <c r="F25" s="71" t="n"/>
-      <c r="G25" s="71" t="n"/>
-      <c r="H25" s="70" t="n"/>
-      <c r="I25" s="70" t="n"/>
+      <c r="A25" s="69" t="n"/>
+      <c r="B25" s="69" t="n"/>
+      <c r="C25" s="69" t="n"/>
+      <c r="D25" s="69" t="n"/>
+      <c r="E25" s="70" t="n"/>
+      <c r="F25" s="70" t="n"/>
+      <c r="G25" s="70" t="n"/>
+      <c r="H25" s="69" t="n"/>
+      <c r="I25" s="69" t="n"/>
       <c r="J25" s="65">
         <f>IFERROR(DATEDIF(F25,G25,"M"),"")</f>
         <v/>
       </c>
-      <c r="K25" s="72" t="n"/>
-      <c r="L25" s="78">
+      <c r="K25" s="71" t="n"/>
+      <c r="L25" s="77">
         <f>IFERROR(IF(K25="","",K25/12),"")</f>
         <v/>
       </c>
-      <c r="M25" s="70" t="n"/>
-      <c r="N25" s="81" t="n"/>
-      <c r="O25" s="80">
+      <c r="M25" s="69" t="n"/>
+      <c r="N25" s="80" t="n"/>
+      <c r="O25" s="79">
         <f>IFERROR(IF(G25="","",G25-365),"")</f>
         <v/>
       </c>
-      <c r="P25" s="70" t="n"/>
+      <c r="P25" s="69" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="73" t="n"/>
-      <c r="B26" s="73" t="n"/>
-      <c r="C26" s="73" t="n"/>
-      <c r="D26" s="73" t="n"/>
-      <c r="E26" s="74" t="n"/>
-      <c r="F26" s="74" t="n"/>
-      <c r="G26" s="74" t="n"/>
-      <c r="H26" s="73" t="n"/>
-      <c r="I26" s="73" t="n"/>
+      <c r="A26" s="72" t="n"/>
+      <c r="B26" s="72" t="n"/>
+      <c r="C26" s="72" t="n"/>
+      <c r="D26" s="72" t="n"/>
+      <c r="E26" s="73" t="n"/>
+      <c r="F26" s="73" t="n"/>
+      <c r="G26" s="73" t="n"/>
+      <c r="H26" s="72" t="n"/>
+      <c r="I26" s="72" t="n"/>
       <c r="J26" s="65">
         <f>IFERROR(DATEDIF(F26,G26,"M"),"")</f>
         <v/>
       </c>
-      <c r="K26" s="75" t="n"/>
-      <c r="L26" s="78">
+      <c r="K26" s="74" t="n"/>
+      <c r="L26" s="77">
         <f>IFERROR(IF(K26="","",K26/12),"")</f>
         <v/>
       </c>
-      <c r="M26" s="73" t="n"/>
-      <c r="N26" s="82" t="n"/>
-      <c r="O26" s="80">
+      <c r="M26" s="72" t="n"/>
+      <c r="N26" s="81" t="n"/>
+      <c r="O26" s="79">
         <f>IFERROR(IF(G26="","",G26-365),"")</f>
         <v/>
       </c>
-      <c r="P26" s="73" t="n"/>
+      <c r="P26" s="72" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="70" t="n"/>
-      <c r="B27" s="70" t="n"/>
-      <c r="C27" s="70" t="n"/>
-      <c r="D27" s="70" t="n"/>
-      <c r="E27" s="71" t="n"/>
-      <c r="F27" s="71" t="n"/>
-      <c r="G27" s="71" t="n"/>
-      <c r="H27" s="70" t="n"/>
-      <c r="I27" s="70" t="n"/>
+      <c r="A27" s="69" t="n"/>
+      <c r="B27" s="69" t="n"/>
+      <c r="C27" s="69" t="n"/>
+      <c r="D27" s="69" t="n"/>
+      <c r="E27" s="70" t="n"/>
+      <c r="F27" s="70" t="n"/>
+      <c r="G27" s="70" t="n"/>
+      <c r="H27" s="69" t="n"/>
+      <c r="I27" s="69" t="n"/>
       <c r="J27" s="65">
         <f>IFERROR(DATEDIF(F27,G27,"M"),"")</f>
         <v/>
       </c>
-      <c r="K27" s="72" t="n"/>
-      <c r="L27" s="78">
+      <c r="K27" s="71" t="n"/>
+      <c r="L27" s="77">
         <f>IFERROR(IF(K27="","",K27/12),"")</f>
         <v/>
       </c>
-      <c r="M27" s="70" t="n"/>
-      <c r="N27" s="81" t="n"/>
-      <c r="O27" s="80">
+      <c r="M27" s="69" t="n"/>
+      <c r="N27" s="80" t="n"/>
+      <c r="O27" s="79">
         <f>IFERROR(IF(G27="","",G27-365),"")</f>
         <v/>
       </c>
-      <c r="P27" s="70" t="n"/>
+      <c r="P27" s="69" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="73" t="n"/>
-      <c r="B28" s="73" t="n"/>
-      <c r="C28" s="73" t="n"/>
-      <c r="D28" s="73" t="n"/>
-      <c r="E28" s="74" t="n"/>
-      <c r="F28" s="74" t="n"/>
-      <c r="G28" s="74" t="n"/>
-      <c r="H28" s="73" t="n"/>
-      <c r="I28" s="73" t="n"/>
+      <c r="A28" s="72" t="n"/>
+      <c r="B28" s="72" t="n"/>
+      <c r="C28" s="72" t="n"/>
+      <c r="D28" s="72" t="n"/>
+      <c r="E28" s="73" t="n"/>
+      <c r="F28" s="73" t="n"/>
+      <c r="G28" s="73" t="n"/>
+      <c r="H28" s="72" t="n"/>
+      <c r="I28" s="72" t="n"/>
       <c r="J28" s="65">
         <f>IFERROR(DATEDIF(F28,G28,"M"),"")</f>
         <v/>
       </c>
-      <c r="K28" s="75" t="n"/>
-      <c r="L28" s="78">
+      <c r="K28" s="74" t="n"/>
+      <c r="L28" s="77">
         <f>IFERROR(IF(K28="","",K28/12),"")</f>
         <v/>
       </c>
-      <c r="M28" s="73" t="n"/>
-      <c r="N28" s="82" t="n"/>
-      <c r="O28" s="80">
+      <c r="M28" s="72" t="n"/>
+      <c r="N28" s="81" t="n"/>
+      <c r="O28" s="79">
         <f>IFERROR(IF(G28="","",G28-365),"")</f>
         <v/>
       </c>
-      <c r="P28" s="73" t="n"/>
+      <c r="P28" s="72" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="70" t="n"/>
-      <c r="B29" s="70" t="n"/>
-      <c r="C29" s="70" t="n"/>
-      <c r="D29" s="70" t="n"/>
-      <c r="E29" s="71" t="n"/>
-      <c r="F29" s="71" t="n"/>
-      <c r="G29" s="71" t="n"/>
-      <c r="H29" s="70" t="n"/>
-      <c r="I29" s="70" t="n"/>
+      <c r="A29" s="69" t="n"/>
+      <c r="B29" s="69" t="n"/>
+      <c r="C29" s="69" t="n"/>
+      <c r="D29" s="69" t="n"/>
+      <c r="E29" s="70" t="n"/>
+      <c r="F29" s="70" t="n"/>
+      <c r="G29" s="70" t="n"/>
+      <c r="H29" s="69" t="n"/>
+      <c r="I29" s="69" t="n"/>
       <c r="J29" s="65">
         <f>IFERROR(DATEDIF(F29,G29,"M"),"")</f>
         <v/>
       </c>
-      <c r="K29" s="72" t="n"/>
-      <c r="L29" s="78">
+      <c r="K29" s="71" t="n"/>
+      <c r="L29" s="77">
         <f>IFERROR(IF(K29="","",K29/12),"")</f>
         <v/>
       </c>
-      <c r="M29" s="70" t="n"/>
-      <c r="N29" s="81" t="n"/>
-      <c r="O29" s="80">
+      <c r="M29" s="69" t="n"/>
+      <c r="N29" s="80" t="n"/>
+      <c r="O29" s="79">
         <f>IFERROR(IF(G29="","",G29-365),"")</f>
         <v/>
       </c>
-      <c r="P29" s="70" t="n"/>
+      <c r="P29" s="69" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="73" t="n"/>
-      <c r="B30" s="73" t="n"/>
-      <c r="C30" s="73" t="n"/>
-      <c r="D30" s="73" t="n"/>
-      <c r="E30" s="74" t="n"/>
-      <c r="F30" s="74" t="n"/>
-      <c r="G30" s="74" t="n"/>
-      <c r="H30" s="73" t="n"/>
-      <c r="I30" s="73" t="n"/>
+      <c r="A30" s="72" t="n"/>
+      <c r="B30" s="72" t="n"/>
+      <c r="C30" s="72" t="n"/>
+      <c r="D30" s="72" t="n"/>
+      <c r="E30" s="73" t="n"/>
+      <c r="F30" s="73" t="n"/>
+      <c r="G30" s="73" t="n"/>
+      <c r="H30" s="72" t="n"/>
+      <c r="I30" s="72" t="n"/>
       <c r="J30" s="65">
         <f>IFERROR(DATEDIF(F30,G30,"M"),"")</f>
         <v/>
       </c>
-      <c r="K30" s="75" t="n"/>
-      <c r="L30" s="78">
+      <c r="K30" s="74" t="n"/>
+      <c r="L30" s="77">
         <f>IFERROR(IF(K30="","",K30/12),"")</f>
         <v/>
       </c>
-      <c r="M30" s="73" t="n"/>
-      <c r="N30" s="82" t="n"/>
-      <c r="O30" s="80">
+      <c r="M30" s="72" t="n"/>
+      <c r="N30" s="81" t="n"/>
+      <c r="O30" s="79">
         <f>IFERROR(IF(G30="","",G30-365),"")</f>
         <v/>
       </c>
-      <c r="P30" s="73" t="n"/>
+      <c r="P30" s="72" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="70" t="n"/>
-      <c r="B31" s="70" t="n"/>
-      <c r="C31" s="70" t="n"/>
-      <c r="D31" s="70" t="n"/>
-      <c r="E31" s="71" t="n"/>
-      <c r="F31" s="71" t="n"/>
-      <c r="G31" s="71" t="n"/>
-      <c r="H31" s="70" t="n"/>
-      <c r="I31" s="70" t="n"/>
+      <c r="A31" s="69" t="n"/>
+      <c r="B31" s="69" t="n"/>
+      <c r="C31" s="69" t="n"/>
+      <c r="D31" s="69" t="n"/>
+      <c r="E31" s="70" t="n"/>
+      <c r="F31" s="70" t="n"/>
+      <c r="G31" s="70" t="n"/>
+      <c r="H31" s="69" t="n"/>
+      <c r="I31" s="69" t="n"/>
       <c r="J31" s="65">
         <f>IFERROR(DATEDIF(F31,G31,"M"),"")</f>
         <v/>
       </c>
-      <c r="K31" s="72" t="n"/>
-      <c r="L31" s="78">
+      <c r="K31" s="71" t="n"/>
+      <c r="L31" s="77">
         <f>IFERROR(IF(K31="","",K31/12),"")</f>
         <v/>
       </c>
-      <c r="M31" s="70" t="n"/>
-      <c r="N31" s="81" t="n"/>
-      <c r="O31" s="80">
+      <c r="M31" s="69" t="n"/>
+      <c r="N31" s="80" t="n"/>
+      <c r="O31" s="79">
         <f>IFERROR(IF(G31="","",G31-365),"")</f>
         <v/>
       </c>
-      <c r="P31" s="70" t="n"/>
+      <c r="P31" s="69" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="73" t="n"/>
-      <c r="B32" s="73" t="n"/>
-      <c r="C32" s="73" t="n"/>
-      <c r="D32" s="73" t="n"/>
-      <c r="E32" s="74" t="n"/>
-      <c r="F32" s="74" t="n"/>
-      <c r="G32" s="74" t="n"/>
-      <c r="H32" s="73" t="n"/>
-      <c r="I32" s="73" t="n"/>
+      <c r="A32" s="72" t="n"/>
+      <c r="B32" s="72" t="n"/>
+      <c r="C32" s="72" t="n"/>
+      <c r="D32" s="72" t="n"/>
+      <c r="E32" s="73" t="n"/>
+      <c r="F32" s="73" t="n"/>
+      <c r="G32" s="73" t="n"/>
+      <c r="H32" s="72" t="n"/>
+      <c r="I32" s="72" t="n"/>
       <c r="J32" s="65">
         <f>IFERROR(DATEDIF(F32,G32,"M"),"")</f>
         <v/>
       </c>
-      <c r="K32" s="75" t="n"/>
-      <c r="L32" s="78">
+      <c r="K32" s="74" t="n"/>
+      <c r="L32" s="77">
         <f>IFERROR(IF(K32="","",K32/12),"")</f>
         <v/>
       </c>
-      <c r="M32" s="73" t="n"/>
-      <c r="N32" s="82" t="n"/>
-      <c r="O32" s="80">
+      <c r="M32" s="72" t="n"/>
+      <c r="N32" s="81" t="n"/>
+      <c r="O32" s="79">
         <f>IFERROR(IF(G32="","",G32-365),"")</f>
         <v/>
       </c>
-      <c r="P32" s="73" t="n"/>
+      <c r="P32" s="72" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="70" t="n"/>
-      <c r="B33" s="70" t="n"/>
-      <c r="C33" s="70" t="n"/>
-      <c r="D33" s="70" t="n"/>
-      <c r="E33" s="71" t="n"/>
-      <c r="F33" s="71" t="n"/>
-      <c r="G33" s="71" t="n"/>
-      <c r="H33" s="70" t="n"/>
-      <c r="I33" s="70" t="n"/>
+      <c r="A33" s="69" t="n"/>
+      <c r="B33" s="69" t="n"/>
+      <c r="C33" s="69" t="n"/>
+      <c r="D33" s="69" t="n"/>
+      <c r="E33" s="70" t="n"/>
+      <c r="F33" s="70" t="n"/>
+      <c r="G33" s="70" t="n"/>
+      <c r="H33" s="69" t="n"/>
+      <c r="I33" s="69" t="n"/>
       <c r="J33" s="65">
         <f>IFERROR(DATEDIF(F33,G33,"M"),"")</f>
         <v/>
       </c>
-      <c r="K33" s="72" t="n"/>
-      <c r="L33" s="78">
+      <c r="K33" s="71" t="n"/>
+      <c r="L33" s="77">
         <f>IFERROR(IF(K33="","",K33/12),"")</f>
         <v/>
       </c>
-      <c r="M33" s="70" t="n"/>
-      <c r="N33" s="81" t="n"/>
-      <c r="O33" s="80">
+      <c r="M33" s="69" t="n"/>
+      <c r="N33" s="80" t="n"/>
+      <c r="O33" s="79">
         <f>IFERROR(IF(G33="","",G33-365),"")</f>
         <v/>
       </c>
-      <c r="P33" s="70" t="n"/>
+      <c r="P33" s="69" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="73" t="n"/>
-      <c r="B34" s="73" t="n"/>
-      <c r="C34" s="73" t="n"/>
-      <c r="D34" s="73" t="n"/>
-      <c r="E34" s="74" t="n"/>
-      <c r="F34" s="74" t="n"/>
-      <c r="G34" s="74" t="n"/>
-      <c r="H34" s="73" t="n"/>
-      <c r="I34" s="73" t="n"/>
+      <c r="A34" s="72" t="n"/>
+      <c r="B34" s="72" t="n"/>
+      <c r="C34" s="72" t="n"/>
+      <c r="D34" s="72" t="n"/>
+      <c r="E34" s="73" t="n"/>
+      <c r="F34" s="73" t="n"/>
+      <c r="G34" s="73" t="n"/>
+      <c r="H34" s="72" t="n"/>
+      <c r="I34" s="72" t="n"/>
       <c r="J34" s="65">
         <f>IFERROR(DATEDIF(F34,G34,"M"),"")</f>
         <v/>
       </c>
-      <c r="K34" s="75" t="n"/>
-      <c r="L34" s="78">
+      <c r="K34" s="74" t="n"/>
+      <c r="L34" s="77">
         <f>IFERROR(IF(K34="","",K34/12),"")</f>
         <v/>
       </c>
-      <c r="M34" s="73" t="n"/>
-      <c r="N34" s="82" t="n"/>
-      <c r="O34" s="80">
+      <c r="M34" s="72" t="n"/>
+      <c r="N34" s="81" t="n"/>
+      <c r="O34" s="79">
         <f>IFERROR(IF(G34="","",G34-365),"")</f>
         <v/>
       </c>
-      <c r="P34" s="73" t="n"/>
+      <c r="P34" s="72" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="70" t="n"/>
-      <c r="B35" s="70" t="n"/>
-      <c r="C35" s="70" t="n"/>
-      <c r="D35" s="70" t="n"/>
-      <c r="E35" s="71" t="n"/>
-      <c r="F35" s="71" t="n"/>
-      <c r="G35" s="71" t="n"/>
-      <c r="H35" s="70" t="n"/>
-      <c r="I35" s="70" t="n"/>
+      <c r="A35" s="69" t="n"/>
+      <c r="B35" s="69" t="n"/>
+      <c r="C35" s="69" t="n"/>
+      <c r="D35" s="69" t="n"/>
+      <c r="E35" s="70" t="n"/>
+      <c r="F35" s="70" t="n"/>
+      <c r="G35" s="70" t="n"/>
+      <c r="H35" s="69" t="n"/>
+      <c r="I35" s="69" t="n"/>
       <c r="J35" s="65">
         <f>IFERROR(DATEDIF(F35,G35,"M"),"")</f>
         <v/>
       </c>
-      <c r="K35" s="72" t="n"/>
-      <c r="L35" s="78">
+      <c r="K35" s="71" t="n"/>
+      <c r="L35" s="77">
         <f>IFERROR(IF(K35="","",K35/12),"")</f>
         <v/>
       </c>
-      <c r="M35" s="70" t="n"/>
-      <c r="N35" s="81" t="n"/>
-      <c r="O35" s="80">
+      <c r="M35" s="69" t="n"/>
+      <c r="N35" s="80" t="n"/>
+      <c r="O35" s="79">
         <f>IFERROR(IF(G35="","",G35-365),"")</f>
         <v/>
       </c>
-      <c r="P35" s="70" t="n"/>
+      <c r="P35" s="69" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="73" t="n"/>
-      <c r="B36" s="73" t="n"/>
-      <c r="C36" s="73" t="n"/>
-      <c r="D36" s="73" t="n"/>
-      <c r="E36" s="74" t="n"/>
-      <c r="F36" s="74" t="n"/>
-      <c r="G36" s="74" t="n"/>
-      <c r="H36" s="73" t="n"/>
-      <c r="I36" s="73" t="n"/>
+      <c r="A36" s="72" t="n"/>
+      <c r="B36" s="72" t="n"/>
+      <c r="C36" s="72" t="n"/>
+      <c r="D36" s="72" t="n"/>
+      <c r="E36" s="73" t="n"/>
+      <c r="F36" s="73" t="n"/>
+      <c r="G36" s="73" t="n"/>
+      <c r="H36" s="72" t="n"/>
+      <c r="I36" s="72" t="n"/>
       <c r="J36" s="65">
         <f>IFERROR(DATEDIF(F36,G36,"M"),"")</f>
         <v/>
       </c>
-      <c r="K36" s="75" t="n"/>
-      <c r="L36" s="78">
+      <c r="K36" s="74" t="n"/>
+      <c r="L36" s="77">
         <f>IFERROR(IF(K36="","",K36/12),"")</f>
         <v/>
       </c>
-      <c r="M36" s="73" t="n"/>
-      <c r="N36" s="82" t="n"/>
-      <c r="O36" s="80">
+      <c r="M36" s="72" t="n"/>
+      <c r="N36" s="81" t="n"/>
+      <c r="O36" s="79">
         <f>IFERROR(IF(G36="","",G36-365),"")</f>
         <v/>
       </c>
-      <c r="P36" s="73" t="n"/>
+      <c r="P36" s="72" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="70" t="n"/>
-      <c r="B37" s="70" t="n"/>
-      <c r="C37" s="70" t="n"/>
-      <c r="D37" s="70" t="n"/>
-      <c r="E37" s="71" t="n"/>
-      <c r="F37" s="71" t="n"/>
-      <c r="G37" s="71" t="n"/>
-      <c r="H37" s="70" t="n"/>
-      <c r="I37" s="70" t="n"/>
+      <c r="A37" s="69" t="n"/>
+      <c r="B37" s="69" t="n"/>
+      <c r="C37" s="69" t="n"/>
+      <c r="D37" s="69" t="n"/>
+      <c r="E37" s="70" t="n"/>
+      <c r="F37" s="70" t="n"/>
+      <c r="G37" s="70" t="n"/>
+      <c r="H37" s="69" t="n"/>
+      <c r="I37" s="69" t="n"/>
       <c r="J37" s="65">
         <f>IFERROR(DATEDIF(F37,G37,"M"),"")</f>
         <v/>
       </c>
-      <c r="K37" s="72" t="n"/>
-      <c r="L37" s="78">
+      <c r="K37" s="71" t="n"/>
+      <c r="L37" s="77">
         <f>IFERROR(IF(K37="","",K37/12),"")</f>
         <v/>
       </c>
-      <c r="M37" s="70" t="n"/>
-      <c r="N37" s="81" t="n"/>
-      <c r="O37" s="80">
+      <c r="M37" s="69" t="n"/>
+      <c r="N37" s="80" t="n"/>
+      <c r="O37" s="79">
         <f>IFERROR(IF(G37="","",G37-365),"")</f>
         <v/>
       </c>
-      <c r="P37" s="70" t="n"/>
+      <c r="P37" s="69" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="73" t="n"/>
-      <c r="B38" s="73" t="n"/>
-      <c r="C38" s="73" t="n"/>
-      <c r="D38" s="73" t="n"/>
-      <c r="E38" s="74" t="n"/>
-      <c r="F38" s="74" t="n"/>
-      <c r="G38" s="74" t="n"/>
-      <c r="H38" s="73" t="n"/>
-      <c r="I38" s="73" t="n"/>
+      <c r="A38" s="72" t="n"/>
+      <c r="B38" s="72" t="n"/>
+      <c r="C38" s="72" t="n"/>
+      <c r="D38" s="72" t="n"/>
+      <c r="E38" s="73" t="n"/>
+      <c r="F38" s="73" t="n"/>
+      <c r="G38" s="73" t="n"/>
+      <c r="H38" s="72" t="n"/>
+      <c r="I38" s="72" t="n"/>
       <c r="J38" s="65">
         <f>IFERROR(DATEDIF(F38,G38,"M"),"")</f>
         <v/>
       </c>
-      <c r="K38" s="75" t="n"/>
-      <c r="L38" s="78">
+      <c r="K38" s="74" t="n"/>
+      <c r="L38" s="77">
         <f>IFERROR(IF(K38="","",K38/12),"")</f>
         <v/>
       </c>
-      <c r="M38" s="73" t="n"/>
-      <c r="N38" s="82" t="n"/>
-      <c r="O38" s="80">
+      <c r="M38" s="72" t="n"/>
+      <c r="N38" s="81" t="n"/>
+      <c r="O38" s="79">
         <f>IFERROR(IF(G38="","",G38-365),"")</f>
         <v/>
       </c>
-      <c r="P38" s="73" t="n"/>
+      <c r="P38" s="72" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="70" t="n"/>
-      <c r="B39" s="70" t="n"/>
-      <c r="C39" s="70" t="n"/>
-      <c r="D39" s="70" t="n"/>
-      <c r="E39" s="71" t="n"/>
-      <c r="F39" s="71" t="n"/>
-      <c r="G39" s="71" t="n"/>
-      <c r="H39" s="70" t="n"/>
-      <c r="I39" s="70" t="n"/>
+      <c r="A39" s="69" t="n"/>
+      <c r="B39" s="69" t="n"/>
+      <c r="C39" s="69" t="n"/>
+      <c r="D39" s="69" t="n"/>
+      <c r="E39" s="70" t="n"/>
+      <c r="F39" s="70" t="n"/>
+      <c r="G39" s="70" t="n"/>
+      <c r="H39" s="69" t="n"/>
+      <c r="I39" s="69" t="n"/>
       <c r="J39" s="65">
         <f>IFERROR(DATEDIF(F39,G39,"M"),"")</f>
         <v/>
       </c>
-      <c r="K39" s="72" t="n"/>
-      <c r="L39" s="78">
+      <c r="K39" s="71" t="n"/>
+      <c r="L39" s="77">
         <f>IFERROR(IF(K39="","",K39/12),"")</f>
         <v/>
       </c>
-      <c r="M39" s="70" t="n"/>
-      <c r="N39" s="81" t="n"/>
-      <c r="O39" s="80">
+      <c r="M39" s="69" t="n"/>
+      <c r="N39" s="80" t="n"/>
+      <c r="O39" s="79">
         <f>IFERROR(IF(G39="","",G39-365),"")</f>
         <v/>
       </c>
-      <c r="P39" s="70" t="n"/>
+      <c r="P39" s="69" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="73" t="n"/>
-      <c r="B40" s="73" t="n"/>
-      <c r="C40" s="73" t="n"/>
-      <c r="D40" s="73" t="n"/>
-      <c r="E40" s="74" t="n"/>
-      <c r="F40" s="74" t="n"/>
-      <c r="G40" s="74" t="n"/>
-      <c r="H40" s="73" t="n"/>
-      <c r="I40" s="73" t="n"/>
+      <c r="A40" s="72" t="n"/>
+      <c r="B40" s="72" t="n"/>
+      <c r="C40" s="72" t="n"/>
+      <c r="D40" s="72" t="n"/>
+      <c r="E40" s="73" t="n"/>
+      <c r="F40" s="73" t="n"/>
+      <c r="G40" s="73" t="n"/>
+      <c r="H40" s="72" t="n"/>
+      <c r="I40" s="72" t="n"/>
       <c r="J40" s="65">
         <f>IFERROR(DATEDIF(F40,G40,"M"),"")</f>
         <v/>
       </c>
-      <c r="K40" s="75" t="n"/>
-      <c r="L40" s="78">
+      <c r="K40" s="74" t="n"/>
+      <c r="L40" s="77">
         <f>IFERROR(IF(K40="","",K40/12),"")</f>
         <v/>
       </c>
-      <c r="M40" s="73" t="n"/>
-      <c r="N40" s="82" t="n"/>
-      <c r="O40" s="80">
+      <c r="M40" s="72" t="n"/>
+      <c r="N40" s="81" t="n"/>
+      <c r="O40" s="79">
         <f>IFERROR(IF(G40="","",G40-365),"")</f>
         <v/>
       </c>
-      <c r="P40" s="73" t="n"/>
+      <c r="P40" s="72" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="70" t="n"/>
-      <c r="B41" s="70" t="n"/>
-      <c r="C41" s="70" t="n"/>
-      <c r="D41" s="70" t="n"/>
-      <c r="E41" s="71" t="n"/>
-      <c r="F41" s="71" t="n"/>
-      <c r="G41" s="71" t="n"/>
-      <c r="H41" s="70" t="n"/>
-      <c r="I41" s="70" t="n"/>
+      <c r="A41" s="69" t="n"/>
+      <c r="B41" s="69" t="n"/>
+      <c r="C41" s="69" t="n"/>
+      <c r="D41" s="69" t="n"/>
+      <c r="E41" s="70" t="n"/>
+      <c r="F41" s="70" t="n"/>
+      <c r="G41" s="70" t="n"/>
+      <c r="H41" s="69" t="n"/>
+      <c r="I41" s="69" t="n"/>
       <c r="J41" s="65">
         <f>IFERROR(DATEDIF(F41,G41,"M"),"")</f>
         <v/>
       </c>
-      <c r="K41" s="72" t="n"/>
-      <c r="L41" s="78">
+      <c r="K41" s="71" t="n"/>
+      <c r="L41" s="77">
         <f>IFERROR(IF(K41="","",K41/12),"")</f>
         <v/>
       </c>
-      <c r="M41" s="70" t="n"/>
-      <c r="N41" s="81" t="n"/>
-      <c r="O41" s="80">
+      <c r="M41" s="69" t="n"/>
+      <c r="N41" s="80" t="n"/>
+      <c r="O41" s="79">
         <f>IFERROR(IF(G41="","",G41-365),"")</f>
         <v/>
       </c>
-      <c r="P41" s="70" t="n"/>
+      <c r="P41" s="69" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="73" t="n"/>
-      <c r="B42" s="73" t="n"/>
-      <c r="C42" s="73" t="n"/>
-      <c r="D42" s="73" t="n"/>
-      <c r="E42" s="74" t="n"/>
-      <c r="F42" s="74" t="n"/>
-      <c r="G42" s="74" t="n"/>
-      <c r="H42" s="73" t="n"/>
-      <c r="I42" s="73" t="n"/>
+      <c r="A42" s="72" t="n"/>
+      <c r="B42" s="72" t="n"/>
+      <c r="C42" s="72" t="n"/>
+      <c r="D42" s="72" t="n"/>
+      <c r="E42" s="73" t="n"/>
+      <c r="F42" s="73" t="n"/>
+      <c r="G42" s="73" t="n"/>
+      <c r="H42" s="72" t="n"/>
+      <c r="I42" s="72" t="n"/>
       <c r="J42" s="65">
         <f>IFERROR(DATEDIF(F42,G42,"M"),"")</f>
         <v/>
       </c>
-      <c r="K42" s="75" t="n"/>
-      <c r="L42" s="78">
+      <c r="K42" s="74" t="n"/>
+      <c r="L42" s="77">
         <f>IFERROR(IF(K42="","",K42/12),"")</f>
         <v/>
       </c>
-      <c r="M42" s="73" t="n"/>
-      <c r="N42" s="82" t="n"/>
-      <c r="O42" s="80">
+      <c r="M42" s="72" t="n"/>
+      <c r="N42" s="81" t="n"/>
+      <c r="O42" s="79">
         <f>IFERROR(IF(G42="","",G42-365),"")</f>
         <v/>
       </c>
-      <c r="P42" s="73" t="n"/>
+      <c r="P42" s="72" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="70" t="n"/>
-      <c r="B43" s="70" t="n"/>
-      <c r="C43" s="70" t="n"/>
-      <c r="D43" s="70" t="n"/>
-      <c r="E43" s="71" t="n"/>
-      <c r="F43" s="71" t="n"/>
-      <c r="G43" s="71" t="n"/>
-      <c r="H43" s="70" t="n"/>
-      <c r="I43" s="70" t="n"/>
+      <c r="A43" s="69" t="n"/>
+      <c r="B43" s="69" t="n"/>
+      <c r="C43" s="69" t="n"/>
+      <c r="D43" s="69" t="n"/>
+      <c r="E43" s="70" t="n"/>
+      <c r="F43" s="70" t="n"/>
+      <c r="G43" s="70" t="n"/>
+      <c r="H43" s="69" t="n"/>
+      <c r="I43" s="69" t="n"/>
       <c r="J43" s="65">
         <f>IFERROR(DATEDIF(F43,G43,"M"),"")</f>
         <v/>
       </c>
-      <c r="K43" s="72" t="n"/>
-      <c r="L43" s="78">
+      <c r="K43" s="71" t="n"/>
+      <c r="L43" s="77">
         <f>IFERROR(IF(K43="","",K43/12),"")</f>
         <v/>
       </c>
-      <c r="M43" s="70" t="n"/>
-      <c r="N43" s="81" t="n"/>
-      <c r="O43" s="80">
+      <c r="M43" s="69" t="n"/>
+      <c r="N43" s="80" t="n"/>
+      <c r="O43" s="79">
         <f>IFERROR(IF(G43="","",G43-365),"")</f>
         <v/>
       </c>
-      <c r="P43" s="70" t="n"/>
+      <c r="P43" s="69" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="73" t="n"/>
-      <c r="B44" s="73" t="n"/>
-      <c r="C44" s="73" t="n"/>
-      <c r="D44" s="73" t="n"/>
-      <c r="E44" s="74" t="n"/>
-      <c r="F44" s="74" t="n"/>
-      <c r="G44" s="74" t="n"/>
-      <c r="H44" s="73" t="n"/>
-      <c r="I44" s="73" t="n"/>
+      <c r="A44" s="72" t="n"/>
+      <c r="B44" s="72" t="n"/>
+      <c r="C44" s="72" t="n"/>
+      <c r="D44" s="72" t="n"/>
+      <c r="E44" s="73" t="n"/>
+      <c r="F44" s="73" t="n"/>
+      <c r="G44" s="73" t="n"/>
+      <c r="H44" s="72" t="n"/>
+      <c r="I44" s="72" t="n"/>
       <c r="J44" s="65">
         <f>IFERROR(DATEDIF(F44,G44,"M"),"")</f>
         <v/>
       </c>
-      <c r="K44" s="75" t="n"/>
-      <c r="L44" s="78">
+      <c r="K44" s="74" t="n"/>
+      <c r="L44" s="77">
         <f>IFERROR(IF(K44="","",K44/12),"")</f>
         <v/>
       </c>
-      <c r="M44" s="73" t="n"/>
-      <c r="N44" s="82" t="n"/>
-      <c r="O44" s="80">
+      <c r="M44" s="72" t="n"/>
+      <c r="N44" s="81" t="n"/>
+      <c r="O44" s="79">
         <f>IFERROR(IF(G44="","",G44-365),"")</f>
         <v/>
       </c>
-      <c r="P44" s="73" t="n"/>
+      <c r="P44" s="72" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="70" t="n"/>
-      <c r="B45" s="70" t="n"/>
-      <c r="C45" s="70" t="n"/>
-      <c r="D45" s="70" t="n"/>
-      <c r="E45" s="71" t="n"/>
-      <c r="F45" s="71" t="n"/>
-      <c r="G45" s="71" t="n"/>
-      <c r="H45" s="70" t="n"/>
-      <c r="I45" s="70" t="n"/>
+      <c r="A45" s="69" t="n"/>
+      <c r="B45" s="69" t="n"/>
+      <c r="C45" s="69" t="n"/>
+      <c r="D45" s="69" t="n"/>
+      <c r="E45" s="70" t="n"/>
+      <c r="F45" s="70" t="n"/>
+      <c r="G45" s="70" t="n"/>
+      <c r="H45" s="69" t="n"/>
+      <c r="I45" s="69" t="n"/>
       <c r="J45" s="65">
         <f>IFERROR(DATEDIF(F45,G45,"M"),"")</f>
         <v/>
       </c>
-      <c r="K45" s="72" t="n"/>
-      <c r="L45" s="78">
+      <c r="K45" s="71" t="n"/>
+      <c r="L45" s="77">
         <f>IFERROR(IF(K45="","",K45/12),"")</f>
         <v/>
       </c>
-      <c r="M45" s="70" t="n"/>
-      <c r="N45" s="81" t="n"/>
-      <c r="O45" s="80">
+      <c r="M45" s="69" t="n"/>
+      <c r="N45" s="80" t="n"/>
+      <c r="O45" s="79">
         <f>IFERROR(IF(G45="","",G45-365),"")</f>
         <v/>
       </c>
-      <c r="P45" s="70" t="n"/>
+      <c r="P45" s="69" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="73" t="n"/>
-      <c r="B46" s="73" t="n"/>
-      <c r="C46" s="73" t="n"/>
-      <c r="D46" s="73" t="n"/>
-      <c r="E46" s="74" t="n"/>
-      <c r="F46" s="74" t="n"/>
-      <c r="G46" s="74" t="n"/>
-      <c r="H46" s="73" t="n"/>
-      <c r="I46" s="73" t="n"/>
+      <c r="A46" s="72" t="n"/>
+      <c r="B46" s="72" t="n"/>
+      <c r="C46" s="72" t="n"/>
+      <c r="D46" s="72" t="n"/>
+      <c r="E46" s="73" t="n"/>
+      <c r="F46" s="73" t="n"/>
+      <c r="G46" s="73" t="n"/>
+      <c r="H46" s="72" t="n"/>
+      <c r="I46" s="72" t="n"/>
       <c r="J46" s="65">
         <f>IFERROR(DATEDIF(F46,G46,"M"),"")</f>
         <v/>
       </c>
-      <c r="K46" s="75" t="n"/>
-      <c r="L46" s="78">
+      <c r="K46" s="74" t="n"/>
+      <c r="L46" s="77">
         <f>IFERROR(IF(K46="","",K46/12),"")</f>
         <v/>
       </c>
-      <c r="M46" s="73" t="n"/>
-      <c r="N46" s="82" t="n"/>
-      <c r="O46" s="80">
+      <c r="M46" s="72" t="n"/>
+      <c r="N46" s="81" t="n"/>
+      <c r="O46" s="79">
         <f>IFERROR(IF(G46="","",G46-365),"")</f>
         <v/>
       </c>
-      <c r="P46" s="73" t="n"/>
+      <c r="P46" s="72" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="70" t="n"/>
-      <c r="B47" s="70" t="n"/>
-      <c r="C47" s="70" t="n"/>
-      <c r="D47" s="70" t="n"/>
-      <c r="E47" s="71" t="n"/>
-      <c r="F47" s="71" t="n"/>
-      <c r="G47" s="71" t="n"/>
-      <c r="H47" s="70" t="n"/>
-      <c r="I47" s="70" t="n"/>
+      <c r="A47" s="69" t="n"/>
+      <c r="B47" s="69" t="n"/>
+      <c r="C47" s="69" t="n"/>
+      <c r="D47" s="69" t="n"/>
+      <c r="E47" s="70" t="n"/>
+      <c r="F47" s="70" t="n"/>
+      <c r="G47" s="70" t="n"/>
+      <c r="H47" s="69" t="n"/>
+      <c r="I47" s="69" t="n"/>
       <c r="J47" s="65">
         <f>IFERROR(DATEDIF(F47,G47,"M"),"")</f>
         <v/>
       </c>
-      <c r="K47" s="72" t="n"/>
-      <c r="L47" s="78">
+      <c r="K47" s="71" t="n"/>
+      <c r="L47" s="77">
         <f>IFERROR(IF(K47="","",K47/12),"")</f>
         <v/>
       </c>
-      <c r="M47" s="70" t="n"/>
-      <c r="N47" s="81" t="n"/>
-      <c r="O47" s="80">
+      <c r="M47" s="69" t="n"/>
+      <c r="N47" s="80" t="n"/>
+      <c r="O47" s="79">
         <f>IFERROR(IF(G47="","",G47-365),"")</f>
         <v/>
       </c>
-      <c r="P47" s="70" t="n"/>
+      <c r="P47" s="69" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="73" t="n"/>
-      <c r="B48" s="73" t="n"/>
-      <c r="C48" s="73" t="n"/>
-      <c r="D48" s="73" t="n"/>
-      <c r="E48" s="74" t="n"/>
-      <c r="F48" s="74" t="n"/>
-      <c r="G48" s="74" t="n"/>
-      <c r="H48" s="73" t="n"/>
-      <c r="I48" s="73" t="n"/>
+      <c r="A48" s="72" t="n"/>
+      <c r="B48" s="72" t="n"/>
+      <c r="C48" s="72" t="n"/>
+      <c r="D48" s="72" t="n"/>
+      <c r="E48" s="73" t="n"/>
+      <c r="F48" s="73" t="n"/>
+      <c r="G48" s="73" t="n"/>
+      <c r="H48" s="72" t="n"/>
+      <c r="I48" s="72" t="n"/>
       <c r="J48" s="65">
         <f>IFERROR(DATEDIF(F48,G48,"M"),"")</f>
         <v/>
       </c>
-      <c r="K48" s="75" t="n"/>
-      <c r="L48" s="78">
+      <c r="K48" s="74" t="n"/>
+      <c r="L48" s="77">
         <f>IFERROR(IF(K48="","",K48/12),"")</f>
         <v/>
       </c>
-      <c r="M48" s="73" t="n"/>
-      <c r="N48" s="82" t="n"/>
-      <c r="O48" s="80">
+      <c r="M48" s="72" t="n"/>
+      <c r="N48" s="81" t="n"/>
+      <c r="O48" s="79">
         <f>IFERROR(IF(G48="","",G48-365),"")</f>
         <v/>
       </c>
-      <c r="P48" s="73" t="n"/>
+      <c r="P48" s="72" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="70" t="n"/>
-      <c r="B49" s="70" t="n"/>
-      <c r="C49" s="70" t="n"/>
-      <c r="D49" s="70" t="n"/>
-      <c r="E49" s="71" t="n"/>
-      <c r="F49" s="71" t="n"/>
-      <c r="G49" s="71" t="n"/>
-      <c r="H49" s="70" t="n"/>
-      <c r="I49" s="70" t="n"/>
+      <c r="A49" s="69" t="n"/>
+      <c r="B49" s="69" t="n"/>
+      <c r="C49" s="69" t="n"/>
+      <c r="D49" s="69" t="n"/>
+      <c r="E49" s="70" t="n"/>
+      <c r="F49" s="70" t="n"/>
+      <c r="G49" s="70" t="n"/>
+      <c r="H49" s="69" t="n"/>
+      <c r="I49" s="69" t="n"/>
       <c r="J49" s="65">
         <f>IFERROR(DATEDIF(F49,G49,"M"),"")</f>
         <v/>
       </c>
-      <c r="K49" s="72" t="n"/>
-      <c r="L49" s="78">
+      <c r="K49" s="71" t="n"/>
+      <c r="L49" s="77">
         <f>IFERROR(IF(K49="","",K49/12),"")</f>
         <v/>
       </c>
-      <c r="M49" s="70" t="n"/>
-      <c r="N49" s="81" t="n"/>
-      <c r="O49" s="80">
+      <c r="M49" s="69" t="n"/>
+      <c r="N49" s="80" t="n"/>
+      <c r="O49" s="79">
         <f>IFERROR(IF(G49="","",G49-365),"")</f>
         <v/>
       </c>
-      <c r="P49" s="70" t="n"/>
+      <c r="P49" s="69" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="73" t="n"/>
-      <c r="B50" s="73" t="n"/>
-      <c r="C50" s="73" t="n"/>
-      <c r="D50" s="73" t="n"/>
-      <c r="E50" s="74" t="n"/>
-      <c r="F50" s="74" t="n"/>
-      <c r="G50" s="74" t="n"/>
-      <c r="H50" s="73" t="n"/>
-      <c r="I50" s="73" t="n"/>
+      <c r="A50" s="72" t="n"/>
+      <c r="B50" s="72" t="n"/>
+      <c r="C50" s="72" t="n"/>
+      <c r="D50" s="72" t="n"/>
+      <c r="E50" s="73" t="n"/>
+      <c r="F50" s="73" t="n"/>
+      <c r="G50" s="73" t="n"/>
+      <c r="H50" s="72" t="n"/>
+      <c r="I50" s="72" t="n"/>
       <c r="J50" s="65">
         <f>IFERROR(DATEDIF(F50,G50,"M"),"")</f>
         <v/>
       </c>
-      <c r="K50" s="75" t="n"/>
-      <c r="L50" s="78">
+      <c r="K50" s="74" t="n"/>
+      <c r="L50" s="77">
         <f>IFERROR(IF(K50="","",K50/12),"")</f>
         <v/>
       </c>
-      <c r="M50" s="73" t="n"/>
-      <c r="N50" s="82" t="n"/>
-      <c r="O50" s="80">
+      <c r="M50" s="72" t="n"/>
+      <c r="N50" s="81" t="n"/>
+      <c r="O50" s="79">
         <f>IFERROR(IF(G50="","",G50-365),"")</f>
         <v/>
       </c>
-      <c r="P50" s="73" t="n"/>
+      <c r="P50" s="72" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="70" t="n"/>
-      <c r="B51" s="70" t="n"/>
-      <c r="C51" s="70" t="n"/>
-      <c r="D51" s="70" t="n"/>
-      <c r="E51" s="71" t="n"/>
-      <c r="F51" s="71" t="n"/>
-      <c r="G51" s="71" t="n"/>
-      <c r="H51" s="70" t="n"/>
-      <c r="I51" s="70" t="n"/>
+      <c r="A51" s="69" t="n"/>
+      <c r="B51" s="69" t="n"/>
+      <c r="C51" s="69" t="n"/>
+      <c r="D51" s="69" t="n"/>
+      <c r="E51" s="70" t="n"/>
+      <c r="F51" s="70" t="n"/>
+      <c r="G51" s="70" t="n"/>
+      <c r="H51" s="69" t="n"/>
+      <c r="I51" s="69" t="n"/>
       <c r="J51" s="65">
         <f>IFERROR(DATEDIF(F51,G51,"M"),"")</f>
         <v/>
       </c>
-      <c r="K51" s="72" t="n"/>
-      <c r="L51" s="78">
+      <c r="K51" s="71" t="n"/>
+      <c r="L51" s="77">
         <f>IFERROR(IF(K51="","",K51/12),"")</f>
         <v/>
       </c>
-      <c r="M51" s="70" t="n"/>
-      <c r="N51" s="81" t="n"/>
-      <c r="O51" s="80">
+      <c r="M51" s="69" t="n"/>
+      <c r="N51" s="80" t="n"/>
+      <c r="O51" s="79">
         <f>IFERROR(IF(G51="","",G51-365),"")</f>
         <v/>
       </c>
-      <c r="P51" s="70" t="n"/>
+      <c r="P51" s="69" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="73" t="n"/>
-      <c r="B52" s="73" t="n"/>
-      <c r="C52" s="73" t="n"/>
-      <c r="D52" s="73" t="n"/>
-      <c r="E52" s="74" t="n"/>
-      <c r="F52" s="74" t="n"/>
-      <c r="G52" s="74" t="n"/>
-      <c r="H52" s="73" t="n"/>
-      <c r="I52" s="73" t="n"/>
+      <c r="A52" s="72" t="n"/>
+      <c r="B52" s="72" t="n"/>
+      <c r="C52" s="72" t="n"/>
+      <c r="D52" s="72" t="n"/>
+      <c r="E52" s="73" t="n"/>
+      <c r="F52" s="73" t="n"/>
+      <c r="G52" s="73" t="n"/>
+      <c r="H52" s="72" t="n"/>
+      <c r="I52" s="72" t="n"/>
       <c r="J52" s="65">
         <f>IFERROR(DATEDIF(F52,G52,"M"),"")</f>
         <v/>
       </c>
-      <c r="K52" s="75" t="n"/>
-      <c r="L52" s="78">
+      <c r="K52" s="74" t="n"/>
+      <c r="L52" s="77">
         <f>IFERROR(IF(K52="","",K52/12),"")</f>
         <v/>
       </c>
-      <c r="M52" s="73" t="n"/>
-      <c r="N52" s="82" t="n"/>
-      <c r="O52" s="80">
+      <c r="M52" s="72" t="n"/>
+      <c r="N52" s="81" t="n"/>
+      <c r="O52" s="79">
         <f>IFERROR(IF(G52="","",G52-365),"")</f>
         <v/>
       </c>
-      <c r="P52" s="73" t="n"/>
+      <c r="P52" s="72" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="70" t="n"/>
-      <c r="B53" s="70" t="n"/>
-      <c r="C53" s="70" t="n"/>
-      <c r="D53" s="70" t="n"/>
-      <c r="E53" s="71" t="n"/>
-      <c r="F53" s="71" t="n"/>
-      <c r="G53" s="71" t="n"/>
-      <c r="H53" s="70" t="n"/>
-      <c r="I53" s="70" t="n"/>
+      <c r="A53" s="69" t="n"/>
+      <c r="B53" s="69" t="n"/>
+      <c r="C53" s="69" t="n"/>
+      <c r="D53" s="69" t="n"/>
+      <c r="E53" s="70" t="n"/>
+      <c r="F53" s="70" t="n"/>
+      <c r="G53" s="70" t="n"/>
+      <c r="H53" s="69" t="n"/>
+      <c r="I53" s="69" t="n"/>
       <c r="J53" s="65">
         <f>IFERROR(DATEDIF(F53,G53,"M"),"")</f>
         <v/>
       </c>
-      <c r="K53" s="72" t="n"/>
-      <c r="L53" s="78">
+      <c r="K53" s="71" t="n"/>
+      <c r="L53" s="77">
         <f>IFERROR(IF(K53="","",K53/12),"")</f>
         <v/>
       </c>
-      <c r="M53" s="70" t="n"/>
-      <c r="N53" s="81" t="n"/>
-      <c r="O53" s="80">
+      <c r="M53" s="69" t="n"/>
+      <c r="N53" s="80" t="n"/>
+      <c r="O53" s="79">
         <f>IFERROR(IF(G53="","",G53-365),"")</f>
         <v/>
       </c>
-      <c r="P53" s="70" t="n"/>
+      <c r="P53" s="69" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Added Previous Agreement Ref to AGREEMENTS
</commit_message>
<xml_diff>
--- a/Tenant_Manager.xlsx
+++ b/Tenant_Manager.xlsx
@@ -4233,7 +4233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P53"/>
+  <dimension ref="A1:Q53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4245,13 +4245,14 @@
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="28" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="28" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -4316,35 +4317,40 @@
       </c>
       <c r="J3" s="76" t="inlineStr">
         <is>
+          <t>Previous Agr. Ref</t>
+        </is>
+      </c>
+      <c r="K3" s="76" t="inlineStr">
+        <is>
           <t>Term (months)</t>
         </is>
       </c>
-      <c r="K3" s="76" t="inlineStr">
+      <c r="L3" s="76" t="inlineStr">
         <is>
           <t>Annual Rent</t>
         </is>
       </c>
-      <c r="L3" s="76" t="inlineStr">
+      <c r="M3" s="76" t="inlineStr">
         <is>
           <t>Monthly Rent</t>
         </is>
       </c>
-      <c r="M3" s="76" t="inlineStr">
+      <c r="N3" s="76" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="N3" s="76" t="inlineStr">
+      <c r="O3" s="76" t="inlineStr">
         <is>
           <t>Rent Increment%</t>
         </is>
       </c>
-      <c r="O3" s="76" t="inlineStr">
+      <c r="P3" s="76" t="inlineStr">
         <is>
           <t>Next Review Date</t>
         </is>
       </c>
-      <c r="P3" s="76" t="inlineStr">
+      <c r="Q3" s="76" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -4412,6 +4418,7 @@
         <v/>
       </c>
       <c r="P4" s="63" t="n"/>
+      <c r="Q4" s="63" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="69" t="n"/>
@@ -4439,6 +4446,7 @@
         <v/>
       </c>
       <c r="P5" s="69" t="n"/>
+      <c r="Q5" s="69" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="72" t="n"/>
@@ -4466,6 +4474,7 @@
         <v/>
       </c>
       <c r="P6" s="72" t="n"/>
+      <c r="Q6" s="72" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="69" t="n"/>
@@ -4493,6 +4502,7 @@
         <v/>
       </c>
       <c r="P7" s="69" t="n"/>
+      <c r="Q7" s="69" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="72" t="n"/>
@@ -4520,6 +4530,7 @@
         <v/>
       </c>
       <c r="P8" s="72" t="n"/>
+      <c r="Q8" s="72" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="69" t="n"/>
@@ -4547,6 +4558,7 @@
         <v/>
       </c>
       <c r="P9" s="69" t="n"/>
+      <c r="Q9" s="69" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="72" t="n"/>
@@ -4574,6 +4586,7 @@
         <v/>
       </c>
       <c r="P10" s="72" t="n"/>
+      <c r="Q10" s="72" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="69" t="n"/>
@@ -4601,6 +4614,7 @@
         <v/>
       </c>
       <c r="P11" s="69" t="n"/>
+      <c r="Q11" s="69" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="72" t="n"/>
@@ -4628,6 +4642,7 @@
         <v/>
       </c>
       <c r="P12" s="72" t="n"/>
+      <c r="Q12" s="72" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="69" t="n"/>
@@ -4655,6 +4670,7 @@
         <v/>
       </c>
       <c r="P13" s="69" t="n"/>
+      <c r="Q13" s="69" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="72" t="n"/>
@@ -4682,6 +4698,7 @@
         <v/>
       </c>
       <c r="P14" s="72" t="n"/>
+      <c r="Q14" s="72" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="69" t="n"/>
@@ -4709,6 +4726,7 @@
         <v/>
       </c>
       <c r="P15" s="69" t="n"/>
+      <c r="Q15" s="69" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="72" t="n"/>
@@ -4736,6 +4754,7 @@
         <v/>
       </c>
       <c r="P16" s="72" t="n"/>
+      <c r="Q16" s="72" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="69" t="n"/>
@@ -4763,6 +4782,7 @@
         <v/>
       </c>
       <c r="P17" s="69" t="n"/>
+      <c r="Q17" s="69" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="72" t="n"/>
@@ -4790,6 +4810,7 @@
         <v/>
       </c>
       <c r="P18" s="72" t="n"/>
+      <c r="Q18" s="72" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="69" t="n"/>
@@ -4817,6 +4838,7 @@
         <v/>
       </c>
       <c r="P19" s="69" t="n"/>
+      <c r="Q19" s="69" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="72" t="n"/>
@@ -4844,6 +4866,7 @@
         <v/>
       </c>
       <c r="P20" s="72" t="n"/>
+      <c r="Q20" s="72" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="69" t="n"/>
@@ -4871,6 +4894,7 @@
         <v/>
       </c>
       <c r="P21" s="69" t="n"/>
+      <c r="Q21" s="69" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="72" t="n"/>
@@ -4898,6 +4922,7 @@
         <v/>
       </c>
       <c r="P22" s="72" t="n"/>
+      <c r="Q22" s="72" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="69" t="n"/>
@@ -4925,6 +4950,7 @@
         <v/>
       </c>
       <c r="P23" s="69" t="n"/>
+      <c r="Q23" s="69" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="72" t="n"/>
@@ -4952,6 +4978,7 @@
         <v/>
       </c>
       <c r="P24" s="72" t="n"/>
+      <c r="Q24" s="72" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="69" t="n"/>
@@ -4979,6 +5006,7 @@
         <v/>
       </c>
       <c r="P25" s="69" t="n"/>
+      <c r="Q25" s="69" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="72" t="n"/>
@@ -5006,6 +5034,7 @@
         <v/>
       </c>
       <c r="P26" s="72" t="n"/>
+      <c r="Q26" s="72" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="69" t="n"/>
@@ -5033,6 +5062,7 @@
         <v/>
       </c>
       <c r="P27" s="69" t="n"/>
+      <c r="Q27" s="69" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="72" t="n"/>
@@ -5060,6 +5090,7 @@
         <v/>
       </c>
       <c r="P28" s="72" t="n"/>
+      <c r="Q28" s="72" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="69" t="n"/>
@@ -5087,6 +5118,7 @@
         <v/>
       </c>
       <c r="P29" s="69" t="n"/>
+      <c r="Q29" s="69" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="72" t="n"/>
@@ -5114,6 +5146,7 @@
         <v/>
       </c>
       <c r="P30" s="72" t="n"/>
+      <c r="Q30" s="72" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="69" t="n"/>
@@ -5141,6 +5174,7 @@
         <v/>
       </c>
       <c r="P31" s="69" t="n"/>
+      <c r="Q31" s="69" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="72" t="n"/>
@@ -5168,6 +5202,7 @@
         <v/>
       </c>
       <c r="P32" s="72" t="n"/>
+      <c r="Q32" s="72" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="69" t="n"/>
@@ -5195,6 +5230,7 @@
         <v/>
       </c>
       <c r="P33" s="69" t="n"/>
+      <c r="Q33" s="69" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="72" t="n"/>
@@ -5222,6 +5258,7 @@
         <v/>
       </c>
       <c r="P34" s="72" t="n"/>
+      <c r="Q34" s="72" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="69" t="n"/>
@@ -5249,6 +5286,7 @@
         <v/>
       </c>
       <c r="P35" s="69" t="n"/>
+      <c r="Q35" s="69" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="72" t="n"/>
@@ -5276,6 +5314,7 @@
         <v/>
       </c>
       <c r="P36" s="72" t="n"/>
+      <c r="Q36" s="72" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="69" t="n"/>
@@ -5303,6 +5342,7 @@
         <v/>
       </c>
       <c r="P37" s="69" t="n"/>
+      <c r="Q37" s="69" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="72" t="n"/>
@@ -5330,6 +5370,7 @@
         <v/>
       </c>
       <c r="P38" s="72" t="n"/>
+      <c r="Q38" s="72" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="69" t="n"/>
@@ -5357,6 +5398,7 @@
         <v/>
       </c>
       <c r="P39" s="69" t="n"/>
+      <c r="Q39" s="69" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="72" t="n"/>
@@ -5384,6 +5426,7 @@
         <v/>
       </c>
       <c r="P40" s="72" t="n"/>
+      <c r="Q40" s="72" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="69" t="n"/>
@@ -5411,6 +5454,7 @@
         <v/>
       </c>
       <c r="P41" s="69" t="n"/>
+      <c r="Q41" s="69" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="72" t="n"/>
@@ -5438,6 +5482,7 @@
         <v/>
       </c>
       <c r="P42" s="72" t="n"/>
+      <c r="Q42" s="72" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="69" t="n"/>
@@ -5465,6 +5510,7 @@
         <v/>
       </c>
       <c r="P43" s="69" t="n"/>
+      <c r="Q43" s="69" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="72" t="n"/>
@@ -5492,6 +5538,7 @@
         <v/>
       </c>
       <c r="P44" s="72" t="n"/>
+      <c r="Q44" s="72" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="69" t="n"/>
@@ -5519,6 +5566,7 @@
         <v/>
       </c>
       <c r="P45" s="69" t="n"/>
+      <c r="Q45" s="69" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="72" t="n"/>
@@ -5546,6 +5594,7 @@
         <v/>
       </c>
       <c r="P46" s="72" t="n"/>
+      <c r="Q46" s="72" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="69" t="n"/>
@@ -5573,6 +5622,7 @@
         <v/>
       </c>
       <c r="P47" s="69" t="n"/>
+      <c r="Q47" s="69" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="72" t="n"/>
@@ -5600,6 +5650,7 @@
         <v/>
       </c>
       <c r="P48" s="72" t="n"/>
+      <c r="Q48" s="72" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="69" t="n"/>
@@ -5627,6 +5678,7 @@
         <v/>
       </c>
       <c r="P49" s="69" t="n"/>
+      <c r="Q49" s="69" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="72" t="n"/>
@@ -5654,6 +5706,7 @@
         <v/>
       </c>
       <c r="P50" s="72" t="n"/>
+      <c r="Q50" s="72" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="69" t="n"/>
@@ -5681,6 +5734,7 @@
         <v/>
       </c>
       <c r="P51" s="69" t="n"/>
+      <c r="Q51" s="69" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="72" t="n"/>
@@ -5708,6 +5762,7 @@
         <v/>
       </c>
       <c r="P52" s="72" t="n"/>
+      <c r="Q52" s="72" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="69" t="n"/>
@@ -5735,11 +5790,12 @@
         <v/>
       </c>
       <c r="P53" s="69" t="n"/>
+      <c r="Q53" s="69" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <conditionalFormatting sqref="H4:H53">
     <cfRule type="expression" priority="1" dxfId="3">

</xml_diff>

<commit_message>
Completed emergency contacts and agreement renewal tracking
</commit_message>
<xml_diff>
--- a/Tenant_Manager.xlsx
+++ b/Tenant_Manager.xlsx
@@ -4394,30 +4394,30 @@
       <c r="I4" s="63" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="65">
+      <c r="J4" s="63" t="inlineStr"/>
+      <c r="K4" s="65">
         <f>IFERROR(DATEDIF(F4,G4,"M"),"")</f>
         <v/>
       </c>
-      <c r="K4" s="66" t="n">
+      <c r="L4" s="66" t="n">
         <v>42000</v>
       </c>
-      <c r="L4" s="77">
-        <f>IFERROR(IF(K4="","",K4/12),"")</f>
-        <v/>
-      </c>
-      <c r="M4" s="63" t="inlineStr">
+      <c r="M4" s="77">
+        <f>IFERROR(IF(L4="","",L4/12),"")</f>
+        <v/>
+      </c>
+      <c r="N4" s="63" t="inlineStr">
         <is>
           <t>GHS</t>
         </is>
       </c>
-      <c r="N4" s="78" t="n">
+      <c r="O4" s="78" t="n">
         <v>0.05</v>
       </c>
-      <c r="O4" s="79">
+      <c r="P4" s="79">
         <f>IFERROR(IF(G4="","",G4-365),"")</f>
         <v/>
       </c>
-      <c r="P4" s="63" t="n"/>
       <c r="Q4" s="63" t="n"/>
     </row>
     <row r="5">
@@ -4430,22 +4430,22 @@
       <c r="G5" s="70" t="n"/>
       <c r="H5" s="69" t="n"/>
       <c r="I5" s="69" t="n"/>
-      <c r="J5" s="65">
+      <c r="J5" s="69" t="n"/>
+      <c r="K5" s="65">
         <f>IFERROR(DATEDIF(F5,G5,"M"),"")</f>
         <v/>
       </c>
-      <c r="K5" s="71" t="n"/>
-      <c r="L5" s="77">
-        <f>IFERROR(IF(K5="","",K5/12),"")</f>
-        <v/>
-      </c>
-      <c r="M5" s="69" t="n"/>
-      <c r="N5" s="80" t="n"/>
-      <c r="O5" s="79">
+      <c r="L5" s="71" t="n"/>
+      <c r="M5" s="77">
+        <f>IFERROR(IF(L5="","",L5/12),"")</f>
+        <v/>
+      </c>
+      <c r="N5" s="69" t="n"/>
+      <c r="O5" s="80" t="n"/>
+      <c r="P5" s="79">
         <f>IFERROR(IF(G5="","",G5-365),"")</f>
         <v/>
       </c>
-      <c r="P5" s="69" t="n"/>
       <c r="Q5" s="69" t="n"/>
     </row>
     <row r="6">
@@ -4458,22 +4458,22 @@
       <c r="G6" s="73" t="n"/>
       <c r="H6" s="72" t="n"/>
       <c r="I6" s="72" t="n"/>
-      <c r="J6" s="65">
+      <c r="J6" s="72" t="n"/>
+      <c r="K6" s="65">
         <f>IFERROR(DATEDIF(F6,G6,"M"),"")</f>
         <v/>
       </c>
-      <c r="K6" s="74" t="n"/>
-      <c r="L6" s="77">
-        <f>IFERROR(IF(K6="","",K6/12),"")</f>
-        <v/>
-      </c>
-      <c r="M6" s="72" t="n"/>
-      <c r="N6" s="81" t="n"/>
-      <c r="O6" s="79">
+      <c r="L6" s="74" t="n"/>
+      <c r="M6" s="77">
+        <f>IFERROR(IF(L6="","",L6/12),"")</f>
+        <v/>
+      </c>
+      <c r="N6" s="72" t="n"/>
+      <c r="O6" s="81" t="n"/>
+      <c r="P6" s="79">
         <f>IFERROR(IF(G6="","",G6-365),"")</f>
         <v/>
       </c>
-      <c r="P6" s="72" t="n"/>
       <c r="Q6" s="72" t="n"/>
     </row>
     <row r="7">
@@ -4486,22 +4486,22 @@
       <c r="G7" s="70" t="n"/>
       <c r="H7" s="69" t="n"/>
       <c r="I7" s="69" t="n"/>
-      <c r="J7" s="65">
+      <c r="J7" s="69" t="n"/>
+      <c r="K7" s="65">
         <f>IFERROR(DATEDIF(F7,G7,"M"),"")</f>
         <v/>
       </c>
-      <c r="K7" s="71" t="n"/>
-      <c r="L7" s="77">
-        <f>IFERROR(IF(K7="","",K7/12),"")</f>
-        <v/>
-      </c>
-      <c r="M7" s="69" t="n"/>
-      <c r="N7" s="80" t="n"/>
-      <c r="O7" s="79">
+      <c r="L7" s="71" t="n"/>
+      <c r="M7" s="77">
+        <f>IFERROR(IF(L7="","",L7/12),"")</f>
+        <v/>
+      </c>
+      <c r="N7" s="69" t="n"/>
+      <c r="O7" s="80" t="n"/>
+      <c r="P7" s="79">
         <f>IFERROR(IF(G7="","",G7-365),"")</f>
         <v/>
       </c>
-      <c r="P7" s="69" t="n"/>
       <c r="Q7" s="69" t="n"/>
     </row>
     <row r="8">
@@ -4514,22 +4514,22 @@
       <c r="G8" s="73" t="n"/>
       <c r="H8" s="72" t="n"/>
       <c r="I8" s="72" t="n"/>
-      <c r="J8" s="65">
+      <c r="J8" s="72" t="n"/>
+      <c r="K8" s="65">
         <f>IFERROR(DATEDIF(F8,G8,"M"),"")</f>
         <v/>
       </c>
-      <c r="K8" s="74" t="n"/>
-      <c r="L8" s="77">
-        <f>IFERROR(IF(K8="","",K8/12),"")</f>
-        <v/>
-      </c>
-      <c r="M8" s="72" t="n"/>
-      <c r="N8" s="81" t="n"/>
-      <c r="O8" s="79">
+      <c r="L8" s="74" t="n"/>
+      <c r="M8" s="77">
+        <f>IFERROR(IF(L8="","",L8/12),"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="72" t="n"/>
+      <c r="O8" s="81" t="n"/>
+      <c r="P8" s="79">
         <f>IFERROR(IF(G8="","",G8-365),"")</f>
         <v/>
       </c>
-      <c r="P8" s="72" t="n"/>
       <c r="Q8" s="72" t="n"/>
     </row>
     <row r="9">
@@ -4542,22 +4542,22 @@
       <c r="G9" s="70" t="n"/>
       <c r="H9" s="69" t="n"/>
       <c r="I9" s="69" t="n"/>
-      <c r="J9" s="65">
+      <c r="J9" s="69" t="n"/>
+      <c r="K9" s="65">
         <f>IFERROR(DATEDIF(F9,G9,"M"),"")</f>
         <v/>
       </c>
-      <c r="K9" s="71" t="n"/>
-      <c r="L9" s="77">
-        <f>IFERROR(IF(K9="","",K9/12),"")</f>
-        <v/>
-      </c>
-      <c r="M9" s="69" t="n"/>
-      <c r="N9" s="80" t="n"/>
-      <c r="O9" s="79">
+      <c r="L9" s="71" t="n"/>
+      <c r="M9" s="77">
+        <f>IFERROR(IF(L9="","",L9/12),"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="69" t="n"/>
+      <c r="O9" s="80" t="n"/>
+      <c r="P9" s="79">
         <f>IFERROR(IF(G9="","",G9-365),"")</f>
         <v/>
       </c>
-      <c r="P9" s="69" t="n"/>
       <c r="Q9" s="69" t="n"/>
     </row>
     <row r="10">
@@ -4570,22 +4570,22 @@
       <c r="G10" s="73" t="n"/>
       <c r="H10" s="72" t="n"/>
       <c r="I10" s="72" t="n"/>
-      <c r="J10" s="65">
+      <c r="J10" s="72" t="n"/>
+      <c r="K10" s="65">
         <f>IFERROR(DATEDIF(F10,G10,"M"),"")</f>
         <v/>
       </c>
-      <c r="K10" s="74" t="n"/>
-      <c r="L10" s="77">
-        <f>IFERROR(IF(K10="","",K10/12),"")</f>
-        <v/>
-      </c>
-      <c r="M10" s="72" t="n"/>
-      <c r="N10" s="81" t="n"/>
-      <c r="O10" s="79">
+      <c r="L10" s="74" t="n"/>
+      <c r="M10" s="77">
+        <f>IFERROR(IF(L10="","",L10/12),"")</f>
+        <v/>
+      </c>
+      <c r="N10" s="72" t="n"/>
+      <c r="O10" s="81" t="n"/>
+      <c r="P10" s="79">
         <f>IFERROR(IF(G10="","",G10-365),"")</f>
         <v/>
       </c>
-      <c r="P10" s="72" t="n"/>
       <c r="Q10" s="72" t="n"/>
     </row>
     <row r="11">
@@ -4598,22 +4598,22 @@
       <c r="G11" s="70" t="n"/>
       <c r="H11" s="69" t="n"/>
       <c r="I11" s="69" t="n"/>
-      <c r="J11" s="65">
+      <c r="J11" s="69" t="n"/>
+      <c r="K11" s="65">
         <f>IFERROR(DATEDIF(F11,G11,"M"),"")</f>
         <v/>
       </c>
-      <c r="K11" s="71" t="n"/>
-      <c r="L11" s="77">
-        <f>IFERROR(IF(K11="","",K11/12),"")</f>
-        <v/>
-      </c>
-      <c r="M11" s="69" t="n"/>
-      <c r="N11" s="80" t="n"/>
-      <c r="O11" s="79">
+      <c r="L11" s="71" t="n"/>
+      <c r="M11" s="77">
+        <f>IFERROR(IF(L11="","",L11/12),"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="69" t="n"/>
+      <c r="O11" s="80" t="n"/>
+      <c r="P11" s="79">
         <f>IFERROR(IF(G11="","",G11-365),"")</f>
         <v/>
       </c>
-      <c r="P11" s="69" t="n"/>
       <c r="Q11" s="69" t="n"/>
     </row>
     <row r="12">
@@ -4626,22 +4626,22 @@
       <c r="G12" s="73" t="n"/>
       <c r="H12" s="72" t="n"/>
       <c r="I12" s="72" t="n"/>
-      <c r="J12" s="65">
+      <c r="J12" s="72" t="n"/>
+      <c r="K12" s="65">
         <f>IFERROR(DATEDIF(F12,G12,"M"),"")</f>
         <v/>
       </c>
-      <c r="K12" s="74" t="n"/>
-      <c r="L12" s="77">
-        <f>IFERROR(IF(K12="","",K12/12),"")</f>
-        <v/>
-      </c>
-      <c r="M12" s="72" t="n"/>
-      <c r="N12" s="81" t="n"/>
-      <c r="O12" s="79">
+      <c r="L12" s="74" t="n"/>
+      <c r="M12" s="77">
+        <f>IFERROR(IF(L12="","",L12/12),"")</f>
+        <v/>
+      </c>
+      <c r="N12" s="72" t="n"/>
+      <c r="O12" s="81" t="n"/>
+      <c r="P12" s="79">
         <f>IFERROR(IF(G12="","",G12-365),"")</f>
         <v/>
       </c>
-      <c r="P12" s="72" t="n"/>
       <c r="Q12" s="72" t="n"/>
     </row>
     <row r="13">
@@ -4654,22 +4654,22 @@
       <c r="G13" s="70" t="n"/>
       <c r="H13" s="69" t="n"/>
       <c r="I13" s="69" t="n"/>
-      <c r="J13" s="65">
+      <c r="J13" s="69" t="n"/>
+      <c r="K13" s="65">
         <f>IFERROR(DATEDIF(F13,G13,"M"),"")</f>
         <v/>
       </c>
-      <c r="K13" s="71" t="n"/>
-      <c r="L13" s="77">
-        <f>IFERROR(IF(K13="","",K13/12),"")</f>
-        <v/>
-      </c>
-      <c r="M13" s="69" t="n"/>
-      <c r="N13" s="80" t="n"/>
-      <c r="O13" s="79">
+      <c r="L13" s="71" t="n"/>
+      <c r="M13" s="77">
+        <f>IFERROR(IF(L13="","",L13/12),"")</f>
+        <v/>
+      </c>
+      <c r="N13" s="69" t="n"/>
+      <c r="O13" s="80" t="n"/>
+      <c r="P13" s="79">
         <f>IFERROR(IF(G13="","",G13-365),"")</f>
         <v/>
       </c>
-      <c r="P13" s="69" t="n"/>
       <c r="Q13" s="69" t="n"/>
     </row>
     <row r="14">
@@ -4682,22 +4682,22 @@
       <c r="G14" s="73" t="n"/>
       <c r="H14" s="72" t="n"/>
       <c r="I14" s="72" t="n"/>
-      <c r="J14" s="65">
+      <c r="J14" s="72" t="n"/>
+      <c r="K14" s="65">
         <f>IFERROR(DATEDIF(F14,G14,"M"),"")</f>
         <v/>
       </c>
-      <c r="K14" s="74" t="n"/>
-      <c r="L14" s="77">
-        <f>IFERROR(IF(K14="","",K14/12),"")</f>
-        <v/>
-      </c>
-      <c r="M14" s="72" t="n"/>
-      <c r="N14" s="81" t="n"/>
-      <c r="O14" s="79">
+      <c r="L14" s="74" t="n"/>
+      <c r="M14" s="77">
+        <f>IFERROR(IF(L14="","",L14/12),"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="72" t="n"/>
+      <c r="O14" s="81" t="n"/>
+      <c r="P14" s="79">
         <f>IFERROR(IF(G14="","",G14-365),"")</f>
         <v/>
       </c>
-      <c r="P14" s="72" t="n"/>
       <c r="Q14" s="72" t="n"/>
     </row>
     <row r="15">
@@ -4710,22 +4710,22 @@
       <c r="G15" s="70" t="n"/>
       <c r="H15" s="69" t="n"/>
       <c r="I15" s="69" t="n"/>
-      <c r="J15" s="65">
+      <c r="J15" s="69" t="n"/>
+      <c r="K15" s="65">
         <f>IFERROR(DATEDIF(F15,G15,"M"),"")</f>
         <v/>
       </c>
-      <c r="K15" s="71" t="n"/>
-      <c r="L15" s="77">
-        <f>IFERROR(IF(K15="","",K15/12),"")</f>
-        <v/>
-      </c>
-      <c r="M15" s="69" t="n"/>
-      <c r="N15" s="80" t="n"/>
-      <c r="O15" s="79">
+      <c r="L15" s="71" t="n"/>
+      <c r="M15" s="77">
+        <f>IFERROR(IF(L15="","",L15/12),"")</f>
+        <v/>
+      </c>
+      <c r="N15" s="69" t="n"/>
+      <c r="O15" s="80" t="n"/>
+      <c r="P15" s="79">
         <f>IFERROR(IF(G15="","",G15-365),"")</f>
         <v/>
       </c>
-      <c r="P15" s="69" t="n"/>
       <c r="Q15" s="69" t="n"/>
     </row>
     <row r="16">
@@ -4738,22 +4738,22 @@
       <c r="G16" s="73" t="n"/>
       <c r="H16" s="72" t="n"/>
       <c r="I16" s="72" t="n"/>
-      <c r="J16" s="65">
+      <c r="J16" s="72" t="n"/>
+      <c r="K16" s="65">
         <f>IFERROR(DATEDIF(F16,G16,"M"),"")</f>
         <v/>
       </c>
-      <c r="K16" s="74" t="n"/>
-      <c r="L16" s="77">
-        <f>IFERROR(IF(K16="","",K16/12),"")</f>
-        <v/>
-      </c>
-      <c r="M16" s="72" t="n"/>
-      <c r="N16" s="81" t="n"/>
-      <c r="O16" s="79">
+      <c r="L16" s="74" t="n"/>
+      <c r="M16" s="77">
+        <f>IFERROR(IF(L16="","",L16/12),"")</f>
+        <v/>
+      </c>
+      <c r="N16" s="72" t="n"/>
+      <c r="O16" s="81" t="n"/>
+      <c r="P16" s="79">
         <f>IFERROR(IF(G16="","",G16-365),"")</f>
         <v/>
       </c>
-      <c r="P16" s="72" t="n"/>
       <c r="Q16" s="72" t="n"/>
     </row>
     <row r="17">
@@ -4766,22 +4766,22 @@
       <c r="G17" s="70" t="n"/>
       <c r="H17" s="69" t="n"/>
       <c r="I17" s="69" t="n"/>
-      <c r="J17" s="65">
+      <c r="J17" s="69" t="n"/>
+      <c r="K17" s="65">
         <f>IFERROR(DATEDIF(F17,G17,"M"),"")</f>
         <v/>
       </c>
-      <c r="K17" s="71" t="n"/>
-      <c r="L17" s="77">
-        <f>IFERROR(IF(K17="","",K17/12),"")</f>
-        <v/>
-      </c>
-      <c r="M17" s="69" t="n"/>
-      <c r="N17" s="80" t="n"/>
-      <c r="O17" s="79">
+      <c r="L17" s="71" t="n"/>
+      <c r="M17" s="77">
+        <f>IFERROR(IF(L17="","",L17/12),"")</f>
+        <v/>
+      </c>
+      <c r="N17" s="69" t="n"/>
+      <c r="O17" s="80" t="n"/>
+      <c r="P17" s="79">
         <f>IFERROR(IF(G17="","",G17-365),"")</f>
         <v/>
       </c>
-      <c r="P17" s="69" t="n"/>
       <c r="Q17" s="69" t="n"/>
     </row>
     <row r="18">
@@ -4794,22 +4794,22 @@
       <c r="G18" s="73" t="n"/>
       <c r="H18" s="72" t="n"/>
       <c r="I18" s="72" t="n"/>
-      <c r="J18" s="65">
+      <c r="J18" s="72" t="n"/>
+      <c r="K18" s="65">
         <f>IFERROR(DATEDIF(F18,G18,"M"),"")</f>
         <v/>
       </c>
-      <c r="K18" s="74" t="n"/>
-      <c r="L18" s="77">
-        <f>IFERROR(IF(K18="","",K18/12),"")</f>
-        <v/>
-      </c>
-      <c r="M18" s="72" t="n"/>
-      <c r="N18" s="81" t="n"/>
-      <c r="O18" s="79">
+      <c r="L18" s="74" t="n"/>
+      <c r="M18" s="77">
+        <f>IFERROR(IF(L18="","",L18/12),"")</f>
+        <v/>
+      </c>
+      <c r="N18" s="72" t="n"/>
+      <c r="O18" s="81" t="n"/>
+      <c r="P18" s="79">
         <f>IFERROR(IF(G18="","",G18-365),"")</f>
         <v/>
       </c>
-      <c r="P18" s="72" t="n"/>
       <c r="Q18" s="72" t="n"/>
     </row>
     <row r="19">
@@ -4822,22 +4822,22 @@
       <c r="G19" s="70" t="n"/>
       <c r="H19" s="69" t="n"/>
       <c r="I19" s="69" t="n"/>
-      <c r="J19" s="65">
+      <c r="J19" s="69" t="n"/>
+      <c r="K19" s="65">
         <f>IFERROR(DATEDIF(F19,G19,"M"),"")</f>
         <v/>
       </c>
-      <c r="K19" s="71" t="n"/>
-      <c r="L19" s="77">
-        <f>IFERROR(IF(K19="","",K19/12),"")</f>
-        <v/>
-      </c>
-      <c r="M19" s="69" t="n"/>
-      <c r="N19" s="80" t="n"/>
-      <c r="O19" s="79">
+      <c r="L19" s="71" t="n"/>
+      <c r="M19" s="77">
+        <f>IFERROR(IF(L19="","",L19/12),"")</f>
+        <v/>
+      </c>
+      <c r="N19" s="69" t="n"/>
+      <c r="O19" s="80" t="n"/>
+      <c r="P19" s="79">
         <f>IFERROR(IF(G19="","",G19-365),"")</f>
         <v/>
       </c>
-      <c r="P19" s="69" t="n"/>
       <c r="Q19" s="69" t="n"/>
     </row>
     <row r="20">
@@ -4850,22 +4850,22 @@
       <c r="G20" s="73" t="n"/>
       <c r="H20" s="72" t="n"/>
       <c r="I20" s="72" t="n"/>
-      <c r="J20" s="65">
+      <c r="J20" s="72" t="n"/>
+      <c r="K20" s="65">
         <f>IFERROR(DATEDIF(F20,G20,"M"),"")</f>
         <v/>
       </c>
-      <c r="K20" s="74" t="n"/>
-      <c r="L20" s="77">
-        <f>IFERROR(IF(K20="","",K20/12),"")</f>
-        <v/>
-      </c>
-      <c r="M20" s="72" t="n"/>
-      <c r="N20" s="81" t="n"/>
-      <c r="O20" s="79">
+      <c r="L20" s="74" t="n"/>
+      <c r="M20" s="77">
+        <f>IFERROR(IF(L20="","",L20/12),"")</f>
+        <v/>
+      </c>
+      <c r="N20" s="72" t="n"/>
+      <c r="O20" s="81" t="n"/>
+      <c r="P20" s="79">
         <f>IFERROR(IF(G20="","",G20-365),"")</f>
         <v/>
       </c>
-      <c r="P20" s="72" t="n"/>
       <c r="Q20" s="72" t="n"/>
     </row>
     <row r="21">
@@ -4878,22 +4878,22 @@
       <c r="G21" s="70" t="n"/>
       <c r="H21" s="69" t="n"/>
       <c r="I21" s="69" t="n"/>
-      <c r="J21" s="65">
+      <c r="J21" s="69" t="n"/>
+      <c r="K21" s="65">
         <f>IFERROR(DATEDIF(F21,G21,"M"),"")</f>
         <v/>
       </c>
-      <c r="K21" s="71" t="n"/>
-      <c r="L21" s="77">
-        <f>IFERROR(IF(K21="","",K21/12),"")</f>
-        <v/>
-      </c>
-      <c r="M21" s="69" t="n"/>
-      <c r="N21" s="80" t="n"/>
-      <c r="O21" s="79">
+      <c r="L21" s="71" t="n"/>
+      <c r="M21" s="77">
+        <f>IFERROR(IF(L21="","",L21/12),"")</f>
+        <v/>
+      </c>
+      <c r="N21" s="69" t="n"/>
+      <c r="O21" s="80" t="n"/>
+      <c r="P21" s="79">
         <f>IFERROR(IF(G21="","",G21-365),"")</f>
         <v/>
       </c>
-      <c r="P21" s="69" t="n"/>
       <c r="Q21" s="69" t="n"/>
     </row>
     <row r="22">
@@ -4906,22 +4906,22 @@
       <c r="G22" s="73" t="n"/>
       <c r="H22" s="72" t="n"/>
       <c r="I22" s="72" t="n"/>
-      <c r="J22" s="65">
+      <c r="J22" s="72" t="n"/>
+      <c r="K22" s="65">
         <f>IFERROR(DATEDIF(F22,G22,"M"),"")</f>
         <v/>
       </c>
-      <c r="K22" s="74" t="n"/>
-      <c r="L22" s="77">
-        <f>IFERROR(IF(K22="","",K22/12),"")</f>
-        <v/>
-      </c>
-      <c r="M22" s="72" t="n"/>
-      <c r="N22" s="81" t="n"/>
-      <c r="O22" s="79">
+      <c r="L22" s="74" t="n"/>
+      <c r="M22" s="77">
+        <f>IFERROR(IF(L22="","",L22/12),"")</f>
+        <v/>
+      </c>
+      <c r="N22" s="72" t="n"/>
+      <c r="O22" s="81" t="n"/>
+      <c r="P22" s="79">
         <f>IFERROR(IF(G22="","",G22-365),"")</f>
         <v/>
       </c>
-      <c r="P22" s="72" t="n"/>
       <c r="Q22" s="72" t="n"/>
     </row>
     <row r="23">
@@ -4934,22 +4934,22 @@
       <c r="G23" s="70" t="n"/>
       <c r="H23" s="69" t="n"/>
       <c r="I23" s="69" t="n"/>
-      <c r="J23" s="65">
+      <c r="J23" s="69" t="n"/>
+      <c r="K23" s="65">
         <f>IFERROR(DATEDIF(F23,G23,"M"),"")</f>
         <v/>
       </c>
-      <c r="K23" s="71" t="n"/>
-      <c r="L23" s="77">
-        <f>IFERROR(IF(K23="","",K23/12),"")</f>
-        <v/>
-      </c>
-      <c r="M23" s="69" t="n"/>
-      <c r="N23" s="80" t="n"/>
-      <c r="O23" s="79">
+      <c r="L23" s="71" t="n"/>
+      <c r="M23" s="77">
+        <f>IFERROR(IF(L23="","",L23/12),"")</f>
+        <v/>
+      </c>
+      <c r="N23" s="69" t="n"/>
+      <c r="O23" s="80" t="n"/>
+      <c r="P23" s="79">
         <f>IFERROR(IF(G23="","",G23-365),"")</f>
         <v/>
       </c>
-      <c r="P23" s="69" t="n"/>
       <c r="Q23" s="69" t="n"/>
     </row>
     <row r="24">
@@ -4962,22 +4962,22 @@
       <c r="G24" s="73" t="n"/>
       <c r="H24" s="72" t="n"/>
       <c r="I24" s="72" t="n"/>
-      <c r="J24" s="65">
+      <c r="J24" s="72" t="n"/>
+      <c r="K24" s="65">
         <f>IFERROR(DATEDIF(F24,G24,"M"),"")</f>
         <v/>
       </c>
-      <c r="K24" s="74" t="n"/>
-      <c r="L24" s="77">
-        <f>IFERROR(IF(K24="","",K24/12),"")</f>
-        <v/>
-      </c>
-      <c r="M24" s="72" t="n"/>
-      <c r="N24" s="81" t="n"/>
-      <c r="O24" s="79">
+      <c r="L24" s="74" t="n"/>
+      <c r="M24" s="77">
+        <f>IFERROR(IF(L24="","",L24/12),"")</f>
+        <v/>
+      </c>
+      <c r="N24" s="72" t="n"/>
+      <c r="O24" s="81" t="n"/>
+      <c r="P24" s="79">
         <f>IFERROR(IF(G24="","",G24-365),"")</f>
         <v/>
       </c>
-      <c r="P24" s="72" t="n"/>
       <c r="Q24" s="72" t="n"/>
     </row>
     <row r="25">
@@ -4990,22 +4990,22 @@
       <c r="G25" s="70" t="n"/>
       <c r="H25" s="69" t="n"/>
       <c r="I25" s="69" t="n"/>
-      <c r="J25" s="65">
+      <c r="J25" s="69" t="n"/>
+      <c r="K25" s="65">
         <f>IFERROR(DATEDIF(F25,G25,"M"),"")</f>
         <v/>
       </c>
-      <c r="K25" s="71" t="n"/>
-      <c r="L25" s="77">
-        <f>IFERROR(IF(K25="","",K25/12),"")</f>
-        <v/>
-      </c>
-      <c r="M25" s="69" t="n"/>
-      <c r="N25" s="80" t="n"/>
-      <c r="O25" s="79">
+      <c r="L25" s="71" t="n"/>
+      <c r="M25" s="77">
+        <f>IFERROR(IF(L25="","",L25/12),"")</f>
+        <v/>
+      </c>
+      <c r="N25" s="69" t="n"/>
+      <c r="O25" s="80" t="n"/>
+      <c r="P25" s="79">
         <f>IFERROR(IF(G25="","",G25-365),"")</f>
         <v/>
       </c>
-      <c r="P25" s="69" t="n"/>
       <c r="Q25" s="69" t="n"/>
     </row>
     <row r="26">
@@ -5018,22 +5018,22 @@
       <c r="G26" s="73" t="n"/>
       <c r="H26" s="72" t="n"/>
       <c r="I26" s="72" t="n"/>
-      <c r="J26" s="65">
+      <c r="J26" s="72" t="n"/>
+      <c r="K26" s="65">
         <f>IFERROR(DATEDIF(F26,G26,"M"),"")</f>
         <v/>
       </c>
-      <c r="K26" s="74" t="n"/>
-      <c r="L26" s="77">
-        <f>IFERROR(IF(K26="","",K26/12),"")</f>
-        <v/>
-      </c>
-      <c r="M26" s="72" t="n"/>
-      <c r="N26" s="81" t="n"/>
-      <c r="O26" s="79">
+      <c r="L26" s="74" t="n"/>
+      <c r="M26" s="77">
+        <f>IFERROR(IF(L26="","",L26/12),"")</f>
+        <v/>
+      </c>
+      <c r="N26" s="72" t="n"/>
+      <c r="O26" s="81" t="n"/>
+      <c r="P26" s="79">
         <f>IFERROR(IF(G26="","",G26-365),"")</f>
         <v/>
       </c>
-      <c r="P26" s="72" t="n"/>
       <c r="Q26" s="72" t="n"/>
     </row>
     <row r="27">
@@ -5046,22 +5046,22 @@
       <c r="G27" s="70" t="n"/>
       <c r="H27" s="69" t="n"/>
       <c r="I27" s="69" t="n"/>
-      <c r="J27" s="65">
+      <c r="J27" s="69" t="n"/>
+      <c r="K27" s="65">
         <f>IFERROR(DATEDIF(F27,G27,"M"),"")</f>
         <v/>
       </c>
-      <c r="K27" s="71" t="n"/>
-      <c r="L27" s="77">
-        <f>IFERROR(IF(K27="","",K27/12),"")</f>
-        <v/>
-      </c>
-      <c r="M27" s="69" t="n"/>
-      <c r="N27" s="80" t="n"/>
-      <c r="O27" s="79">
+      <c r="L27" s="71" t="n"/>
+      <c r="M27" s="77">
+        <f>IFERROR(IF(L27="","",L27/12),"")</f>
+        <v/>
+      </c>
+      <c r="N27" s="69" t="n"/>
+      <c r="O27" s="80" t="n"/>
+      <c r="P27" s="79">
         <f>IFERROR(IF(G27="","",G27-365),"")</f>
         <v/>
       </c>
-      <c r="P27" s="69" t="n"/>
       <c r="Q27" s="69" t="n"/>
     </row>
     <row r="28">
@@ -5074,22 +5074,22 @@
       <c r="G28" s="73" t="n"/>
       <c r="H28" s="72" t="n"/>
       <c r="I28" s="72" t="n"/>
-      <c r="J28" s="65">
+      <c r="J28" s="72" t="n"/>
+      <c r="K28" s="65">
         <f>IFERROR(DATEDIF(F28,G28,"M"),"")</f>
         <v/>
       </c>
-      <c r="K28" s="74" t="n"/>
-      <c r="L28" s="77">
-        <f>IFERROR(IF(K28="","",K28/12),"")</f>
-        <v/>
-      </c>
-      <c r="M28" s="72" t="n"/>
-      <c r="N28" s="81" t="n"/>
-      <c r="O28" s="79">
+      <c r="L28" s="74" t="n"/>
+      <c r="M28" s="77">
+        <f>IFERROR(IF(L28="","",L28/12),"")</f>
+        <v/>
+      </c>
+      <c r="N28" s="72" t="n"/>
+      <c r="O28" s="81" t="n"/>
+      <c r="P28" s="79">
         <f>IFERROR(IF(G28="","",G28-365),"")</f>
         <v/>
       </c>
-      <c r="P28" s="72" t="n"/>
       <c r="Q28" s="72" t="n"/>
     </row>
     <row r="29">
@@ -5102,22 +5102,22 @@
       <c r="G29" s="70" t="n"/>
       <c r="H29" s="69" t="n"/>
       <c r="I29" s="69" t="n"/>
-      <c r="J29" s="65">
+      <c r="J29" s="69" t="n"/>
+      <c r="K29" s="65">
         <f>IFERROR(DATEDIF(F29,G29,"M"),"")</f>
         <v/>
       </c>
-      <c r="K29" s="71" t="n"/>
-      <c r="L29" s="77">
-        <f>IFERROR(IF(K29="","",K29/12),"")</f>
-        <v/>
-      </c>
-      <c r="M29" s="69" t="n"/>
-      <c r="N29" s="80" t="n"/>
-      <c r="O29" s="79">
+      <c r="L29" s="71" t="n"/>
+      <c r="M29" s="77">
+        <f>IFERROR(IF(L29="","",L29/12),"")</f>
+        <v/>
+      </c>
+      <c r="N29" s="69" t="n"/>
+      <c r="O29" s="80" t="n"/>
+      <c r="P29" s="79">
         <f>IFERROR(IF(G29="","",G29-365),"")</f>
         <v/>
       </c>
-      <c r="P29" s="69" t="n"/>
       <c r="Q29" s="69" t="n"/>
     </row>
     <row r="30">
@@ -5130,22 +5130,22 @@
       <c r="G30" s="73" t="n"/>
       <c r="H30" s="72" t="n"/>
       <c r="I30" s="72" t="n"/>
-      <c r="J30" s="65">
+      <c r="J30" s="72" t="n"/>
+      <c r="K30" s="65">
         <f>IFERROR(DATEDIF(F30,G30,"M"),"")</f>
         <v/>
       </c>
-      <c r="K30" s="74" t="n"/>
-      <c r="L30" s="77">
-        <f>IFERROR(IF(K30="","",K30/12),"")</f>
-        <v/>
-      </c>
-      <c r="M30" s="72" t="n"/>
-      <c r="N30" s="81" t="n"/>
-      <c r="O30" s="79">
+      <c r="L30" s="74" t="n"/>
+      <c r="M30" s="77">
+        <f>IFERROR(IF(L30="","",L30/12),"")</f>
+        <v/>
+      </c>
+      <c r="N30" s="72" t="n"/>
+      <c r="O30" s="81" t="n"/>
+      <c r="P30" s="79">
         <f>IFERROR(IF(G30="","",G30-365),"")</f>
         <v/>
       </c>
-      <c r="P30" s="72" t="n"/>
       <c r="Q30" s="72" t="n"/>
     </row>
     <row r="31">
@@ -5158,22 +5158,22 @@
       <c r="G31" s="70" t="n"/>
       <c r="H31" s="69" t="n"/>
       <c r="I31" s="69" t="n"/>
-      <c r="J31" s="65">
+      <c r="J31" s="69" t="n"/>
+      <c r="K31" s="65">
         <f>IFERROR(DATEDIF(F31,G31,"M"),"")</f>
         <v/>
       </c>
-      <c r="K31" s="71" t="n"/>
-      <c r="L31" s="77">
-        <f>IFERROR(IF(K31="","",K31/12),"")</f>
-        <v/>
-      </c>
-      <c r="M31" s="69" t="n"/>
-      <c r="N31" s="80" t="n"/>
-      <c r="O31" s="79">
+      <c r="L31" s="71" t="n"/>
+      <c r="M31" s="77">
+        <f>IFERROR(IF(L31="","",L31/12),"")</f>
+        <v/>
+      </c>
+      <c r="N31" s="69" t="n"/>
+      <c r="O31" s="80" t="n"/>
+      <c r="P31" s="79">
         <f>IFERROR(IF(G31="","",G31-365),"")</f>
         <v/>
       </c>
-      <c r="P31" s="69" t="n"/>
       <c r="Q31" s="69" t="n"/>
     </row>
     <row r="32">
@@ -5186,22 +5186,22 @@
       <c r="G32" s="73" t="n"/>
       <c r="H32" s="72" t="n"/>
       <c r="I32" s="72" t="n"/>
-      <c r="J32" s="65">
+      <c r="J32" s="72" t="n"/>
+      <c r="K32" s="65">
         <f>IFERROR(DATEDIF(F32,G32,"M"),"")</f>
         <v/>
       </c>
-      <c r="K32" s="74" t="n"/>
-      <c r="L32" s="77">
-        <f>IFERROR(IF(K32="","",K32/12),"")</f>
-        <v/>
-      </c>
-      <c r="M32" s="72" t="n"/>
-      <c r="N32" s="81" t="n"/>
-      <c r="O32" s="79">
+      <c r="L32" s="74" t="n"/>
+      <c r="M32" s="77">
+        <f>IFERROR(IF(L32="","",L32/12),"")</f>
+        <v/>
+      </c>
+      <c r="N32" s="72" t="n"/>
+      <c r="O32" s="81" t="n"/>
+      <c r="P32" s="79">
         <f>IFERROR(IF(G32="","",G32-365),"")</f>
         <v/>
       </c>
-      <c r="P32" s="72" t="n"/>
       <c r="Q32" s="72" t="n"/>
     </row>
     <row r="33">
@@ -5214,22 +5214,22 @@
       <c r="G33" s="70" t="n"/>
       <c r="H33" s="69" t="n"/>
       <c r="I33" s="69" t="n"/>
-      <c r="J33" s="65">
+      <c r="J33" s="69" t="n"/>
+      <c r="K33" s="65">
         <f>IFERROR(DATEDIF(F33,G33,"M"),"")</f>
         <v/>
       </c>
-      <c r="K33" s="71" t="n"/>
-      <c r="L33" s="77">
-        <f>IFERROR(IF(K33="","",K33/12),"")</f>
-        <v/>
-      </c>
-      <c r="M33" s="69" t="n"/>
-      <c r="N33" s="80" t="n"/>
-      <c r="O33" s="79">
+      <c r="L33" s="71" t="n"/>
+      <c r="M33" s="77">
+        <f>IFERROR(IF(L33="","",L33/12),"")</f>
+        <v/>
+      </c>
+      <c r="N33" s="69" t="n"/>
+      <c r="O33" s="80" t="n"/>
+      <c r="P33" s="79">
         <f>IFERROR(IF(G33="","",G33-365),"")</f>
         <v/>
       </c>
-      <c r="P33" s="69" t="n"/>
       <c r="Q33" s="69" t="n"/>
     </row>
     <row r="34">
@@ -5242,22 +5242,22 @@
       <c r="G34" s="73" t="n"/>
       <c r="H34" s="72" t="n"/>
       <c r="I34" s="72" t="n"/>
-      <c r="J34" s="65">
+      <c r="J34" s="72" t="n"/>
+      <c r="K34" s="65">
         <f>IFERROR(DATEDIF(F34,G34,"M"),"")</f>
         <v/>
       </c>
-      <c r="K34" s="74" t="n"/>
-      <c r="L34" s="77">
-        <f>IFERROR(IF(K34="","",K34/12),"")</f>
-        <v/>
-      </c>
-      <c r="M34" s="72" t="n"/>
-      <c r="N34" s="81" t="n"/>
-      <c r="O34" s="79">
+      <c r="L34" s="74" t="n"/>
+      <c r="M34" s="77">
+        <f>IFERROR(IF(L34="","",L34/12),"")</f>
+        <v/>
+      </c>
+      <c r="N34" s="72" t="n"/>
+      <c r="O34" s="81" t="n"/>
+      <c r="P34" s="79">
         <f>IFERROR(IF(G34="","",G34-365),"")</f>
         <v/>
       </c>
-      <c r="P34" s="72" t="n"/>
       <c r="Q34" s="72" t="n"/>
     </row>
     <row r="35">
@@ -5270,22 +5270,22 @@
       <c r="G35" s="70" t="n"/>
       <c r="H35" s="69" t="n"/>
       <c r="I35" s="69" t="n"/>
-      <c r="J35" s="65">
+      <c r="J35" s="69" t="n"/>
+      <c r="K35" s="65">
         <f>IFERROR(DATEDIF(F35,G35,"M"),"")</f>
         <v/>
       </c>
-      <c r="K35" s="71" t="n"/>
-      <c r="L35" s="77">
-        <f>IFERROR(IF(K35="","",K35/12),"")</f>
-        <v/>
-      </c>
-      <c r="M35" s="69" t="n"/>
-      <c r="N35" s="80" t="n"/>
-      <c r="O35" s="79">
+      <c r="L35" s="71" t="n"/>
+      <c r="M35" s="77">
+        <f>IFERROR(IF(L35="","",L35/12),"")</f>
+        <v/>
+      </c>
+      <c r="N35" s="69" t="n"/>
+      <c r="O35" s="80" t="n"/>
+      <c r="P35" s="79">
         <f>IFERROR(IF(G35="","",G35-365),"")</f>
         <v/>
       </c>
-      <c r="P35" s="69" t="n"/>
       <c r="Q35" s="69" t="n"/>
     </row>
     <row r="36">
@@ -5298,22 +5298,22 @@
       <c r="G36" s="73" t="n"/>
       <c r="H36" s="72" t="n"/>
       <c r="I36" s="72" t="n"/>
-      <c r="J36" s="65">
+      <c r="J36" s="72" t="n"/>
+      <c r="K36" s="65">
         <f>IFERROR(DATEDIF(F36,G36,"M"),"")</f>
         <v/>
       </c>
-      <c r="K36" s="74" t="n"/>
-      <c r="L36" s="77">
-        <f>IFERROR(IF(K36="","",K36/12),"")</f>
-        <v/>
-      </c>
-      <c r="M36" s="72" t="n"/>
-      <c r="N36" s="81" t="n"/>
-      <c r="O36" s="79">
+      <c r="L36" s="74" t="n"/>
+      <c r="M36" s="77">
+        <f>IFERROR(IF(L36="","",L36/12),"")</f>
+        <v/>
+      </c>
+      <c r="N36" s="72" t="n"/>
+      <c r="O36" s="81" t="n"/>
+      <c r="P36" s="79">
         <f>IFERROR(IF(G36="","",G36-365),"")</f>
         <v/>
       </c>
-      <c r="P36" s="72" t="n"/>
       <c r="Q36" s="72" t="n"/>
     </row>
     <row r="37">
@@ -5326,22 +5326,22 @@
       <c r="G37" s="70" t="n"/>
       <c r="H37" s="69" t="n"/>
       <c r="I37" s="69" t="n"/>
-      <c r="J37" s="65">
+      <c r="J37" s="69" t="n"/>
+      <c r="K37" s="65">
         <f>IFERROR(DATEDIF(F37,G37,"M"),"")</f>
         <v/>
       </c>
-      <c r="K37" s="71" t="n"/>
-      <c r="L37" s="77">
-        <f>IFERROR(IF(K37="","",K37/12),"")</f>
-        <v/>
-      </c>
-      <c r="M37" s="69" t="n"/>
-      <c r="N37" s="80" t="n"/>
-      <c r="O37" s="79">
+      <c r="L37" s="71" t="n"/>
+      <c r="M37" s="77">
+        <f>IFERROR(IF(L37="","",L37/12),"")</f>
+        <v/>
+      </c>
+      <c r="N37" s="69" t="n"/>
+      <c r="O37" s="80" t="n"/>
+      <c r="P37" s="79">
         <f>IFERROR(IF(G37="","",G37-365),"")</f>
         <v/>
       </c>
-      <c r="P37" s="69" t="n"/>
       <c r="Q37" s="69" t="n"/>
     </row>
     <row r="38">
@@ -5354,22 +5354,22 @@
       <c r="G38" s="73" t="n"/>
       <c r="H38" s="72" t="n"/>
       <c r="I38" s="72" t="n"/>
-      <c r="J38" s="65">
+      <c r="J38" s="72" t="n"/>
+      <c r="K38" s="65">
         <f>IFERROR(DATEDIF(F38,G38,"M"),"")</f>
         <v/>
       </c>
-      <c r="K38" s="74" t="n"/>
-      <c r="L38" s="77">
-        <f>IFERROR(IF(K38="","",K38/12),"")</f>
-        <v/>
-      </c>
-      <c r="M38" s="72" t="n"/>
-      <c r="N38" s="81" t="n"/>
-      <c r="O38" s="79">
+      <c r="L38" s="74" t="n"/>
+      <c r="M38" s="77">
+        <f>IFERROR(IF(L38="","",L38/12),"")</f>
+        <v/>
+      </c>
+      <c r="N38" s="72" t="n"/>
+      <c r="O38" s="81" t="n"/>
+      <c r="P38" s="79">
         <f>IFERROR(IF(G38="","",G38-365),"")</f>
         <v/>
       </c>
-      <c r="P38" s="72" t="n"/>
       <c r="Q38" s="72" t="n"/>
     </row>
     <row r="39">
@@ -5382,22 +5382,22 @@
       <c r="G39" s="70" t="n"/>
       <c r="H39" s="69" t="n"/>
       <c r="I39" s="69" t="n"/>
-      <c r="J39" s="65">
+      <c r="J39" s="69" t="n"/>
+      <c r="K39" s="65">
         <f>IFERROR(DATEDIF(F39,G39,"M"),"")</f>
         <v/>
       </c>
-      <c r="K39" s="71" t="n"/>
-      <c r="L39" s="77">
-        <f>IFERROR(IF(K39="","",K39/12),"")</f>
-        <v/>
-      </c>
-      <c r="M39" s="69" t="n"/>
-      <c r="N39" s="80" t="n"/>
-      <c r="O39" s="79">
+      <c r="L39" s="71" t="n"/>
+      <c r="M39" s="77">
+        <f>IFERROR(IF(L39="","",L39/12),"")</f>
+        <v/>
+      </c>
+      <c r="N39" s="69" t="n"/>
+      <c r="O39" s="80" t="n"/>
+      <c r="P39" s="79">
         <f>IFERROR(IF(G39="","",G39-365),"")</f>
         <v/>
       </c>
-      <c r="P39" s="69" t="n"/>
       <c r="Q39" s="69" t="n"/>
     </row>
     <row r="40">
@@ -5410,22 +5410,22 @@
       <c r="G40" s="73" t="n"/>
       <c r="H40" s="72" t="n"/>
       <c r="I40" s="72" t="n"/>
-      <c r="J40" s="65">
+      <c r="J40" s="72" t="n"/>
+      <c r="K40" s="65">
         <f>IFERROR(DATEDIF(F40,G40,"M"),"")</f>
         <v/>
       </c>
-      <c r="K40" s="74" t="n"/>
-      <c r="L40" s="77">
-        <f>IFERROR(IF(K40="","",K40/12),"")</f>
-        <v/>
-      </c>
-      <c r="M40" s="72" t="n"/>
-      <c r="N40" s="81" t="n"/>
-      <c r="O40" s="79">
+      <c r="L40" s="74" t="n"/>
+      <c r="M40" s="77">
+        <f>IFERROR(IF(L40="","",L40/12),"")</f>
+        <v/>
+      </c>
+      <c r="N40" s="72" t="n"/>
+      <c r="O40" s="81" t="n"/>
+      <c r="P40" s="79">
         <f>IFERROR(IF(G40="","",G40-365),"")</f>
         <v/>
       </c>
-      <c r="P40" s="72" t="n"/>
       <c r="Q40" s="72" t="n"/>
     </row>
     <row r="41">
@@ -5438,22 +5438,22 @@
       <c r="G41" s="70" t="n"/>
       <c r="H41" s="69" t="n"/>
       <c r="I41" s="69" t="n"/>
-      <c r="J41" s="65">
+      <c r="J41" s="69" t="n"/>
+      <c r="K41" s="65">
         <f>IFERROR(DATEDIF(F41,G41,"M"),"")</f>
         <v/>
       </c>
-      <c r="K41" s="71" t="n"/>
-      <c r="L41" s="77">
-        <f>IFERROR(IF(K41="","",K41/12),"")</f>
-        <v/>
-      </c>
-      <c r="M41" s="69" t="n"/>
-      <c r="N41" s="80" t="n"/>
-      <c r="O41" s="79">
+      <c r="L41" s="71" t="n"/>
+      <c r="M41" s="77">
+        <f>IFERROR(IF(L41="","",L41/12),"")</f>
+        <v/>
+      </c>
+      <c r="N41" s="69" t="n"/>
+      <c r="O41" s="80" t="n"/>
+      <c r="P41" s="79">
         <f>IFERROR(IF(G41="","",G41-365),"")</f>
         <v/>
       </c>
-      <c r="P41" s="69" t="n"/>
       <c r="Q41" s="69" t="n"/>
     </row>
     <row r="42">
@@ -5466,22 +5466,22 @@
       <c r="G42" s="73" t="n"/>
       <c r="H42" s="72" t="n"/>
       <c r="I42" s="72" t="n"/>
-      <c r="J42" s="65">
+      <c r="J42" s="72" t="n"/>
+      <c r="K42" s="65">
         <f>IFERROR(DATEDIF(F42,G42,"M"),"")</f>
         <v/>
       </c>
-      <c r="K42" s="74" t="n"/>
-      <c r="L42" s="77">
-        <f>IFERROR(IF(K42="","",K42/12),"")</f>
-        <v/>
-      </c>
-      <c r="M42" s="72" t="n"/>
-      <c r="N42" s="81" t="n"/>
-      <c r="O42" s="79">
+      <c r="L42" s="74" t="n"/>
+      <c r="M42" s="77">
+        <f>IFERROR(IF(L42="","",L42/12),"")</f>
+        <v/>
+      </c>
+      <c r="N42" s="72" t="n"/>
+      <c r="O42" s="81" t="n"/>
+      <c r="P42" s="79">
         <f>IFERROR(IF(G42="","",G42-365),"")</f>
         <v/>
       </c>
-      <c r="P42" s="72" t="n"/>
       <c r="Q42" s="72" t="n"/>
     </row>
     <row r="43">
@@ -5494,22 +5494,22 @@
       <c r="G43" s="70" t="n"/>
       <c r="H43" s="69" t="n"/>
       <c r="I43" s="69" t="n"/>
-      <c r="J43" s="65">
+      <c r="J43" s="69" t="n"/>
+      <c r="K43" s="65">
         <f>IFERROR(DATEDIF(F43,G43,"M"),"")</f>
         <v/>
       </c>
-      <c r="K43" s="71" t="n"/>
-      <c r="L43" s="77">
-        <f>IFERROR(IF(K43="","",K43/12),"")</f>
-        <v/>
-      </c>
-      <c r="M43" s="69" t="n"/>
-      <c r="N43" s="80" t="n"/>
-      <c r="O43" s="79">
+      <c r="L43" s="71" t="n"/>
+      <c r="M43" s="77">
+        <f>IFERROR(IF(L43="","",L43/12),"")</f>
+        <v/>
+      </c>
+      <c r="N43" s="69" t="n"/>
+      <c r="O43" s="80" t="n"/>
+      <c r="P43" s="79">
         <f>IFERROR(IF(G43="","",G43-365),"")</f>
         <v/>
       </c>
-      <c r="P43" s="69" t="n"/>
       <c r="Q43" s="69" t="n"/>
     </row>
     <row r="44">
@@ -5522,22 +5522,22 @@
       <c r="G44" s="73" t="n"/>
       <c r="H44" s="72" t="n"/>
       <c r="I44" s="72" t="n"/>
-      <c r="J44" s="65">
+      <c r="J44" s="72" t="n"/>
+      <c r="K44" s="65">
         <f>IFERROR(DATEDIF(F44,G44,"M"),"")</f>
         <v/>
       </c>
-      <c r="K44" s="74" t="n"/>
-      <c r="L44" s="77">
-        <f>IFERROR(IF(K44="","",K44/12),"")</f>
-        <v/>
-      </c>
-      <c r="M44" s="72" t="n"/>
-      <c r="N44" s="81" t="n"/>
-      <c r="O44" s="79">
+      <c r="L44" s="74" t="n"/>
+      <c r="M44" s="77">
+        <f>IFERROR(IF(L44="","",L44/12),"")</f>
+        <v/>
+      </c>
+      <c r="N44" s="72" t="n"/>
+      <c r="O44" s="81" t="n"/>
+      <c r="P44" s="79">
         <f>IFERROR(IF(G44="","",G44-365),"")</f>
         <v/>
       </c>
-      <c r="P44" s="72" t="n"/>
       <c r="Q44" s="72" t="n"/>
     </row>
     <row r="45">
@@ -5550,22 +5550,22 @@
       <c r="G45" s="70" t="n"/>
       <c r="H45" s="69" t="n"/>
       <c r="I45" s="69" t="n"/>
-      <c r="J45" s="65">
+      <c r="J45" s="69" t="n"/>
+      <c r="K45" s="65">
         <f>IFERROR(DATEDIF(F45,G45,"M"),"")</f>
         <v/>
       </c>
-      <c r="K45" s="71" t="n"/>
-      <c r="L45" s="77">
-        <f>IFERROR(IF(K45="","",K45/12),"")</f>
-        <v/>
-      </c>
-      <c r="M45" s="69" t="n"/>
-      <c r="N45" s="80" t="n"/>
-      <c r="O45" s="79">
+      <c r="L45" s="71" t="n"/>
+      <c r="M45" s="77">
+        <f>IFERROR(IF(L45="","",L45/12),"")</f>
+        <v/>
+      </c>
+      <c r="N45" s="69" t="n"/>
+      <c r="O45" s="80" t="n"/>
+      <c r="P45" s="79">
         <f>IFERROR(IF(G45="","",G45-365),"")</f>
         <v/>
       </c>
-      <c r="P45" s="69" t="n"/>
       <c r="Q45" s="69" t="n"/>
     </row>
     <row r="46">
@@ -5578,22 +5578,22 @@
       <c r="G46" s="73" t="n"/>
       <c r="H46" s="72" t="n"/>
       <c r="I46" s="72" t="n"/>
-      <c r="J46" s="65">
+      <c r="J46" s="72" t="n"/>
+      <c r="K46" s="65">
         <f>IFERROR(DATEDIF(F46,G46,"M"),"")</f>
         <v/>
       </c>
-      <c r="K46" s="74" t="n"/>
-      <c r="L46" s="77">
-        <f>IFERROR(IF(K46="","",K46/12),"")</f>
-        <v/>
-      </c>
-      <c r="M46" s="72" t="n"/>
-      <c r="N46" s="81" t="n"/>
-      <c r="O46" s="79">
+      <c r="L46" s="74" t="n"/>
+      <c r="M46" s="77">
+        <f>IFERROR(IF(L46="","",L46/12),"")</f>
+        <v/>
+      </c>
+      <c r="N46" s="72" t="n"/>
+      <c r="O46" s="81" t="n"/>
+      <c r="P46" s="79">
         <f>IFERROR(IF(G46="","",G46-365),"")</f>
         <v/>
       </c>
-      <c r="P46" s="72" t="n"/>
       <c r="Q46" s="72" t="n"/>
     </row>
     <row r="47">
@@ -5606,22 +5606,22 @@
       <c r="G47" s="70" t="n"/>
       <c r="H47" s="69" t="n"/>
       <c r="I47" s="69" t="n"/>
-      <c r="J47" s="65">
+      <c r="J47" s="69" t="n"/>
+      <c r="K47" s="65">
         <f>IFERROR(DATEDIF(F47,G47,"M"),"")</f>
         <v/>
       </c>
-      <c r="K47" s="71" t="n"/>
-      <c r="L47" s="77">
-        <f>IFERROR(IF(K47="","",K47/12),"")</f>
-        <v/>
-      </c>
-      <c r="M47" s="69" t="n"/>
-      <c r="N47" s="80" t="n"/>
-      <c r="O47" s="79">
+      <c r="L47" s="71" t="n"/>
+      <c r="M47" s="77">
+        <f>IFERROR(IF(L47="","",L47/12),"")</f>
+        <v/>
+      </c>
+      <c r="N47" s="69" t="n"/>
+      <c r="O47" s="80" t="n"/>
+      <c r="P47" s="79">
         <f>IFERROR(IF(G47="","",G47-365),"")</f>
         <v/>
       </c>
-      <c r="P47" s="69" t="n"/>
       <c r="Q47" s="69" t="n"/>
     </row>
     <row r="48">
@@ -5634,22 +5634,22 @@
       <c r="G48" s="73" t="n"/>
       <c r="H48" s="72" t="n"/>
       <c r="I48" s="72" t="n"/>
-      <c r="J48" s="65">
+      <c r="J48" s="72" t="n"/>
+      <c r="K48" s="65">
         <f>IFERROR(DATEDIF(F48,G48,"M"),"")</f>
         <v/>
       </c>
-      <c r="K48" s="74" t="n"/>
-      <c r="L48" s="77">
-        <f>IFERROR(IF(K48="","",K48/12),"")</f>
-        <v/>
-      </c>
-      <c r="M48" s="72" t="n"/>
-      <c r="N48" s="81" t="n"/>
-      <c r="O48" s="79">
+      <c r="L48" s="74" t="n"/>
+      <c r="M48" s="77">
+        <f>IFERROR(IF(L48="","",L48/12),"")</f>
+        <v/>
+      </c>
+      <c r="N48" s="72" t="n"/>
+      <c r="O48" s="81" t="n"/>
+      <c r="P48" s="79">
         <f>IFERROR(IF(G48="","",G48-365),"")</f>
         <v/>
       </c>
-      <c r="P48" s="72" t="n"/>
       <c r="Q48" s="72" t="n"/>
     </row>
     <row r="49">
@@ -5662,22 +5662,22 @@
       <c r="G49" s="70" t="n"/>
       <c r="H49" s="69" t="n"/>
       <c r="I49" s="69" t="n"/>
-      <c r="J49" s="65">
+      <c r="J49" s="69" t="n"/>
+      <c r="K49" s="65">
         <f>IFERROR(DATEDIF(F49,G49,"M"),"")</f>
         <v/>
       </c>
-      <c r="K49" s="71" t="n"/>
-      <c r="L49" s="77">
-        <f>IFERROR(IF(K49="","",K49/12),"")</f>
-        <v/>
-      </c>
-      <c r="M49" s="69" t="n"/>
-      <c r="N49" s="80" t="n"/>
-      <c r="O49" s="79">
+      <c r="L49" s="71" t="n"/>
+      <c r="M49" s="77">
+        <f>IFERROR(IF(L49="","",L49/12),"")</f>
+        <v/>
+      </c>
+      <c r="N49" s="69" t="n"/>
+      <c r="O49" s="80" t="n"/>
+      <c r="P49" s="79">
         <f>IFERROR(IF(G49="","",G49-365),"")</f>
         <v/>
       </c>
-      <c r="P49" s="69" t="n"/>
       <c r="Q49" s="69" t="n"/>
     </row>
     <row r="50">
@@ -5690,22 +5690,22 @@
       <c r="G50" s="73" t="n"/>
       <c r="H50" s="72" t="n"/>
       <c r="I50" s="72" t="n"/>
-      <c r="J50" s="65">
+      <c r="J50" s="72" t="n"/>
+      <c r="K50" s="65">
         <f>IFERROR(DATEDIF(F50,G50,"M"),"")</f>
         <v/>
       </c>
-      <c r="K50" s="74" t="n"/>
-      <c r="L50" s="77">
-        <f>IFERROR(IF(K50="","",K50/12),"")</f>
-        <v/>
-      </c>
-      <c r="M50" s="72" t="n"/>
-      <c r="N50" s="81" t="n"/>
-      <c r="O50" s="79">
+      <c r="L50" s="74" t="n"/>
+      <c r="M50" s="77">
+        <f>IFERROR(IF(L50="","",L50/12),"")</f>
+        <v/>
+      </c>
+      <c r="N50" s="72" t="n"/>
+      <c r="O50" s="81" t="n"/>
+      <c r="P50" s="79">
         <f>IFERROR(IF(G50="","",G50-365),"")</f>
         <v/>
       </c>
-      <c r="P50" s="72" t="n"/>
       <c r="Q50" s="72" t="n"/>
     </row>
     <row r="51">
@@ -5718,22 +5718,22 @@
       <c r="G51" s="70" t="n"/>
       <c r="H51" s="69" t="n"/>
       <c r="I51" s="69" t="n"/>
-      <c r="J51" s="65">
+      <c r="J51" s="69" t="n"/>
+      <c r="K51" s="65">
         <f>IFERROR(DATEDIF(F51,G51,"M"),"")</f>
         <v/>
       </c>
-      <c r="K51" s="71" t="n"/>
-      <c r="L51" s="77">
-        <f>IFERROR(IF(K51="","",K51/12),"")</f>
-        <v/>
-      </c>
-      <c r="M51" s="69" t="n"/>
-      <c r="N51" s="80" t="n"/>
-      <c r="O51" s="79">
+      <c r="L51" s="71" t="n"/>
+      <c r="M51" s="77">
+        <f>IFERROR(IF(L51="","",L51/12),"")</f>
+        <v/>
+      </c>
+      <c r="N51" s="69" t="n"/>
+      <c r="O51" s="80" t="n"/>
+      <c r="P51" s="79">
         <f>IFERROR(IF(G51="","",G51-365),"")</f>
         <v/>
       </c>
-      <c r="P51" s="69" t="n"/>
       <c r="Q51" s="69" t="n"/>
     </row>
     <row r="52">
@@ -5746,22 +5746,22 @@
       <c r="G52" s="73" t="n"/>
       <c r="H52" s="72" t="n"/>
       <c r="I52" s="72" t="n"/>
-      <c r="J52" s="65">
+      <c r="J52" s="72" t="n"/>
+      <c r="K52" s="65">
         <f>IFERROR(DATEDIF(F52,G52,"M"),"")</f>
         <v/>
       </c>
-      <c r="K52" s="74" t="n"/>
-      <c r="L52" s="77">
-        <f>IFERROR(IF(K52="","",K52/12),"")</f>
-        <v/>
-      </c>
-      <c r="M52" s="72" t="n"/>
-      <c r="N52" s="81" t="n"/>
-      <c r="O52" s="79">
+      <c r="L52" s="74" t="n"/>
+      <c r="M52" s="77">
+        <f>IFERROR(IF(L52="","",L52/12),"")</f>
+        <v/>
+      </c>
+      <c r="N52" s="72" t="n"/>
+      <c r="O52" s="81" t="n"/>
+      <c r="P52" s="79">
         <f>IFERROR(IF(G52="","",G52-365),"")</f>
         <v/>
       </c>
-      <c r="P52" s="72" t="n"/>
       <c r="Q52" s="72" t="n"/>
     </row>
     <row r="53">
@@ -5774,22 +5774,22 @@
       <c r="G53" s="70" t="n"/>
       <c r="H53" s="69" t="n"/>
       <c r="I53" s="69" t="n"/>
-      <c r="J53" s="65">
+      <c r="J53" s="69" t="n"/>
+      <c r="K53" s="65">
         <f>IFERROR(DATEDIF(F53,G53,"M"),"")</f>
         <v/>
       </c>
-      <c r="K53" s="71" t="n"/>
-      <c r="L53" s="77">
-        <f>IFERROR(IF(K53="","",K53/12),"")</f>
-        <v/>
-      </c>
-      <c r="M53" s="69" t="n"/>
-      <c r="N53" s="80" t="n"/>
-      <c r="O53" s="79">
+      <c r="L53" s="71" t="n"/>
+      <c r="M53" s="77">
+        <f>IFERROR(IF(L53="","",L53/12),"")</f>
+        <v/>
+      </c>
+      <c r="N53" s="69" t="n"/>
+      <c r="O53" s="80" t="n"/>
+      <c r="P53" s="79">
         <f>IFERROR(IF(G53="","",G53-365),"")</f>
         <v/>
       </c>
-      <c r="P53" s="69" t="n"/>
       <c r="Q53" s="69" t="n"/>
     </row>
   </sheetData>
@@ -5806,7 +5806,7 @@
     <dataValidation sqref="H4:H53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>LOOKUP!$B$28:$B$29</formula1>
     </dataValidation>
-    <dataValidation sqref="M4:M53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N4:N53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>LOOKUP!$B$18:$B$22</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Added ROOMS occupancy and tenant lookup formulas
</commit_message>
<xml_diff>
--- a/Tenant_Manager.xlsx
+++ b/Tenant_Manager.xlsx
@@ -4144,6 +4144,18 @@
           <t>RM-01</t>
         </is>
       </c>
+      <c r="C2">
+        <f>IFERROR(INDEX(TENANTS!$B$4:$B$53,MATCH(A2,TENANTS!$F$4:$F$53,0)),"Vacant")</f>
+        <v/>
+      </c>
+      <c r="D2">
+        <f>IFERROR(INDEX(TENANTS!$L$4:$L$53,MATCH(A2,TENANTS!$F$4:$F$53,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>IF(C2="Vacant","Vacant","Occupied")</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4151,6 +4163,18 @@
           <t>RM-02</t>
         </is>
       </c>
+      <c r="C3">
+        <f>IFERROR(INDEX(TENANTS!$B$4:$B$53,MATCH(A3,TENANTS!$F$4:$F$53,0)),"Vacant")</f>
+        <v/>
+      </c>
+      <c r="D3">
+        <f>IFERROR(INDEX(TENANTS!$L$4:$L$53,MATCH(A3,TENANTS!$F$4:$F$53,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>IF(C3="Vacant","Vacant","Occupied")</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4158,6 +4182,18 @@
           <t>RM-03</t>
         </is>
       </c>
+      <c r="C4">
+        <f>IFERROR(INDEX(TENANTS!$B$4:$B$53,MATCH(A4,TENANTS!$F$4:$F$53,0)),"Vacant")</f>
+        <v/>
+      </c>
+      <c r="D4">
+        <f>IFERROR(INDEX(TENANTS!$L$4:$L$53,MATCH(A4,TENANTS!$F$4:$F$53,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>IF(C4="Vacant","Vacant","Occupied")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4165,6 +4201,18 @@
           <t>RM-04</t>
         </is>
       </c>
+      <c r="C5">
+        <f>IFERROR(INDEX(TENANTS!$B$4:$B$53,MATCH(A5,TENANTS!$F$4:$F$53,0)),"Vacant")</f>
+        <v/>
+      </c>
+      <c r="D5">
+        <f>IFERROR(INDEX(TENANTS!$L$4:$L$53,MATCH(A5,TENANTS!$F$4:$F$53,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>IF(C5="Vacant","Vacant","Occupied")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4172,6 +4220,18 @@
           <t>RM-05</t>
         </is>
       </c>
+      <c r="C6">
+        <f>IFERROR(INDEX(TENANTS!$B$4:$B$53,MATCH(A6,TENANTS!$F$4:$F$53,0)),"Vacant")</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>IFERROR(INDEX(TENANTS!$L$4:$L$53,MATCH(A6,TENANTS!$F$4:$F$53,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>IF(C6="Vacant","Vacant","Occupied")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4179,6 +4239,18 @@
           <t>RM-06</t>
         </is>
       </c>
+      <c r="C7">
+        <f>IFERROR(INDEX(TENANTS!$B$4:$B$53,MATCH(A7,TENANTS!$F$4:$F$53,0)),"Vacant")</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>IFERROR(INDEX(TENANTS!$L$4:$L$53,MATCH(A7,TENANTS!$F$4:$F$53,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>IF(C7="Vacant","Vacant","Occupied")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4186,6 +4258,18 @@
           <t>RM-07</t>
         </is>
       </c>
+      <c r="C8">
+        <f>IFERROR(INDEX(TENANTS!$B$4:$B$53,MATCH(A8,TENANTS!$F$4:$F$53,0)),"Vacant")</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IFERROR(INDEX(TENANTS!$L$4:$L$53,MATCH(A8,TENANTS!$F$4:$F$53,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IF(C8="Vacant","Vacant","Occupied")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4193,6 +4277,18 @@
           <t>RM-08</t>
         </is>
       </c>
+      <c r="C9">
+        <f>IFERROR(INDEX(TENANTS!$B$4:$B$53,MATCH(A9,TENANTS!$F$4:$F$53,0)),"Vacant")</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>IFERROR(INDEX(TENANTS!$L$4:$L$53,MATCH(A9,TENANTS!$F$4:$F$53,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>IF(C9="Vacant","Vacant","Occupied")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4200,6 +4296,18 @@
           <t>RM-09</t>
         </is>
       </c>
+      <c r="C10">
+        <f>IFERROR(INDEX(TENANTS!$B$4:$B$53,MATCH(A10,TENANTS!$F$4:$F$53,0)),"Vacant")</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>IFERROR(INDEX(TENANTS!$L$4:$L$53,MATCH(A10,TENANTS!$F$4:$F$53,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>IF(C10="Vacant","Vacant","Occupied")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4207,6 +4315,18 @@
           <t>RM-10</t>
         </is>
       </c>
+      <c r="C11">
+        <f>IFERROR(INDEX(TENANTS!$B$4:$B$53,MATCH(A11,TENANTS!$F$4:$F$53,0)),"Vacant")</f>
+        <v/>
+      </c>
+      <c r="D11">
+        <f>IFERROR(INDEX(TENANTS!$L$4:$L$53,MATCH(A11,TENANTS!$F$4:$F$53,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>IF(C11="Vacant","Vacant","Occupied")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4214,6 +4334,18 @@
           <t>RM-11</t>
         </is>
       </c>
+      <c r="C12">
+        <f>IFERROR(INDEX(TENANTS!$B$4:$B$53,MATCH(A12,TENANTS!$F$4:$F$53,0)),"Vacant")</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>IFERROR(INDEX(TENANTS!$L$4:$L$53,MATCH(A12,TENANTS!$F$4:$F$53,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>IF(C12="Vacant","Vacant","Occupied")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4221,8 +4353,28 @@
           <t>RM-12</t>
         </is>
       </c>
+      <c r="C13">
+        <f>IFERROR(INDEX(TENANTS!$B$4:$B$53,MATCH(A13,TENANTS!$F$4:$F$53,0)),"Vacant")</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>IFERROR(INDEX(TENANTS!$L$4:$L$53,MATCH(A13,TENANTS!$F$4:$F$53,0)),"")</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>IF(C13="Vacant","Vacant","Occupied")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="E2:E13">
+    <cfRule type="expression" priority="1" dxfId="2">
+      <formula>=E2="Occupied"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>=E2="Vacant"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>